<commit_message>
Atualiza dashboards Aura - 2026-07-28 03:53:46
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixas_42l.xlsx
+++ b/relatorio_analitico_caixas_42l.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Caixa 42L" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Caixa 42L'!$A$1:$L$443</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Caixa 42L'!$A$1:$L$446</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L443"/>
+  <dimension ref="A1:L446"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -3740,7 +3740,7 @@
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
@@ -3988,7 +3988,7 @@
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
@@ -4608,7 +4608,7 @@
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
@@ -6034,7 +6034,7 @@
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D91" s="2" t="inlineStr">
@@ -6592,7 +6592,7 @@
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D100" s="2" t="inlineStr">
@@ -10436,7 +10436,7 @@
       </c>
       <c r="C162" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D162" s="2" t="inlineStr">
@@ -10560,7 +10560,7 @@
       </c>
       <c r="C164" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D164" s="2" t="inlineStr">
@@ -10622,7 +10622,7 @@
       </c>
       <c r="C165" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D165" s="2" t="inlineStr">
@@ -14342,7 +14342,7 @@
       </c>
       <c r="C225" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D225" s="2" t="inlineStr">
@@ -14404,7 +14404,7 @@
       </c>
       <c r="C226" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D226" s="2" t="inlineStr">
@@ -19302,7 +19302,7 @@
       </c>
       <c r="C305" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D305" s="2" t="inlineStr">
@@ -19674,27 +19674,27 @@
       </c>
       <c r="C311" s="2" t="inlineStr">
         <is>
-          <t>-90 C a -60 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D311" s="2" t="inlineStr">
         <is>
-          <t>557493</t>
+          <t>562261</t>
         </is>
       </c>
       <c r="E311" s="2" t="inlineStr">
         <is>
-          <t>RN</t>
+          <t>RJ</t>
         </is>
       </c>
       <c r="F311" s="2" t="inlineStr">
         <is>
-          <t>AS-0511</t>
+          <t>A3676</t>
         </is>
       </c>
       <c r="G311" s="2" t="inlineStr">
         <is>
-          <t>00019200000013252739</t>
+          <t>00019200000013778277</t>
         </is>
       </c>
       <c r="H311" s="2" t="inlineStr">
@@ -19704,22 +19704,22 @@
       </c>
       <c r="I311" s="2" t="inlineStr">
         <is>
-          <t>01/07/2026 01:19</t>
+          <t>28/07/2026 03:41</t>
         </is>
       </c>
       <c r="J311" s="2" t="inlineStr">
         <is>
-          <t>03/07/2026 15:30</t>
+          <t>-</t>
         </is>
       </c>
       <c r="K311" s="2" t="inlineStr">
         <is>
-          <t>01/07/2026 01:19</t>
+          <t>28/07/2026 03:41</t>
         </is>
       </c>
       <c r="L311" s="2" t="inlineStr">
         <is>
-          <t>03/07/2026 15:30</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -19736,27 +19736,27 @@
       </c>
       <c r="C312" s="2" t="inlineStr">
         <is>
-          <t>-90 C a -60 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D312" s="2" t="inlineStr">
         <is>
-          <t>557493</t>
+          <t>562261</t>
         </is>
       </c>
       <c r="E312" s="2" t="inlineStr">
         <is>
-          <t>RN</t>
+          <t>RJ</t>
         </is>
       </c>
       <c r="F312" s="2" t="inlineStr">
         <is>
-          <t>AS-0615</t>
+          <t>A8624</t>
         </is>
       </c>
       <c r="G312" s="2" t="inlineStr">
         <is>
-          <t>00019200000013252747</t>
+          <t>00019200000013778285</t>
         </is>
       </c>
       <c r="H312" s="2" t="inlineStr">
@@ -19766,22 +19766,22 @@
       </c>
       <c r="I312" s="2" t="inlineStr">
         <is>
-          <t>01/07/2026 01:19</t>
+          <t>28/07/2026 03:41</t>
         </is>
       </c>
       <c r="J312" s="2" t="inlineStr">
         <is>
-          <t>03/07/2026 15:30</t>
+          <t>-</t>
         </is>
       </c>
       <c r="K312" s="2" t="inlineStr">
         <is>
-          <t>01/07/2026 01:19</t>
+          <t>28/07/2026 03:41</t>
         </is>
       </c>
       <c r="L312" s="2" t="inlineStr">
         <is>
-          <t>03/07/2026 15:30</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -19813,12 +19813,12 @@
       </c>
       <c r="F313" s="2" t="inlineStr">
         <is>
-          <t>AS-0425</t>
+          <t>AS-0511</t>
         </is>
       </c>
       <c r="G313" s="2" t="inlineStr">
         <is>
-          <t>00019200000013252755</t>
+          <t>00019200000013252739</t>
         </is>
       </c>
       <c r="H313" s="2" t="inlineStr">
@@ -19875,12 +19875,12 @@
       </c>
       <c r="F314" s="2" t="inlineStr">
         <is>
-          <t>AS-0138</t>
+          <t>AS-0615</t>
         </is>
       </c>
       <c r="G314" s="2" t="inlineStr">
         <is>
-          <t>00019200000013252763</t>
+          <t>00019200000013252747</t>
         </is>
       </c>
       <c r="H314" s="2" t="inlineStr">
@@ -19937,12 +19937,12 @@
       </c>
       <c r="F315" s="2" t="inlineStr">
         <is>
-          <t>AS-0245</t>
+          <t>AS-0425</t>
         </is>
       </c>
       <c r="G315" s="2" t="inlineStr">
         <is>
-          <t>00019200000013252771</t>
+          <t>00019200000013252755</t>
         </is>
       </c>
       <c r="H315" s="2" t="inlineStr">
@@ -19999,12 +19999,12 @@
       </c>
       <c r="F316" s="2" t="inlineStr">
         <is>
-          <t>AS-0762</t>
+          <t>AS-0138</t>
         </is>
       </c>
       <c r="G316" s="2" t="inlineStr">
         <is>
-          <t>00019200000013252780</t>
+          <t>00019200000013252763</t>
         </is>
       </c>
       <c r="H316" s="2" t="inlineStr">
@@ -20061,12 +20061,12 @@
       </c>
       <c r="F317" s="2" t="inlineStr">
         <is>
-          <t>AS-0462</t>
+          <t>AS-0245</t>
         </is>
       </c>
       <c r="G317" s="2" t="inlineStr">
         <is>
-          <t>00019200000013252798</t>
+          <t>00019200000013252771</t>
         </is>
       </c>
       <c r="H317" s="2" t="inlineStr">
@@ -20123,12 +20123,12 @@
       </c>
       <c r="F318" s="2" t="inlineStr">
         <is>
-          <t>AS-0702</t>
+          <t>AS-0762</t>
         </is>
       </c>
       <c r="G318" s="2" t="inlineStr">
         <is>
-          <t>00019200000013252801</t>
+          <t>00019200000013252780</t>
         </is>
       </c>
       <c r="H318" s="2" t="inlineStr">
@@ -20185,12 +20185,12 @@
       </c>
       <c r="F319" s="2" t="inlineStr">
         <is>
-          <t>AS-0513</t>
+          <t>AS-0462</t>
         </is>
       </c>
       <c r="G319" s="2" t="inlineStr">
         <is>
-          <t>00019200000013254510</t>
+          <t>00019200000013252798</t>
         </is>
       </c>
       <c r="H319" s="2" t="inlineStr">
@@ -20247,12 +20247,12 @@
       </c>
       <c r="F320" s="2" t="inlineStr">
         <is>
-          <t>AS-0172</t>
+          <t>AS-0702</t>
         </is>
       </c>
       <c r="G320" s="2" t="inlineStr">
         <is>
-          <t>00019200000013254529</t>
+          <t>00019200000013252801</t>
         </is>
       </c>
       <c r="H320" s="2" t="inlineStr">
@@ -20309,12 +20309,12 @@
       </c>
       <c r="F321" s="2" t="inlineStr">
         <is>
-          <t>AS-0019</t>
+          <t>AS-0513</t>
         </is>
       </c>
       <c r="G321" s="2" t="inlineStr">
         <is>
-          <t>00019200000013429450</t>
+          <t>00019200000013254510</t>
         </is>
       </c>
       <c r="H321" s="2" t="inlineStr">
@@ -20371,12 +20371,12 @@
       </c>
       <c r="F322" s="2" t="inlineStr">
         <is>
-          <t>AS-0426</t>
+          <t>AS-0172</t>
         </is>
       </c>
       <c r="G322" s="2" t="inlineStr">
         <is>
-          <t>00019200000013429469</t>
+          <t>00019200000013254529</t>
         </is>
       </c>
       <c r="H322" s="2" t="inlineStr">
@@ -20433,12 +20433,12 @@
       </c>
       <c r="F323" s="2" t="inlineStr">
         <is>
-          <t>AS-0699</t>
+          <t>AS-0019</t>
         </is>
       </c>
       <c r="G323" s="2" t="inlineStr">
         <is>
-          <t>00019200000013429477</t>
+          <t>00019200000013429450</t>
         </is>
       </c>
       <c r="H323" s="2" t="inlineStr">
@@ -20495,12 +20495,12 @@
       </c>
       <c r="F324" s="2" t="inlineStr">
         <is>
-          <t>AS-0376</t>
+          <t>AS-0426</t>
         </is>
       </c>
       <c r="G324" s="2" t="inlineStr">
         <is>
-          <t>00019200000013429485</t>
+          <t>00019200000013429469</t>
         </is>
       </c>
       <c r="H324" s="2" t="inlineStr">
@@ -20557,12 +20557,12 @@
       </c>
       <c r="F325" s="2" t="inlineStr">
         <is>
-          <t>AS-0683</t>
+          <t>AS-0699</t>
         </is>
       </c>
       <c r="G325" s="2" t="inlineStr">
         <is>
-          <t>00019200000013429493</t>
+          <t>00019200000013429477</t>
         </is>
       </c>
       <c r="H325" s="2" t="inlineStr">
@@ -20619,12 +20619,12 @@
       </c>
       <c r="F326" s="2" t="inlineStr">
         <is>
-          <t>AS-0078</t>
+          <t>AS-0376</t>
         </is>
       </c>
       <c r="G326" s="2" t="inlineStr">
         <is>
-          <t>00019200000013429507</t>
+          <t>00019200000013429485</t>
         </is>
       </c>
       <c r="H326" s="2" t="inlineStr">
@@ -20681,12 +20681,12 @@
       </c>
       <c r="F327" s="2" t="inlineStr">
         <is>
-          <t>AS-0077</t>
+          <t>AS-0683</t>
         </is>
       </c>
       <c r="G327" s="2" t="inlineStr">
         <is>
-          <t>00019200000013429515</t>
+          <t>00019200000013429493</t>
         </is>
       </c>
       <c r="H327" s="2" t="inlineStr">
@@ -20743,12 +20743,12 @@
       </c>
       <c r="F328" s="2" t="inlineStr">
         <is>
-          <t>AS-0499</t>
+          <t>AS-0078</t>
         </is>
       </c>
       <c r="G328" s="2" t="inlineStr">
         <is>
-          <t>00019200000013429523</t>
+          <t>00019200000013429507</t>
         </is>
       </c>
       <c r="H328" s="2" t="inlineStr">
@@ -20805,12 +20805,12 @@
       </c>
       <c r="F329" s="2" t="inlineStr">
         <is>
-          <t>AS-0518</t>
+          <t>AS-0077</t>
         </is>
       </c>
       <c r="G329" s="2" t="inlineStr">
         <is>
-          <t>00019200000013429531</t>
+          <t>00019200000013429515</t>
         </is>
       </c>
       <c r="H329" s="2" t="inlineStr">
@@ -20867,12 +20867,12 @@
       </c>
       <c r="F330" s="2" t="inlineStr">
         <is>
-          <t>AS-0494</t>
+          <t>AS-0499</t>
         </is>
       </c>
       <c r="G330" s="2" t="inlineStr">
         <is>
-          <t>00019200000013429540</t>
+          <t>00019200000013429523</t>
         </is>
       </c>
       <c r="H330" s="2" t="inlineStr">
@@ -20929,12 +20929,12 @@
       </c>
       <c r="F331" s="2" t="inlineStr">
         <is>
-          <t>AS-0269</t>
+          <t>AS-0518</t>
         </is>
       </c>
       <c r="G331" s="2" t="inlineStr">
         <is>
-          <t>00019200000013429558</t>
+          <t>00019200000013429531</t>
         </is>
       </c>
       <c r="H331" s="2" t="inlineStr">
@@ -20991,12 +20991,12 @@
       </c>
       <c r="F332" s="2" t="inlineStr">
         <is>
-          <t>AS-0201</t>
+          <t>AS-0494</t>
         </is>
       </c>
       <c r="G332" s="2" t="inlineStr">
         <is>
-          <t>00019200000013429566</t>
+          <t>00019200000013429540</t>
         </is>
       </c>
       <c r="H332" s="2" t="inlineStr">
@@ -21038,12 +21038,12 @@
       </c>
       <c r="C333" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-90 C a -60 C</t>
         </is>
       </c>
       <c r="D333" s="2" t="inlineStr">
         <is>
-          <t>559981</t>
+          <t>557493</t>
         </is>
       </c>
       <c r="E333" s="2" t="inlineStr">
@@ -21053,12 +21053,12 @@
       </c>
       <c r="F333" s="2" t="inlineStr">
         <is>
-          <t>A6263</t>
+          <t>AS-0269</t>
         </is>
       </c>
       <c r="G333" s="2" t="inlineStr">
         <is>
-          <t>00019200000013419153</t>
+          <t>00019200000013429558</t>
         </is>
       </c>
       <c r="H333" s="2" t="inlineStr">
@@ -21068,22 +21068,22 @@
       </c>
       <c r="I333" s="2" t="inlineStr">
         <is>
-          <t>07/07/2026 05:52</t>
+          <t>01/07/2026 01:19</t>
         </is>
       </c>
       <c r="J333" s="2" t="inlineStr">
         <is>
-          <t>08/07/2026 17:32</t>
+          <t>03/07/2026 15:30</t>
         </is>
       </c>
       <c r="K333" s="2" t="inlineStr">
         <is>
-          <t>07/07/2026 05:52</t>
+          <t>01/07/2026 01:19</t>
         </is>
       </c>
       <c r="L333" s="2" t="inlineStr">
         <is>
-          <t>08/07/2026 17:32</t>
+          <t>03/07/2026 15:30</t>
         </is>
       </c>
     </row>
@@ -21105,7 +21105,7 @@
       </c>
       <c r="D334" s="2" t="inlineStr">
         <is>
-          <t>560570</t>
+          <t>557493</t>
         </is>
       </c>
       <c r="E334" s="2" t="inlineStr">
@@ -21115,12 +21115,12 @@
       </c>
       <c r="F334" s="2" t="inlineStr">
         <is>
-          <t>869170034877747</t>
+          <t>AS-0201</t>
         </is>
       </c>
       <c r="G334" s="2" t="inlineStr">
         <is>
-          <t>00019200000013776150</t>
+          <t>00019200000013429566</t>
         </is>
       </c>
       <c r="H334" s="2" t="inlineStr">
@@ -21130,22 +21130,22 @@
       </c>
       <c r="I334" s="2" t="inlineStr">
         <is>
-          <t>27/07/2026 22:34</t>
+          <t>01/07/2026 01:19</t>
         </is>
       </c>
       <c r="J334" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>03/07/2026 15:30</t>
         </is>
       </c>
       <c r="K334" s="2" t="inlineStr">
         <is>
-          <t>27/07/2026 22:34</t>
+          <t>01/07/2026 01:19</t>
         </is>
       </c>
       <c r="L334" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>03/07/2026 15:30</t>
         </is>
       </c>
     </row>
@@ -21162,12 +21162,12 @@
       </c>
       <c r="C335" s="2" t="inlineStr">
         <is>
-          <t>-90 C a -60 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D335" s="2" t="inlineStr">
         <is>
-          <t>560570</t>
+          <t>559981</t>
         </is>
       </c>
       <c r="E335" s="2" t="inlineStr">
@@ -21177,12 +21177,12 @@
       </c>
       <c r="F335" s="2" t="inlineStr">
         <is>
-          <t>300100</t>
+          <t>A6263</t>
         </is>
       </c>
       <c r="G335" s="2" t="inlineStr">
         <is>
-          <t>00019200000013776169</t>
+          <t>00019200000013419153</t>
         </is>
       </c>
       <c r="H335" s="2" t="inlineStr">
@@ -21192,22 +21192,22 @@
       </c>
       <c r="I335" s="2" t="inlineStr">
         <is>
-          <t>27/07/2026 22:34</t>
+          <t>07/07/2026 05:52</t>
         </is>
       </c>
       <c r="J335" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>08/07/2026 17:32</t>
         </is>
       </c>
       <c r="K335" s="2" t="inlineStr">
         <is>
-          <t>27/07/2026 22:34</t>
+          <t>07/07/2026 05:52</t>
         </is>
       </c>
       <c r="L335" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>08/07/2026 17:32</t>
         </is>
       </c>
     </row>
@@ -21239,12 +21239,12 @@
       </c>
       <c r="F336" s="2" t="inlineStr">
         <is>
-          <t>300054</t>
+          <t>869170034877747</t>
         </is>
       </c>
       <c r="G336" s="2" t="inlineStr">
         <is>
-          <t>00019200000013776177</t>
+          <t>00019200000013776150</t>
         </is>
       </c>
       <c r="H336" s="2" t="inlineStr">
@@ -21301,12 +21301,12 @@
       </c>
       <c r="F337" s="2" t="inlineStr">
         <is>
-          <t>300056</t>
+          <t>300100</t>
         </is>
       </c>
       <c r="G337" s="2" t="inlineStr">
         <is>
-          <t>00019200000013776185</t>
+          <t>00019200000013776169</t>
         </is>
       </c>
       <c r="H337" s="2" t="inlineStr">
@@ -21363,12 +21363,12 @@
       </c>
       <c r="F338" s="2" t="inlineStr">
         <is>
-          <t>300163</t>
+          <t>300054</t>
         </is>
       </c>
       <c r="G338" s="2" t="inlineStr">
         <is>
-          <t>00019200000013776193</t>
+          <t>00019200000013776177</t>
         </is>
       </c>
       <c r="H338" s="2" t="inlineStr">
@@ -21425,12 +21425,12 @@
       </c>
       <c r="F339" s="2" t="inlineStr">
         <is>
-          <t>300059</t>
+          <t>300056</t>
         </is>
       </c>
       <c r="G339" s="2" t="inlineStr">
         <is>
-          <t>00019200000013776207</t>
+          <t>00019200000013776185</t>
         </is>
       </c>
       <c r="H339" s="2" t="inlineStr">
@@ -21487,12 +21487,12 @@
       </c>
       <c r="F340" s="2" t="inlineStr">
         <is>
-          <t>869170035504837</t>
+          <t>300163</t>
         </is>
       </c>
       <c r="G340" s="2" t="inlineStr">
         <is>
-          <t>00019200000013776215</t>
+          <t>00019200000013776193</t>
         </is>
       </c>
       <c r="H340" s="2" t="inlineStr">
@@ -21549,12 +21549,12 @@
       </c>
       <c r="F341" s="2" t="inlineStr">
         <is>
-          <t>869170035520866</t>
+          <t>300059</t>
         </is>
       </c>
       <c r="G341" s="2" t="inlineStr">
         <is>
-          <t>00019200000013776223</t>
+          <t>00019200000013776207</t>
         </is>
       </c>
       <c r="H341" s="2" t="inlineStr">
@@ -21611,12 +21611,12 @@
       </c>
       <c r="F342" s="2" t="inlineStr">
         <is>
-          <t>869170035517771</t>
+          <t>869170035504837</t>
         </is>
       </c>
       <c r="G342" s="2" t="inlineStr">
         <is>
-          <t>00019200000013776231</t>
+          <t>00019200000013776215</t>
         </is>
       </c>
       <c r="H342" s="2" t="inlineStr">
@@ -21673,12 +21673,12 @@
       </c>
       <c r="F343" s="2" t="inlineStr">
         <is>
-          <t>869170034881269</t>
+          <t>869170035520866</t>
         </is>
       </c>
       <c r="G343" s="2" t="inlineStr">
         <is>
-          <t>00019200000013776240</t>
+          <t>00019200000013776223</t>
         </is>
       </c>
       <c r="H343" s="2" t="inlineStr">
@@ -21735,12 +21735,12 @@
       </c>
       <c r="F344" s="2" t="inlineStr">
         <is>
-          <t>869170034876806</t>
+          <t>869170035517771</t>
         </is>
       </c>
       <c r="G344" s="2" t="inlineStr">
         <is>
-          <t>00019200000013776258</t>
+          <t>00019200000013776231</t>
         </is>
       </c>
       <c r="H344" s="2" t="inlineStr">
@@ -21797,12 +21797,12 @@
       </c>
       <c r="F345" s="2" t="inlineStr">
         <is>
-          <t>AS-0213</t>
+          <t>869170034881269</t>
         </is>
       </c>
       <c r="G345" s="2" t="inlineStr">
         <is>
-          <t>00019200000013776266</t>
+          <t>00019200000013776240</t>
         </is>
       </c>
       <c r="H345" s="2" t="inlineStr">
@@ -21859,12 +21859,12 @@
       </c>
       <c r="F346" s="2" t="inlineStr">
         <is>
-          <t>300027</t>
+          <t>869170034876806</t>
         </is>
       </c>
       <c r="G346" s="2" t="inlineStr">
         <is>
-          <t>00019200000013776274</t>
+          <t>00019200000013776258</t>
         </is>
       </c>
       <c r="H346" s="2" t="inlineStr">
@@ -21921,12 +21921,12 @@
       </c>
       <c r="F347" s="2" t="inlineStr">
         <is>
-          <t>300173</t>
+          <t>AS-0213</t>
         </is>
       </c>
       <c r="G347" s="2" t="inlineStr">
         <is>
-          <t>00019200000013776282</t>
+          <t>00019200000013776266</t>
         </is>
       </c>
       <c r="H347" s="2" t="inlineStr">
@@ -21983,12 +21983,12 @@
       </c>
       <c r="F348" s="2" t="inlineStr">
         <is>
-          <t>300181</t>
+          <t>300027</t>
         </is>
       </c>
       <c r="G348" s="2" t="inlineStr">
         <is>
-          <t>00019200000013776290</t>
+          <t>00019200000013776274</t>
         </is>
       </c>
       <c r="H348" s="2" t="inlineStr">
@@ -22030,27 +22030,27 @@
       </c>
       <c r="C349" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-90 C a -60 C</t>
         </is>
       </c>
       <c r="D349" s="2" t="inlineStr">
         <is>
-          <t>559957</t>
+          <t>560570</t>
         </is>
       </c>
       <c r="E349" s="2" t="inlineStr">
         <is>
-          <t>RO</t>
+          <t>RN</t>
         </is>
       </c>
       <c r="F349" s="2" t="inlineStr">
         <is>
-          <t>A9354</t>
+          <t>300173</t>
         </is>
       </c>
       <c r="G349" s="2" t="inlineStr">
         <is>
-          <t>00019200000013418211</t>
+          <t>00019200000013776282</t>
         </is>
       </c>
       <c r="H349" s="2" t="inlineStr">
@@ -22060,22 +22060,22 @@
       </c>
       <c r="I349" s="2" t="inlineStr">
         <is>
-          <t>07/07/2026 01:00</t>
+          <t>27/07/2026 22:34</t>
         </is>
       </c>
       <c r="J349" s="2" t="inlineStr">
         <is>
-          <t>08/07/2026 18:00</t>
+          <t>-</t>
         </is>
       </c>
       <c r="K349" s="2" t="inlineStr">
         <is>
-          <t>07/07/2026 01:00</t>
+          <t>27/07/2026 22:34</t>
         </is>
       </c>
       <c r="L349" s="2" t="inlineStr">
         <is>
-          <t>08/07/2026 18:00</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -22092,27 +22092,27 @@
       </c>
       <c r="C350" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-90 C a -60 C</t>
         </is>
       </c>
       <c r="D350" s="2" t="inlineStr">
         <is>
-          <t>559957</t>
+          <t>560570</t>
         </is>
       </c>
       <c r="E350" s="2" t="inlineStr">
         <is>
-          <t>RO</t>
+          <t>RN</t>
         </is>
       </c>
       <c r="F350" s="2" t="inlineStr">
         <is>
-          <t>A3754</t>
+          <t>300181</t>
         </is>
       </c>
       <c r="G350" s="2" t="inlineStr">
         <is>
-          <t>00019200000013418220</t>
+          <t>00019200000013776290</t>
         </is>
       </c>
       <c r="H350" s="2" t="inlineStr">
@@ -22122,22 +22122,22 @@
       </c>
       <c r="I350" s="2" t="inlineStr">
         <is>
-          <t>07/07/2026 01:00</t>
+          <t>27/07/2026 22:34</t>
         </is>
       </c>
       <c r="J350" s="2" t="inlineStr">
         <is>
-          <t>08/07/2026 18:00</t>
+          <t>-</t>
         </is>
       </c>
       <c r="K350" s="2" t="inlineStr">
         <is>
-          <t>07/07/2026 01:00</t>
+          <t>27/07/2026 22:34</t>
         </is>
       </c>
       <c r="L350" s="2" t="inlineStr">
         <is>
-          <t>08/07/2026 18:00</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -22154,12 +22154,12 @@
       </c>
       <c r="C351" s="2" t="inlineStr">
         <is>
-          <t>-90 C a -60 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D351" s="2" t="inlineStr">
         <is>
-          <t>560527</t>
+          <t>559957</t>
         </is>
       </c>
       <c r="E351" s="2" t="inlineStr">
@@ -22169,12 +22169,12 @@
       </c>
       <c r="F351" s="2" t="inlineStr">
         <is>
-          <t>869170035519140</t>
+          <t>A9354</t>
         </is>
       </c>
       <c r="G351" s="2" t="inlineStr">
         <is>
-          <t>00019200000013778544</t>
+          <t>00019200000013418211</t>
         </is>
       </c>
       <c r="H351" s="2" t="inlineStr">
@@ -22184,22 +22184,22 @@
       </c>
       <c r="I351" s="2" t="inlineStr">
         <is>
-          <t>27/07/2026 22:33</t>
+          <t>07/07/2026 01:00</t>
         </is>
       </c>
       <c r="J351" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>08/07/2026 18:00</t>
         </is>
       </c>
       <c r="K351" s="2" t="inlineStr">
         <is>
-          <t>27/07/2026 22:33</t>
+          <t>07/07/2026 01:00</t>
         </is>
       </c>
       <c r="L351" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>08/07/2026 18:00</t>
         </is>
       </c>
     </row>
@@ -22216,12 +22216,12 @@
       </c>
       <c r="C352" s="2" t="inlineStr">
         <is>
-          <t>-90 C a -60 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D352" s="2" t="inlineStr">
         <is>
-          <t>560576</t>
+          <t>559957</t>
         </is>
       </c>
       <c r="E352" s="2" t="inlineStr">
@@ -22231,12 +22231,12 @@
       </c>
       <c r="F352" s="2" t="inlineStr">
         <is>
-          <t>V5561022</t>
+          <t>A3754</t>
         </is>
       </c>
       <c r="G352" s="2" t="inlineStr">
         <is>
-          <t>00019200000013471686</t>
+          <t>00019200000013418220</t>
         </is>
       </c>
       <c r="H352" s="2" t="inlineStr">
@@ -22246,22 +22246,22 @@
       </c>
       <c r="I352" s="2" t="inlineStr">
         <is>
-          <t>19/07/2026 23:45</t>
+          <t>07/07/2026 01:00</t>
         </is>
       </c>
       <c r="J352" s="2" t="inlineStr">
         <is>
-          <t>21/07/2026 17:30</t>
+          <t>08/07/2026 18:00</t>
         </is>
       </c>
       <c r="K352" s="2" t="inlineStr">
         <is>
-          <t>19/07/2026 23:45</t>
+          <t>07/07/2026 01:00</t>
         </is>
       </c>
       <c r="L352" s="2" t="inlineStr">
         <is>
-          <t>21/07/2026 17:30</t>
+          <t>08/07/2026 18:00</t>
         </is>
       </c>
     </row>
@@ -22283,7 +22283,7 @@
       </c>
       <c r="D353" s="2" t="inlineStr">
         <is>
-          <t>560576</t>
+          <t>560527</t>
         </is>
       </c>
       <c r="E353" s="2" t="inlineStr">
@@ -22293,12 +22293,12 @@
       </c>
       <c r="F353" s="2" t="inlineStr">
         <is>
-          <t>V56M3023</t>
+          <t>869170035519140</t>
         </is>
       </c>
       <c r="G353" s="2" t="inlineStr">
         <is>
-          <t>00019200000013471694</t>
+          <t>00019200000013778544</t>
         </is>
       </c>
       <c r="H353" s="2" t="inlineStr">
@@ -22308,22 +22308,22 @@
       </c>
       <c r="I353" s="2" t="inlineStr">
         <is>
-          <t>19/07/2026 23:45</t>
+          <t>27/07/2026 22:33</t>
         </is>
       </c>
       <c r="J353" s="2" t="inlineStr">
         <is>
-          <t>21/07/2026 17:30</t>
+          <t>-</t>
         </is>
       </c>
       <c r="K353" s="2" t="inlineStr">
         <is>
-          <t>19/07/2026 23:45</t>
+          <t>27/07/2026 22:33</t>
         </is>
       </c>
       <c r="L353" s="2" t="inlineStr">
         <is>
-          <t>21/07/2026 17:30</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -22355,12 +22355,12 @@
       </c>
       <c r="F354" s="2" t="inlineStr">
         <is>
-          <t>V56M300F</t>
+          <t>V5561022</t>
         </is>
       </c>
       <c r="G354" s="2" t="inlineStr">
         <is>
-          <t>00019200000013471708</t>
+          <t>00019200000013471686</t>
         </is>
       </c>
       <c r="H354" s="2" t="inlineStr">
@@ -22417,12 +22417,12 @@
       </c>
       <c r="F355" s="2" t="inlineStr">
         <is>
-          <t>V54101A9</t>
+          <t>V56M3023</t>
         </is>
       </c>
       <c r="G355" s="2" t="inlineStr">
         <is>
-          <t>00019200000013471716</t>
+          <t>00019200000013471694</t>
         </is>
       </c>
       <c r="H355" s="2" t="inlineStr">
@@ -22479,12 +22479,12 @@
       </c>
       <c r="F356" s="2" t="inlineStr">
         <is>
-          <t>V556101C</t>
+          <t>V56M300F</t>
         </is>
       </c>
       <c r="G356" s="2" t="inlineStr">
         <is>
-          <t>00019200000013471724</t>
+          <t>00019200000013471708</t>
         </is>
       </c>
       <c r="H356" s="2" t="inlineStr">
@@ -22541,12 +22541,12 @@
       </c>
       <c r="F357" s="2" t="inlineStr">
         <is>
-          <t>V56M3016</t>
+          <t>V54101A9</t>
         </is>
       </c>
       <c r="G357" s="2" t="inlineStr">
         <is>
-          <t>00019200000013471732</t>
+          <t>00019200000013471716</t>
         </is>
       </c>
       <c r="H357" s="2" t="inlineStr">
@@ -22603,12 +22603,12 @@
       </c>
       <c r="F358" s="2" t="inlineStr">
         <is>
-          <t>V54100A1</t>
+          <t>V556101C</t>
         </is>
       </c>
       <c r="G358" s="2" t="inlineStr">
         <is>
-          <t>00019200000013471740</t>
+          <t>00019200000013471724</t>
         </is>
       </c>
       <c r="H358" s="2" t="inlineStr">
@@ -22665,12 +22665,12 @@
       </c>
       <c r="F359" s="2" t="inlineStr">
         <is>
-          <t>V556102F</t>
+          <t>V56M3016</t>
         </is>
       </c>
       <c r="G359" s="2" t="inlineStr">
         <is>
-          <t>00019200000013471872</t>
+          <t>00019200000013471732</t>
         </is>
       </c>
       <c r="H359" s="2" t="inlineStr">
@@ -22727,12 +22727,12 @@
       </c>
       <c r="F360" s="2" t="inlineStr">
         <is>
-          <t>V5561002</t>
+          <t>V54100A1</t>
         </is>
       </c>
       <c r="G360" s="2" t="inlineStr">
         <is>
-          <t>00019200000013471880</t>
+          <t>00019200000013471740</t>
         </is>
       </c>
       <c r="H360" s="2" t="inlineStr">
@@ -22789,12 +22789,12 @@
       </c>
       <c r="F361" s="2" t="inlineStr">
         <is>
-          <t>V56M301E</t>
+          <t>V556102F</t>
         </is>
       </c>
       <c r="G361" s="2" t="inlineStr">
         <is>
-          <t>00019200000013471899</t>
+          <t>00019200000013471872</t>
         </is>
       </c>
       <c r="H361" s="2" t="inlineStr">
@@ -22851,12 +22851,12 @@
       </c>
       <c r="F362" s="2" t="inlineStr">
         <is>
-          <t>V5561015</t>
+          <t>V5561002</t>
         </is>
       </c>
       <c r="G362" s="2" t="inlineStr">
         <is>
-          <t>00019200000013475789</t>
+          <t>00019200000013471880</t>
         </is>
       </c>
       <c r="H362" s="2" t="inlineStr">
@@ -22913,12 +22913,12 @@
       </c>
       <c r="F363" s="2" t="inlineStr">
         <is>
-          <t>V5560004</t>
+          <t>V56M301E</t>
         </is>
       </c>
       <c r="G363" s="2" t="inlineStr">
         <is>
-          <t>00019200000013475797</t>
+          <t>00019200000013471899</t>
         </is>
       </c>
       <c r="H363" s="2" t="inlineStr">
@@ -22960,12 +22960,12 @@
       </c>
       <c r="C364" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-90 C a -60 C</t>
         </is>
       </c>
       <c r="D364" s="2" t="inlineStr">
         <is>
-          <t>561418</t>
+          <t>560576</t>
         </is>
       </c>
       <c r="E364" s="2" t="inlineStr">
@@ -22975,12 +22975,12 @@
       </c>
       <c r="F364" s="2" t="inlineStr">
         <is>
-          <t>A8179</t>
+          <t>V5561015</t>
         </is>
       </c>
       <c r="G364" s="2" t="inlineStr">
         <is>
-          <t>00019200000013472151</t>
+          <t>00019200000013475789</t>
         </is>
       </c>
       <c r="H364" s="2" t="inlineStr">
@@ -22990,22 +22990,22 @@
       </c>
       <c r="I364" s="2" t="inlineStr">
         <is>
-          <t>19/07/2026 03:54</t>
+          <t>19/07/2026 23:45</t>
         </is>
       </c>
       <c r="J364" s="2" t="inlineStr">
         <is>
-          <t>24/07/2026 20:25</t>
+          <t>21/07/2026 17:30</t>
         </is>
       </c>
       <c r="K364" s="2" t="inlineStr">
         <is>
-          <t>19/07/2026 03:54</t>
+          <t>19/07/2026 23:45</t>
         </is>
       </c>
       <c r="L364" s="2" t="inlineStr">
         <is>
-          <t>24/07/2026 20:25</t>
+          <t>21/07/2026 17:30</t>
         </is>
       </c>
     </row>
@@ -23022,12 +23022,12 @@
       </c>
       <c r="C365" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-90 C a -60 C</t>
         </is>
       </c>
       <c r="D365" s="2" t="inlineStr">
         <is>
-          <t>561418</t>
+          <t>560576</t>
         </is>
       </c>
       <c r="E365" s="2" t="inlineStr">
@@ -23037,12 +23037,12 @@
       </c>
       <c r="F365" s="2" t="inlineStr">
         <is>
-          <t>A9611</t>
+          <t>V5560004</t>
         </is>
       </c>
       <c r="G365" s="2" t="inlineStr">
         <is>
-          <t>00019200000013472160</t>
+          <t>00019200000013475797</t>
         </is>
       </c>
       <c r="H365" s="2" t="inlineStr">
@@ -23052,22 +23052,22 @@
       </c>
       <c r="I365" s="2" t="inlineStr">
         <is>
-          <t>19/07/2026 03:54</t>
+          <t>19/07/2026 23:45</t>
         </is>
       </c>
       <c r="J365" s="2" t="inlineStr">
         <is>
-          <t>24/07/2026 20:25</t>
+          <t>21/07/2026 17:30</t>
         </is>
       </c>
       <c r="K365" s="2" t="inlineStr">
         <is>
-          <t>19/07/2026 03:54</t>
+          <t>19/07/2026 23:45</t>
         </is>
       </c>
       <c r="L365" s="2" t="inlineStr">
         <is>
-          <t>24/07/2026 20:25</t>
+          <t>21/07/2026 17:30</t>
         </is>
       </c>
     </row>
@@ -23099,12 +23099,12 @@
       </c>
       <c r="F366" s="2" t="inlineStr">
         <is>
-          <t>TA0310</t>
+          <t>A8179</t>
         </is>
       </c>
       <c r="G366" s="2" t="inlineStr">
         <is>
-          <t>00019200000013472178</t>
+          <t>00019200000013472151</t>
         </is>
       </c>
       <c r="H366" s="2" t="inlineStr">
@@ -23161,12 +23161,12 @@
       </c>
       <c r="F367" s="2" t="inlineStr">
         <is>
-          <t>TA0493</t>
+          <t>A9611</t>
         </is>
       </c>
       <c r="G367" s="2" t="inlineStr">
         <is>
-          <t>00019200000013472186</t>
+          <t>00019200000013472160</t>
         </is>
       </c>
       <c r="H367" s="2" t="inlineStr">
@@ -23223,12 +23223,12 @@
       </c>
       <c r="F368" s="2" t="inlineStr">
         <is>
-          <t>A2344</t>
+          <t>TA0310</t>
         </is>
       </c>
       <c r="G368" s="2" t="inlineStr">
         <is>
-          <t>00019200000013472194</t>
+          <t>00019200000013472178</t>
         </is>
       </c>
       <c r="H368" s="2" t="inlineStr">
@@ -23270,7 +23270,7 @@
       </c>
       <c r="C369" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D369" s="2" t="inlineStr">
@@ -23285,12 +23285,12 @@
       </c>
       <c r="F369" s="2" t="inlineStr">
         <is>
-          <t>A8458</t>
+          <t>TA0493</t>
         </is>
       </c>
       <c r="G369" s="2" t="inlineStr">
         <is>
-          <t>00019200000013472208</t>
+          <t>00019200000013472186</t>
         </is>
       </c>
       <c r="H369" s="2" t="inlineStr">
@@ -23332,7 +23332,7 @@
       </c>
       <c r="C370" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D370" s="2" t="inlineStr">
@@ -23347,12 +23347,12 @@
       </c>
       <c r="F370" s="2" t="inlineStr">
         <is>
-          <t>A7945</t>
+          <t>A2344</t>
         </is>
       </c>
       <c r="G370" s="2" t="inlineStr">
         <is>
-          <t>00019200000013472216</t>
+          <t>00019200000013472194</t>
         </is>
       </c>
       <c r="H370" s="2" t="inlineStr">
@@ -23409,12 +23409,12 @@
       </c>
       <c r="F371" s="2" t="inlineStr">
         <is>
-          <t>A5377</t>
+          <t>A8458</t>
         </is>
       </c>
       <c r="G371" s="2" t="inlineStr">
         <is>
-          <t>00019200000013472224</t>
+          <t>00019200000013472208</t>
         </is>
       </c>
       <c r="H371" s="2" t="inlineStr">
@@ -23471,12 +23471,12 @@
       </c>
       <c r="F372" s="2" t="inlineStr">
         <is>
-          <t>A7312</t>
+          <t>A7945</t>
         </is>
       </c>
       <c r="G372" s="2" t="inlineStr">
         <is>
-          <t>00019200000013472232</t>
+          <t>00019200000013472216</t>
         </is>
       </c>
       <c r="H372" s="2" t="inlineStr">
@@ -23533,12 +23533,12 @@
       </c>
       <c r="F373" s="2" t="inlineStr">
         <is>
-          <t>A6642</t>
+          <t>A5377</t>
         </is>
       </c>
       <c r="G373" s="2" t="inlineStr">
         <is>
-          <t>00019200000013472259</t>
+          <t>00019200000013472224</t>
         </is>
       </c>
       <c r="H373" s="2" t="inlineStr">
@@ -23595,12 +23595,12 @@
       </c>
       <c r="F374" s="2" t="inlineStr">
         <is>
-          <t>A6142</t>
+          <t>A7312</t>
         </is>
       </c>
       <c r="G374" s="2" t="inlineStr">
         <is>
-          <t>00019200000013472267</t>
+          <t>00019200000013472232</t>
         </is>
       </c>
       <c r="H374" s="2" t="inlineStr">
@@ -23657,12 +23657,12 @@
       </c>
       <c r="F375" s="2" t="inlineStr">
         <is>
-          <t>TA0826</t>
+          <t>A6642</t>
         </is>
       </c>
       <c r="G375" s="2" t="inlineStr">
         <is>
-          <t>00019200000013472275</t>
+          <t>00019200000013472259</t>
         </is>
       </c>
       <c r="H375" s="2" t="inlineStr">
@@ -23719,12 +23719,12 @@
       </c>
       <c r="F376" s="2" t="inlineStr">
         <is>
-          <t>A8679</t>
+          <t>A6142</t>
         </is>
       </c>
       <c r="G376" s="2" t="inlineStr">
         <is>
-          <t>00019200000013472283</t>
+          <t>00019200000013472267</t>
         </is>
       </c>
       <c r="H376" s="2" t="inlineStr">
@@ -23781,12 +23781,12 @@
       </c>
       <c r="F377" s="2" t="inlineStr">
         <is>
-          <t>TA1135</t>
+          <t>TA0826</t>
         </is>
       </c>
       <c r="G377" s="2" t="inlineStr">
         <is>
-          <t>00019200000013472291</t>
+          <t>00019200000013472275</t>
         </is>
       </c>
       <c r="H377" s="2" t="inlineStr">
@@ -23843,12 +23843,12 @@
       </c>
       <c r="F378" s="2" t="inlineStr">
         <is>
-          <t>TA0895</t>
+          <t>A8679</t>
         </is>
       </c>
       <c r="G378" s="2" t="inlineStr">
         <is>
-          <t>00019200000013472305</t>
+          <t>00019200000013472283</t>
         </is>
       </c>
       <c r="H378" s="2" t="inlineStr">
@@ -23905,12 +23905,12 @@
       </c>
       <c r="F379" s="2" t="inlineStr">
         <is>
-          <t>A7095</t>
+          <t>TA1135</t>
         </is>
       </c>
       <c r="G379" s="2" t="inlineStr">
         <is>
-          <t>00019200000013472313</t>
+          <t>00019200000013472291</t>
         </is>
       </c>
       <c r="H379" s="2" t="inlineStr">
@@ -23967,12 +23967,12 @@
       </c>
       <c r="F380" s="2" t="inlineStr">
         <is>
-          <t>A6569</t>
+          <t>TA0895</t>
         </is>
       </c>
       <c r="G380" s="2" t="inlineStr">
         <is>
-          <t>00019200000013472321</t>
+          <t>00019200000013472305</t>
         </is>
       </c>
       <c r="H380" s="2" t="inlineStr">
@@ -24029,12 +24029,12 @@
       </c>
       <c r="F381" s="2" t="inlineStr">
         <is>
-          <t>TA1062</t>
+          <t>A7095</t>
         </is>
       </c>
       <c r="G381" s="2" t="inlineStr">
         <is>
-          <t>00019200000013472330</t>
+          <t>00019200000013472313</t>
         </is>
       </c>
       <c r="H381" s="2" t="inlineStr">
@@ -24091,12 +24091,12 @@
       </c>
       <c r="F382" s="2" t="inlineStr">
         <is>
-          <t>A5533</t>
+          <t>A6569</t>
         </is>
       </c>
       <c r="G382" s="2" t="inlineStr">
         <is>
-          <t>00019200000013472348</t>
+          <t>00019200000013472321</t>
         </is>
       </c>
       <c r="H382" s="2" t="inlineStr">
@@ -24153,12 +24153,12 @@
       </c>
       <c r="F383" s="2" t="inlineStr">
         <is>
-          <t>A9128</t>
+          <t>TA1062</t>
         </is>
       </c>
       <c r="G383" s="2" t="inlineStr">
         <is>
-          <t>00019200000013472356</t>
+          <t>00019200000013472330</t>
         </is>
       </c>
       <c r="H383" s="2" t="inlineStr">
@@ -24215,12 +24215,12 @@
       </c>
       <c r="F384" s="2" t="inlineStr">
         <is>
-          <t>A8531</t>
+          <t>A5533</t>
         </is>
       </c>
       <c r="G384" s="2" t="inlineStr">
         <is>
-          <t>00019200000013472364</t>
+          <t>00019200000013472348</t>
         </is>
       </c>
       <c r="H384" s="2" t="inlineStr">
@@ -24277,12 +24277,12 @@
       </c>
       <c r="F385" s="2" t="inlineStr">
         <is>
-          <t>A0259</t>
+          <t>A9128</t>
         </is>
       </c>
       <c r="G385" s="2" t="inlineStr">
         <is>
-          <t>00019200000013472372</t>
+          <t>00019200000013472356</t>
         </is>
       </c>
       <c r="H385" s="2" t="inlineStr">
@@ -24339,12 +24339,12 @@
       </c>
       <c r="F386" s="2" t="inlineStr">
         <is>
-          <t>A3195</t>
+          <t>A8531</t>
         </is>
       </c>
       <c r="G386" s="2" t="inlineStr">
         <is>
-          <t>00019200000013472380</t>
+          <t>00019200000013472364</t>
         </is>
       </c>
       <c r="H386" s="2" t="inlineStr">
@@ -24401,12 +24401,12 @@
       </c>
       <c r="F387" s="2" t="inlineStr">
         <is>
-          <t>A5061</t>
+          <t>A0259</t>
         </is>
       </c>
       <c r="G387" s="2" t="inlineStr">
         <is>
-          <t>00019200000013472399</t>
+          <t>00019200000013472372</t>
         </is>
       </c>
       <c r="H387" s="2" t="inlineStr">
@@ -24463,12 +24463,12 @@
       </c>
       <c r="F388" s="2" t="inlineStr">
         <is>
-          <t>A5097</t>
+          <t>A3195</t>
         </is>
       </c>
       <c r="G388" s="2" t="inlineStr">
         <is>
-          <t>00019200000013472402</t>
+          <t>00019200000013472380</t>
         </is>
       </c>
       <c r="H388" s="2" t="inlineStr">
@@ -24525,12 +24525,12 @@
       </c>
       <c r="F389" s="2" t="inlineStr">
         <is>
-          <t>A3193</t>
+          <t>A5061</t>
         </is>
       </c>
       <c r="G389" s="2" t="inlineStr">
         <is>
-          <t>00019200000013472410</t>
+          <t>00019200000013472399</t>
         </is>
       </c>
       <c r="H389" s="2" t="inlineStr">
@@ -24572,7 +24572,7 @@
       </c>
       <c r="C390" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D390" s="2" t="inlineStr">
@@ -24587,12 +24587,12 @@
       </c>
       <c r="F390" s="2" t="inlineStr">
         <is>
-          <t>A5035</t>
+          <t>A5097</t>
         </is>
       </c>
       <c r="G390" s="2" t="inlineStr">
         <is>
-          <t>00019200000013473760</t>
+          <t>00019200000013472402</t>
         </is>
       </c>
       <c r="H390" s="2" t="inlineStr">
@@ -24639,22 +24639,22 @@
       </c>
       <c r="D391" s="2" t="inlineStr">
         <is>
-          <t>559944</t>
+          <t>561418</t>
         </is>
       </c>
       <c r="E391" s="2" t="inlineStr">
         <is>
-          <t>RR</t>
+          <t>RO</t>
         </is>
       </c>
       <c r="F391" s="2" t="inlineStr">
         <is>
-          <t>A3432</t>
+          <t>A3193</t>
         </is>
       </c>
       <c r="G391" s="2" t="inlineStr">
         <is>
-          <t>00019200000013419030</t>
+          <t>00019200000013472410</t>
         </is>
       </c>
       <c r="H391" s="2" t="inlineStr">
@@ -24664,22 +24664,22 @@
       </c>
       <c r="I391" s="2" t="inlineStr">
         <is>
-          <t>07/07/2026 06:51</t>
+          <t>19/07/2026 03:54</t>
         </is>
       </c>
       <c r="J391" s="2" t="inlineStr">
         <is>
-          <t>10/07/2026 18:00</t>
+          <t>24/07/2026 20:25</t>
         </is>
       </c>
       <c r="K391" s="2" t="inlineStr">
         <is>
-          <t>07/07/2026 06:51</t>
+          <t>19/07/2026 03:54</t>
         </is>
       </c>
       <c r="L391" s="2" t="inlineStr">
         <is>
-          <t>10/07/2026 18:00</t>
+          <t>24/07/2026 20:25</t>
         </is>
       </c>
     </row>
@@ -24696,27 +24696,27 @@
       </c>
       <c r="C392" s="2" t="inlineStr">
         <is>
-          <t>-90 C a -60 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D392" s="2" t="inlineStr">
         <is>
-          <t>560780</t>
+          <t>561418</t>
         </is>
       </c>
       <c r="E392" s="2" t="inlineStr">
         <is>
-          <t>RR</t>
+          <t>RO</t>
         </is>
       </c>
       <c r="F392" s="2" t="inlineStr">
         <is>
-          <t>300017</t>
+          <t>A5035</t>
         </is>
       </c>
       <c r="G392" s="2" t="inlineStr">
         <is>
-          <t>00019200000013778609</t>
+          <t>00019200000013473760</t>
         </is>
       </c>
       <c r="H392" s="2" t="inlineStr">
@@ -24726,22 +24726,22 @@
       </c>
       <c r="I392" s="2" t="inlineStr">
         <is>
-          <t>27/07/2026 22:35</t>
+          <t>19/07/2026 03:54</t>
         </is>
       </c>
       <c r="J392" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>24/07/2026 20:25</t>
         </is>
       </c>
       <c r="K392" s="2" t="inlineStr">
         <is>
-          <t>27/07/2026 22:35</t>
+          <t>19/07/2026 03:54</t>
         </is>
       </c>
       <c r="L392" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>24/07/2026 20:25</t>
         </is>
       </c>
     </row>
@@ -24763,22 +24763,22 @@
       </c>
       <c r="D393" s="2" t="inlineStr">
         <is>
-          <t>559925</t>
+          <t>559944</t>
         </is>
       </c>
       <c r="E393" s="2" t="inlineStr">
         <is>
-          <t>RS</t>
+          <t>RR</t>
         </is>
       </c>
       <c r="F393" s="2" t="inlineStr">
         <is>
-          <t>A7594</t>
+          <t>A3432</t>
         </is>
       </c>
       <c r="G393" s="2" t="inlineStr">
         <is>
-          <t>00019200000013419137</t>
+          <t>00019200000013419030</t>
         </is>
       </c>
       <c r="H393" s="2" t="inlineStr">
@@ -24793,7 +24793,7 @@
       </c>
       <c r="J393" s="2" t="inlineStr">
         <is>
-          <t>09/07/2026 13:09</t>
+          <t>10/07/2026 18:00</t>
         </is>
       </c>
       <c r="K393" s="2" t="inlineStr">
@@ -24803,7 +24803,7 @@
       </c>
       <c r="L393" s="2" t="inlineStr">
         <is>
-          <t>09/07/2026 13:09</t>
+          <t>10/07/2026 18:00</t>
         </is>
       </c>
     </row>
@@ -24825,22 +24825,22 @@
       </c>
       <c r="D394" s="2" t="inlineStr">
         <is>
-          <t>560574</t>
+          <t>560780</t>
         </is>
       </c>
       <c r="E394" s="2" t="inlineStr">
         <is>
-          <t>RS</t>
+          <t>RR</t>
         </is>
       </c>
       <c r="F394" s="2" t="inlineStr">
         <is>
-          <t>AS-0499</t>
+          <t>300017</t>
         </is>
       </c>
       <c r="G394" s="2" t="inlineStr">
         <is>
-          <t>00019200000013463969</t>
+          <t>00019200000013778609</t>
         </is>
       </c>
       <c r="H394" s="2" t="inlineStr">
@@ -24850,22 +24850,22 @@
       </c>
       <c r="I394" s="2" t="inlineStr">
         <is>
-          <t>21/07/2026 22:28</t>
+          <t>27/07/2026 22:35</t>
         </is>
       </c>
       <c r="J394" s="2" t="inlineStr">
         <is>
-          <t>23/07/2026 15:00</t>
+          <t>-</t>
         </is>
       </c>
       <c r="K394" s="2" t="inlineStr">
         <is>
-          <t>21/07/2026 22:28</t>
+          <t>27/07/2026 22:35</t>
         </is>
       </c>
       <c r="L394" s="2" t="inlineStr">
         <is>
-          <t>23/07/2026 13:15</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -24882,12 +24882,12 @@
       </c>
       <c r="C395" s="2" t="inlineStr">
         <is>
-          <t>-90 C a -60 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D395" s="2" t="inlineStr">
         <is>
-          <t>560574</t>
+          <t>559925</t>
         </is>
       </c>
       <c r="E395" s="2" t="inlineStr">
@@ -24897,12 +24897,12 @@
       </c>
       <c r="F395" s="2" t="inlineStr">
         <is>
-          <t>AS-0683</t>
+          <t>A7594</t>
         </is>
       </c>
       <c r="G395" s="2" t="inlineStr">
         <is>
-          <t>00019200000013463977</t>
+          <t>00019200000013419137</t>
         </is>
       </c>
       <c r="H395" s="2" t="inlineStr">
@@ -24912,22 +24912,22 @@
       </c>
       <c r="I395" s="2" t="inlineStr">
         <is>
-          <t>21/07/2026 22:28</t>
+          <t>07/07/2026 06:51</t>
         </is>
       </c>
       <c r="J395" s="2" t="inlineStr">
         <is>
-          <t>23/07/2026 15:00</t>
+          <t>09/07/2026 13:09</t>
         </is>
       </c>
       <c r="K395" s="2" t="inlineStr">
         <is>
-          <t>21/07/2026 22:28</t>
+          <t>07/07/2026 06:51</t>
         </is>
       </c>
       <c r="L395" s="2" t="inlineStr">
         <is>
-          <t>23/07/2026 13:15</t>
+          <t>09/07/2026 13:09</t>
         </is>
       </c>
     </row>
@@ -24959,12 +24959,12 @@
       </c>
       <c r="F396" s="2" t="inlineStr">
         <is>
-          <t>AS-0426</t>
+          <t>AS-0499</t>
         </is>
       </c>
       <c r="G396" s="2" t="inlineStr">
         <is>
-          <t>00019200000013463985</t>
+          <t>00019200000013463969</t>
         </is>
       </c>
       <c r="H396" s="2" t="inlineStr">
@@ -25021,12 +25021,12 @@
       </c>
       <c r="F397" s="2" t="inlineStr">
         <is>
-          <t>AS-0702</t>
+          <t>AS-0683</t>
         </is>
       </c>
       <c r="G397" s="2" t="inlineStr">
         <is>
-          <t>00019200000013463993</t>
+          <t>00019200000013463977</t>
         </is>
       </c>
       <c r="H397" s="2" t="inlineStr">
@@ -25083,12 +25083,12 @@
       </c>
       <c r="F398" s="2" t="inlineStr">
         <is>
-          <t>AS-0869</t>
+          <t>AS-0426</t>
         </is>
       </c>
       <c r="G398" s="2" t="inlineStr">
         <is>
-          <t>00019200000013464019</t>
+          <t>00019200000013463985</t>
         </is>
       </c>
       <c r="H398" s="2" t="inlineStr">
@@ -25145,12 +25145,12 @@
       </c>
       <c r="F399" s="2" t="inlineStr">
         <is>
-          <t>AS-0837</t>
+          <t>AS-0702</t>
         </is>
       </c>
       <c r="G399" s="2" t="inlineStr">
         <is>
-          <t>00019200000013464027</t>
+          <t>00019200000013463993</t>
         </is>
       </c>
       <c r="H399" s="2" t="inlineStr">
@@ -25207,12 +25207,12 @@
       </c>
       <c r="F400" s="2" t="inlineStr">
         <is>
-          <t>AS-0201</t>
+          <t>AS-0869</t>
         </is>
       </c>
       <c r="G400" s="2" t="inlineStr">
         <is>
-          <t>00019200000013464035</t>
+          <t>00019200000013464019</t>
         </is>
       </c>
       <c r="H400" s="2" t="inlineStr">
@@ -25237,7 +25237,7 @@
       </c>
       <c r="L400" s="2" t="inlineStr">
         <is>
-          <t>23/07/2026 15:00</t>
+          <t>23/07/2026 13:15</t>
         </is>
       </c>
     </row>
@@ -25269,12 +25269,12 @@
       </c>
       <c r="F401" s="2" t="inlineStr">
         <is>
-          <t>AS-0487</t>
+          <t>AS-0837</t>
         </is>
       </c>
       <c r="G401" s="2" t="inlineStr">
         <is>
-          <t>00019200000013464043</t>
+          <t>00019200000013464027</t>
         </is>
       </c>
       <c r="H401" s="2" t="inlineStr">
@@ -25331,12 +25331,12 @@
       </c>
       <c r="F402" s="2" t="inlineStr">
         <is>
-          <t>AS-0356</t>
+          <t>AS-0201</t>
         </is>
       </c>
       <c r="G402" s="2" t="inlineStr">
         <is>
-          <t>00019200000013464051</t>
+          <t>00019200000013464035</t>
         </is>
       </c>
       <c r="H402" s="2" t="inlineStr">
@@ -25393,12 +25393,12 @@
       </c>
       <c r="F403" s="2" t="inlineStr">
         <is>
-          <t>AS-0414</t>
+          <t>AS-0487</t>
         </is>
       </c>
       <c r="G403" s="2" t="inlineStr">
         <is>
-          <t>00019200000013464078</t>
+          <t>00019200000013464043</t>
         </is>
       </c>
       <c r="H403" s="2" t="inlineStr">
@@ -25455,12 +25455,12 @@
       </c>
       <c r="F404" s="2" t="inlineStr">
         <is>
-          <t>AS-0078</t>
+          <t>AS-0356</t>
         </is>
       </c>
       <c r="G404" s="2" t="inlineStr">
         <is>
-          <t>00019200000013464086</t>
+          <t>00019200000013464051</t>
         </is>
       </c>
       <c r="H404" s="2" t="inlineStr">
@@ -25517,12 +25517,12 @@
       </c>
       <c r="F405" s="2" t="inlineStr">
         <is>
-          <t>AS-0019</t>
+          <t>AS-0414</t>
         </is>
       </c>
       <c r="G405" s="2" t="inlineStr">
         <is>
-          <t>00019200000013464094</t>
+          <t>00019200000013464078</t>
         </is>
       </c>
       <c r="H405" s="2" t="inlineStr">
@@ -25547,7 +25547,7 @@
       </c>
       <c r="L405" s="2" t="inlineStr">
         <is>
-          <t>23/07/2026 15:00</t>
+          <t>23/07/2026 13:15</t>
         </is>
       </c>
     </row>
@@ -25579,12 +25579,12 @@
       </c>
       <c r="F406" s="2" t="inlineStr">
         <is>
-          <t>AS-0252</t>
+          <t>AS-0078</t>
         </is>
       </c>
       <c r="G406" s="2" t="inlineStr">
         <is>
-          <t>00019200000013464108</t>
+          <t>00019200000013464086</t>
         </is>
       </c>
       <c r="H406" s="2" t="inlineStr">
@@ -25641,12 +25641,12 @@
       </c>
       <c r="F407" s="2" t="inlineStr">
         <is>
-          <t>AS-0160</t>
+          <t>AS-0019</t>
         </is>
       </c>
       <c r="G407" s="2" t="inlineStr">
         <is>
-          <t>00019200000013464116</t>
+          <t>00019200000013464094</t>
         </is>
       </c>
       <c r="H407" s="2" t="inlineStr">
@@ -25703,12 +25703,12 @@
       </c>
       <c r="F408" s="2" t="inlineStr">
         <is>
-          <t>AS-0513</t>
+          <t>AS-0252</t>
         </is>
       </c>
       <c r="G408" s="2" t="inlineStr">
         <is>
-          <t>00019200000013464124</t>
+          <t>00019200000013464108</t>
         </is>
       </c>
       <c r="H408" s="2" t="inlineStr">
@@ -25733,7 +25733,7 @@
       </c>
       <c r="L408" s="2" t="inlineStr">
         <is>
-          <t>23/07/2026 13:15</t>
+          <t>23/07/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -25765,12 +25765,12 @@
       </c>
       <c r="F409" s="2" t="inlineStr">
         <is>
-          <t>AS-0234</t>
+          <t>AS-0160</t>
         </is>
       </c>
       <c r="G409" s="2" t="inlineStr">
         <is>
-          <t>00019200000013464132</t>
+          <t>00019200000013464116</t>
         </is>
       </c>
       <c r="H409" s="2" t="inlineStr">
@@ -25827,12 +25827,12 @@
       </c>
       <c r="F410" s="2" t="inlineStr">
         <is>
-          <t>AS-0494</t>
+          <t>AS-0513</t>
         </is>
       </c>
       <c r="G410" s="2" t="inlineStr">
         <is>
-          <t>00019200000013464140</t>
+          <t>00019200000013464124</t>
         </is>
       </c>
       <c r="H410" s="2" t="inlineStr">
@@ -25857,7 +25857,7 @@
       </c>
       <c r="L410" s="2" t="inlineStr">
         <is>
-          <t>23/07/2026 15:00</t>
+          <t>23/07/2026 13:15</t>
         </is>
       </c>
     </row>
@@ -25889,12 +25889,12 @@
       </c>
       <c r="F411" s="2" t="inlineStr">
         <is>
-          <t>AS-0850</t>
+          <t>AS-0234</t>
         </is>
       </c>
       <c r="G411" s="2" t="inlineStr">
         <is>
-          <t>00019200000013464159</t>
+          <t>00019200000013464132</t>
         </is>
       </c>
       <c r="H411" s="2" t="inlineStr">
@@ -25951,12 +25951,12 @@
       </c>
       <c r="F412" s="2" t="inlineStr">
         <is>
-          <t>AS-0107</t>
+          <t>AS-0494</t>
         </is>
       </c>
       <c r="G412" s="2" t="inlineStr">
         <is>
-          <t>00019200000013464167</t>
+          <t>00019200000013464140</t>
         </is>
       </c>
       <c r="H412" s="2" t="inlineStr">
@@ -26013,12 +26013,12 @@
       </c>
       <c r="F413" s="2" t="inlineStr">
         <is>
-          <t>AS-0845</t>
+          <t>AS-0850</t>
         </is>
       </c>
       <c r="G413" s="2" t="inlineStr">
         <is>
-          <t>00019200000013464175</t>
+          <t>00019200000013464159</t>
         </is>
       </c>
       <c r="H413" s="2" t="inlineStr">
@@ -26075,12 +26075,12 @@
       </c>
       <c r="F414" s="2" t="inlineStr">
         <is>
-          <t>AS-0511</t>
+          <t>AS-0107</t>
         </is>
       </c>
       <c r="G414" s="2" t="inlineStr">
         <is>
-          <t>00019200000013464183</t>
+          <t>00019200000013464167</t>
         </is>
       </c>
       <c r="H414" s="2" t="inlineStr">
@@ -26137,12 +26137,12 @@
       </c>
       <c r="F415" s="2" t="inlineStr">
         <is>
-          <t>AS-0363</t>
+          <t>AS-0845</t>
         </is>
       </c>
       <c r="G415" s="2" t="inlineStr">
         <is>
-          <t>00019200000013464191</t>
+          <t>00019200000013464175</t>
         </is>
       </c>
       <c r="H415" s="2" t="inlineStr">
@@ -26167,7 +26167,7 @@
       </c>
       <c r="L415" s="2" t="inlineStr">
         <is>
-          <t>23/07/2026 13:15</t>
+          <t>23/07/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -26199,12 +26199,12 @@
       </c>
       <c r="F416" s="2" t="inlineStr">
         <is>
-          <t>AS-0269</t>
+          <t>AS-0511</t>
         </is>
       </c>
       <c r="G416" s="2" t="inlineStr">
         <is>
-          <t>00019200000013464205</t>
+          <t>00019200000013464183</t>
         </is>
       </c>
       <c r="H416" s="2" t="inlineStr">
@@ -26229,7 +26229,7 @@
       </c>
       <c r="L416" s="2" t="inlineStr">
         <is>
-          <t>23/07/2026 13:15</t>
+          <t>23/07/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -26261,12 +26261,12 @@
       </c>
       <c r="F417" s="2" t="inlineStr">
         <is>
-          <t>AS-0643</t>
+          <t>AS-0363</t>
         </is>
       </c>
       <c r="G417" s="2" t="inlineStr">
         <is>
-          <t>00019200000013464213</t>
+          <t>00019200000013464191</t>
         </is>
       </c>
       <c r="H417" s="2" t="inlineStr">
@@ -26323,12 +26323,12 @@
       </c>
       <c r="F418" s="2" t="inlineStr">
         <is>
-          <t>AS-0263</t>
+          <t>AS-0269</t>
         </is>
       </c>
       <c r="G418" s="2" t="inlineStr">
         <is>
-          <t>00019200000013464221</t>
+          <t>00019200000013464205</t>
         </is>
       </c>
       <c r="H418" s="2" t="inlineStr">
@@ -26370,12 +26370,12 @@
       </c>
       <c r="C419" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-90 C a -60 C</t>
         </is>
       </c>
       <c r="D419" s="2" t="inlineStr">
         <is>
-          <t>560688</t>
+          <t>560574</t>
         </is>
       </c>
       <c r="E419" s="2" t="inlineStr">
@@ -26385,37 +26385,37 @@
       </c>
       <c r="F419" s="2" t="inlineStr">
         <is>
-          <t>A5913</t>
+          <t>AS-0643</t>
         </is>
       </c>
       <c r="G419" s="2" t="inlineStr">
         <is>
-          <t>00019200000013694359</t>
+          <t>00019200000013464213</t>
         </is>
       </c>
       <c r="H419" s="2" t="inlineStr">
         <is>
-          <t>Rodoviário</t>
+          <t>MultiModal</t>
         </is>
       </c>
       <c r="I419" s="2" t="inlineStr">
         <is>
-          <t>27/07/2026 06:04</t>
+          <t>21/07/2026 22:28</t>
         </is>
       </c>
       <c r="J419" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>23/07/2026 15:00</t>
         </is>
       </c>
       <c r="K419" s="2" t="inlineStr">
         <is>
-          <t>27/07/2026 06:04</t>
+          <t>21/07/2026 22:28</t>
         </is>
       </c>
       <c r="L419" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>23/07/2026 13:15</t>
         </is>
       </c>
     </row>
@@ -26432,27 +26432,27 @@
       </c>
       <c r="C420" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-90 C a -60 C</t>
         </is>
       </c>
       <c r="D420" s="2" t="inlineStr">
         <is>
-          <t>559880</t>
+          <t>560574</t>
         </is>
       </c>
       <c r="E420" s="2" t="inlineStr">
         <is>
-          <t>SC</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="F420" s="2" t="inlineStr">
         <is>
-          <t>A8482</t>
+          <t>AS-0263</t>
         </is>
       </c>
       <c r="G420" s="2" t="inlineStr">
         <is>
-          <t>00019200000013407147</t>
+          <t>00019200000013464221</t>
         </is>
       </c>
       <c r="H420" s="2" t="inlineStr">
@@ -26462,22 +26462,22 @@
       </c>
       <c r="I420" s="2" t="inlineStr">
         <is>
-          <t>09/07/2026 05:48</t>
+          <t>21/07/2026 22:28</t>
         </is>
       </c>
       <c r="J420" s="2" t="inlineStr">
         <is>
-          <t>10/07/2026 17:00</t>
+          <t>23/07/2026 15:00</t>
         </is>
       </c>
       <c r="K420" s="2" t="inlineStr">
         <is>
-          <t>09/07/2026 05:48</t>
+          <t>21/07/2026 22:28</t>
         </is>
       </c>
       <c r="L420" s="2" t="inlineStr">
         <is>
-          <t>10/07/2026 17:00</t>
+          <t>23/07/2026 13:15</t>
         </is>
       </c>
     </row>
@@ -26494,52 +26494,52 @@
       </c>
       <c r="C421" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D421" s="2" t="inlineStr">
         <is>
-          <t>559880</t>
+          <t>560688</t>
         </is>
       </c>
       <c r="E421" s="2" t="inlineStr">
         <is>
-          <t>SC</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="F421" s="2" t="inlineStr">
         <is>
-          <t>A4021</t>
+          <t>A5913</t>
         </is>
       </c>
       <c r="G421" s="2" t="inlineStr">
         <is>
-          <t>00019200000013407180</t>
+          <t>00019200000013694359</t>
         </is>
       </c>
       <c r="H421" s="2" t="inlineStr">
         <is>
-          <t>MultiModal</t>
+          <t>Rodoviário</t>
         </is>
       </c>
       <c r="I421" s="2" t="inlineStr">
         <is>
-          <t>09/07/2026 05:48</t>
+          <t>27/07/2026 06:04</t>
         </is>
       </c>
       <c r="J421" s="2" t="inlineStr">
         <is>
-          <t>10/07/2026 17:00</t>
+          <t>-</t>
         </is>
       </c>
       <c r="K421" s="2" t="inlineStr">
         <is>
-          <t>09/07/2026 05:48</t>
+          <t>27/07/2026 06:04</t>
         </is>
       </c>
       <c r="L421" s="2" t="inlineStr">
         <is>
-          <t>10/07/2026 17:00</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -26561,22 +26561,22 @@
       </c>
       <c r="D422" s="2" t="inlineStr">
         <is>
-          <t>559880</t>
+          <t>562154</t>
         </is>
       </c>
       <c r="E422" s="2" t="inlineStr">
         <is>
-          <t>SC</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="F422" s="2" t="inlineStr">
         <is>
-          <t>A7212</t>
+          <t>A4440</t>
         </is>
       </c>
       <c r="G422" s="2" t="inlineStr">
         <is>
-          <t>00019200000013407198</t>
+          <t>00019200000013778293</t>
         </is>
       </c>
       <c r="H422" s="2" t="inlineStr">
@@ -26586,22 +26586,22 @@
       </c>
       <c r="I422" s="2" t="inlineStr">
         <is>
-          <t>09/07/2026 05:48</t>
+          <t>28/07/2026 03:39</t>
         </is>
       </c>
       <c r="J422" s="2" t="inlineStr">
         <is>
-          <t>10/07/2026 17:00</t>
+          <t>-</t>
         </is>
       </c>
       <c r="K422" s="2" t="inlineStr">
         <is>
-          <t>09/07/2026 05:48</t>
+          <t>28/07/2026 03:39</t>
         </is>
       </c>
       <c r="L422" s="2" t="inlineStr">
         <is>
-          <t>10/07/2026 17:00</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -26618,7 +26618,7 @@
       </c>
       <c r="C423" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D423" s="2" t="inlineStr">
@@ -26633,12 +26633,12 @@
       </c>
       <c r="F423" s="2" t="inlineStr">
         <is>
-          <t>A3672</t>
+          <t>A8482</t>
         </is>
       </c>
       <c r="G423" s="2" t="inlineStr">
         <is>
-          <t>00019200000013407201</t>
+          <t>00019200000013407147</t>
         </is>
       </c>
       <c r="H423" s="2" t="inlineStr">
@@ -26680,7 +26680,7 @@
       </c>
       <c r="C424" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D424" s="2" t="inlineStr">
@@ -26695,12 +26695,12 @@
       </c>
       <c r="F424" s="2" t="inlineStr">
         <is>
-          <t>TA0241</t>
+          <t>A4021</t>
         </is>
       </c>
       <c r="G424" s="2" t="inlineStr">
         <is>
-          <t>00019200000013407210</t>
+          <t>00019200000013407180</t>
         </is>
       </c>
       <c r="H424" s="2" t="inlineStr">
@@ -26747,22 +26747,22 @@
       </c>
       <c r="D425" s="2" t="inlineStr">
         <is>
-          <t>559876</t>
+          <t>559880</t>
         </is>
       </c>
       <c r="E425" s="2" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>SC</t>
         </is>
       </c>
       <c r="F425" s="2" t="inlineStr">
         <is>
-          <t>A1817</t>
+          <t>A7212</t>
         </is>
       </c>
       <c r="G425" s="2" t="inlineStr">
         <is>
-          <t>00019200000013419021</t>
+          <t>00019200000013407198</t>
         </is>
       </c>
       <c r="H425" s="2" t="inlineStr">
@@ -26772,22 +26772,22 @@
       </c>
       <c r="I425" s="2" t="inlineStr">
         <is>
-          <t>07/07/2026 00:57</t>
+          <t>09/07/2026 05:48</t>
         </is>
       </c>
       <c r="J425" s="2" t="inlineStr">
         <is>
-          <t>17/07/2026 15:00</t>
+          <t>10/07/2026 17:00</t>
         </is>
       </c>
       <c r="K425" s="2" t="inlineStr">
         <is>
-          <t>07/07/2026 00:57</t>
+          <t>09/07/2026 05:48</t>
         </is>
       </c>
       <c r="L425" s="2" t="inlineStr">
         <is>
-          <t>17/07/2026 15:00</t>
+          <t>10/07/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -26804,27 +26804,27 @@
       </c>
       <c r="C426" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D426" s="2" t="inlineStr">
         <is>
-          <t>560503</t>
+          <t>559880</t>
         </is>
       </c>
       <c r="E426" s="2" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>SC</t>
         </is>
       </c>
       <c r="F426" s="2" t="inlineStr">
         <is>
-          <t>A0727</t>
+          <t>A3672</t>
         </is>
       </c>
       <c r="G426" s="2" t="inlineStr">
         <is>
-          <t>00019200000013454420</t>
+          <t>00019200000013407201</t>
         </is>
       </c>
       <c r="H426" s="2" t="inlineStr">
@@ -26834,22 +26834,22 @@
       </c>
       <c r="I426" s="2" t="inlineStr">
         <is>
-          <t>15/07/2026 23:21</t>
+          <t>09/07/2026 05:48</t>
         </is>
       </c>
       <c r="J426" s="2" t="inlineStr">
         <is>
-          <t>17/07/2026 12:20</t>
+          <t>10/07/2026 17:00</t>
         </is>
       </c>
       <c r="K426" s="2" t="inlineStr">
         <is>
-          <t>15/07/2026 23:21</t>
+          <t>09/07/2026 05:48</t>
         </is>
       </c>
       <c r="L426" s="2" t="inlineStr">
         <is>
-          <t>17/07/2026 12:20</t>
+          <t>10/07/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -26866,52 +26866,52 @@
       </c>
       <c r="C427" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D427" s="2" t="inlineStr">
         <is>
-          <t>559319</t>
+          <t>559880</t>
         </is>
       </c>
       <c r="E427" s="2" t="inlineStr">
         <is>
-          <t>SP</t>
+          <t>SC</t>
         </is>
       </c>
       <c r="F427" s="2" t="inlineStr">
         <is>
-          <t>A8356</t>
+          <t>TA0241</t>
         </is>
       </c>
       <c r="G427" s="2" t="inlineStr">
         <is>
-          <t>00019200000013247638</t>
+          <t>00019200000013407210</t>
         </is>
       </c>
       <c r="H427" s="2" t="inlineStr">
         <is>
-          <t>Rodoviário</t>
+          <t>MultiModal</t>
         </is>
       </c>
       <c r="I427" s="2" t="inlineStr">
         <is>
-          <t>01/07/2026 03:55</t>
+          <t>09/07/2026 05:48</t>
         </is>
       </c>
       <c r="J427" s="2" t="inlineStr">
         <is>
-          <t>01/07/2026 13:54</t>
+          <t>10/07/2026 17:00</t>
         </is>
       </c>
       <c r="K427" s="2" t="inlineStr">
         <is>
-          <t>01/07/2026 03:55</t>
+          <t>09/07/2026 05:48</t>
         </is>
       </c>
       <c r="L427" s="2" t="inlineStr">
         <is>
-          <t>01/07/2026 13:54</t>
+          <t>10/07/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -26928,52 +26928,52 @@
       </c>
       <c r="C428" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D428" s="2" t="inlineStr">
         <is>
-          <t>559697</t>
+          <t>559876</t>
         </is>
       </c>
       <c r="E428" s="2" t="inlineStr">
         <is>
-          <t>SP</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="F428" s="2" t="inlineStr">
         <is>
-          <t>A5033</t>
+          <t>A1817</t>
         </is>
       </c>
       <c r="G428" s="2" t="inlineStr">
         <is>
-          <t>00019200000013422723</t>
+          <t>00019200000013419021</t>
         </is>
       </c>
       <c r="H428" s="2" t="inlineStr">
         <is>
-          <t>Rodoviário</t>
+          <t>MultiModal</t>
         </is>
       </c>
       <c r="I428" s="2" t="inlineStr">
         <is>
-          <t>03/07/2026 05:14</t>
+          <t>07/07/2026 00:57</t>
         </is>
       </c>
       <c r="J428" s="2" t="inlineStr">
         <is>
-          <t>03/07/2026 12:42</t>
+          <t>17/07/2026 15:00</t>
         </is>
       </c>
       <c r="K428" s="2" t="inlineStr">
         <is>
-          <t>03/07/2026 05:14</t>
+          <t>07/07/2026 00:57</t>
         </is>
       </c>
       <c r="L428" s="2" t="inlineStr">
         <is>
-          <t>03/07/2026 12:42</t>
+          <t>17/07/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -26995,47 +26995,47 @@
       </c>
       <c r="D429" s="2" t="inlineStr">
         <is>
-          <t>559870</t>
+          <t>560503</t>
         </is>
       </c>
       <c r="E429" s="2" t="inlineStr">
         <is>
-          <t>SP</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="F429" s="2" t="inlineStr">
         <is>
-          <t>A5209</t>
+          <t>A0727</t>
         </is>
       </c>
       <c r="G429" s="2" t="inlineStr">
         <is>
-          <t>00019200000013415280</t>
+          <t>00019200000013454420</t>
         </is>
       </c>
       <c r="H429" s="2" t="inlineStr">
         <is>
-          <t>Rodoviário</t>
+          <t>MultiModal</t>
         </is>
       </c>
       <c r="I429" s="2" t="inlineStr">
         <is>
-          <t>17/07/2026 04:54</t>
+          <t>15/07/2026 23:21</t>
         </is>
       </c>
       <c r="J429" s="2" t="inlineStr">
         <is>
-          <t>17/07/2026 10:18</t>
+          <t>17/07/2026 12:20</t>
         </is>
       </c>
       <c r="K429" s="2" t="inlineStr">
         <is>
-          <t>17/07/2026 04:54</t>
+          <t>15/07/2026 23:21</t>
         </is>
       </c>
       <c r="L429" s="2" t="inlineStr">
         <is>
-          <t>20/07/2026 14:05</t>
+          <t>17/07/2026 12:20</t>
         </is>
       </c>
     </row>
@@ -27057,7 +27057,7 @@
       </c>
       <c r="D430" s="2" t="inlineStr">
         <is>
-          <t>559870</t>
+          <t>559319</t>
         </is>
       </c>
       <c r="E430" s="2" t="inlineStr">
@@ -27067,12 +27067,12 @@
       </c>
       <c r="F430" s="2" t="inlineStr">
         <is>
-          <t>A4755</t>
+          <t>A8356</t>
         </is>
       </c>
       <c r="G430" s="2" t="inlineStr">
         <is>
-          <t>00019200000013415298</t>
+          <t>00019200000013247638</t>
         </is>
       </c>
       <c r="H430" s="2" t="inlineStr">
@@ -27082,22 +27082,22 @@
       </c>
       <c r="I430" s="2" t="inlineStr">
         <is>
-          <t>17/07/2026 04:54</t>
+          <t>01/07/2026 03:55</t>
         </is>
       </c>
       <c r="J430" s="2" t="inlineStr">
         <is>
-          <t>17/07/2026 10:18</t>
+          <t>01/07/2026 13:54</t>
         </is>
       </c>
       <c r="K430" s="2" t="inlineStr">
         <is>
-          <t>17/07/2026 04:54</t>
+          <t>01/07/2026 03:55</t>
         </is>
       </c>
       <c r="L430" s="2" t="inlineStr">
         <is>
-          <t>20/07/2026 14:05</t>
+          <t>01/07/2026 13:54</t>
         </is>
       </c>
     </row>
@@ -27114,12 +27114,12 @@
       </c>
       <c r="C431" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D431" s="2" t="inlineStr">
         <is>
-          <t>559870</t>
+          <t>559697</t>
         </is>
       </c>
       <c r="E431" s="2" t="inlineStr">
@@ -27129,12 +27129,12 @@
       </c>
       <c r="F431" s="2" t="inlineStr">
         <is>
-          <t>A4555</t>
+          <t>A5033</t>
         </is>
       </c>
       <c r="G431" s="2" t="inlineStr">
         <is>
-          <t>00019200000013415301</t>
+          <t>00019200000013422723</t>
         </is>
       </c>
       <c r="H431" s="2" t="inlineStr">
@@ -27144,22 +27144,22 @@
       </c>
       <c r="I431" s="2" t="inlineStr">
         <is>
-          <t>17/07/2026 04:54</t>
+          <t>03/07/2026 05:14</t>
         </is>
       </c>
       <c r="J431" s="2" t="inlineStr">
         <is>
-          <t>17/07/2026 10:18</t>
+          <t>03/07/2026 12:42</t>
         </is>
       </c>
       <c r="K431" s="2" t="inlineStr">
         <is>
-          <t>17/07/2026 04:54</t>
+          <t>03/07/2026 05:14</t>
         </is>
       </c>
       <c r="L431" s="2" t="inlineStr">
         <is>
-          <t>20/07/2026 14:05</t>
+          <t>03/07/2026 12:42</t>
         </is>
       </c>
     </row>
@@ -27176,7 +27176,7 @@
       </c>
       <c r="C432" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D432" s="2" t="inlineStr">
@@ -27191,12 +27191,12 @@
       </c>
       <c r="F432" s="2" t="inlineStr">
         <is>
-          <t>A4843</t>
+          <t>A5209</t>
         </is>
       </c>
       <c r="G432" s="2" t="inlineStr">
         <is>
-          <t>00019200000013415310</t>
+          <t>00019200000013415280</t>
         </is>
       </c>
       <c r="H432" s="2" t="inlineStr">
@@ -27238,12 +27238,12 @@
       </c>
       <c r="C433" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D433" s="2" t="inlineStr">
         <is>
-          <t>560113</t>
+          <t>559870</t>
         </is>
       </c>
       <c r="E433" s="2" t="inlineStr">
@@ -27253,12 +27253,12 @@
       </c>
       <c r="F433" s="2" t="inlineStr">
         <is>
-          <t>A3818</t>
+          <t>A4755</t>
         </is>
       </c>
       <c r="G433" s="2" t="inlineStr">
         <is>
-          <t>00019200000013451758</t>
+          <t>00019200000013415298</t>
         </is>
       </c>
       <c r="H433" s="2" t="inlineStr">
@@ -27268,22 +27268,22 @@
       </c>
       <c r="I433" s="2" t="inlineStr">
         <is>
-          <t>15/07/2026 02:34</t>
+          <t>17/07/2026 04:54</t>
         </is>
       </c>
       <c r="J433" s="2" t="inlineStr">
         <is>
-          <t>15/07/2026 10:05</t>
+          <t>17/07/2026 10:18</t>
         </is>
       </c>
       <c r="K433" s="2" t="inlineStr">
         <is>
-          <t>15/07/2026 02:34</t>
+          <t>17/07/2026 04:54</t>
         </is>
       </c>
       <c r="L433" s="2" t="inlineStr">
         <is>
-          <t>15/07/2026 10:05</t>
+          <t>20/07/2026 14:05</t>
         </is>
       </c>
     </row>
@@ -27300,12 +27300,12 @@
       </c>
       <c r="C434" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D434" s="2" t="inlineStr">
         <is>
-          <t>561125</t>
+          <t>559870</t>
         </is>
       </c>
       <c r="E434" s="2" t="inlineStr">
@@ -27315,12 +27315,12 @@
       </c>
       <c r="F434" s="2" t="inlineStr">
         <is>
-          <t>A8303</t>
+          <t>A4555</t>
         </is>
       </c>
       <c r="G434" s="2" t="inlineStr">
         <is>
-          <t>00019200000013478745</t>
+          <t>00019200000013415301</t>
         </is>
       </c>
       <c r="H434" s="2" t="inlineStr">
@@ -27330,22 +27330,22 @@
       </c>
       <c r="I434" s="2" t="inlineStr">
         <is>
-          <t>16/07/2026 01:43</t>
+          <t>17/07/2026 04:54</t>
         </is>
       </c>
       <c r="J434" s="2" t="inlineStr">
         <is>
-          <t>16/07/2026 09:34</t>
+          <t>17/07/2026 10:18</t>
         </is>
       </c>
       <c r="K434" s="2" t="inlineStr">
         <is>
-          <t>16/07/2026 01:43</t>
+          <t>17/07/2026 04:54</t>
         </is>
       </c>
       <c r="L434" s="2" t="inlineStr">
         <is>
-          <t>16/07/2026 09:34</t>
+          <t>20/07/2026 14:05</t>
         </is>
       </c>
     </row>
@@ -27362,12 +27362,12 @@
       </c>
       <c r="C435" s="2" t="inlineStr">
         <is>
-          <t>-90 C a -60 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D435" s="2" t="inlineStr">
         <is>
-          <t>561435</t>
+          <t>559870</t>
         </is>
       </c>
       <c r="E435" s="2" t="inlineStr">
@@ -27377,12 +27377,12 @@
       </c>
       <c r="F435" s="2" t="inlineStr">
         <is>
-          <t>869170035491621</t>
+          <t>A4843</t>
         </is>
       </c>
       <c r="G435" s="2" t="inlineStr">
         <is>
-          <t>00019200000013751824</t>
+          <t>00019200000013415310</t>
         </is>
       </c>
       <c r="H435" s="2" t="inlineStr">
@@ -27392,22 +27392,22 @@
       </c>
       <c r="I435" s="2" t="inlineStr">
         <is>
-          <t>27/07/2026 01:06</t>
+          <t>17/07/2026 04:54</t>
         </is>
       </c>
       <c r="J435" s="2" t="inlineStr">
         <is>
-          <t>27/07/2026 09:08</t>
+          <t>17/07/2026 10:18</t>
         </is>
       </c>
       <c r="K435" s="2" t="inlineStr">
         <is>
-          <t>27/07/2026 01:06</t>
+          <t>17/07/2026 04:54</t>
         </is>
       </c>
       <c r="L435" s="2" t="inlineStr">
         <is>
-          <t>27/07/2026 09:11</t>
+          <t>20/07/2026 14:05</t>
         </is>
       </c>
     </row>
@@ -27424,12 +27424,12 @@
       </c>
       <c r="C436" s="2" t="inlineStr">
         <is>
-          <t>-90 C a -60 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D436" s="2" t="inlineStr">
         <is>
-          <t>561435</t>
+          <t>560113</t>
         </is>
       </c>
       <c r="E436" s="2" t="inlineStr">
@@ -27439,12 +27439,12 @@
       </c>
       <c r="F436" s="2" t="inlineStr">
         <is>
-          <t>869170034887332</t>
+          <t>A3818</t>
         </is>
       </c>
       <c r="G436" s="2" t="inlineStr">
         <is>
-          <t>00019200000013751832</t>
+          <t>00019200000013451758</t>
         </is>
       </c>
       <c r="H436" s="2" t="inlineStr">
@@ -27454,22 +27454,22 @@
       </c>
       <c r="I436" s="2" t="inlineStr">
         <is>
-          <t>27/07/2026 01:06</t>
+          <t>15/07/2026 02:34</t>
         </is>
       </c>
       <c r="J436" s="2" t="inlineStr">
         <is>
-          <t>27/07/2026 09:08</t>
+          <t>15/07/2026 10:05</t>
         </is>
       </c>
       <c r="K436" s="2" t="inlineStr">
         <is>
-          <t>27/07/2026 01:06</t>
+          <t>15/07/2026 02:34</t>
         </is>
       </c>
       <c r="L436" s="2" t="inlineStr">
         <is>
-          <t>27/07/2026 09:11</t>
+          <t>15/07/2026 10:05</t>
         </is>
       </c>
     </row>
@@ -27486,12 +27486,12 @@
       </c>
       <c r="C437" s="2" t="inlineStr">
         <is>
-          <t>-90 C a -60 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D437" s="2" t="inlineStr">
         <is>
-          <t>561435</t>
+          <t>561125</t>
         </is>
       </c>
       <c r="E437" s="2" t="inlineStr">
@@ -27501,12 +27501,12 @@
       </c>
       <c r="F437" s="2" t="inlineStr">
         <is>
-          <t>869170034874710</t>
+          <t>A8303</t>
         </is>
       </c>
       <c r="G437" s="2" t="inlineStr">
         <is>
-          <t>00019200000013751840</t>
+          <t>00019200000013478745</t>
         </is>
       </c>
       <c r="H437" s="2" t="inlineStr">
@@ -27516,22 +27516,22 @@
       </c>
       <c r="I437" s="2" t="inlineStr">
         <is>
-          <t>27/07/2026 01:06</t>
+          <t>16/07/2026 01:43</t>
         </is>
       </c>
       <c r="J437" s="2" t="inlineStr">
         <is>
-          <t>27/07/2026 09:08</t>
+          <t>16/07/2026 09:34</t>
         </is>
       </c>
       <c r="K437" s="2" t="inlineStr">
         <is>
-          <t>27/07/2026 01:06</t>
+          <t>16/07/2026 01:43</t>
         </is>
       </c>
       <c r="L437" s="2" t="inlineStr">
         <is>
-          <t>27/07/2026 09:11</t>
+          <t>16/07/2026 09:34</t>
         </is>
       </c>
     </row>
@@ -27563,12 +27563,12 @@
       </c>
       <c r="F438" s="2" t="inlineStr">
         <is>
-          <t>869170035511287</t>
+          <t>869170035491621</t>
         </is>
       </c>
       <c r="G438" s="2" t="inlineStr">
         <is>
-          <t>00019200000013751859</t>
+          <t>00019200000013751824</t>
         </is>
       </c>
       <c r="H438" s="2" t="inlineStr">
@@ -27625,12 +27625,12 @@
       </c>
       <c r="F439" s="2" t="inlineStr">
         <is>
-          <t>869170035511360</t>
+          <t>869170034887332</t>
         </is>
       </c>
       <c r="G439" s="2" t="inlineStr">
         <is>
-          <t>00019200000013751867</t>
+          <t>00019200000013751832</t>
         </is>
       </c>
       <c r="H439" s="2" t="inlineStr">
@@ -27687,12 +27687,12 @@
       </c>
       <c r="F440" s="2" t="inlineStr">
         <is>
-          <t>869170035518605</t>
+          <t>869170034874710</t>
         </is>
       </c>
       <c r="G440" s="2" t="inlineStr">
         <is>
-          <t>00019200000013751875</t>
+          <t>00019200000013751840</t>
         </is>
       </c>
       <c r="H440" s="2" t="inlineStr">
@@ -27734,12 +27734,12 @@
       </c>
       <c r="C441" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-90 C a -60 C</t>
         </is>
       </c>
       <c r="D441" s="2" t="inlineStr">
         <is>
-          <t>562000</t>
+          <t>561435</t>
         </is>
       </c>
       <c r="E441" s="2" t="inlineStr">
@@ -27749,12 +27749,12 @@
       </c>
       <c r="F441" s="2" t="inlineStr">
         <is>
-          <t>A3766</t>
+          <t>869170035511287</t>
         </is>
       </c>
       <c r="G441" s="2" t="inlineStr">
         <is>
-          <t>00019200000013595202</t>
+          <t>00019200000013751859</t>
         </is>
       </c>
       <c r="H441" s="2" t="inlineStr">
@@ -27764,22 +27764,22 @@
       </c>
       <c r="I441" s="2" t="inlineStr">
         <is>
-          <t>23/07/2026 03:21</t>
+          <t>27/07/2026 01:06</t>
         </is>
       </c>
       <c r="J441" s="2" t="inlineStr">
         <is>
-          <t>23/07/2026 12:49</t>
+          <t>27/07/2026 09:08</t>
         </is>
       </c>
       <c r="K441" s="2" t="inlineStr">
         <is>
-          <t>23/07/2026 03:21</t>
+          <t>27/07/2026 01:06</t>
         </is>
       </c>
       <c r="L441" s="2" t="inlineStr">
         <is>
-          <t>23/07/2026 12:49</t>
+          <t>27/07/2026 09:11</t>
         </is>
       </c>
     </row>
@@ -27796,52 +27796,52 @@
       </c>
       <c r="C442" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-90 C a -60 C</t>
         </is>
       </c>
       <c r="D442" s="2" t="inlineStr">
         <is>
-          <t>559781</t>
+          <t>561435</t>
         </is>
       </c>
       <c r="E442" s="2" t="inlineStr">
         <is>
-          <t>TO</t>
+          <t>SP</t>
         </is>
       </c>
       <c r="F442" s="2" t="inlineStr">
         <is>
-          <t>A8445</t>
+          <t>869170035511360</t>
         </is>
       </c>
       <c r="G442" s="2" t="inlineStr">
         <is>
-          <t>00019200000013419129</t>
+          <t>00019200000013751867</t>
         </is>
       </c>
       <c r="H442" s="2" t="inlineStr">
         <is>
-          <t>MultiModal</t>
+          <t>Rodoviário</t>
         </is>
       </c>
       <c r="I442" s="2" t="inlineStr">
         <is>
-          <t>07/07/2026 01:13</t>
+          <t>27/07/2026 01:06</t>
         </is>
       </c>
       <c r="J442" s="2" t="inlineStr">
         <is>
-          <t>08/07/2026 18:00</t>
+          <t>27/07/2026 09:08</t>
         </is>
       </c>
       <c r="K442" s="2" t="inlineStr">
         <is>
-          <t>07/07/2026 01:13</t>
+          <t>27/07/2026 01:06</t>
         </is>
       </c>
       <c r="L442" s="2" t="inlineStr">
         <is>
-          <t>08/07/2026 18:00</t>
+          <t>27/07/2026 09:11</t>
         </is>
       </c>
     </row>
@@ -27858,57 +27858,243 @@
       </c>
       <c r="C443" s="2" t="inlineStr">
         <is>
+          <t>-90 C a -60 C</t>
+        </is>
+      </c>
+      <c r="D443" s="2" t="inlineStr">
+        <is>
+          <t>561435</t>
+        </is>
+      </c>
+      <c r="E443" s="2" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F443" s="2" t="inlineStr">
+        <is>
+          <t>869170035518605</t>
+        </is>
+      </c>
+      <c r="G443" s="2" t="inlineStr">
+        <is>
+          <t>00019200000013751875</t>
+        </is>
+      </c>
+      <c r="H443" s="2" t="inlineStr">
+        <is>
+          <t>Rodoviário</t>
+        </is>
+      </c>
+      <c r="I443" s="2" t="inlineStr">
+        <is>
+          <t>27/07/2026 01:06</t>
+        </is>
+      </c>
+      <c r="J443" s="2" t="inlineStr">
+        <is>
+          <t>27/07/2026 09:08</t>
+        </is>
+      </c>
+      <c r="K443" s="2" t="inlineStr">
+        <is>
+          <t>27/07/2026 01:06</t>
+        </is>
+      </c>
+      <c r="L443" s="2" t="inlineStr">
+        <is>
+          <t>27/07/2026 09:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" s="2" t="inlineStr">
+        <is>
+          <t>CAIXA 42L</t>
+        </is>
+      </c>
+      <c r="B444" s="2" t="inlineStr">
+        <is>
+          <t>CAIXA 42L SEM BERÇO</t>
+        </is>
+      </c>
+      <c r="C444" s="2" t="inlineStr">
+        <is>
+          <t>-15 C a -30 C</t>
+        </is>
+      </c>
+      <c r="D444" s="2" t="inlineStr">
+        <is>
+          <t>562000</t>
+        </is>
+      </c>
+      <c r="E444" s="2" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F444" s="2" t="inlineStr">
+        <is>
+          <t>A3766</t>
+        </is>
+      </c>
+      <c r="G444" s="2" t="inlineStr">
+        <is>
+          <t>00019200000013595202</t>
+        </is>
+      </c>
+      <c r="H444" s="2" t="inlineStr">
+        <is>
+          <t>Rodoviário</t>
+        </is>
+      </c>
+      <c r="I444" s="2" t="inlineStr">
+        <is>
+          <t>23/07/2026 03:21</t>
+        </is>
+      </c>
+      <c r="J444" s="2" t="inlineStr">
+        <is>
+          <t>23/07/2026 12:49</t>
+        </is>
+      </c>
+      <c r="K444" s="2" t="inlineStr">
+        <is>
+          <t>23/07/2026 03:21</t>
+        </is>
+      </c>
+      <c r="L444" s="2" t="inlineStr">
+        <is>
+          <t>23/07/2026 12:49</t>
+        </is>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" s="2" t="inlineStr">
+        <is>
+          <t>CAIXA 42L</t>
+        </is>
+      </c>
+      <c r="B445" s="2" t="inlineStr">
+        <is>
+          <t>CAIXA 42L SEM BERÇO</t>
+        </is>
+      </c>
+      <c r="C445" s="2" t="inlineStr">
+        <is>
+          <t>-35 C a -15 C</t>
+        </is>
+      </c>
+      <c r="D445" s="2" t="inlineStr">
+        <is>
+          <t>559781</t>
+        </is>
+      </c>
+      <c r="E445" s="2" t="inlineStr">
+        <is>
+          <t>TO</t>
+        </is>
+      </c>
+      <c r="F445" s="2" t="inlineStr">
+        <is>
+          <t>A8445</t>
+        </is>
+      </c>
+      <c r="G445" s="2" t="inlineStr">
+        <is>
+          <t>00019200000013419129</t>
+        </is>
+      </c>
+      <c r="H445" s="2" t="inlineStr">
+        <is>
+          <t>MultiModal</t>
+        </is>
+      </c>
+      <c r="I445" s="2" t="inlineStr">
+        <is>
+          <t>07/07/2026 01:13</t>
+        </is>
+      </c>
+      <c r="J445" s="2" t="inlineStr">
+        <is>
+          <t>08/07/2026 18:00</t>
+        </is>
+      </c>
+      <c r="K445" s="2" t="inlineStr">
+        <is>
+          <t>07/07/2026 01:13</t>
+        </is>
+      </c>
+      <c r="L445" s="2" t="inlineStr">
+        <is>
+          <t>08/07/2026 18:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" s="2" t="inlineStr">
+        <is>
+          <t>CAIXA 42L</t>
+        </is>
+      </c>
+      <c r="B446" s="2" t="inlineStr">
+        <is>
+          <t>CAIXA 42L SEM BERÇO</t>
+        </is>
+      </c>
+      <c r="C446" s="2" t="inlineStr">
+        <is>
           <t>-25 C a -15 C</t>
         </is>
       </c>
-      <c r="D443" s="2" t="inlineStr">
+      <c r="D446" s="2" t="inlineStr">
         <is>
           <t>560364</t>
         </is>
       </c>
-      <c r="E443" s="2" t="inlineStr">
+      <c r="E446" s="2" t="inlineStr">
         <is>
           <t>TO</t>
         </is>
       </c>
-      <c r="F443" s="2" t="inlineStr">
+      <c r="F446" s="2" t="inlineStr">
         <is>
           <t>A8870</t>
         </is>
       </c>
-      <c r="G443" s="2" t="inlineStr">
+      <c r="G446" s="2" t="inlineStr">
         <is>
           <t>00019200000013491555</t>
         </is>
       </c>
-      <c r="H443" s="2" t="inlineStr">
-        <is>
-          <t>MultiModal</t>
-        </is>
-      </c>
-      <c r="I443" s="2" t="inlineStr">
+      <c r="H446" s="2" t="inlineStr">
+        <is>
+          <t>MultiModal</t>
+        </is>
+      </c>
+      <c r="I446" s="2" t="inlineStr">
         <is>
           <t>13/07/2026 01:44</t>
         </is>
       </c>
-      <c r="J443" s="2" t="inlineStr">
+      <c r="J446" s="2" t="inlineStr">
         <is>
           <t>15/07/2026 17:22</t>
         </is>
       </c>
-      <c r="K443" s="2" t="inlineStr">
+      <c r="K446" s="2" t="inlineStr">
         <is>
           <t>13/07/2026 01:44</t>
         </is>
       </c>
-      <c r="L443" s="2" t="inlineStr">
+      <c r="L446" s="2" t="inlineStr">
         <is>
           <t>15/07/2026 17:22</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L443"/>
+  <autoFilter ref="A1:L446"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-29 23:11:24
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixas_42l.xlsx
+++ b/relatorio_analitico_caixas_42l.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Caixa 42L" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Caixa 42L'!$A$1:$L$446</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Caixa 42L'!$A$1:$L$447</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L446"/>
+  <dimension ref="A1:L447"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -3740,7 +3740,7 @@
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
@@ -4050,7 +4050,7 @@
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
@@ -4608,7 +4608,7 @@
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
@@ -5910,7 +5910,7 @@
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D89" s="2" t="inlineStr">
@@ -10560,7 +10560,7 @@
       </c>
       <c r="C164" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D164" s="2" t="inlineStr">
@@ -10622,7 +10622,7 @@
       </c>
       <c r="C165" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D165" s="2" t="inlineStr">
@@ -14342,7 +14342,7 @@
       </c>
       <c r="C225" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D225" s="2" t="inlineStr">
@@ -14962,7 +14962,7 @@
       </c>
       <c r="C235" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D235" s="2" t="inlineStr">
@@ -17442,7 +17442,7 @@
       </c>
       <c r="C275" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D275" s="2" t="inlineStr">
@@ -19612,7 +19612,7 @@
       </c>
       <c r="C310" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D310" s="2" t="inlineStr">
@@ -19798,27 +19798,27 @@
       </c>
       <c r="C313" s="2" t="inlineStr">
         <is>
-          <t>-90 C a -60 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D313" s="2" t="inlineStr">
         <is>
-          <t>557493</t>
+          <t>562577</t>
         </is>
       </c>
       <c r="E313" s="2" t="inlineStr">
         <is>
-          <t>RN</t>
+          <t>RJ</t>
         </is>
       </c>
       <c r="F313" s="2" t="inlineStr">
         <is>
-          <t>AS-0511</t>
+          <t>TA0260</t>
         </is>
       </c>
       <c r="G313" s="2" t="inlineStr">
         <is>
-          <t>00019200000013252739</t>
+          <t>00019200000013824139</t>
         </is>
       </c>
       <c r="H313" s="2" t="inlineStr">
@@ -19828,22 +19828,22 @@
       </c>
       <c r="I313" s="2" t="inlineStr">
         <is>
-          <t>01/07/2026 01:19</t>
+          <t>29/07/2026 22:57</t>
         </is>
       </c>
       <c r="J313" s="2" t="inlineStr">
         <is>
-          <t>03/07/2026 15:30</t>
+          <t>-</t>
         </is>
       </c>
       <c r="K313" s="2" t="inlineStr">
         <is>
-          <t>01/07/2026 01:19</t>
+          <t>29/07/2026 22:57</t>
         </is>
       </c>
       <c r="L313" s="2" t="inlineStr">
         <is>
-          <t>03/07/2026 15:30</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -19875,12 +19875,12 @@
       </c>
       <c r="F314" s="2" t="inlineStr">
         <is>
-          <t>AS-0615</t>
+          <t>AS-0511</t>
         </is>
       </c>
       <c r="G314" s="2" t="inlineStr">
         <is>
-          <t>00019200000013252747</t>
+          <t>00019200000013252739</t>
         </is>
       </c>
       <c r="H314" s="2" t="inlineStr">
@@ -19937,12 +19937,12 @@
       </c>
       <c r="F315" s="2" t="inlineStr">
         <is>
-          <t>AS-0425</t>
+          <t>AS-0615</t>
         </is>
       </c>
       <c r="G315" s="2" t="inlineStr">
         <is>
-          <t>00019200000013252755</t>
+          <t>00019200000013252747</t>
         </is>
       </c>
       <c r="H315" s="2" t="inlineStr">
@@ -19999,12 +19999,12 @@
       </c>
       <c r="F316" s="2" t="inlineStr">
         <is>
-          <t>AS-0138</t>
+          <t>AS-0425</t>
         </is>
       </c>
       <c r="G316" s="2" t="inlineStr">
         <is>
-          <t>00019200000013252763</t>
+          <t>00019200000013252755</t>
         </is>
       </c>
       <c r="H316" s="2" t="inlineStr">
@@ -20061,12 +20061,12 @@
       </c>
       <c r="F317" s="2" t="inlineStr">
         <is>
-          <t>AS-0245</t>
+          <t>AS-0138</t>
         </is>
       </c>
       <c r="G317" s="2" t="inlineStr">
         <is>
-          <t>00019200000013252771</t>
+          <t>00019200000013252763</t>
         </is>
       </c>
       <c r="H317" s="2" t="inlineStr">
@@ -20123,12 +20123,12 @@
       </c>
       <c r="F318" s="2" t="inlineStr">
         <is>
-          <t>AS-0762</t>
+          <t>AS-0245</t>
         </is>
       </c>
       <c r="G318" s="2" t="inlineStr">
         <is>
-          <t>00019200000013252780</t>
+          <t>00019200000013252771</t>
         </is>
       </c>
       <c r="H318" s="2" t="inlineStr">
@@ -20185,12 +20185,12 @@
       </c>
       <c r="F319" s="2" t="inlineStr">
         <is>
-          <t>AS-0462</t>
+          <t>AS-0762</t>
         </is>
       </c>
       <c r="G319" s="2" t="inlineStr">
         <is>
-          <t>00019200000013252798</t>
+          <t>00019200000013252780</t>
         </is>
       </c>
       <c r="H319" s="2" t="inlineStr">
@@ -20247,12 +20247,12 @@
       </c>
       <c r="F320" s="2" t="inlineStr">
         <is>
-          <t>AS-0702</t>
+          <t>AS-0462</t>
         </is>
       </c>
       <c r="G320" s="2" t="inlineStr">
         <is>
-          <t>00019200000013252801</t>
+          <t>00019200000013252798</t>
         </is>
       </c>
       <c r="H320" s="2" t="inlineStr">
@@ -20309,12 +20309,12 @@
       </c>
       <c r="F321" s="2" t="inlineStr">
         <is>
-          <t>AS-0513</t>
+          <t>AS-0702</t>
         </is>
       </c>
       <c r="G321" s="2" t="inlineStr">
         <is>
-          <t>00019200000013254510</t>
+          <t>00019200000013252801</t>
         </is>
       </c>
       <c r="H321" s="2" t="inlineStr">
@@ -20371,12 +20371,12 @@
       </c>
       <c r="F322" s="2" t="inlineStr">
         <is>
-          <t>AS-0172</t>
+          <t>AS-0513</t>
         </is>
       </c>
       <c r="G322" s="2" t="inlineStr">
         <is>
-          <t>00019200000013254529</t>
+          <t>00019200000013254510</t>
         </is>
       </c>
       <c r="H322" s="2" t="inlineStr">
@@ -20433,12 +20433,12 @@
       </c>
       <c r="F323" s="2" t="inlineStr">
         <is>
-          <t>AS-0019</t>
+          <t>AS-0172</t>
         </is>
       </c>
       <c r="G323" s="2" t="inlineStr">
         <is>
-          <t>00019200000013429450</t>
+          <t>00019200000013254529</t>
         </is>
       </c>
       <c r="H323" s="2" t="inlineStr">
@@ -20495,12 +20495,12 @@
       </c>
       <c r="F324" s="2" t="inlineStr">
         <is>
-          <t>AS-0426</t>
+          <t>AS-0019</t>
         </is>
       </c>
       <c r="G324" s="2" t="inlineStr">
         <is>
-          <t>00019200000013429469</t>
+          <t>00019200000013429450</t>
         </is>
       </c>
       <c r="H324" s="2" t="inlineStr">
@@ -20557,12 +20557,12 @@
       </c>
       <c r="F325" s="2" t="inlineStr">
         <is>
-          <t>AS-0699</t>
+          <t>AS-0426</t>
         </is>
       </c>
       <c r="G325" s="2" t="inlineStr">
         <is>
-          <t>00019200000013429477</t>
+          <t>00019200000013429469</t>
         </is>
       </c>
       <c r="H325" s="2" t="inlineStr">
@@ -20619,12 +20619,12 @@
       </c>
       <c r="F326" s="2" t="inlineStr">
         <is>
-          <t>AS-0376</t>
+          <t>AS-0699</t>
         </is>
       </c>
       <c r="G326" s="2" t="inlineStr">
         <is>
-          <t>00019200000013429485</t>
+          <t>00019200000013429477</t>
         </is>
       </c>
       <c r="H326" s="2" t="inlineStr">
@@ -20681,12 +20681,12 @@
       </c>
       <c r="F327" s="2" t="inlineStr">
         <is>
-          <t>AS-0683</t>
+          <t>AS-0376</t>
         </is>
       </c>
       <c r="G327" s="2" t="inlineStr">
         <is>
-          <t>00019200000013429493</t>
+          <t>00019200000013429485</t>
         </is>
       </c>
       <c r="H327" s="2" t="inlineStr">
@@ -20743,12 +20743,12 @@
       </c>
       <c r="F328" s="2" t="inlineStr">
         <is>
-          <t>AS-0078</t>
+          <t>AS-0683</t>
         </is>
       </c>
       <c r="G328" s="2" t="inlineStr">
         <is>
-          <t>00019200000013429507</t>
+          <t>00019200000013429493</t>
         </is>
       </c>
       <c r="H328" s="2" t="inlineStr">
@@ -20805,12 +20805,12 @@
       </c>
       <c r="F329" s="2" t="inlineStr">
         <is>
-          <t>AS-0077</t>
+          <t>AS-0078</t>
         </is>
       </c>
       <c r="G329" s="2" t="inlineStr">
         <is>
-          <t>00019200000013429515</t>
+          <t>00019200000013429507</t>
         </is>
       </c>
       <c r="H329" s="2" t="inlineStr">
@@ -20867,12 +20867,12 @@
       </c>
       <c r="F330" s="2" t="inlineStr">
         <is>
-          <t>AS-0499</t>
+          <t>AS-0077</t>
         </is>
       </c>
       <c r="G330" s="2" t="inlineStr">
         <is>
-          <t>00019200000013429523</t>
+          <t>00019200000013429515</t>
         </is>
       </c>
       <c r="H330" s="2" t="inlineStr">
@@ -20929,12 +20929,12 @@
       </c>
       <c r="F331" s="2" t="inlineStr">
         <is>
-          <t>AS-0518</t>
+          <t>AS-0499</t>
         </is>
       </c>
       <c r="G331" s="2" t="inlineStr">
         <is>
-          <t>00019200000013429531</t>
+          <t>00019200000013429523</t>
         </is>
       </c>
       <c r="H331" s="2" t="inlineStr">
@@ -20991,12 +20991,12 @@
       </c>
       <c r="F332" s="2" t="inlineStr">
         <is>
-          <t>AS-0494</t>
+          <t>AS-0518</t>
         </is>
       </c>
       <c r="G332" s="2" t="inlineStr">
         <is>
-          <t>00019200000013429540</t>
+          <t>00019200000013429531</t>
         </is>
       </c>
       <c r="H332" s="2" t="inlineStr">
@@ -21053,12 +21053,12 @@
       </c>
       <c r="F333" s="2" t="inlineStr">
         <is>
-          <t>AS-0269</t>
+          <t>AS-0494</t>
         </is>
       </c>
       <c r="G333" s="2" t="inlineStr">
         <is>
-          <t>00019200000013429558</t>
+          <t>00019200000013429540</t>
         </is>
       </c>
       <c r="H333" s="2" t="inlineStr">
@@ -21115,12 +21115,12 @@
       </c>
       <c r="F334" s="2" t="inlineStr">
         <is>
-          <t>AS-0201</t>
+          <t>AS-0269</t>
         </is>
       </c>
       <c r="G334" s="2" t="inlineStr">
         <is>
-          <t>00019200000013429566</t>
+          <t>00019200000013429558</t>
         </is>
       </c>
       <c r="H334" s="2" t="inlineStr">
@@ -21162,12 +21162,12 @@
       </c>
       <c r="C335" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-90 C a -60 C</t>
         </is>
       </c>
       <c r="D335" s="2" t="inlineStr">
         <is>
-          <t>559981</t>
+          <t>557493</t>
         </is>
       </c>
       <c r="E335" s="2" t="inlineStr">
@@ -21177,12 +21177,12 @@
       </c>
       <c r="F335" s="2" t="inlineStr">
         <is>
-          <t>A6263</t>
+          <t>AS-0201</t>
         </is>
       </c>
       <c r="G335" s="2" t="inlineStr">
         <is>
-          <t>00019200000013419153</t>
+          <t>00019200000013429566</t>
         </is>
       </c>
       <c r="H335" s="2" t="inlineStr">
@@ -21192,22 +21192,22 @@
       </c>
       <c r="I335" s="2" t="inlineStr">
         <is>
-          <t>07/07/2026 05:52</t>
+          <t>01/07/2026 01:19</t>
         </is>
       </c>
       <c r="J335" s="2" t="inlineStr">
         <is>
-          <t>08/07/2026 17:32</t>
+          <t>03/07/2026 15:30</t>
         </is>
       </c>
       <c r="K335" s="2" t="inlineStr">
         <is>
-          <t>07/07/2026 05:52</t>
+          <t>01/07/2026 01:19</t>
         </is>
       </c>
       <c r="L335" s="2" t="inlineStr">
         <is>
-          <t>08/07/2026 17:32</t>
+          <t>03/07/2026 15:30</t>
         </is>
       </c>
     </row>
@@ -21224,12 +21224,12 @@
       </c>
       <c r="C336" s="2" t="inlineStr">
         <is>
-          <t>-90 C a -60 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D336" s="2" t="inlineStr">
         <is>
-          <t>560570</t>
+          <t>559981</t>
         </is>
       </c>
       <c r="E336" s="2" t="inlineStr">
@@ -21239,12 +21239,12 @@
       </c>
       <c r="F336" s="2" t="inlineStr">
         <is>
-          <t>869170034877747</t>
+          <t>A6263</t>
         </is>
       </c>
       <c r="G336" s="2" t="inlineStr">
         <is>
-          <t>00019200000013776150</t>
+          <t>00019200000013419153</t>
         </is>
       </c>
       <c r="H336" s="2" t="inlineStr">
@@ -21254,22 +21254,22 @@
       </c>
       <c r="I336" s="2" t="inlineStr">
         <is>
-          <t>27/07/2026 22:34</t>
+          <t>07/07/2026 05:52</t>
         </is>
       </c>
       <c r="J336" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>08/07/2026 17:32</t>
         </is>
       </c>
       <c r="K336" s="2" t="inlineStr">
         <is>
-          <t>27/07/2026 22:34</t>
+          <t>07/07/2026 05:52</t>
         </is>
       </c>
       <c r="L336" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>08/07/2026 17:32</t>
         </is>
       </c>
     </row>
@@ -21301,12 +21301,12 @@
       </c>
       <c r="F337" s="2" t="inlineStr">
         <is>
-          <t>300100</t>
+          <t>869170034877747</t>
         </is>
       </c>
       <c r="G337" s="2" t="inlineStr">
         <is>
-          <t>00019200000013776169</t>
+          <t>00019200000013776150</t>
         </is>
       </c>
       <c r="H337" s="2" t="inlineStr">
@@ -21363,12 +21363,12 @@
       </c>
       <c r="F338" s="2" t="inlineStr">
         <is>
-          <t>300054</t>
+          <t>300100</t>
         </is>
       </c>
       <c r="G338" s="2" t="inlineStr">
         <is>
-          <t>00019200000013776177</t>
+          <t>00019200000013776169</t>
         </is>
       </c>
       <c r="H338" s="2" t="inlineStr">
@@ -21425,12 +21425,12 @@
       </c>
       <c r="F339" s="2" t="inlineStr">
         <is>
-          <t>300056</t>
+          <t>300054</t>
         </is>
       </c>
       <c r="G339" s="2" t="inlineStr">
         <is>
-          <t>00019200000013776185</t>
+          <t>00019200000013776177</t>
         </is>
       </c>
       <c r="H339" s="2" t="inlineStr">
@@ -21487,12 +21487,12 @@
       </c>
       <c r="F340" s="2" t="inlineStr">
         <is>
-          <t>300163</t>
+          <t>300056</t>
         </is>
       </c>
       <c r="G340" s="2" t="inlineStr">
         <is>
-          <t>00019200000013776193</t>
+          <t>00019200000013776185</t>
         </is>
       </c>
       <c r="H340" s="2" t="inlineStr">
@@ -21549,12 +21549,12 @@
       </c>
       <c r="F341" s="2" t="inlineStr">
         <is>
-          <t>300059</t>
+          <t>300163</t>
         </is>
       </c>
       <c r="G341" s="2" t="inlineStr">
         <is>
-          <t>00019200000013776207</t>
+          <t>00019200000013776193</t>
         </is>
       </c>
       <c r="H341" s="2" t="inlineStr">
@@ -21611,12 +21611,12 @@
       </c>
       <c r="F342" s="2" t="inlineStr">
         <is>
-          <t>869170035504837</t>
+          <t>300059</t>
         </is>
       </c>
       <c r="G342" s="2" t="inlineStr">
         <is>
-          <t>00019200000013776215</t>
+          <t>00019200000013776207</t>
         </is>
       </c>
       <c r="H342" s="2" t="inlineStr">
@@ -21673,12 +21673,12 @@
       </c>
       <c r="F343" s="2" t="inlineStr">
         <is>
-          <t>869170035520866</t>
+          <t>869170035504837</t>
         </is>
       </c>
       <c r="G343" s="2" t="inlineStr">
         <is>
-          <t>00019200000013776223</t>
+          <t>00019200000013776215</t>
         </is>
       </c>
       <c r="H343" s="2" t="inlineStr">
@@ -21735,12 +21735,12 @@
       </c>
       <c r="F344" s="2" t="inlineStr">
         <is>
-          <t>869170035517771</t>
+          <t>869170035520866</t>
         </is>
       </c>
       <c r="G344" s="2" t="inlineStr">
         <is>
-          <t>00019200000013776231</t>
+          <t>00019200000013776223</t>
         </is>
       </c>
       <c r="H344" s="2" t="inlineStr">
@@ -21797,12 +21797,12 @@
       </c>
       <c r="F345" s="2" t="inlineStr">
         <is>
-          <t>869170034881269</t>
+          <t>869170035517771</t>
         </is>
       </c>
       <c r="G345" s="2" t="inlineStr">
         <is>
-          <t>00019200000013776240</t>
+          <t>00019200000013776231</t>
         </is>
       </c>
       <c r="H345" s="2" t="inlineStr">
@@ -21859,12 +21859,12 @@
       </c>
       <c r="F346" s="2" t="inlineStr">
         <is>
-          <t>869170034876806</t>
+          <t>869170034881269</t>
         </is>
       </c>
       <c r="G346" s="2" t="inlineStr">
         <is>
-          <t>00019200000013776258</t>
+          <t>00019200000013776240</t>
         </is>
       </c>
       <c r="H346" s="2" t="inlineStr">
@@ -21921,12 +21921,12 @@
       </c>
       <c r="F347" s="2" t="inlineStr">
         <is>
-          <t>AS-0213</t>
+          <t>869170034876806</t>
         </is>
       </c>
       <c r="G347" s="2" t="inlineStr">
         <is>
-          <t>00019200000013776266</t>
+          <t>00019200000013776258</t>
         </is>
       </c>
       <c r="H347" s="2" t="inlineStr">
@@ -21983,12 +21983,12 @@
       </c>
       <c r="F348" s="2" t="inlineStr">
         <is>
-          <t>300027</t>
+          <t>AS-0213</t>
         </is>
       </c>
       <c r="G348" s="2" t="inlineStr">
         <is>
-          <t>00019200000013776274</t>
+          <t>00019200000013776266</t>
         </is>
       </c>
       <c r="H348" s="2" t="inlineStr">
@@ -22045,12 +22045,12 @@
       </c>
       <c r="F349" s="2" t="inlineStr">
         <is>
-          <t>300173</t>
+          <t>300027</t>
         </is>
       </c>
       <c r="G349" s="2" t="inlineStr">
         <is>
-          <t>00019200000013776282</t>
+          <t>00019200000013776274</t>
         </is>
       </c>
       <c r="H349" s="2" t="inlineStr">
@@ -22107,12 +22107,12 @@
       </c>
       <c r="F350" s="2" t="inlineStr">
         <is>
-          <t>300181</t>
+          <t>300173</t>
         </is>
       </c>
       <c r="G350" s="2" t="inlineStr">
         <is>
-          <t>00019200000013776290</t>
+          <t>00019200000013776282</t>
         </is>
       </c>
       <c r="H350" s="2" t="inlineStr">
@@ -22154,27 +22154,27 @@
       </c>
       <c r="C351" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-90 C a -60 C</t>
         </is>
       </c>
       <c r="D351" s="2" t="inlineStr">
         <is>
-          <t>559957</t>
+          <t>560570</t>
         </is>
       </c>
       <c r="E351" s="2" t="inlineStr">
         <is>
-          <t>RO</t>
+          <t>RN</t>
         </is>
       </c>
       <c r="F351" s="2" t="inlineStr">
         <is>
-          <t>A9354</t>
+          <t>300181</t>
         </is>
       </c>
       <c r="G351" s="2" t="inlineStr">
         <is>
-          <t>00019200000013418211</t>
+          <t>00019200000013776290</t>
         </is>
       </c>
       <c r="H351" s="2" t="inlineStr">
@@ -22184,22 +22184,22 @@
       </c>
       <c r="I351" s="2" t="inlineStr">
         <is>
-          <t>07/07/2026 01:00</t>
+          <t>27/07/2026 22:34</t>
         </is>
       </c>
       <c r="J351" s="2" t="inlineStr">
         <is>
-          <t>08/07/2026 18:00</t>
+          <t>-</t>
         </is>
       </c>
       <c r="K351" s="2" t="inlineStr">
         <is>
-          <t>07/07/2026 01:00</t>
+          <t>27/07/2026 22:34</t>
         </is>
       </c>
       <c r="L351" s="2" t="inlineStr">
         <is>
-          <t>08/07/2026 18:00</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -22231,12 +22231,12 @@
       </c>
       <c r="F352" s="2" t="inlineStr">
         <is>
-          <t>A3754</t>
+          <t>A9354</t>
         </is>
       </c>
       <c r="G352" s="2" t="inlineStr">
         <is>
-          <t>00019200000013418220</t>
+          <t>00019200000013418211</t>
         </is>
       </c>
       <c r="H352" s="2" t="inlineStr">
@@ -22278,12 +22278,12 @@
       </c>
       <c r="C353" s="2" t="inlineStr">
         <is>
-          <t>-90 C a -60 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D353" s="2" t="inlineStr">
         <is>
-          <t>560527</t>
+          <t>559957</t>
         </is>
       </c>
       <c r="E353" s="2" t="inlineStr">
@@ -22293,12 +22293,12 @@
       </c>
       <c r="F353" s="2" t="inlineStr">
         <is>
-          <t>869170035519140</t>
+          <t>A3754</t>
         </is>
       </c>
       <c r="G353" s="2" t="inlineStr">
         <is>
-          <t>00019200000013778544</t>
+          <t>00019200000013418220</t>
         </is>
       </c>
       <c r="H353" s="2" t="inlineStr">
@@ -22308,22 +22308,22 @@
       </c>
       <c r="I353" s="2" t="inlineStr">
         <is>
-          <t>27/07/2026 22:33</t>
+          <t>07/07/2026 01:00</t>
         </is>
       </c>
       <c r="J353" s="2" t="inlineStr">
         <is>
-          <t>29/07/2026 12:05</t>
+          <t>08/07/2026 18:00</t>
         </is>
       </c>
       <c r="K353" s="2" t="inlineStr">
         <is>
-          <t>27/07/2026 22:33</t>
+          <t>07/07/2026 01:00</t>
         </is>
       </c>
       <c r="L353" s="2" t="inlineStr">
         <is>
-          <t>29/07/2026 12:05</t>
+          <t>08/07/2026 18:00</t>
         </is>
       </c>
     </row>
@@ -22345,7 +22345,7 @@
       </c>
       <c r="D354" s="2" t="inlineStr">
         <is>
-          <t>560576</t>
+          <t>560527</t>
         </is>
       </c>
       <c r="E354" s="2" t="inlineStr">
@@ -22355,12 +22355,12 @@
       </c>
       <c r="F354" s="2" t="inlineStr">
         <is>
-          <t>V5561022</t>
+          <t>869170035519140</t>
         </is>
       </c>
       <c r="G354" s="2" t="inlineStr">
         <is>
-          <t>00019200000013471686</t>
+          <t>00019200000013778544</t>
         </is>
       </c>
       <c r="H354" s="2" t="inlineStr">
@@ -22370,22 +22370,22 @@
       </c>
       <c r="I354" s="2" t="inlineStr">
         <is>
-          <t>19/07/2026 23:45</t>
+          <t>27/07/2026 22:33</t>
         </is>
       </c>
       <c r="J354" s="2" t="inlineStr">
         <is>
-          <t>21/07/2026 17:30</t>
+          <t>29/07/2026 12:05</t>
         </is>
       </c>
       <c r="K354" s="2" t="inlineStr">
         <is>
-          <t>19/07/2026 23:45</t>
+          <t>27/07/2026 22:33</t>
         </is>
       </c>
       <c r="L354" s="2" t="inlineStr">
         <is>
-          <t>21/07/2026 17:30</t>
+          <t>29/07/2026 12:05</t>
         </is>
       </c>
     </row>
@@ -22417,12 +22417,12 @@
       </c>
       <c r="F355" s="2" t="inlineStr">
         <is>
-          <t>V56M3023</t>
+          <t>V5561022</t>
         </is>
       </c>
       <c r="G355" s="2" t="inlineStr">
         <is>
-          <t>00019200000013471694</t>
+          <t>00019200000013471686</t>
         </is>
       </c>
       <c r="H355" s="2" t="inlineStr">
@@ -22479,12 +22479,12 @@
       </c>
       <c r="F356" s="2" t="inlineStr">
         <is>
-          <t>V56M300F</t>
+          <t>V56M3023</t>
         </is>
       </c>
       <c r="G356" s="2" t="inlineStr">
         <is>
-          <t>00019200000013471708</t>
+          <t>00019200000013471694</t>
         </is>
       </c>
       <c r="H356" s="2" t="inlineStr">
@@ -22541,12 +22541,12 @@
       </c>
       <c r="F357" s="2" t="inlineStr">
         <is>
-          <t>V54101A9</t>
+          <t>V56M300F</t>
         </is>
       </c>
       <c r="G357" s="2" t="inlineStr">
         <is>
-          <t>00019200000013471716</t>
+          <t>00019200000013471708</t>
         </is>
       </c>
       <c r="H357" s="2" t="inlineStr">
@@ -22603,12 +22603,12 @@
       </c>
       <c r="F358" s="2" t="inlineStr">
         <is>
-          <t>V556101C</t>
+          <t>V54101A9</t>
         </is>
       </c>
       <c r="G358" s="2" t="inlineStr">
         <is>
-          <t>00019200000013471724</t>
+          <t>00019200000013471716</t>
         </is>
       </c>
       <c r="H358" s="2" t="inlineStr">
@@ -22665,12 +22665,12 @@
       </c>
       <c r="F359" s="2" t="inlineStr">
         <is>
-          <t>V56M3016</t>
+          <t>V556101C</t>
         </is>
       </c>
       <c r="G359" s="2" t="inlineStr">
         <is>
-          <t>00019200000013471732</t>
+          <t>00019200000013471724</t>
         </is>
       </c>
       <c r="H359" s="2" t="inlineStr">
@@ -22727,12 +22727,12 @@
       </c>
       <c r="F360" s="2" t="inlineStr">
         <is>
-          <t>V54100A1</t>
+          <t>V56M3016</t>
         </is>
       </c>
       <c r="G360" s="2" t="inlineStr">
         <is>
-          <t>00019200000013471740</t>
+          <t>00019200000013471732</t>
         </is>
       </c>
       <c r="H360" s="2" t="inlineStr">
@@ -22789,12 +22789,12 @@
       </c>
       <c r="F361" s="2" t="inlineStr">
         <is>
-          <t>V556102F</t>
+          <t>V54100A1</t>
         </is>
       </c>
       <c r="G361" s="2" t="inlineStr">
         <is>
-          <t>00019200000013471872</t>
+          <t>00019200000013471740</t>
         </is>
       </c>
       <c r="H361" s="2" t="inlineStr">
@@ -22851,12 +22851,12 @@
       </c>
       <c r="F362" s="2" t="inlineStr">
         <is>
-          <t>V5561002</t>
+          <t>V556102F</t>
         </is>
       </c>
       <c r="G362" s="2" t="inlineStr">
         <is>
-          <t>00019200000013471880</t>
+          <t>00019200000013471872</t>
         </is>
       </c>
       <c r="H362" s="2" t="inlineStr">
@@ -22913,12 +22913,12 @@
       </c>
       <c r="F363" s="2" t="inlineStr">
         <is>
-          <t>V56M301E</t>
+          <t>V5561002</t>
         </is>
       </c>
       <c r="G363" s="2" t="inlineStr">
         <is>
-          <t>00019200000013471899</t>
+          <t>00019200000013471880</t>
         </is>
       </c>
       <c r="H363" s="2" t="inlineStr">
@@ -22975,12 +22975,12 @@
       </c>
       <c r="F364" s="2" t="inlineStr">
         <is>
-          <t>V5561015</t>
+          <t>V56M301E</t>
         </is>
       </c>
       <c r="G364" s="2" t="inlineStr">
         <is>
-          <t>00019200000013475789</t>
+          <t>00019200000013471899</t>
         </is>
       </c>
       <c r="H364" s="2" t="inlineStr">
@@ -23037,12 +23037,12 @@
       </c>
       <c r="F365" s="2" t="inlineStr">
         <is>
-          <t>V5560004</t>
+          <t>V5561015</t>
         </is>
       </c>
       <c r="G365" s="2" t="inlineStr">
         <is>
-          <t>00019200000013475797</t>
+          <t>00019200000013475789</t>
         </is>
       </c>
       <c r="H365" s="2" t="inlineStr">
@@ -23084,12 +23084,12 @@
       </c>
       <c r="C366" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-90 C a -60 C</t>
         </is>
       </c>
       <c r="D366" s="2" t="inlineStr">
         <is>
-          <t>561418</t>
+          <t>560576</t>
         </is>
       </c>
       <c r="E366" s="2" t="inlineStr">
@@ -23099,12 +23099,12 @@
       </c>
       <c r="F366" s="2" t="inlineStr">
         <is>
-          <t>A8179</t>
+          <t>V5560004</t>
         </is>
       </c>
       <c r="G366" s="2" t="inlineStr">
         <is>
-          <t>00019200000013472151</t>
+          <t>00019200000013475797</t>
         </is>
       </c>
       <c r="H366" s="2" t="inlineStr">
@@ -23114,22 +23114,22 @@
       </c>
       <c r="I366" s="2" t="inlineStr">
         <is>
-          <t>19/07/2026 03:54</t>
+          <t>19/07/2026 23:45</t>
         </is>
       </c>
       <c r="J366" s="2" t="inlineStr">
         <is>
-          <t>24/07/2026 20:25</t>
+          <t>21/07/2026 17:30</t>
         </is>
       </c>
       <c r="K366" s="2" t="inlineStr">
         <is>
-          <t>19/07/2026 03:54</t>
+          <t>19/07/2026 23:45</t>
         </is>
       </c>
       <c r="L366" s="2" t="inlineStr">
         <is>
-          <t>24/07/2026 20:25</t>
+          <t>21/07/2026 17:30</t>
         </is>
       </c>
     </row>
@@ -23161,12 +23161,12 @@
       </c>
       <c r="F367" s="2" t="inlineStr">
         <is>
-          <t>A9611</t>
+          <t>A8179</t>
         </is>
       </c>
       <c r="G367" s="2" t="inlineStr">
         <is>
-          <t>00019200000013472160</t>
+          <t>00019200000013472151</t>
         </is>
       </c>
       <c r="H367" s="2" t="inlineStr">
@@ -23223,12 +23223,12 @@
       </c>
       <c r="F368" s="2" t="inlineStr">
         <is>
-          <t>TA0310</t>
+          <t>A9611</t>
         </is>
       </c>
       <c r="G368" s="2" t="inlineStr">
         <is>
-          <t>00019200000013472178</t>
+          <t>00019200000013472160</t>
         </is>
       </c>
       <c r="H368" s="2" t="inlineStr">
@@ -23285,12 +23285,12 @@
       </c>
       <c r="F369" s="2" t="inlineStr">
         <is>
-          <t>TA0493</t>
+          <t>TA0310</t>
         </is>
       </c>
       <c r="G369" s="2" t="inlineStr">
         <is>
-          <t>00019200000013472186</t>
+          <t>00019200000013472178</t>
         </is>
       </c>
       <c r="H369" s="2" t="inlineStr">
@@ -23347,12 +23347,12 @@
       </c>
       <c r="F370" s="2" t="inlineStr">
         <is>
-          <t>A2344</t>
+          <t>TA0493</t>
         </is>
       </c>
       <c r="G370" s="2" t="inlineStr">
         <is>
-          <t>00019200000013472194</t>
+          <t>00019200000013472186</t>
         </is>
       </c>
       <c r="H370" s="2" t="inlineStr">
@@ -23409,12 +23409,12 @@
       </c>
       <c r="F371" s="2" t="inlineStr">
         <is>
-          <t>A8458</t>
+          <t>A2344</t>
         </is>
       </c>
       <c r="G371" s="2" t="inlineStr">
         <is>
-          <t>00019200000013472208</t>
+          <t>00019200000013472194</t>
         </is>
       </c>
       <c r="H371" s="2" t="inlineStr">
@@ -23456,7 +23456,7 @@
       </c>
       <c r="C372" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D372" s="2" t="inlineStr">
@@ -23471,12 +23471,12 @@
       </c>
       <c r="F372" s="2" t="inlineStr">
         <is>
-          <t>A7945</t>
+          <t>A8458</t>
         </is>
       </c>
       <c r="G372" s="2" t="inlineStr">
         <is>
-          <t>00019200000013472216</t>
+          <t>00019200000013472208</t>
         </is>
       </c>
       <c r="H372" s="2" t="inlineStr">
@@ -23533,12 +23533,12 @@
       </c>
       <c r="F373" s="2" t="inlineStr">
         <is>
-          <t>A5377</t>
+          <t>A7945</t>
         </is>
       </c>
       <c r="G373" s="2" t="inlineStr">
         <is>
-          <t>00019200000013472224</t>
+          <t>00019200000013472216</t>
         </is>
       </c>
       <c r="H373" s="2" t="inlineStr">
@@ -23595,12 +23595,12 @@
       </c>
       <c r="F374" s="2" t="inlineStr">
         <is>
-          <t>A7312</t>
+          <t>A5377</t>
         </is>
       </c>
       <c r="G374" s="2" t="inlineStr">
         <is>
-          <t>00019200000013472232</t>
+          <t>00019200000013472224</t>
         </is>
       </c>
       <c r="H374" s="2" t="inlineStr">
@@ -23657,12 +23657,12 @@
       </c>
       <c r="F375" s="2" t="inlineStr">
         <is>
-          <t>A6642</t>
+          <t>A7312</t>
         </is>
       </c>
       <c r="G375" s="2" t="inlineStr">
         <is>
-          <t>00019200000013472259</t>
+          <t>00019200000013472232</t>
         </is>
       </c>
       <c r="H375" s="2" t="inlineStr">
@@ -23719,12 +23719,12 @@
       </c>
       <c r="F376" s="2" t="inlineStr">
         <is>
-          <t>A6142</t>
+          <t>A6642</t>
         </is>
       </c>
       <c r="G376" s="2" t="inlineStr">
         <is>
-          <t>00019200000013472267</t>
+          <t>00019200000013472259</t>
         </is>
       </c>
       <c r="H376" s="2" t="inlineStr">
@@ -23781,12 +23781,12 @@
       </c>
       <c r="F377" s="2" t="inlineStr">
         <is>
-          <t>TA0826</t>
+          <t>A6142</t>
         </is>
       </c>
       <c r="G377" s="2" t="inlineStr">
         <is>
-          <t>00019200000013472275</t>
+          <t>00019200000013472267</t>
         </is>
       </c>
       <c r="H377" s="2" t="inlineStr">
@@ -23843,12 +23843,12 @@
       </c>
       <c r="F378" s="2" t="inlineStr">
         <is>
-          <t>A8679</t>
+          <t>TA0826</t>
         </is>
       </c>
       <c r="G378" s="2" t="inlineStr">
         <is>
-          <t>00019200000013472283</t>
+          <t>00019200000013472275</t>
         </is>
       </c>
       <c r="H378" s="2" t="inlineStr">
@@ -23905,12 +23905,12 @@
       </c>
       <c r="F379" s="2" t="inlineStr">
         <is>
-          <t>TA1135</t>
+          <t>A8679</t>
         </is>
       </c>
       <c r="G379" s="2" t="inlineStr">
         <is>
-          <t>00019200000013472291</t>
+          <t>00019200000013472283</t>
         </is>
       </c>
       <c r="H379" s="2" t="inlineStr">
@@ -23967,12 +23967,12 @@
       </c>
       <c r="F380" s="2" t="inlineStr">
         <is>
-          <t>TA0895</t>
+          <t>TA1135</t>
         </is>
       </c>
       <c r="G380" s="2" t="inlineStr">
         <is>
-          <t>00019200000013472305</t>
+          <t>00019200000013472291</t>
         </is>
       </c>
       <c r="H380" s="2" t="inlineStr">
@@ -24029,12 +24029,12 @@
       </c>
       <c r="F381" s="2" t="inlineStr">
         <is>
-          <t>A7095</t>
+          <t>TA0895</t>
         </is>
       </c>
       <c r="G381" s="2" t="inlineStr">
         <is>
-          <t>00019200000013472313</t>
+          <t>00019200000013472305</t>
         </is>
       </c>
       <c r="H381" s="2" t="inlineStr">
@@ -24091,12 +24091,12 @@
       </c>
       <c r="F382" s="2" t="inlineStr">
         <is>
-          <t>A6569</t>
+          <t>A7095</t>
         </is>
       </c>
       <c r="G382" s="2" t="inlineStr">
         <is>
-          <t>00019200000013472321</t>
+          <t>00019200000013472313</t>
         </is>
       </c>
       <c r="H382" s="2" t="inlineStr">
@@ -24153,12 +24153,12 @@
       </c>
       <c r="F383" s="2" t="inlineStr">
         <is>
-          <t>TA1062</t>
+          <t>A6569</t>
         </is>
       </c>
       <c r="G383" s="2" t="inlineStr">
         <is>
-          <t>00019200000013472330</t>
+          <t>00019200000013472321</t>
         </is>
       </c>
       <c r="H383" s="2" t="inlineStr">
@@ -24215,12 +24215,12 @@
       </c>
       <c r="F384" s="2" t="inlineStr">
         <is>
-          <t>A5533</t>
+          <t>TA1062</t>
         </is>
       </c>
       <c r="G384" s="2" t="inlineStr">
         <is>
-          <t>00019200000013472348</t>
+          <t>00019200000013472330</t>
         </is>
       </c>
       <c r="H384" s="2" t="inlineStr">
@@ -24277,12 +24277,12 @@
       </c>
       <c r="F385" s="2" t="inlineStr">
         <is>
-          <t>A9128</t>
+          <t>A5533</t>
         </is>
       </c>
       <c r="G385" s="2" t="inlineStr">
         <is>
-          <t>00019200000013472356</t>
+          <t>00019200000013472348</t>
         </is>
       </c>
       <c r="H385" s="2" t="inlineStr">
@@ -24339,12 +24339,12 @@
       </c>
       <c r="F386" s="2" t="inlineStr">
         <is>
-          <t>A8531</t>
+          <t>A9128</t>
         </is>
       </c>
       <c r="G386" s="2" t="inlineStr">
         <is>
-          <t>00019200000013472364</t>
+          <t>00019200000013472356</t>
         </is>
       </c>
       <c r="H386" s="2" t="inlineStr">
@@ -24401,12 +24401,12 @@
       </c>
       <c r="F387" s="2" t="inlineStr">
         <is>
-          <t>A0259</t>
+          <t>A8531</t>
         </is>
       </c>
       <c r="G387" s="2" t="inlineStr">
         <is>
-          <t>00019200000013472372</t>
+          <t>00019200000013472364</t>
         </is>
       </c>
       <c r="H387" s="2" t="inlineStr">
@@ -24463,12 +24463,12 @@
       </c>
       <c r="F388" s="2" t="inlineStr">
         <is>
-          <t>A3195</t>
+          <t>A0259</t>
         </is>
       </c>
       <c r="G388" s="2" t="inlineStr">
         <is>
-          <t>00019200000013472380</t>
+          <t>00019200000013472372</t>
         </is>
       </c>
       <c r="H388" s="2" t="inlineStr">
@@ -24525,12 +24525,12 @@
       </c>
       <c r="F389" s="2" t="inlineStr">
         <is>
-          <t>A5061</t>
+          <t>A3195</t>
         </is>
       </c>
       <c r="G389" s="2" t="inlineStr">
         <is>
-          <t>00019200000013472399</t>
+          <t>00019200000013472380</t>
         </is>
       </c>
       <c r="H389" s="2" t="inlineStr">
@@ -24587,12 +24587,12 @@
       </c>
       <c r="F390" s="2" t="inlineStr">
         <is>
-          <t>A5097</t>
+          <t>A5061</t>
         </is>
       </c>
       <c r="G390" s="2" t="inlineStr">
         <is>
-          <t>00019200000013472402</t>
+          <t>00019200000013472399</t>
         </is>
       </c>
       <c r="H390" s="2" t="inlineStr">
@@ -24649,12 +24649,12 @@
       </c>
       <c r="F391" s="2" t="inlineStr">
         <is>
-          <t>A3193</t>
+          <t>A5097</t>
         </is>
       </c>
       <c r="G391" s="2" t="inlineStr">
         <is>
-          <t>00019200000013472410</t>
+          <t>00019200000013472402</t>
         </is>
       </c>
       <c r="H391" s="2" t="inlineStr">
@@ -24696,7 +24696,7 @@
       </c>
       <c r="C392" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D392" s="2" t="inlineStr">
@@ -24711,12 +24711,12 @@
       </c>
       <c r="F392" s="2" t="inlineStr">
         <is>
-          <t>A5035</t>
+          <t>A3193</t>
         </is>
       </c>
       <c r="G392" s="2" t="inlineStr">
         <is>
-          <t>00019200000013473760</t>
+          <t>00019200000013472410</t>
         </is>
       </c>
       <c r="H392" s="2" t="inlineStr">
@@ -24758,27 +24758,27 @@
       </c>
       <c r="C393" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D393" s="2" t="inlineStr">
         <is>
-          <t>559944</t>
+          <t>561418</t>
         </is>
       </c>
       <c r="E393" s="2" t="inlineStr">
         <is>
-          <t>RR</t>
+          <t>RO</t>
         </is>
       </c>
       <c r="F393" s="2" t="inlineStr">
         <is>
-          <t>A3432</t>
+          <t>A5035</t>
         </is>
       </c>
       <c r="G393" s="2" t="inlineStr">
         <is>
-          <t>00019200000013419030</t>
+          <t>00019200000013473760</t>
         </is>
       </c>
       <c r="H393" s="2" t="inlineStr">
@@ -24788,22 +24788,22 @@
       </c>
       <c r="I393" s="2" t="inlineStr">
         <is>
-          <t>07/07/2026 06:51</t>
+          <t>19/07/2026 03:54</t>
         </is>
       </c>
       <c r="J393" s="2" t="inlineStr">
         <is>
-          <t>10/07/2026 18:00</t>
+          <t>24/07/2026 20:25</t>
         </is>
       </c>
       <c r="K393" s="2" t="inlineStr">
         <is>
-          <t>07/07/2026 06:51</t>
+          <t>19/07/2026 03:54</t>
         </is>
       </c>
       <c r="L393" s="2" t="inlineStr">
         <is>
-          <t>10/07/2026 18:00</t>
+          <t>24/07/2026 20:25</t>
         </is>
       </c>
     </row>
@@ -24820,12 +24820,12 @@
       </c>
       <c r="C394" s="2" t="inlineStr">
         <is>
-          <t>-90 C a -60 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D394" s="2" t="inlineStr">
         <is>
-          <t>560780</t>
+          <t>559944</t>
         </is>
       </c>
       <c r="E394" s="2" t="inlineStr">
@@ -24835,12 +24835,12 @@
       </c>
       <c r="F394" s="2" t="inlineStr">
         <is>
-          <t>300017</t>
+          <t>A3432</t>
         </is>
       </c>
       <c r="G394" s="2" t="inlineStr">
         <is>
-          <t>00019200000013778609</t>
+          <t>00019200000013419030</t>
         </is>
       </c>
       <c r="H394" s="2" t="inlineStr">
@@ -24850,22 +24850,22 @@
       </c>
       <c r="I394" s="2" t="inlineStr">
         <is>
-          <t>27/07/2026 22:35</t>
+          <t>07/07/2026 06:51</t>
         </is>
       </c>
       <c r="J394" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 18:00</t>
         </is>
       </c>
       <c r="K394" s="2" t="inlineStr">
         <is>
-          <t>27/07/2026 22:35</t>
+          <t>07/07/2026 06:51</t>
         </is>
       </c>
       <c r="L394" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 18:00</t>
         </is>
       </c>
     </row>
@@ -24882,27 +24882,27 @@
       </c>
       <c r="C395" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-90 C a -60 C</t>
         </is>
       </c>
       <c r="D395" s="2" t="inlineStr">
         <is>
-          <t>559925</t>
+          <t>560780</t>
         </is>
       </c>
       <c r="E395" s="2" t="inlineStr">
         <is>
-          <t>RS</t>
+          <t>RR</t>
         </is>
       </c>
       <c r="F395" s="2" t="inlineStr">
         <is>
-          <t>A7594</t>
+          <t>300017</t>
         </is>
       </c>
       <c r="G395" s="2" t="inlineStr">
         <is>
-          <t>00019200000013419137</t>
+          <t>00019200000013778609</t>
         </is>
       </c>
       <c r="H395" s="2" t="inlineStr">
@@ -24912,22 +24912,22 @@
       </c>
       <c r="I395" s="2" t="inlineStr">
         <is>
-          <t>07/07/2026 06:51</t>
+          <t>27/07/2026 22:35</t>
         </is>
       </c>
       <c r="J395" s="2" t="inlineStr">
         <is>
-          <t>09/07/2026 13:09</t>
+          <t>-</t>
         </is>
       </c>
       <c r="K395" s="2" t="inlineStr">
         <is>
-          <t>07/07/2026 06:51</t>
+          <t>27/07/2026 22:35</t>
         </is>
       </c>
       <c r="L395" s="2" t="inlineStr">
         <is>
-          <t>09/07/2026 13:09</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -24944,12 +24944,12 @@
       </c>
       <c r="C396" s="2" t="inlineStr">
         <is>
-          <t>-90 C a -60 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D396" s="2" t="inlineStr">
         <is>
-          <t>560574</t>
+          <t>559925</t>
         </is>
       </c>
       <c r="E396" s="2" t="inlineStr">
@@ -24959,12 +24959,12 @@
       </c>
       <c r="F396" s="2" t="inlineStr">
         <is>
-          <t>AS-0499</t>
+          <t>A7594</t>
         </is>
       </c>
       <c r="G396" s="2" t="inlineStr">
         <is>
-          <t>00019200000013463969</t>
+          <t>00019200000013419137</t>
         </is>
       </c>
       <c r="H396" s="2" t="inlineStr">
@@ -24974,22 +24974,22 @@
       </c>
       <c r="I396" s="2" t="inlineStr">
         <is>
-          <t>21/07/2026 22:28</t>
+          <t>07/07/2026 06:51</t>
         </is>
       </c>
       <c r="J396" s="2" t="inlineStr">
         <is>
-          <t>23/07/2026 15:00</t>
+          <t>09/07/2026 13:09</t>
         </is>
       </c>
       <c r="K396" s="2" t="inlineStr">
         <is>
-          <t>21/07/2026 22:28</t>
+          <t>07/07/2026 06:51</t>
         </is>
       </c>
       <c r="L396" s="2" t="inlineStr">
         <is>
-          <t>23/07/2026 13:15</t>
+          <t>09/07/2026 13:09</t>
         </is>
       </c>
     </row>
@@ -25021,12 +25021,12 @@
       </c>
       <c r="F397" s="2" t="inlineStr">
         <is>
-          <t>AS-0683</t>
+          <t>AS-0499</t>
         </is>
       </c>
       <c r="G397" s="2" t="inlineStr">
         <is>
-          <t>00019200000013463977</t>
+          <t>00019200000013463969</t>
         </is>
       </c>
       <c r="H397" s="2" t="inlineStr">
@@ -25083,12 +25083,12 @@
       </c>
       <c r="F398" s="2" t="inlineStr">
         <is>
-          <t>AS-0426</t>
+          <t>AS-0683</t>
         </is>
       </c>
       <c r="G398" s="2" t="inlineStr">
         <is>
-          <t>00019200000013463985</t>
+          <t>00019200000013463977</t>
         </is>
       </c>
       <c r="H398" s="2" t="inlineStr">
@@ -25145,12 +25145,12 @@
       </c>
       <c r="F399" s="2" t="inlineStr">
         <is>
-          <t>AS-0702</t>
+          <t>AS-0426</t>
         </is>
       </c>
       <c r="G399" s="2" t="inlineStr">
         <is>
-          <t>00019200000013463993</t>
+          <t>00019200000013463985</t>
         </is>
       </c>
       <c r="H399" s="2" t="inlineStr">
@@ -25207,12 +25207,12 @@
       </c>
       <c r="F400" s="2" t="inlineStr">
         <is>
-          <t>AS-0869</t>
+          <t>AS-0702</t>
         </is>
       </c>
       <c r="G400" s="2" t="inlineStr">
         <is>
-          <t>00019200000013464019</t>
+          <t>00019200000013463993</t>
         </is>
       </c>
       <c r="H400" s="2" t="inlineStr">
@@ -25269,12 +25269,12 @@
       </c>
       <c r="F401" s="2" t="inlineStr">
         <is>
-          <t>AS-0837</t>
+          <t>AS-0869</t>
         </is>
       </c>
       <c r="G401" s="2" t="inlineStr">
         <is>
-          <t>00019200000013464027</t>
+          <t>00019200000013464019</t>
         </is>
       </c>
       <c r="H401" s="2" t="inlineStr">
@@ -25331,12 +25331,12 @@
       </c>
       <c r="F402" s="2" t="inlineStr">
         <is>
-          <t>AS-0201</t>
+          <t>AS-0837</t>
         </is>
       </c>
       <c r="G402" s="2" t="inlineStr">
         <is>
-          <t>00019200000013464035</t>
+          <t>00019200000013464027</t>
         </is>
       </c>
       <c r="H402" s="2" t="inlineStr">
@@ -25361,7 +25361,7 @@
       </c>
       <c r="L402" s="2" t="inlineStr">
         <is>
-          <t>23/07/2026 15:00</t>
+          <t>23/07/2026 13:15</t>
         </is>
       </c>
     </row>
@@ -25393,12 +25393,12 @@
       </c>
       <c r="F403" s="2" t="inlineStr">
         <is>
-          <t>AS-0487</t>
+          <t>AS-0201</t>
         </is>
       </c>
       <c r="G403" s="2" t="inlineStr">
         <is>
-          <t>00019200000013464043</t>
+          <t>00019200000013464035</t>
         </is>
       </c>
       <c r="H403" s="2" t="inlineStr">
@@ -25423,7 +25423,7 @@
       </c>
       <c r="L403" s="2" t="inlineStr">
         <is>
-          <t>23/07/2026 13:15</t>
+          <t>23/07/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -25455,12 +25455,12 @@
       </c>
       <c r="F404" s="2" t="inlineStr">
         <is>
-          <t>AS-0356</t>
+          <t>AS-0487</t>
         </is>
       </c>
       <c r="G404" s="2" t="inlineStr">
         <is>
-          <t>00019200000013464051</t>
+          <t>00019200000013464043</t>
         </is>
       </c>
       <c r="H404" s="2" t="inlineStr">
@@ -25485,7 +25485,7 @@
       </c>
       <c r="L404" s="2" t="inlineStr">
         <is>
-          <t>23/07/2026 15:00</t>
+          <t>23/07/2026 13:15</t>
         </is>
       </c>
     </row>
@@ -25517,12 +25517,12 @@
       </c>
       <c r="F405" s="2" t="inlineStr">
         <is>
-          <t>AS-0414</t>
+          <t>AS-0356</t>
         </is>
       </c>
       <c r="G405" s="2" t="inlineStr">
         <is>
-          <t>00019200000013464078</t>
+          <t>00019200000013464051</t>
         </is>
       </c>
       <c r="H405" s="2" t="inlineStr">
@@ -25547,7 +25547,7 @@
       </c>
       <c r="L405" s="2" t="inlineStr">
         <is>
-          <t>23/07/2026 13:15</t>
+          <t>23/07/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -25579,12 +25579,12 @@
       </c>
       <c r="F406" s="2" t="inlineStr">
         <is>
-          <t>AS-0078</t>
+          <t>AS-0414</t>
         </is>
       </c>
       <c r="G406" s="2" t="inlineStr">
         <is>
-          <t>00019200000013464086</t>
+          <t>00019200000013464078</t>
         </is>
       </c>
       <c r="H406" s="2" t="inlineStr">
@@ -25609,7 +25609,7 @@
       </c>
       <c r="L406" s="2" t="inlineStr">
         <is>
-          <t>23/07/2026 15:00</t>
+          <t>23/07/2026 13:15</t>
         </is>
       </c>
     </row>
@@ -25641,12 +25641,12 @@
       </c>
       <c r="F407" s="2" t="inlineStr">
         <is>
-          <t>AS-0019</t>
+          <t>AS-0078</t>
         </is>
       </c>
       <c r="G407" s="2" t="inlineStr">
         <is>
-          <t>00019200000013464094</t>
+          <t>00019200000013464086</t>
         </is>
       </c>
       <c r="H407" s="2" t="inlineStr">
@@ -25703,12 +25703,12 @@
       </c>
       <c r="F408" s="2" t="inlineStr">
         <is>
-          <t>AS-0252</t>
+          <t>AS-0019</t>
         </is>
       </c>
       <c r="G408" s="2" t="inlineStr">
         <is>
-          <t>00019200000013464108</t>
+          <t>00019200000013464094</t>
         </is>
       </c>
       <c r="H408" s="2" t="inlineStr">
@@ -25765,12 +25765,12 @@
       </c>
       <c r="F409" s="2" t="inlineStr">
         <is>
-          <t>AS-0160</t>
+          <t>AS-0252</t>
         </is>
       </c>
       <c r="G409" s="2" t="inlineStr">
         <is>
-          <t>00019200000013464116</t>
+          <t>00019200000013464108</t>
         </is>
       </c>
       <c r="H409" s="2" t="inlineStr">
@@ -25827,12 +25827,12 @@
       </c>
       <c r="F410" s="2" t="inlineStr">
         <is>
-          <t>AS-0513</t>
+          <t>AS-0160</t>
         </is>
       </c>
       <c r="G410" s="2" t="inlineStr">
         <is>
-          <t>00019200000013464124</t>
+          <t>00019200000013464116</t>
         </is>
       </c>
       <c r="H410" s="2" t="inlineStr">
@@ -25857,7 +25857,7 @@
       </c>
       <c r="L410" s="2" t="inlineStr">
         <is>
-          <t>23/07/2026 13:15</t>
+          <t>23/07/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -25889,12 +25889,12 @@
       </c>
       <c r="F411" s="2" t="inlineStr">
         <is>
-          <t>AS-0234</t>
+          <t>AS-0513</t>
         </is>
       </c>
       <c r="G411" s="2" t="inlineStr">
         <is>
-          <t>00019200000013464132</t>
+          <t>00019200000013464124</t>
         </is>
       </c>
       <c r="H411" s="2" t="inlineStr">
@@ -25919,7 +25919,7 @@
       </c>
       <c r="L411" s="2" t="inlineStr">
         <is>
-          <t>23/07/2026 15:00</t>
+          <t>23/07/2026 13:15</t>
         </is>
       </c>
     </row>
@@ -25951,12 +25951,12 @@
       </c>
       <c r="F412" s="2" t="inlineStr">
         <is>
-          <t>AS-0494</t>
+          <t>AS-0234</t>
         </is>
       </c>
       <c r="G412" s="2" t="inlineStr">
         <is>
-          <t>00019200000013464140</t>
+          <t>00019200000013464132</t>
         </is>
       </c>
       <c r="H412" s="2" t="inlineStr">
@@ -26013,12 +26013,12 @@
       </c>
       <c r="F413" s="2" t="inlineStr">
         <is>
-          <t>AS-0850</t>
+          <t>AS-0494</t>
         </is>
       </c>
       <c r="G413" s="2" t="inlineStr">
         <is>
-          <t>00019200000013464159</t>
+          <t>00019200000013464140</t>
         </is>
       </c>
       <c r="H413" s="2" t="inlineStr">
@@ -26075,12 +26075,12 @@
       </c>
       <c r="F414" s="2" t="inlineStr">
         <is>
-          <t>AS-0107</t>
+          <t>AS-0850</t>
         </is>
       </c>
       <c r="G414" s="2" t="inlineStr">
         <is>
-          <t>00019200000013464167</t>
+          <t>00019200000013464159</t>
         </is>
       </c>
       <c r="H414" s="2" t="inlineStr">
@@ -26137,12 +26137,12 @@
       </c>
       <c r="F415" s="2" t="inlineStr">
         <is>
-          <t>AS-0845</t>
+          <t>AS-0107</t>
         </is>
       </c>
       <c r="G415" s="2" t="inlineStr">
         <is>
-          <t>00019200000013464175</t>
+          <t>00019200000013464167</t>
         </is>
       </c>
       <c r="H415" s="2" t="inlineStr">
@@ -26199,12 +26199,12 @@
       </c>
       <c r="F416" s="2" t="inlineStr">
         <is>
-          <t>AS-0511</t>
+          <t>AS-0845</t>
         </is>
       </c>
       <c r="G416" s="2" t="inlineStr">
         <is>
-          <t>00019200000013464183</t>
+          <t>00019200000013464175</t>
         </is>
       </c>
       <c r="H416" s="2" t="inlineStr">
@@ -26261,12 +26261,12 @@
       </c>
       <c r="F417" s="2" t="inlineStr">
         <is>
-          <t>AS-0363</t>
+          <t>AS-0511</t>
         </is>
       </c>
       <c r="G417" s="2" t="inlineStr">
         <is>
-          <t>00019200000013464191</t>
+          <t>00019200000013464183</t>
         </is>
       </c>
       <c r="H417" s="2" t="inlineStr">
@@ -26291,7 +26291,7 @@
       </c>
       <c r="L417" s="2" t="inlineStr">
         <is>
-          <t>23/07/2026 13:15</t>
+          <t>23/07/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -26323,12 +26323,12 @@
       </c>
       <c r="F418" s="2" t="inlineStr">
         <is>
-          <t>AS-0269</t>
+          <t>AS-0363</t>
         </is>
       </c>
       <c r="G418" s="2" t="inlineStr">
         <is>
-          <t>00019200000013464205</t>
+          <t>00019200000013464191</t>
         </is>
       </c>
       <c r="H418" s="2" t="inlineStr">
@@ -26385,12 +26385,12 @@
       </c>
       <c r="F419" s="2" t="inlineStr">
         <is>
-          <t>AS-0643</t>
+          <t>AS-0269</t>
         </is>
       </c>
       <c r="G419" s="2" t="inlineStr">
         <is>
-          <t>00019200000013464213</t>
+          <t>00019200000013464205</t>
         </is>
       </c>
       <c r="H419" s="2" t="inlineStr">
@@ -26447,12 +26447,12 @@
       </c>
       <c r="F420" s="2" t="inlineStr">
         <is>
-          <t>AS-0263</t>
+          <t>AS-0643</t>
         </is>
       </c>
       <c r="G420" s="2" t="inlineStr">
         <is>
-          <t>00019200000013464221</t>
+          <t>00019200000013464213</t>
         </is>
       </c>
       <c r="H420" s="2" t="inlineStr">
@@ -26494,12 +26494,12 @@
       </c>
       <c r="C421" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-90 C a -60 C</t>
         </is>
       </c>
       <c r="D421" s="2" t="inlineStr">
         <is>
-          <t>560688</t>
+          <t>560574</t>
         </is>
       </c>
       <c r="E421" s="2" t="inlineStr">
@@ -26509,37 +26509,37 @@
       </c>
       <c r="F421" s="2" t="inlineStr">
         <is>
-          <t>A5913</t>
+          <t>AS-0263</t>
         </is>
       </c>
       <c r="G421" s="2" t="inlineStr">
         <is>
-          <t>00019200000013694359</t>
+          <t>00019200000013464221</t>
         </is>
       </c>
       <c r="H421" s="2" t="inlineStr">
         <is>
-          <t>Rodoviário</t>
+          <t>MultiModal</t>
         </is>
       </c>
       <c r="I421" s="2" t="inlineStr">
         <is>
-          <t>27/07/2026 06:04</t>
+          <t>21/07/2026 22:28</t>
         </is>
       </c>
       <c r="J421" s="2" t="inlineStr">
         <is>
-          <t>29/07/2026 10:36</t>
+          <t>23/07/2026 15:00</t>
         </is>
       </c>
       <c r="K421" s="2" t="inlineStr">
         <is>
-          <t>27/07/2026 06:04</t>
+          <t>21/07/2026 22:28</t>
         </is>
       </c>
       <c r="L421" s="2" t="inlineStr">
         <is>
-          <t>29/07/2026 10:23</t>
+          <t>23/07/2026 13:15</t>
         </is>
       </c>
     </row>
@@ -26556,12 +26556,12 @@
       </c>
       <c r="C422" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D422" s="2" t="inlineStr">
         <is>
-          <t>562154</t>
+          <t>560688</t>
         </is>
       </c>
       <c r="E422" s="2" t="inlineStr">
@@ -26571,37 +26571,37 @@
       </c>
       <c r="F422" s="2" t="inlineStr">
         <is>
-          <t>A4440</t>
+          <t>A5913</t>
         </is>
       </c>
       <c r="G422" s="2" t="inlineStr">
         <is>
-          <t>00019200000013778293</t>
+          <t>00019200000013694359</t>
         </is>
       </c>
       <c r="H422" s="2" t="inlineStr">
         <is>
-          <t>MultiModal</t>
+          <t>Rodoviário</t>
         </is>
       </c>
       <c r="I422" s="2" t="inlineStr">
         <is>
-          <t>28/07/2026 03:39</t>
+          <t>27/07/2026 06:04</t>
         </is>
       </c>
       <c r="J422" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>29/07/2026 10:36</t>
         </is>
       </c>
       <c r="K422" s="2" t="inlineStr">
         <is>
-          <t>28/07/2026 03:39</t>
+          <t>27/07/2026 06:04</t>
         </is>
       </c>
       <c r="L422" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>29/07/2026 10:23</t>
         </is>
       </c>
     </row>
@@ -26618,27 +26618,27 @@
       </c>
       <c r="C423" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D423" s="2" t="inlineStr">
         <is>
-          <t>559880</t>
+          <t>562154</t>
         </is>
       </c>
       <c r="E423" s="2" t="inlineStr">
         <is>
-          <t>SC</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="F423" s="2" t="inlineStr">
         <is>
-          <t>A8482</t>
+          <t>A4440</t>
         </is>
       </c>
       <c r="G423" s="2" t="inlineStr">
         <is>
-          <t>00019200000013407147</t>
+          <t>00019200000013778293</t>
         </is>
       </c>
       <c r="H423" s="2" t="inlineStr">
@@ -26648,22 +26648,22 @@
       </c>
       <c r="I423" s="2" t="inlineStr">
         <is>
-          <t>09/07/2026 05:48</t>
+          <t>28/07/2026 03:39</t>
         </is>
       </c>
       <c r="J423" s="2" t="inlineStr">
         <is>
-          <t>10/07/2026 17:00</t>
+          <t>-</t>
         </is>
       </c>
       <c r="K423" s="2" t="inlineStr">
         <is>
-          <t>09/07/2026 05:48</t>
+          <t>28/07/2026 03:39</t>
         </is>
       </c>
       <c r="L423" s="2" t="inlineStr">
         <is>
-          <t>10/07/2026 17:00</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -26695,12 +26695,12 @@
       </c>
       <c r="F424" s="2" t="inlineStr">
         <is>
-          <t>A4021</t>
+          <t>A8482</t>
         </is>
       </c>
       <c r="G424" s="2" t="inlineStr">
         <is>
-          <t>00019200000013407180</t>
+          <t>00019200000013407147</t>
         </is>
       </c>
       <c r="H424" s="2" t="inlineStr">
@@ -26757,12 +26757,12 @@
       </c>
       <c r="F425" s="2" t="inlineStr">
         <is>
-          <t>A7212</t>
+          <t>A4021</t>
         </is>
       </c>
       <c r="G425" s="2" t="inlineStr">
         <is>
-          <t>00019200000013407198</t>
+          <t>00019200000013407180</t>
         </is>
       </c>
       <c r="H425" s="2" t="inlineStr">
@@ -26819,12 +26819,12 @@
       </c>
       <c r="F426" s="2" t="inlineStr">
         <is>
-          <t>A3672</t>
+          <t>A7212</t>
         </is>
       </c>
       <c r="G426" s="2" t="inlineStr">
         <is>
-          <t>00019200000013407201</t>
+          <t>00019200000013407198</t>
         </is>
       </c>
       <c r="H426" s="2" t="inlineStr">
@@ -26881,12 +26881,12 @@
       </c>
       <c r="F427" s="2" t="inlineStr">
         <is>
-          <t>TA0241</t>
+          <t>A3672</t>
         </is>
       </c>
       <c r="G427" s="2" t="inlineStr">
         <is>
-          <t>00019200000013407210</t>
+          <t>00019200000013407201</t>
         </is>
       </c>
       <c r="H427" s="2" t="inlineStr">
@@ -26928,27 +26928,27 @@
       </c>
       <c r="C428" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D428" s="2" t="inlineStr">
         <is>
-          <t>559876</t>
+          <t>559880</t>
         </is>
       </c>
       <c r="E428" s="2" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>SC</t>
         </is>
       </c>
       <c r="F428" s="2" t="inlineStr">
         <is>
-          <t>A1817</t>
+          <t>TA0241</t>
         </is>
       </c>
       <c r="G428" s="2" t="inlineStr">
         <is>
-          <t>00019200000013419021</t>
+          <t>00019200000013407210</t>
         </is>
       </c>
       <c r="H428" s="2" t="inlineStr">
@@ -26958,22 +26958,22 @@
       </c>
       <c r="I428" s="2" t="inlineStr">
         <is>
-          <t>07/07/2026 00:57</t>
+          <t>09/07/2026 05:48</t>
         </is>
       </c>
       <c r="J428" s="2" t="inlineStr">
         <is>
-          <t>17/07/2026 15:00</t>
+          <t>10/07/2026 17:00</t>
         </is>
       </c>
       <c r="K428" s="2" t="inlineStr">
         <is>
-          <t>07/07/2026 00:57</t>
+          <t>09/07/2026 05:48</t>
         </is>
       </c>
       <c r="L428" s="2" t="inlineStr">
         <is>
-          <t>17/07/2026 15:00</t>
+          <t>10/07/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -26995,7 +26995,7 @@
       </c>
       <c r="D429" s="2" t="inlineStr">
         <is>
-          <t>560503</t>
+          <t>559876</t>
         </is>
       </c>
       <c r="E429" s="2" t="inlineStr">
@@ -27005,12 +27005,12 @@
       </c>
       <c r="F429" s="2" t="inlineStr">
         <is>
-          <t>A0727</t>
+          <t>A1817</t>
         </is>
       </c>
       <c r="G429" s="2" t="inlineStr">
         <is>
-          <t>00019200000013454420</t>
+          <t>00019200000013419021</t>
         </is>
       </c>
       <c r="H429" s="2" t="inlineStr">
@@ -27020,22 +27020,22 @@
       </c>
       <c r="I429" s="2" t="inlineStr">
         <is>
-          <t>15/07/2026 23:21</t>
+          <t>07/07/2026 00:57</t>
         </is>
       </c>
       <c r="J429" s="2" t="inlineStr">
         <is>
-          <t>17/07/2026 12:20</t>
+          <t>17/07/2026 15:00</t>
         </is>
       </c>
       <c r="K429" s="2" t="inlineStr">
         <is>
-          <t>15/07/2026 23:21</t>
+          <t>07/07/2026 00:57</t>
         </is>
       </c>
       <c r="L429" s="2" t="inlineStr">
         <is>
-          <t>17/07/2026 12:20</t>
+          <t>17/07/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -27052,52 +27052,52 @@
       </c>
       <c r="C430" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D430" s="2" t="inlineStr">
         <is>
-          <t>559319</t>
+          <t>560503</t>
         </is>
       </c>
       <c r="E430" s="2" t="inlineStr">
         <is>
-          <t>SP</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="F430" s="2" t="inlineStr">
         <is>
-          <t>A8356</t>
+          <t>A0727</t>
         </is>
       </c>
       <c r="G430" s="2" t="inlineStr">
         <is>
-          <t>00019200000013247638</t>
+          <t>00019200000013454420</t>
         </is>
       </c>
       <c r="H430" s="2" t="inlineStr">
         <is>
-          <t>Rodoviário</t>
+          <t>MultiModal</t>
         </is>
       </c>
       <c r="I430" s="2" t="inlineStr">
         <is>
-          <t>01/07/2026 03:55</t>
+          <t>15/07/2026 23:21</t>
         </is>
       </c>
       <c r="J430" s="2" t="inlineStr">
         <is>
-          <t>01/07/2026 13:54</t>
+          <t>17/07/2026 12:20</t>
         </is>
       </c>
       <c r="K430" s="2" t="inlineStr">
         <is>
-          <t>01/07/2026 03:55</t>
+          <t>15/07/2026 23:21</t>
         </is>
       </c>
       <c r="L430" s="2" t="inlineStr">
         <is>
-          <t>01/07/2026 13:54</t>
+          <t>17/07/2026 12:20</t>
         </is>
       </c>
     </row>
@@ -27119,7 +27119,7 @@
       </c>
       <c r="D431" s="2" t="inlineStr">
         <is>
-          <t>559697</t>
+          <t>559319</t>
         </is>
       </c>
       <c r="E431" s="2" t="inlineStr">
@@ -27129,12 +27129,12 @@
       </c>
       <c r="F431" s="2" t="inlineStr">
         <is>
-          <t>A5033</t>
+          <t>A8356</t>
         </is>
       </c>
       <c r="G431" s="2" t="inlineStr">
         <is>
-          <t>00019200000013422723</t>
+          <t>00019200000013247638</t>
         </is>
       </c>
       <c r="H431" s="2" t="inlineStr">
@@ -27144,22 +27144,22 @@
       </c>
       <c r="I431" s="2" t="inlineStr">
         <is>
-          <t>03/07/2026 05:14</t>
+          <t>01/07/2026 03:55</t>
         </is>
       </c>
       <c r="J431" s="2" t="inlineStr">
         <is>
-          <t>03/07/2026 12:42</t>
+          <t>01/07/2026 13:54</t>
         </is>
       </c>
       <c r="K431" s="2" t="inlineStr">
         <is>
-          <t>03/07/2026 05:14</t>
+          <t>01/07/2026 03:55</t>
         </is>
       </c>
       <c r="L431" s="2" t="inlineStr">
         <is>
-          <t>03/07/2026 12:42</t>
+          <t>01/07/2026 13:54</t>
         </is>
       </c>
     </row>
@@ -27176,12 +27176,12 @@
       </c>
       <c r="C432" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D432" s="2" t="inlineStr">
         <is>
-          <t>559870</t>
+          <t>559697</t>
         </is>
       </c>
       <c r="E432" s="2" t="inlineStr">
@@ -27191,12 +27191,12 @@
       </c>
       <c r="F432" s="2" t="inlineStr">
         <is>
-          <t>A5209</t>
+          <t>A5033</t>
         </is>
       </c>
       <c r="G432" s="2" t="inlineStr">
         <is>
-          <t>00019200000013415280</t>
+          <t>00019200000013422723</t>
         </is>
       </c>
       <c r="H432" s="2" t="inlineStr">
@@ -27206,22 +27206,22 @@
       </c>
       <c r="I432" s="2" t="inlineStr">
         <is>
-          <t>17/07/2026 04:54</t>
+          <t>03/07/2026 05:14</t>
         </is>
       </c>
       <c r="J432" s="2" t="inlineStr">
         <is>
-          <t>17/07/2026 10:18</t>
+          <t>03/07/2026 12:42</t>
         </is>
       </c>
       <c r="K432" s="2" t="inlineStr">
         <is>
-          <t>17/07/2026 04:54</t>
+          <t>03/07/2026 05:14</t>
         </is>
       </c>
       <c r="L432" s="2" t="inlineStr">
         <is>
-          <t>20/07/2026 14:05</t>
+          <t>03/07/2026 12:42</t>
         </is>
       </c>
     </row>
@@ -27253,12 +27253,12 @@
       </c>
       <c r="F433" s="2" t="inlineStr">
         <is>
-          <t>A4755</t>
+          <t>A5209</t>
         </is>
       </c>
       <c r="G433" s="2" t="inlineStr">
         <is>
-          <t>00019200000013415298</t>
+          <t>00019200000013415280</t>
         </is>
       </c>
       <c r="H433" s="2" t="inlineStr">
@@ -27315,12 +27315,12 @@
       </c>
       <c r="F434" s="2" t="inlineStr">
         <is>
-          <t>A4555</t>
+          <t>A4755</t>
         </is>
       </c>
       <c r="G434" s="2" t="inlineStr">
         <is>
-          <t>00019200000013415301</t>
+          <t>00019200000013415298</t>
         </is>
       </c>
       <c r="H434" s="2" t="inlineStr">
@@ -27377,12 +27377,12 @@
       </c>
       <c r="F435" s="2" t="inlineStr">
         <is>
-          <t>A4843</t>
+          <t>A4555</t>
         </is>
       </c>
       <c r="G435" s="2" t="inlineStr">
         <is>
-          <t>00019200000013415310</t>
+          <t>00019200000013415301</t>
         </is>
       </c>
       <c r="H435" s="2" t="inlineStr">
@@ -27429,7 +27429,7 @@
       </c>
       <c r="D436" s="2" t="inlineStr">
         <is>
-          <t>560113</t>
+          <t>559870</t>
         </is>
       </c>
       <c r="E436" s="2" t="inlineStr">
@@ -27439,12 +27439,12 @@
       </c>
       <c r="F436" s="2" t="inlineStr">
         <is>
-          <t>A3818</t>
+          <t>A4843</t>
         </is>
       </c>
       <c r="G436" s="2" t="inlineStr">
         <is>
-          <t>00019200000013451758</t>
+          <t>00019200000013415310</t>
         </is>
       </c>
       <c r="H436" s="2" t="inlineStr">
@@ -27454,22 +27454,22 @@
       </c>
       <c r="I436" s="2" t="inlineStr">
         <is>
-          <t>15/07/2026 02:34</t>
+          <t>17/07/2026 04:54</t>
         </is>
       </c>
       <c r="J436" s="2" t="inlineStr">
         <is>
-          <t>15/07/2026 10:05</t>
+          <t>17/07/2026 10:18</t>
         </is>
       </c>
       <c r="K436" s="2" t="inlineStr">
         <is>
-          <t>15/07/2026 02:34</t>
+          <t>17/07/2026 04:54</t>
         </is>
       </c>
       <c r="L436" s="2" t="inlineStr">
         <is>
-          <t>15/07/2026 10:05</t>
+          <t>20/07/2026 14:05</t>
         </is>
       </c>
     </row>
@@ -27486,12 +27486,12 @@
       </c>
       <c r="C437" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D437" s="2" t="inlineStr">
         <is>
-          <t>561125</t>
+          <t>560113</t>
         </is>
       </c>
       <c r="E437" s="2" t="inlineStr">
@@ -27501,12 +27501,12 @@
       </c>
       <c r="F437" s="2" t="inlineStr">
         <is>
-          <t>A8303</t>
+          <t>A3818</t>
         </is>
       </c>
       <c r="G437" s="2" t="inlineStr">
         <is>
-          <t>00019200000013478745</t>
+          <t>00019200000013451758</t>
         </is>
       </c>
       <c r="H437" s="2" t="inlineStr">
@@ -27516,22 +27516,22 @@
       </c>
       <c r="I437" s="2" t="inlineStr">
         <is>
-          <t>16/07/2026 01:43</t>
+          <t>15/07/2026 02:34</t>
         </is>
       </c>
       <c r="J437" s="2" t="inlineStr">
         <is>
-          <t>16/07/2026 09:34</t>
+          <t>15/07/2026 10:05</t>
         </is>
       </c>
       <c r="K437" s="2" t="inlineStr">
         <is>
-          <t>16/07/2026 01:43</t>
+          <t>15/07/2026 02:34</t>
         </is>
       </c>
       <c r="L437" s="2" t="inlineStr">
         <is>
-          <t>16/07/2026 09:34</t>
+          <t>15/07/2026 10:05</t>
         </is>
       </c>
     </row>
@@ -27548,12 +27548,12 @@
       </c>
       <c r="C438" s="2" t="inlineStr">
         <is>
-          <t>-90 C a -60 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D438" s="2" t="inlineStr">
         <is>
-          <t>561435</t>
+          <t>561125</t>
         </is>
       </c>
       <c r="E438" s="2" t="inlineStr">
@@ -27563,12 +27563,12 @@
       </c>
       <c r="F438" s="2" t="inlineStr">
         <is>
-          <t>869170035491621</t>
+          <t>A8303</t>
         </is>
       </c>
       <c r="G438" s="2" t="inlineStr">
         <is>
-          <t>00019200000013751824</t>
+          <t>00019200000013478745</t>
         </is>
       </c>
       <c r="H438" s="2" t="inlineStr">
@@ -27578,22 +27578,22 @@
       </c>
       <c r="I438" s="2" t="inlineStr">
         <is>
-          <t>27/07/2026 01:06</t>
+          <t>16/07/2026 01:43</t>
         </is>
       </c>
       <c r="J438" s="2" t="inlineStr">
         <is>
-          <t>27/07/2026 09:08</t>
+          <t>16/07/2026 09:34</t>
         </is>
       </c>
       <c r="K438" s="2" t="inlineStr">
         <is>
-          <t>27/07/2026 01:06</t>
+          <t>16/07/2026 01:43</t>
         </is>
       </c>
       <c r="L438" s="2" t="inlineStr">
         <is>
-          <t>27/07/2026 09:11</t>
+          <t>16/07/2026 09:34</t>
         </is>
       </c>
     </row>
@@ -27625,12 +27625,12 @@
       </c>
       <c r="F439" s="2" t="inlineStr">
         <is>
-          <t>869170034887332</t>
+          <t>869170035491621</t>
         </is>
       </c>
       <c r="G439" s="2" t="inlineStr">
         <is>
-          <t>00019200000013751832</t>
+          <t>00019200000013751824</t>
         </is>
       </c>
       <c r="H439" s="2" t="inlineStr">
@@ -27687,12 +27687,12 @@
       </c>
       <c r="F440" s="2" t="inlineStr">
         <is>
-          <t>869170034874710</t>
+          <t>869170034887332</t>
         </is>
       </c>
       <c r="G440" s="2" t="inlineStr">
         <is>
-          <t>00019200000013751840</t>
+          <t>00019200000013751832</t>
         </is>
       </c>
       <c r="H440" s="2" t="inlineStr">
@@ -27749,12 +27749,12 @@
       </c>
       <c r="F441" s="2" t="inlineStr">
         <is>
-          <t>869170035511287</t>
+          <t>869170034874710</t>
         </is>
       </c>
       <c r="G441" s="2" t="inlineStr">
         <is>
-          <t>00019200000013751859</t>
+          <t>00019200000013751840</t>
         </is>
       </c>
       <c r="H441" s="2" t="inlineStr">
@@ -27811,12 +27811,12 @@
       </c>
       <c r="F442" s="2" t="inlineStr">
         <is>
-          <t>869170035511360</t>
+          <t>869170035511287</t>
         </is>
       </c>
       <c r="G442" s="2" t="inlineStr">
         <is>
-          <t>00019200000013751867</t>
+          <t>00019200000013751859</t>
         </is>
       </c>
       <c r="H442" s="2" t="inlineStr">
@@ -27873,12 +27873,12 @@
       </c>
       <c r="F443" s="2" t="inlineStr">
         <is>
-          <t>869170035518605</t>
+          <t>869170035511360</t>
         </is>
       </c>
       <c r="G443" s="2" t="inlineStr">
         <is>
-          <t>00019200000013751875</t>
+          <t>00019200000013751867</t>
         </is>
       </c>
       <c r="H443" s="2" t="inlineStr">
@@ -27920,12 +27920,12 @@
       </c>
       <c r="C444" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-90 C a -60 C</t>
         </is>
       </c>
       <c r="D444" s="2" t="inlineStr">
         <is>
-          <t>562000</t>
+          <t>561435</t>
         </is>
       </c>
       <c r="E444" s="2" t="inlineStr">
@@ -27935,12 +27935,12 @@
       </c>
       <c r="F444" s="2" t="inlineStr">
         <is>
-          <t>A3766</t>
+          <t>869170035518605</t>
         </is>
       </c>
       <c r="G444" s="2" t="inlineStr">
         <is>
-          <t>00019200000013595202</t>
+          <t>00019200000013751875</t>
         </is>
       </c>
       <c r="H444" s="2" t="inlineStr">
@@ -27950,22 +27950,22 @@
       </c>
       <c r="I444" s="2" t="inlineStr">
         <is>
-          <t>23/07/2026 03:21</t>
+          <t>27/07/2026 01:06</t>
         </is>
       </c>
       <c r="J444" s="2" t="inlineStr">
         <is>
-          <t>23/07/2026 12:49</t>
+          <t>27/07/2026 09:08</t>
         </is>
       </c>
       <c r="K444" s="2" t="inlineStr">
         <is>
-          <t>23/07/2026 03:21</t>
+          <t>27/07/2026 01:06</t>
         </is>
       </c>
       <c r="L444" s="2" t="inlineStr">
         <is>
-          <t>23/07/2026 12:49</t>
+          <t>27/07/2026 09:11</t>
         </is>
       </c>
     </row>
@@ -27982,52 +27982,52 @@
       </c>
       <c r="C445" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D445" s="2" t="inlineStr">
         <is>
-          <t>559781</t>
+          <t>562000</t>
         </is>
       </c>
       <c r="E445" s="2" t="inlineStr">
         <is>
-          <t>TO</t>
+          <t>SP</t>
         </is>
       </c>
       <c r="F445" s="2" t="inlineStr">
         <is>
-          <t>A8445</t>
+          <t>A3766</t>
         </is>
       </c>
       <c r="G445" s="2" t="inlineStr">
         <is>
-          <t>00019200000013419129</t>
+          <t>00019200000013595202</t>
         </is>
       </c>
       <c r="H445" s="2" t="inlineStr">
         <is>
-          <t>MultiModal</t>
+          <t>Rodoviário</t>
         </is>
       </c>
       <c r="I445" s="2" t="inlineStr">
         <is>
-          <t>07/07/2026 01:13</t>
+          <t>23/07/2026 03:21</t>
         </is>
       </c>
       <c r="J445" s="2" t="inlineStr">
         <is>
-          <t>08/07/2026 18:00</t>
+          <t>23/07/2026 12:49</t>
         </is>
       </c>
       <c r="K445" s="2" t="inlineStr">
         <is>
-          <t>07/07/2026 01:13</t>
+          <t>23/07/2026 03:21</t>
         </is>
       </c>
       <c r="L445" s="2" t="inlineStr">
         <is>
-          <t>08/07/2026 18:00</t>
+          <t>23/07/2026 12:49</t>
         </is>
       </c>
     </row>
@@ -28044,57 +28044,119 @@
       </c>
       <c r="C446" s="2" t="inlineStr">
         <is>
+          <t>-35 C a -15 C</t>
+        </is>
+      </c>
+      <c r="D446" s="2" t="inlineStr">
+        <is>
+          <t>559781</t>
+        </is>
+      </c>
+      <c r="E446" s="2" t="inlineStr">
+        <is>
+          <t>TO</t>
+        </is>
+      </c>
+      <c r="F446" s="2" t="inlineStr">
+        <is>
+          <t>A8445</t>
+        </is>
+      </c>
+      <c r="G446" s="2" t="inlineStr">
+        <is>
+          <t>00019200000013419129</t>
+        </is>
+      </c>
+      <c r="H446" s="2" t="inlineStr">
+        <is>
+          <t>MultiModal</t>
+        </is>
+      </c>
+      <c r="I446" s="2" t="inlineStr">
+        <is>
+          <t>07/07/2026 01:13</t>
+        </is>
+      </c>
+      <c r="J446" s="2" t="inlineStr">
+        <is>
+          <t>08/07/2026 18:00</t>
+        </is>
+      </c>
+      <c r="K446" s="2" t="inlineStr">
+        <is>
+          <t>07/07/2026 01:13</t>
+        </is>
+      </c>
+      <c r="L446" s="2" t="inlineStr">
+        <is>
+          <t>08/07/2026 18:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" s="2" t="inlineStr">
+        <is>
+          <t>CAIXA 42L</t>
+        </is>
+      </c>
+      <c r="B447" s="2" t="inlineStr">
+        <is>
+          <t>CAIXA 42L SEM BERÇO</t>
+        </is>
+      </c>
+      <c r="C447" s="2" t="inlineStr">
+        <is>
           <t>-25 C a -15 C</t>
         </is>
       </c>
-      <c r="D446" s="2" t="inlineStr">
+      <c r="D447" s="2" t="inlineStr">
         <is>
           <t>560364</t>
         </is>
       </c>
-      <c r="E446" s="2" t="inlineStr">
+      <c r="E447" s="2" t="inlineStr">
         <is>
           <t>TO</t>
         </is>
       </c>
-      <c r="F446" s="2" t="inlineStr">
+      <c r="F447" s="2" t="inlineStr">
         <is>
           <t>A8870</t>
         </is>
       </c>
-      <c r="G446" s="2" t="inlineStr">
+      <c r="G447" s="2" t="inlineStr">
         <is>
           <t>00019200000013491555</t>
         </is>
       </c>
-      <c r="H446" s="2" t="inlineStr">
-        <is>
-          <t>MultiModal</t>
-        </is>
-      </c>
-      <c r="I446" s="2" t="inlineStr">
+      <c r="H447" s="2" t="inlineStr">
+        <is>
+          <t>MultiModal</t>
+        </is>
+      </c>
+      <c r="I447" s="2" t="inlineStr">
         <is>
           <t>13/07/2026 01:44</t>
         </is>
       </c>
-      <c r="J446" s="2" t="inlineStr">
+      <c r="J447" s="2" t="inlineStr">
         <is>
           <t>15/07/2026 17:22</t>
         </is>
       </c>
-      <c r="K446" s="2" t="inlineStr">
+      <c r="K447" s="2" t="inlineStr">
         <is>
           <t>13/07/2026 01:44</t>
         </is>
       </c>
-      <c r="L446" s="2" t="inlineStr">
+      <c r="L447" s="2" t="inlineStr">
         <is>
           <t>15/07/2026 17:22</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L446"/>
+  <autoFilter ref="A1:L447"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-08-25 19:32:58
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixas_42l.xlsx
+++ b/relatorio_analitico_caixas_42l.xlsx
@@ -1795,7 +1795,7 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -6284,7 +6284,7 @@
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
@@ -7021,7 +7021,7 @@
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
@@ -7423,7 +7423,7 @@
       </c>
       <c r="C105" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D105" s="2" t="inlineStr">
@@ -14994,7 +14994,7 @@
       </c>
       <c r="C218" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D218" s="2" t="inlineStr">
@@ -18545,7 +18545,7 @@
       </c>
       <c r="C271" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D271" s="2" t="inlineStr">
@@ -18679,7 +18679,7 @@
       </c>
       <c r="C273" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D273" s="2" t="inlineStr">
@@ -19215,7 +19215,7 @@
       </c>
       <c r="C281" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D281" s="2" t="inlineStr">
@@ -19550,7 +19550,7 @@
       </c>
       <c r="C286" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D286" s="2" t="inlineStr">
@@ -22096,7 +22096,7 @@
       </c>
       <c r="C324" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D324" s="2" t="inlineStr">
@@ -24508,7 +24508,7 @@
       </c>
       <c r="C360" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D360" s="2" t="inlineStr">
@@ -24776,7 +24776,7 @@
       </c>
       <c r="C364" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D364" s="2" t="inlineStr">
@@ -25513,7 +25513,7 @@
       </c>
       <c r="C375" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D375" s="2" t="inlineStr">
@@ -31007,7 +31007,7 @@
       </c>
       <c r="C457" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D457" s="2" t="inlineStr">
@@ -31342,7 +31342,7 @@
       </c>
       <c r="C462" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D462" s="2" t="inlineStr">
@@ -31610,7 +31610,7 @@
       </c>
       <c r="C466" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D466" s="2" t="inlineStr">
@@ -31677,7 +31677,7 @@
       </c>
       <c r="C467" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D467" s="2" t="inlineStr">
@@ -34089,7 +34089,7 @@
       </c>
       <c r="C503" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D503" s="2" t="inlineStr">
@@ -36434,7 +36434,7 @@
       </c>
       <c r="C538" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D538" s="2" t="inlineStr">
@@ -39583,7 +39583,7 @@
       </c>
       <c r="C585" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D585" s="2" t="inlineStr">
@@ -42866,7 +42866,7 @@
       </c>
       <c r="C634" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D634" s="2" t="inlineStr">
@@ -43268,7 +43268,7 @@
       </c>
       <c r="C640" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D640" s="2" t="inlineStr">
@@ -43402,7 +43402,7 @@
       </c>
       <c r="C642" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D642" s="2" t="inlineStr">
@@ -45144,7 +45144,7 @@
       </c>
       <c r="C668" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D668" s="2" t="inlineStr">
@@ -46216,7 +46216,7 @@
       </c>
       <c r="C684" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D684" s="2" t="inlineStr">
@@ -46417,7 +46417,7 @@
       </c>
       <c r="C687" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D687" s="2" t="inlineStr">
@@ -46484,7 +46484,7 @@
       </c>
       <c r="C688" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D688" s="2" t="inlineStr">
@@ -49231,7 +49231,7 @@
       </c>
       <c r="C729" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D729" s="2" t="inlineStr">
@@ -49365,7 +49365,7 @@
       </c>
       <c r="C731" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D731" s="2" t="inlineStr">
@@ -50303,7 +50303,7 @@
       </c>
       <c r="C745" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D745" s="2" t="inlineStr">
@@ -51040,7 +51040,7 @@
       </c>
       <c r="C756" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D756" s="2" t="inlineStr">
@@ -55060,7 +55060,7 @@
       </c>
       <c r="C816" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D816" s="2" t="inlineStr">
@@ -55663,7 +55663,7 @@
       </c>
       <c r="C825" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D825" s="2" t="inlineStr">
@@ -55797,7 +55797,7 @@
       </c>
       <c r="C827" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D827" s="2" t="inlineStr">
@@ -57472,7 +57472,7 @@
       </c>
       <c r="C852" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D852" s="2" t="inlineStr">
@@ -58008,7 +58008,7 @@
       </c>
       <c r="C860" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D860" s="2" t="inlineStr">
@@ -58075,7 +58075,7 @@
       </c>
       <c r="C861" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D861" s="2" t="inlineStr">
@@ -59415,7 +59415,7 @@
       </c>
       <c r="C881" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D881" s="2" t="inlineStr">
@@ -60152,7 +60152,7 @@
       </c>
       <c r="C892" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D892" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-08-26 10:22:21
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixas_42l.xlsx
+++ b/relatorio_analitico_caixas_42l.xlsx
@@ -1728,7 +1728,7 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -4140,7 +4140,7 @@
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
@@ -6284,7 +6284,7 @@
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
@@ -7021,7 +7021,7 @@
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
@@ -7423,7 +7423,7 @@
       </c>
       <c r="C105" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D105" s="2" t="inlineStr">
@@ -14994,7 +14994,7 @@
       </c>
       <c r="C218" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D218" s="2" t="inlineStr">
@@ -16133,7 +16133,7 @@
       </c>
       <c r="C235" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D235" s="2" t="inlineStr">
@@ -18411,7 +18411,7 @@
       </c>
       <c r="C269" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D269" s="2" t="inlineStr">
@@ -18679,7 +18679,7 @@
       </c>
       <c r="C273" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D273" s="2" t="inlineStr">
@@ -22096,7 +22096,7 @@
       </c>
       <c r="C324" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D324" s="2" t="inlineStr">
@@ -22297,7 +22297,7 @@
       </c>
       <c r="C327" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D327" s="2" t="inlineStr">
@@ -24642,7 +24642,7 @@
       </c>
       <c r="C362" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D362" s="2" t="inlineStr">
@@ -24843,7 +24843,7 @@
       </c>
       <c r="C365" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D365" s="2" t="inlineStr">
@@ -31007,7 +31007,7 @@
       </c>
       <c r="C457" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D457" s="2" t="inlineStr">
@@ -31610,7 +31610,7 @@
       </c>
       <c r="C466" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D466" s="2" t="inlineStr">
@@ -31677,7 +31677,7 @@
       </c>
       <c r="C467" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D467" s="2" t="inlineStr">
@@ -36434,7 +36434,7 @@
       </c>
       <c r="C538" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D538" s="2" t="inlineStr">
@@ -36635,7 +36635,7 @@
       </c>
       <c r="C541" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D541" s="2" t="inlineStr">
@@ -39449,7 +39449,7 @@
       </c>
       <c r="C583" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D583" s="2" t="inlineStr">
@@ -39583,7 +39583,7 @@
       </c>
       <c r="C585" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D585" s="2" t="inlineStr">
@@ -42866,7 +42866,7 @@
       </c>
       <c r="C634" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D634" s="2" t="inlineStr">
@@ -43268,7 +43268,7 @@
       </c>
       <c r="C640" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D640" s="2" t="inlineStr">
@@ -43402,7 +43402,7 @@
       </c>
       <c r="C642" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D642" s="2" t="inlineStr">
@@ -46216,7 +46216,7 @@
       </c>
       <c r="C684" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D684" s="2" t="inlineStr">
@@ -46283,7 +46283,7 @@
       </c>
       <c r="C685" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D685" s="2" t="inlineStr">
@@ -47757,7 +47757,7 @@
       </c>
       <c r="C707" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D707" s="2" t="inlineStr">
@@ -49231,7 +49231,7 @@
       </c>
       <c r="C729" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D729" s="2" t="inlineStr">
@@ -49365,7 +49365,7 @@
       </c>
       <c r="C731" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D731" s="2" t="inlineStr">
@@ -49432,7 +49432,7 @@
       </c>
       <c r="C732" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D732" s="2" t="inlineStr">
@@ -50839,7 +50839,7 @@
       </c>
       <c r="C753" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D753" s="2" t="inlineStr">
@@ -55194,7 +55194,7 @@
       </c>
       <c r="C818" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D818" s="2" t="inlineStr">
@@ -55663,7 +55663,7 @@
       </c>
       <c r="C825" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D825" s="2" t="inlineStr">
@@ -57472,7 +57472,7 @@
       </c>
       <c r="C852" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D852" s="2" t="inlineStr">
@@ -58008,7 +58008,7 @@
       </c>
       <c r="C860" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D860" s="2" t="inlineStr">
@@ -58812,7 +58812,7 @@
       </c>
       <c r="C872" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D872" s="2" t="inlineStr">
@@ -59080,7 +59080,7 @@
       </c>
       <c r="C876" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D876" s="2" t="inlineStr">
@@ -60152,7 +60152,7 @@
       </c>
       <c r="C892" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D892" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-08-26 11:33:10
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixas_42l.xlsx
+++ b/relatorio_analitico_caixas_42l.xlsx
@@ -1728,7 +1728,7 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -1795,7 +1795,7 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -4140,7 +4140,7 @@
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
@@ -7423,7 +7423,7 @@
       </c>
       <c r="C105" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D105" s="2" t="inlineStr">
@@ -16133,7 +16133,7 @@
       </c>
       <c r="C235" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D235" s="2" t="inlineStr">
@@ -18411,7 +18411,7 @@
       </c>
       <c r="C269" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D269" s="2" t="inlineStr">
@@ -24642,7 +24642,7 @@
       </c>
       <c r="C362" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D362" s="2" t="inlineStr">
@@ -24776,7 +24776,7 @@
       </c>
       <c r="C364" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D364" s="2" t="inlineStr">
@@ -24843,7 +24843,7 @@
       </c>
       <c r="C365" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D365" s="2" t="inlineStr">
@@ -25513,7 +25513,7 @@
       </c>
       <c r="C375" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D375" s="2" t="inlineStr">
@@ -30940,7 +30940,7 @@
       </c>
       <c r="C456" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D456" s="2" t="inlineStr">
@@ -31007,7 +31007,7 @@
       </c>
       <c r="C457" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D457" s="2" t="inlineStr">
@@ -31342,7 +31342,7 @@
       </c>
       <c r="C462" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D462" s="2" t="inlineStr">
@@ -31543,7 +31543,7 @@
       </c>
       <c r="C465" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D465" s="2" t="inlineStr">
@@ -31610,7 +31610,7 @@
       </c>
       <c r="C466" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D466" s="2" t="inlineStr">
@@ -31677,7 +31677,7 @@
       </c>
       <c r="C467" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D467" s="2" t="inlineStr">
@@ -34089,7 +34089,7 @@
       </c>
       <c r="C503" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D503" s="2" t="inlineStr">
@@ -36501,7 +36501,7 @@
       </c>
       <c r="C539" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D539" s="2" t="inlineStr">
@@ -36635,7 +36635,7 @@
       </c>
       <c r="C541" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D541" s="2" t="inlineStr">
@@ -42397,7 +42397,7 @@
       </c>
       <c r="C627" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D627" s="2" t="inlineStr">
@@ -42464,7 +42464,7 @@
       </c>
       <c r="C628" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D628" s="2" t="inlineStr">
@@ -42866,7 +42866,7 @@
       </c>
       <c r="C634" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D634" s="2" t="inlineStr">
@@ -43268,7 +43268,7 @@
       </c>
       <c r="C640" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D640" s="2" t="inlineStr">
@@ -43469,7 +43469,7 @@
       </c>
       <c r="C643" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D643" s="2" t="inlineStr">
@@ -45144,7 +45144,7 @@
       </c>
       <c r="C668" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D668" s="2" t="inlineStr">
@@ -46216,7 +46216,7 @@
       </c>
       <c r="C684" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D684" s="2" t="inlineStr">
@@ -46283,7 +46283,7 @@
       </c>
       <c r="C685" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D685" s="2" t="inlineStr">
@@ -46484,7 +46484,7 @@
       </c>
       <c r="C688" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D688" s="2" t="inlineStr">
@@ -47757,7 +47757,7 @@
       </c>
       <c r="C707" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D707" s="2" t="inlineStr">
@@ -49298,7 +49298,7 @@
       </c>
       <c r="C730" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D730" s="2" t="inlineStr">
@@ -49365,7 +49365,7 @@
       </c>
       <c r="C731" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D731" s="2" t="inlineStr">
@@ -49432,7 +49432,7 @@
       </c>
       <c r="C732" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D732" s="2" t="inlineStr">
@@ -50303,7 +50303,7 @@
       </c>
       <c r="C745" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D745" s="2" t="inlineStr">
@@ -50839,7 +50839,7 @@
       </c>
       <c r="C753" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D753" s="2" t="inlineStr">
@@ -55194,7 +55194,7 @@
       </c>
       <c r="C818" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D818" s="2" t="inlineStr">
@@ -55328,7 +55328,7 @@
       </c>
       <c r="C820" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D820" s="2" t="inlineStr">
@@ -55663,7 +55663,7 @@
       </c>
       <c r="C825" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D825" s="2" t="inlineStr">
@@ -57472,7 +57472,7 @@
       </c>
       <c r="C852" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D852" s="2" t="inlineStr">
@@ -58812,7 +58812,7 @@
       </c>
       <c r="C872" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D872" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-08-26 14:41:37
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixas_42l.xlsx
+++ b/relatorio_analitico_caixas_42l.xlsx
@@ -4140,7 +4140,7 @@
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
@@ -6284,7 +6284,7 @@
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
@@ -16133,7 +16133,7 @@
       </c>
       <c r="C235" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D235" s="2" t="inlineStr">
@@ -18411,7 +18411,7 @@
       </c>
       <c r="C269" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D269" s="2" t="inlineStr">
@@ -18545,7 +18545,7 @@
       </c>
       <c r="C271" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D271" s="2" t="inlineStr">
@@ -19215,7 +19215,7 @@
       </c>
       <c r="C281" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D281" s="2" t="inlineStr">
@@ -25513,7 +25513,7 @@
       </c>
       <c r="C375" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D375" s="2" t="inlineStr">
@@ -31476,7 +31476,7 @@
       </c>
       <c r="C464" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D464" s="2" t="inlineStr">
@@ -36501,7 +36501,7 @@
       </c>
       <c r="C539" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D539" s="2" t="inlineStr">
@@ -39583,7 +39583,7 @@
       </c>
       <c r="C585" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D585" s="2" t="inlineStr">
@@ -42397,7 +42397,7 @@
       </c>
       <c r="C627" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D627" s="2" t="inlineStr">
@@ -43268,7 +43268,7 @@
       </c>
       <c r="C640" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D640" s="2" t="inlineStr">
@@ -45144,7 +45144,7 @@
       </c>
       <c r="C668" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D668" s="2" t="inlineStr">
@@ -46283,7 +46283,7 @@
       </c>
       <c r="C685" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D685" s="2" t="inlineStr">
@@ -46417,7 +46417,7 @@
       </c>
       <c r="C687" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D687" s="2" t="inlineStr">
@@ -47757,7 +47757,7 @@
       </c>
       <c r="C707" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D707" s="2" t="inlineStr">
@@ -49231,7 +49231,7 @@
       </c>
       <c r="C729" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D729" s="2" t="inlineStr">
@@ -49365,7 +49365,7 @@
       </c>
       <c r="C731" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D731" s="2" t="inlineStr">
@@ -50303,7 +50303,7 @@
       </c>
       <c r="C745" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D745" s="2" t="inlineStr">
@@ -51040,7 +51040,7 @@
       </c>
       <c r="C756" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D756" s="2" t="inlineStr">
@@ -55194,7 +55194,7 @@
       </c>
       <c r="C818" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D818" s="2" t="inlineStr">
@@ -55529,7 +55529,7 @@
       </c>
       <c r="C823" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D823" s="2" t="inlineStr">
@@ -55663,7 +55663,7 @@
       </c>
       <c r="C825" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D825" s="2" t="inlineStr">
@@ -55797,7 +55797,7 @@
       </c>
       <c r="C827" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D827" s="2" t="inlineStr">
@@ -55998,7 +55998,7 @@
       </c>
       <c r="C830" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D830" s="2" t="inlineStr">
@@ -57405,7 +57405,7 @@
       </c>
       <c r="C851" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D851" s="2" t="inlineStr">
@@ -59415,7 +59415,7 @@
       </c>
       <c r="C881" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D881" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-08-26 15:51:09
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixas_42l.xlsx
+++ b/relatorio_analitico_caixas_42l.xlsx
@@ -1795,7 +1795,7 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -4140,7 +4140,7 @@
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
@@ -7021,7 +7021,7 @@
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
@@ -15262,7 +15262,7 @@
       </c>
       <c r="C222" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D222" s="2" t="inlineStr">
@@ -15396,7 +15396,7 @@
       </c>
       <c r="C224" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D224" s="2" t="inlineStr">
@@ -16669,7 +16669,7 @@
       </c>
       <c r="C243" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D243" s="2" t="inlineStr">
@@ -17808,7 +17808,7 @@
       </c>
       <c r="C260" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D260" s="2" t="inlineStr">
@@ -18411,7 +18411,7 @@
       </c>
       <c r="C269" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D269" s="2" t="inlineStr">
@@ -22096,7 +22096,7 @@
       </c>
       <c r="C324" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D324" s="2" t="inlineStr">
@@ -24642,7 +24642,7 @@
       </c>
       <c r="C362" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D362" s="2" t="inlineStr">
@@ -24843,7 +24843,7 @@
       </c>
       <c r="C365" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D365" s="2" t="inlineStr">
@@ -27389,7 +27389,7 @@
       </c>
       <c r="C403" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D403" s="2" t="inlineStr">
@@ -34089,7 +34089,7 @@
       </c>
       <c r="C503" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D503" s="2" t="inlineStr">
@@ -36501,7 +36501,7 @@
       </c>
       <c r="C539" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D539" s="2" t="inlineStr">
@@ -42464,7 +42464,7 @@
       </c>
       <c r="C628" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D628" s="2" t="inlineStr">
@@ -42866,7 +42866,7 @@
       </c>
       <c r="C634" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D634" s="2" t="inlineStr">
@@ -43268,7 +43268,7 @@
       </c>
       <c r="C640" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D640" s="2" t="inlineStr">
@@ -46216,7 +46216,7 @@
       </c>
       <c r="C684" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D684" s="2" t="inlineStr">
@@ -46283,7 +46283,7 @@
       </c>
       <c r="C685" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D685" s="2" t="inlineStr">
@@ -46350,7 +46350,7 @@
       </c>
       <c r="C686" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D686" s="2" t="inlineStr">
@@ -46484,7 +46484,7 @@
       </c>
       <c r="C688" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D688" s="2" t="inlineStr">
@@ -49365,7 +49365,7 @@
       </c>
       <c r="C731" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D731" s="2" t="inlineStr">
@@ -50839,7 +50839,7 @@
       </c>
       <c r="C753" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D753" s="2" t="inlineStr">
@@ -55060,7 +55060,7 @@
       </c>
       <c r="C816" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D816" s="2" t="inlineStr">
@@ -55194,7 +55194,7 @@
       </c>
       <c r="C818" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D818" s="2" t="inlineStr">
@@ -58812,7 +58812,7 @@
       </c>
       <c r="C872" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D872" s="2" t="inlineStr">
@@ -59080,7 +59080,7 @@
       </c>
       <c r="C876" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D876" s="2" t="inlineStr">
@@ -59415,7 +59415,7 @@
       </c>
       <c r="C881" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D881" s="2" t="inlineStr">
@@ -60152,7 +60152,7 @@
       </c>
       <c r="C892" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D892" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-08-26 19:22:06
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixas_42l.xlsx
+++ b/relatorio_analitico_caixas_42l.xlsx
@@ -4140,7 +4140,7 @@
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
@@ -15396,7 +15396,7 @@
       </c>
       <c r="C224" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D224" s="2" t="inlineStr">
@@ -15463,7 +15463,7 @@
       </c>
       <c r="C225" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D225" s="2" t="inlineStr">
@@ -17808,7 +17808,7 @@
       </c>
       <c r="C260" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D260" s="2" t="inlineStr">
@@ -18411,7 +18411,7 @@
       </c>
       <c r="C269" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D269" s="2" t="inlineStr">
@@ -18679,7 +18679,7 @@
       </c>
       <c r="C273" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D273" s="2" t="inlineStr">
@@ -19215,7 +19215,7 @@
       </c>
       <c r="C281" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D281" s="2" t="inlineStr">
@@ -19550,7 +19550,7 @@
       </c>
       <c r="C286" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D286" s="2" t="inlineStr">
@@ -19684,7 +19684,7 @@
       </c>
       <c r="C288" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D288" s="2" t="inlineStr">
@@ -24508,7 +24508,7 @@
       </c>
       <c r="C360" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D360" s="2" t="inlineStr">
@@ -25513,7 +25513,7 @@
       </c>
       <c r="C375" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D375" s="2" t="inlineStr">
@@ -30940,7 +30940,7 @@
       </c>
       <c r="C456" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D456" s="2" t="inlineStr">
@@ -31007,7 +31007,7 @@
       </c>
       <c r="C457" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D457" s="2" t="inlineStr">
@@ -31476,7 +31476,7 @@
       </c>
       <c r="C464" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D464" s="2" t="inlineStr">
@@ -31610,7 +31610,7 @@
       </c>
       <c r="C466" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D466" s="2" t="inlineStr">
@@ -31677,7 +31677,7 @@
       </c>
       <c r="C467" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D467" s="2" t="inlineStr">
@@ -34089,7 +34089,7 @@
       </c>
       <c r="C503" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D503" s="2" t="inlineStr">
@@ -39583,7 +39583,7 @@
       </c>
       <c r="C585" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D585" s="2" t="inlineStr">
@@ -42397,7 +42397,7 @@
       </c>
       <c r="C627" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D627" s="2" t="inlineStr">
@@ -42464,7 +42464,7 @@
       </c>
       <c r="C628" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D628" s="2" t="inlineStr">
@@ -42866,7 +42866,7 @@
       </c>
       <c r="C634" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D634" s="2" t="inlineStr">
@@ -46283,7 +46283,7 @@
       </c>
       <c r="C685" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D685" s="2" t="inlineStr">
@@ -46417,7 +46417,7 @@
       </c>
       <c r="C687" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D687" s="2" t="inlineStr">
@@ -49365,7 +49365,7 @@
       </c>
       <c r="C731" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D731" s="2" t="inlineStr">
@@ -50839,7 +50839,7 @@
       </c>
       <c r="C753" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D753" s="2" t="inlineStr">
@@ -51040,7 +51040,7 @@
       </c>
       <c r="C756" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D756" s="2" t="inlineStr">
@@ -55060,7 +55060,7 @@
       </c>
       <c r="C816" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D816" s="2" t="inlineStr">
@@ -55194,7 +55194,7 @@
       </c>
       <c r="C818" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D818" s="2" t="inlineStr">
@@ -55328,7 +55328,7 @@
       </c>
       <c r="C820" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D820" s="2" t="inlineStr">
@@ -55529,7 +55529,7 @@
       </c>
       <c r="C823" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D823" s="2" t="inlineStr">
@@ -55663,7 +55663,7 @@
       </c>
       <c r="C825" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D825" s="2" t="inlineStr">
@@ -57405,7 +57405,7 @@
       </c>
       <c r="C851" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D851" s="2" t="inlineStr">
@@ -57941,7 +57941,7 @@
       </c>
       <c r="C859" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D859" s="2" t="inlineStr">
@@ -58075,7 +58075,7 @@
       </c>
       <c r="C861" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D861" s="2" t="inlineStr">
@@ -58812,7 +58812,7 @@
       </c>
       <c r="C872" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D872" s="2" t="inlineStr">
@@ -59080,7 +59080,7 @@
       </c>
       <c r="C876" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D876" s="2" t="inlineStr">
@@ -60152,7 +60152,7 @@
       </c>
       <c r="C892" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D892" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-08-27 00:01:26
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixas_42l.xlsx
+++ b/relatorio_analitico_caixas_42l.xlsx
@@ -1728,7 +1728,7 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -6284,7 +6284,7 @@
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
@@ -15396,7 +15396,7 @@
       </c>
       <c r="C224" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D224" s="2" t="inlineStr">
@@ -16669,7 +16669,7 @@
       </c>
       <c r="C243" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D243" s="2" t="inlineStr">
@@ -17808,7 +17808,7 @@
       </c>
       <c r="C260" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D260" s="2" t="inlineStr">
@@ -19215,7 +19215,7 @@
       </c>
       <c r="C281" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D281" s="2" t="inlineStr">
@@ -22297,7 +22297,7 @@
       </c>
       <c r="C327" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D327" s="2" t="inlineStr">
@@ -24508,7 +24508,7 @@
       </c>
       <c r="C360" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D360" s="2" t="inlineStr">
@@ -24843,7 +24843,7 @@
       </c>
       <c r="C365" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D365" s="2" t="inlineStr">
@@ -25513,7 +25513,7 @@
       </c>
       <c r="C375" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D375" s="2" t="inlineStr">
@@ -31543,7 +31543,7 @@
       </c>
       <c r="C465" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D465" s="2" t="inlineStr">
@@ -31677,7 +31677,7 @@
       </c>
       <c r="C467" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D467" s="2" t="inlineStr">
@@ -36434,7 +36434,7 @@
       </c>
       <c r="C538" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D538" s="2" t="inlineStr">
@@ -39449,7 +39449,7 @@
       </c>
       <c r="C583" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D583" s="2" t="inlineStr">
@@ -39583,7 +39583,7 @@
       </c>
       <c r="C585" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D585" s="2" t="inlineStr">
@@ -42866,7 +42866,7 @@
       </c>
       <c r="C634" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D634" s="2" t="inlineStr">
@@ -43268,7 +43268,7 @@
       </c>
       <c r="C640" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D640" s="2" t="inlineStr">
@@ -43402,7 +43402,7 @@
       </c>
       <c r="C642" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D642" s="2" t="inlineStr">
@@ -43469,7 +43469,7 @@
       </c>
       <c r="C643" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D643" s="2" t="inlineStr">
@@ -46283,7 +46283,7 @@
       </c>
       <c r="C685" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D685" s="2" t="inlineStr">
@@ -46484,7 +46484,7 @@
       </c>
       <c r="C688" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D688" s="2" t="inlineStr">
@@ -47757,7 +47757,7 @@
       </c>
       <c r="C707" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D707" s="2" t="inlineStr">
@@ -49231,7 +49231,7 @@
       </c>
       <c r="C729" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D729" s="2" t="inlineStr">
@@ -50303,7 +50303,7 @@
       </c>
       <c r="C745" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D745" s="2" t="inlineStr">
@@ -50839,7 +50839,7 @@
       </c>
       <c r="C753" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D753" s="2" t="inlineStr">
@@ -51040,7 +51040,7 @@
       </c>
       <c r="C756" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D756" s="2" t="inlineStr">
@@ -55194,7 +55194,7 @@
       </c>
       <c r="C818" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D818" s="2" t="inlineStr">
@@ -55663,7 +55663,7 @@
       </c>
       <c r="C825" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D825" s="2" t="inlineStr">
@@ -55998,7 +55998,7 @@
       </c>
       <c r="C830" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D830" s="2" t="inlineStr">
@@ -57405,7 +57405,7 @@
       </c>
       <c r="C851" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D851" s="2" t="inlineStr">
@@ -58075,7 +58075,7 @@
       </c>
       <c r="C861" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D861" s="2" t="inlineStr">
@@ -59415,7 +59415,7 @@
       </c>
       <c r="C881" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D881" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-08-27 01:41:49
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixas_42l.xlsx
+++ b/relatorio_analitico_caixas_42l.xlsx
@@ -1795,7 +1795,7 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -7423,7 +7423,7 @@
       </c>
       <c r="C105" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D105" s="2" t="inlineStr">
@@ -14994,7 +14994,7 @@
       </c>
       <c r="C218" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D218" s="2" t="inlineStr">
@@ -15262,7 +15262,7 @@
       </c>
       <c r="C222" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D222" s="2" t="inlineStr">
@@ -17808,7 +17808,7 @@
       </c>
       <c r="C260" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D260" s="2" t="inlineStr">
@@ -18411,7 +18411,7 @@
       </c>
       <c r="C269" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D269" s="2" t="inlineStr">
@@ -19684,7 +19684,7 @@
       </c>
       <c r="C288" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D288" s="2" t="inlineStr">
@@ -22096,7 +22096,7 @@
       </c>
       <c r="C324" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D324" s="2" t="inlineStr">
@@ -22297,7 +22297,7 @@
       </c>
       <c r="C327" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D327" s="2" t="inlineStr">
@@ -24843,7 +24843,7 @@
       </c>
       <c r="C365" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D365" s="2" t="inlineStr">
@@ -25513,7 +25513,7 @@
       </c>
       <c r="C375" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D375" s="2" t="inlineStr">
@@ -30940,7 +30940,7 @@
       </c>
       <c r="C456" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D456" s="2" t="inlineStr">
@@ -31476,7 +31476,7 @@
       </c>
       <c r="C464" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D464" s="2" t="inlineStr">
@@ -31543,7 +31543,7 @@
       </c>
       <c r="C465" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D465" s="2" t="inlineStr">
@@ -31610,7 +31610,7 @@
       </c>
       <c r="C466" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D466" s="2" t="inlineStr">
@@ -31677,7 +31677,7 @@
       </c>
       <c r="C467" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D467" s="2" t="inlineStr">
@@ -36635,7 +36635,7 @@
       </c>
       <c r="C541" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D541" s="2" t="inlineStr">
@@ -39583,7 +39583,7 @@
       </c>
       <c r="C585" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D585" s="2" t="inlineStr">
@@ -43469,7 +43469,7 @@
       </c>
       <c r="C643" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D643" s="2" t="inlineStr">
@@ -46283,7 +46283,7 @@
       </c>
       <c r="C685" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D685" s="2" t="inlineStr">
@@ -46484,7 +46484,7 @@
       </c>
       <c r="C688" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D688" s="2" t="inlineStr">
@@ -47757,7 +47757,7 @@
       </c>
       <c r="C707" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D707" s="2" t="inlineStr">
@@ -49365,7 +49365,7 @@
       </c>
       <c r="C731" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D731" s="2" t="inlineStr">
@@ -49432,7 +49432,7 @@
       </c>
       <c r="C732" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D732" s="2" t="inlineStr">
@@ -55194,7 +55194,7 @@
       </c>
       <c r="C818" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D818" s="2" t="inlineStr">
@@ -55328,7 +55328,7 @@
       </c>
       <c r="C820" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D820" s="2" t="inlineStr">
@@ -55663,7 +55663,7 @@
       </c>
       <c r="C825" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D825" s="2" t="inlineStr">
@@ -55998,7 +55998,7 @@
       </c>
       <c r="C830" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D830" s="2" t="inlineStr">
@@ -58008,7 +58008,7 @@
       </c>
       <c r="C860" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D860" s="2" t="inlineStr">
@@ -60152,7 +60152,7 @@
       </c>
       <c r="C892" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D892" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-08-27 02:01:40
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixas_42l.xlsx
+++ b/relatorio_analitico_caixas_42l.xlsx
@@ -1728,7 +1728,7 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -6284,7 +6284,7 @@
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
@@ -7423,7 +7423,7 @@
       </c>
       <c r="C105" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D105" s="2" t="inlineStr">
@@ -14994,7 +14994,7 @@
       </c>
       <c r="C218" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D218" s="2" t="inlineStr">
@@ -15262,7 +15262,7 @@
       </c>
       <c r="C222" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D222" s="2" t="inlineStr">
@@ -17808,7 +17808,7 @@
       </c>
       <c r="C260" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D260" s="2" t="inlineStr">
@@ -18411,7 +18411,7 @@
       </c>
       <c r="C269" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D269" s="2" t="inlineStr">
@@ -18679,7 +18679,7 @@
       </c>
       <c r="C273" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D273" s="2" t="inlineStr">
@@ -19215,7 +19215,7 @@
       </c>
       <c r="C281" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D281" s="2" t="inlineStr">
@@ -19550,7 +19550,7 @@
       </c>
       <c r="C286" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D286" s="2" t="inlineStr">
@@ -19684,7 +19684,7 @@
       </c>
       <c r="C288" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D288" s="2" t="inlineStr">
@@ -22096,7 +22096,7 @@
       </c>
       <c r="C324" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D324" s="2" t="inlineStr">
@@ -24508,7 +24508,7 @@
       </c>
       <c r="C360" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D360" s="2" t="inlineStr">
@@ -24776,7 +24776,7 @@
       </c>
       <c r="C364" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D364" s="2" t="inlineStr">
@@ -30940,7 +30940,7 @@
       </c>
       <c r="C456" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D456" s="2" t="inlineStr">
@@ -31476,7 +31476,7 @@
       </c>
       <c r="C464" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D464" s="2" t="inlineStr">
@@ -31543,7 +31543,7 @@
       </c>
       <c r="C465" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D465" s="2" t="inlineStr">
@@ -31610,7 +31610,7 @@
       </c>
       <c r="C466" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D466" s="2" t="inlineStr">
@@ -34089,7 +34089,7 @@
       </c>
       <c r="C503" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D503" s="2" t="inlineStr">
@@ -36501,7 +36501,7 @@
       </c>
       <c r="C539" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D539" s="2" t="inlineStr">
@@ -42397,7 +42397,7 @@
       </c>
       <c r="C627" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D627" s="2" t="inlineStr">
@@ -42464,7 +42464,7 @@
       </c>
       <c r="C628" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D628" s="2" t="inlineStr">
@@ -43268,7 +43268,7 @@
       </c>
       <c r="C640" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D640" s="2" t="inlineStr">
@@ -43402,7 +43402,7 @@
       </c>
       <c r="C642" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D642" s="2" t="inlineStr">
@@ -46417,7 +46417,7 @@
       </c>
       <c r="C687" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D687" s="2" t="inlineStr">
@@ -47757,7 +47757,7 @@
       </c>
       <c r="C707" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D707" s="2" t="inlineStr">
@@ -49432,7 +49432,7 @@
       </c>
       <c r="C732" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D732" s="2" t="inlineStr">
@@ -50303,7 +50303,7 @@
       </c>
       <c r="C745" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D745" s="2" t="inlineStr">
@@ -51040,7 +51040,7 @@
       </c>
       <c r="C756" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D756" s="2" t="inlineStr">
@@ -55328,7 +55328,7 @@
       </c>
       <c r="C820" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D820" s="2" t="inlineStr">
@@ -55529,7 +55529,7 @@
       </c>
       <c r="C823" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D823" s="2" t="inlineStr">
@@ -57941,7 +57941,7 @@
       </c>
       <c r="C859" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D859" s="2" t="inlineStr">
@@ -60152,7 +60152,7 @@
       </c>
       <c r="C892" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D892" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-08-27 06:31:58
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixas_42l.xlsx
+++ b/relatorio_analitico_caixas_42l.xlsx
@@ -1795,7 +1795,7 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -7423,7 +7423,7 @@
       </c>
       <c r="C105" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D105" s="2" t="inlineStr">
@@ -14994,7 +14994,7 @@
       </c>
       <c r="C218" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D218" s="2" t="inlineStr">
@@ -17808,7 +17808,7 @@
       </c>
       <c r="C260" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D260" s="2" t="inlineStr">
@@ -18411,7 +18411,7 @@
       </c>
       <c r="C269" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D269" s="2" t="inlineStr">
@@ -18679,7 +18679,7 @@
       </c>
       <c r="C273" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D273" s="2" t="inlineStr">
@@ -19684,7 +19684,7 @@
       </c>
       <c r="C288" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D288" s="2" t="inlineStr">
@@ -22096,7 +22096,7 @@
       </c>
       <c r="C324" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D324" s="2" t="inlineStr">
@@ -22297,7 +22297,7 @@
       </c>
       <c r="C327" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D327" s="2" t="inlineStr">
@@ -24776,7 +24776,7 @@
       </c>
       <c r="C364" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D364" s="2" t="inlineStr">
@@ -24843,7 +24843,7 @@
       </c>
       <c r="C365" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D365" s="2" t="inlineStr">
@@ -31007,7 +31007,7 @@
       </c>
       <c r="C457" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D457" s="2" t="inlineStr">
@@ -31476,7 +31476,7 @@
       </c>
       <c r="C464" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D464" s="2" t="inlineStr">
@@ -31543,7 +31543,7 @@
       </c>
       <c r="C465" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D465" s="2" t="inlineStr">
@@ -31610,7 +31610,7 @@
       </c>
       <c r="C466" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D466" s="2" t="inlineStr">
@@ -34089,7 +34089,7 @@
       </c>
       <c r="C503" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D503" s="2" t="inlineStr">
@@ -36434,7 +36434,7 @@
       </c>
       <c r="C538" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D538" s="2" t="inlineStr">
@@ -39449,7 +39449,7 @@
       </c>
       <c r="C583" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D583" s="2" t="inlineStr">
@@ -43268,7 +43268,7 @@
       </c>
       <c r="C640" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D640" s="2" t="inlineStr">
@@ -43402,7 +43402,7 @@
       </c>
       <c r="C642" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D642" s="2" t="inlineStr">
@@ -43469,7 +43469,7 @@
       </c>
       <c r="C643" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D643" s="2" t="inlineStr">
@@ -45144,7 +45144,7 @@
       </c>
       <c r="C668" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D668" s="2" t="inlineStr">
@@ -49365,7 +49365,7 @@
       </c>
       <c r="C731" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D731" s="2" t="inlineStr">
@@ -55060,7 +55060,7 @@
       </c>
       <c r="C816" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D816" s="2" t="inlineStr">
@@ -55194,7 +55194,7 @@
       </c>
       <c r="C818" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D818" s="2" t="inlineStr">
@@ -55328,7 +55328,7 @@
       </c>
       <c r="C820" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D820" s="2" t="inlineStr">
@@ -55529,7 +55529,7 @@
       </c>
       <c r="C823" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D823" s="2" t="inlineStr">
@@ -55797,7 +55797,7 @@
       </c>
       <c r="C827" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D827" s="2" t="inlineStr">
@@ -57472,7 +57472,7 @@
       </c>
       <c r="C852" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D852" s="2" t="inlineStr">
@@ -57941,7 +57941,7 @@
       </c>
       <c r="C859" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D859" s="2" t="inlineStr">
@@ -58008,7 +58008,7 @@
       </c>
       <c r="C860" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D860" s="2" t="inlineStr">
@@ -58075,7 +58075,7 @@
       </c>
       <c r="C861" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D861" s="2" t="inlineStr">
@@ -58812,7 +58812,7 @@
       </c>
       <c r="C872" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D872" s="2" t="inlineStr">
@@ -59080,7 +59080,7 @@
       </c>
       <c r="C876" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D876" s="2" t="inlineStr">
@@ -59415,7 +59415,7 @@
       </c>
       <c r="C881" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D881" s="2" t="inlineStr">
@@ -60152,7 +60152,7 @@
       </c>
       <c r="C892" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D892" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-08-31 15:12:58
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixas_42l.xlsx
+++ b/relatorio_analitico_caixas_42l.xlsx
@@ -4207,7 +4207,7 @@
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
@@ -6552,7 +6552,7 @@
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
@@ -7691,7 +7691,7 @@
       </c>
       <c r="C109" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D109" s="2" t="inlineStr">
@@ -15262,7 +15262,7 @@
       </c>
       <c r="C222" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D222" s="2" t="inlineStr">
@@ -15664,7 +15664,7 @@
       </c>
       <c r="C228" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D228" s="2" t="inlineStr">
@@ -16401,7 +16401,7 @@
       </c>
       <c r="C239" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D239" s="2" t="inlineStr">
@@ -18947,7 +18947,7 @@
       </c>
       <c r="C277" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D277" s="2" t="inlineStr">
@@ -20622,7 +20622,7 @@
       </c>
       <c r="C302" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D302" s="2" t="inlineStr">
@@ -20756,7 +20756,7 @@
       </c>
       <c r="C304" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D304" s="2" t="inlineStr">
@@ -25848,7 +25848,7 @@
       </c>
       <c r="C380" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D380" s="2" t="inlineStr">
@@ -25915,7 +25915,7 @@
       </c>
       <c r="C381" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D381" s="2" t="inlineStr">
@@ -26585,7 +26585,7 @@
       </c>
       <c r="C391" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D391" s="2" t="inlineStr">
@@ -32615,7 +32615,7 @@
       </c>
       <c r="C481" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D481" s="2" t="inlineStr">
@@ -32749,7 +32749,7 @@
       </c>
       <c r="C483" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D483" s="2" t="inlineStr">
@@ -35228,7 +35228,7 @@
       </c>
       <c r="C520" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D520" s="2" t="inlineStr">
@@ -37573,7 +37573,7 @@
       </c>
       <c r="C555" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D555" s="2" t="inlineStr">
@@ -37640,7 +37640,7 @@
       </c>
       <c r="C556" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D556" s="2" t="inlineStr">
@@ -39918,7 +39918,7 @@
       </c>
       <c r="C590" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D590" s="2" t="inlineStr">
@@ -46819,7 +46819,7 @@
       </c>
       <c r="C693" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D693" s="2" t="inlineStr">
@@ -47690,7 +47690,7 @@
       </c>
       <c r="C706" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D706" s="2" t="inlineStr">
@@ -47824,7 +47824,7 @@
       </c>
       <c r="C708" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D708" s="2" t="inlineStr">
@@ -50705,7 +50705,7 @@
       </c>
       <c r="C751" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D751" s="2" t="inlineStr">
@@ -50772,7 +50772,7 @@
       </c>
       <c r="C752" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D752" s="2" t="inlineStr">
@@ -53854,7 +53854,7 @@
       </c>
       <c r="C798" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D798" s="2" t="inlineStr">
@@ -55328,7 +55328,7 @@
       </c>
       <c r="C820" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D820" s="2" t="inlineStr">
@@ -59549,7 +59549,7 @@
       </c>
       <c r="C883" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D883" s="2" t="inlineStr">
@@ -59683,7 +59683,7 @@
       </c>
       <c r="C885" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D885" s="2" t="inlineStr">
@@ -59750,7 +59750,7 @@
       </c>
       <c r="C886" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D886" s="2" t="inlineStr">
@@ -59884,7 +59884,7 @@
       </c>
       <c r="C888" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D888" s="2" t="inlineStr">
@@ -60085,7 +60085,7 @@
       </c>
       <c r="C891" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D891" s="2" t="inlineStr">
@@ -60219,7 +60219,7 @@
       </c>
       <c r="C893" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D893" s="2" t="inlineStr">
@@ -60353,7 +60353,7 @@
       </c>
       <c r="C895" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D895" s="2" t="inlineStr">
@@ -62028,7 +62028,7 @@
       </c>
       <c r="C920" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D920" s="2" t="inlineStr">
@@ -62497,7 +62497,7 @@
       </c>
       <c r="C927" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D927" s="2" t="inlineStr">
@@ -63636,7 +63636,7 @@
       </c>
       <c r="C944" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D944" s="2" t="inlineStr">
@@ -64842,7 +64842,7 @@
       </c>
       <c r="C962" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D962" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-01 17:28:08
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixas_42l.xlsx
+++ b/relatorio_analitico_caixas_42l.xlsx
@@ -1996,7 +1996,7 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -4341,7 +4341,7 @@
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
@@ -6753,7 +6753,7 @@
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
@@ -15530,7 +15530,7 @@
       </c>
       <c r="C226" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D226" s="2" t="inlineStr">
@@ -15798,7 +15798,7 @@
       </c>
       <c r="C230" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D230" s="2" t="inlineStr">
@@ -17205,7 +17205,7 @@
       </c>
       <c r="C251" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D251" s="2" t="inlineStr">
@@ -18344,7 +18344,7 @@
       </c>
       <c r="C268" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D268" s="2" t="inlineStr">
@@ -18947,7 +18947,7 @@
       </c>
       <c r="C277" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D277" s="2" t="inlineStr">
@@ -19081,7 +19081,7 @@
       </c>
       <c r="C279" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D279" s="2" t="inlineStr">
@@ -19215,7 +19215,7 @@
       </c>
       <c r="C281" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D281" s="2" t="inlineStr">
@@ -20890,7 +20890,7 @@
       </c>
       <c r="C306" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D306" s="2" t="inlineStr">
@@ -26183,7 +26183,7 @@
       </c>
       <c r="C385" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D385" s="2" t="inlineStr">
@@ -26853,7 +26853,7 @@
       </c>
       <c r="C395" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D395" s="2" t="inlineStr">
@@ -28729,7 +28729,7 @@
       </c>
       <c r="C423" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D423" s="2" t="inlineStr">
@@ -32347,7 +32347,7 @@
       </c>
       <c r="C477" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D477" s="2" t="inlineStr">
@@ -32749,7 +32749,7 @@
       </c>
       <c r="C483" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D483" s="2" t="inlineStr">
@@ -32883,7 +32883,7 @@
       </c>
       <c r="C485" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D485" s="2" t="inlineStr">
@@ -37908,7 +37908,7 @@
       </c>
       <c r="C560" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D560" s="2" t="inlineStr">
@@ -48427,7 +48427,7 @@
       </c>
       <c r="C717" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D717" s="2" t="inlineStr">
@@ -48494,7 +48494,7 @@
       </c>
       <c r="C718" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D718" s="2" t="inlineStr">
@@ -49365,7 +49365,7 @@
       </c>
       <c r="C731" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D731" s="2" t="inlineStr">
@@ -52648,7 +52648,7 @@
       </c>
       <c r="C780" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D780" s="2" t="inlineStr">
@@ -53921,7 +53921,7 @@
       </c>
       <c r="C799" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D799" s="2" t="inlineStr">
@@ -55395,7 +55395,7 @@
       </c>
       <c r="C821" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D821" s="2" t="inlineStr">
@@ -55529,7 +55529,7 @@
       </c>
       <c r="C823" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D823" s="2" t="inlineStr">
@@ -56467,7 +56467,7 @@
       </c>
       <c r="C837" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D837" s="2" t="inlineStr">
@@ -57003,7 +57003,7 @@
       </c>
       <c r="C845" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D845" s="2" t="inlineStr">
@@ -61425,7 +61425,7 @@
       </c>
       <c r="C911" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D911" s="2" t="inlineStr">
@@ -61894,7 +61894,7 @@
       </c>
       <c r="C918" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D918" s="2" t="inlineStr">
@@ -63703,7 +63703,7 @@
       </c>
       <c r="C945" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D945" s="2" t="inlineStr">
@@ -66517,7 +66517,7 @@
       </c>
       <c r="C987" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D987" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-01 19:26:00
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixas_42l.xlsx
+++ b/relatorio_analitico_caixas_42l.xlsx
@@ -1996,7 +1996,7 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -4341,7 +4341,7 @@
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
@@ -6753,7 +6753,7 @@
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
@@ -7490,7 +7490,7 @@
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D106" s="2" t="inlineStr">
@@ -7959,7 +7959,7 @@
       </c>
       <c r="C113" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D113" s="2" t="inlineStr">
@@ -15530,7 +15530,7 @@
       </c>
       <c r="C226" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D226" s="2" t="inlineStr">
@@ -15798,7 +15798,7 @@
       </c>
       <c r="C230" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D230" s="2" t="inlineStr">
@@ -15932,7 +15932,7 @@
       </c>
       <c r="C232" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D232" s="2" t="inlineStr">
@@ -16669,7 +16669,7 @@
       </c>
       <c r="C243" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D243" s="2" t="inlineStr">
@@ -18344,7 +18344,7 @@
       </c>
       <c r="C268" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D268" s="2" t="inlineStr">
@@ -18947,7 +18947,7 @@
       </c>
       <c r="C277" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D277" s="2" t="inlineStr">
@@ -19081,7 +19081,7 @@
       </c>
       <c r="C279" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D279" s="2" t="inlineStr">
@@ -20890,7 +20890,7 @@
       </c>
       <c r="C306" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D306" s="2" t="inlineStr">
@@ -23436,7 +23436,7 @@
       </c>
       <c r="C344" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D344" s="2" t="inlineStr">
@@ -25982,7 +25982,7 @@
       </c>
       <c r="C382" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D382" s="2" t="inlineStr">
@@ -28729,7 +28729,7 @@
       </c>
       <c r="C423" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D423" s="2" t="inlineStr">
@@ -32414,7 +32414,7 @@
       </c>
       <c r="C478" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D478" s="2" t="inlineStr">
@@ -32883,7 +32883,7 @@
       </c>
       <c r="C485" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D485" s="2" t="inlineStr">
@@ -33017,7 +33017,7 @@
       </c>
       <c r="C487" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D487" s="2" t="inlineStr">
@@ -33084,7 +33084,7 @@
       </c>
       <c r="C488" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D488" s="2" t="inlineStr">
@@ -37841,7 +37841,7 @@
       </c>
       <c r="C559" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D559" s="2" t="inlineStr">
@@ -37908,7 +37908,7 @@
       </c>
       <c r="C560" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D560" s="2" t="inlineStr">
@@ -40186,7 +40186,7 @@
       </c>
       <c r="C594" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D594" s="2" t="inlineStr">
@@ -43000,7 +43000,7 @@
       </c>
       <c r="C636" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D636" s="2" t="inlineStr">
@@ -45613,7 +45613,7 @@
       </c>
       <c r="C675" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D675" s="2" t="inlineStr">
@@ -49365,7 +49365,7 @@
       </c>
       <c r="C731" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D731" s="2" t="inlineStr">
@@ -49566,7 +49566,7 @@
       </c>
       <c r="C734" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D734" s="2" t="inlineStr">
@@ -51308,7 +51308,7 @@
       </c>
       <c r="C760" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D760" s="2" t="inlineStr">
@@ -52447,7 +52447,7 @@
       </c>
       <c r="C777" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D777" s="2" t="inlineStr">
@@ -55395,7 +55395,7 @@
       </c>
       <c r="C821" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D821" s="2" t="inlineStr">
@@ -57003,7 +57003,7 @@
       </c>
       <c r="C845" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D845" s="2" t="inlineStr">
@@ -57204,7 +57204,7 @@
       </c>
       <c r="C848" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D848" s="2" t="inlineStr">
@@ -61224,7 +61224,7 @@
       </c>
       <c r="C908" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D908" s="2" t="inlineStr">
@@ -61358,7 +61358,7 @@
       </c>
       <c r="C910" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D910" s="2" t="inlineStr">
@@ -61425,7 +61425,7 @@
       </c>
       <c r="C911" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D911" s="2" t="inlineStr">
@@ -61894,7 +61894,7 @@
       </c>
       <c r="C918" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D918" s="2" t="inlineStr">
@@ -62028,7 +62028,7 @@
       </c>
       <c r="C920" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D920" s="2" t="inlineStr">
@@ -62229,7 +62229,7 @@
       </c>
       <c r="C923" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D923" s="2" t="inlineStr">
@@ -63636,7 +63636,7 @@
       </c>
       <c r="C944" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D944" s="2" t="inlineStr">
@@ -64172,7 +64172,7 @@
       </c>
       <c r="C952" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D952" s="2" t="inlineStr">
@@ -64239,7 +64239,7 @@
       </c>
       <c r="C953" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D953" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-02 18:39:13
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixas_42l.xlsx
+++ b/relatorio_analitico_caixas_42l.xlsx
@@ -1795,7 +1795,7 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -4341,7 +4341,7 @@
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
@@ -6753,7 +6753,7 @@
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
@@ -7959,7 +7959,7 @@
       </c>
       <c r="C113" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D113" s="2" t="inlineStr">
@@ -15798,7 +15798,7 @@
       </c>
       <c r="C230" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D230" s="2" t="inlineStr">
@@ -15932,7 +15932,7 @@
       </c>
       <c r="C232" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D232" s="2" t="inlineStr">
@@ -15999,7 +15999,7 @@
       </c>
       <c r="C233" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D233" s="2" t="inlineStr">
@@ -16669,7 +16669,7 @@
       </c>
       <c r="C243" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D243" s="2" t="inlineStr">
@@ -17205,7 +17205,7 @@
       </c>
       <c r="C251" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D251" s="2" t="inlineStr">
@@ -18947,7 +18947,7 @@
       </c>
       <c r="C277" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D277" s="2" t="inlineStr">
@@ -20555,7 +20555,7 @@
       </c>
       <c r="C301" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D301" s="2" t="inlineStr">
@@ -23436,7 +23436,7 @@
       </c>
       <c r="C344" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D344" s="2" t="inlineStr">
@@ -23637,7 +23637,7 @@
       </c>
       <c r="C347" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D347" s="2" t="inlineStr">
@@ -26116,7 +26116,7 @@
       </c>
       <c r="C384" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D384" s="2" t="inlineStr">
@@ -26183,7 +26183,7 @@
       </c>
       <c r="C385" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D385" s="2" t="inlineStr">
@@ -26853,7 +26853,7 @@
       </c>
       <c r="C395" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D395" s="2" t="inlineStr">
@@ -28729,7 +28729,7 @@
       </c>
       <c r="C423" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D423" s="2" t="inlineStr">
@@ -32883,7 +32883,7 @@
       </c>
       <c r="C485" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D485" s="2" t="inlineStr">
@@ -32950,7 +32950,7 @@
       </c>
       <c r="C486" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D486" s="2" t="inlineStr">
@@ -33017,7 +33017,7 @@
       </c>
       <c r="C487" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D487" s="2" t="inlineStr">
@@ -33084,7 +33084,7 @@
       </c>
       <c r="C488" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D488" s="2" t="inlineStr">
@@ -35496,7 +35496,7 @@
       </c>
       <c r="C524" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D524" s="2" t="inlineStr">
@@ -37841,7 +37841,7 @@
       </c>
       <c r="C559" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D559" s="2" t="inlineStr">
@@ -37908,7 +37908,7 @@
       </c>
       <c r="C560" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D560" s="2" t="inlineStr">
@@ -48494,7 +48494,7 @@
       </c>
       <c r="C718" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D718" s="2" t="inlineStr">
@@ -49365,7 +49365,7 @@
       </c>
       <c r="C731" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D731" s="2" t="inlineStr">
@@ -49499,7 +49499,7 @@
       </c>
       <c r="C733" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D733" s="2" t="inlineStr">
@@ -49566,7 +49566,7 @@
       </c>
       <c r="C734" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D734" s="2" t="inlineStr">
@@ -52648,7 +52648,7 @@
       </c>
       <c r="C780" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D780" s="2" t="inlineStr">
@@ -55462,7 +55462,7 @@
       </c>
       <c r="C822" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D822" s="2" t="inlineStr">
@@ -55529,7 +55529,7 @@
       </c>
       <c r="C823" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D823" s="2" t="inlineStr">
@@ -56467,7 +56467,7 @@
       </c>
       <c r="C837" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D837" s="2" t="inlineStr">
@@ -57204,7 +57204,7 @@
       </c>
       <c r="C848" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D848" s="2" t="inlineStr">
@@ -61224,7 +61224,7 @@
       </c>
       <c r="C908" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D908" s="2" t="inlineStr">
@@ -61760,7 +61760,7 @@
       </c>
       <c r="C916" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D916" s="2" t="inlineStr">
@@ -64172,7 +64172,7 @@
       </c>
       <c r="C952" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D952" s="2" t="inlineStr">
@@ -64306,7 +64306,7 @@
       </c>
       <c r="C954" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D954" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-02 20:10:00
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixas_42l.xlsx
+++ b/relatorio_analitico_caixas_42l.xlsx
@@ -1795,7 +1795,7 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -1996,7 +1996,7 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -6552,7 +6552,7 @@
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
@@ -7490,7 +7490,7 @@
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D106" s="2" t="inlineStr">
@@ -17205,7 +17205,7 @@
       </c>
       <c r="C251" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D251" s="2" t="inlineStr">
@@ -20555,7 +20555,7 @@
       </c>
       <c r="C301" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D301" s="2" t="inlineStr">
@@ -23637,7 +23637,7 @@
       </c>
       <c r="C347" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D347" s="2" t="inlineStr">
@@ -26116,7 +26116,7 @@
       </c>
       <c r="C384" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D384" s="2" t="inlineStr">
@@ -26183,7 +26183,7 @@
       </c>
       <c r="C385" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D385" s="2" t="inlineStr">
@@ -26853,7 +26853,7 @@
       </c>
       <c r="C395" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D395" s="2" t="inlineStr">
@@ -28729,7 +28729,7 @@
       </c>
       <c r="C423" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D423" s="2" t="inlineStr">
@@ -32347,7 +32347,7 @@
       </c>
       <c r="C477" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D477" s="2" t="inlineStr">
@@ -32749,7 +32749,7 @@
       </c>
       <c r="C483" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D483" s="2" t="inlineStr">
@@ -33017,7 +33017,7 @@
       </c>
       <c r="C487" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D487" s="2" t="inlineStr">
@@ -33084,7 +33084,7 @@
       </c>
       <c r="C488" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D488" s="2" t="inlineStr">
@@ -37841,7 +37841,7 @@
       </c>
       <c r="C559" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D559" s="2" t="inlineStr">
@@ -40186,7 +40186,7 @@
       </c>
       <c r="C594" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D594" s="2" t="inlineStr">
@@ -48427,7 +48427,7 @@
       </c>
       <c r="C717" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D717" s="2" t="inlineStr">
@@ -48494,7 +48494,7 @@
       </c>
       <c r="C718" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D718" s="2" t="inlineStr">
@@ -48963,7 +48963,7 @@
       </c>
       <c r="C725" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D725" s="2" t="inlineStr">
@@ -49499,7 +49499,7 @@
       </c>
       <c r="C733" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D733" s="2" t="inlineStr">
@@ -49566,7 +49566,7 @@
       </c>
       <c r="C734" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D734" s="2" t="inlineStr">
@@ -51308,7 +51308,7 @@
       </c>
       <c r="C760" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D760" s="2" t="inlineStr">
@@ -52380,7 +52380,7 @@
       </c>
       <c r="C776" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D776" s="2" t="inlineStr">
@@ -52447,7 +52447,7 @@
       </c>
       <c r="C777" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D777" s="2" t="inlineStr">
@@ -52514,7 +52514,7 @@
       </c>
       <c r="C778" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D778" s="2" t="inlineStr">
@@ -53921,7 +53921,7 @@
       </c>
       <c r="C799" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D799" s="2" t="inlineStr">
@@ -55462,7 +55462,7 @@
       </c>
       <c r="C822" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D822" s="2" t="inlineStr">
@@ -57204,7 +57204,7 @@
       </c>
       <c r="C848" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D848" s="2" t="inlineStr">
@@ -61224,7 +61224,7 @@
       </c>
       <c r="C908" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D908" s="2" t="inlineStr">
@@ -61358,7 +61358,7 @@
       </c>
       <c r="C910" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D910" s="2" t="inlineStr">
@@ -62028,7 +62028,7 @@
       </c>
       <c r="C920" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D920" s="2" t="inlineStr">
@@ -62229,7 +62229,7 @@
       </c>
       <c r="C923" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D923" s="2" t="inlineStr">
@@ -64239,7 +64239,7 @@
       </c>
       <c r="C953" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D953" s="2" t="inlineStr">
@@ -65311,7 +65311,7 @@
       </c>
       <c r="C969" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D969" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-03 00:48:23
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixas_42l.xlsx
+++ b/relatorio_analitico_caixas_42l.xlsx
@@ -1795,7 +1795,7 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -4341,7 +4341,7 @@
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
@@ -6552,7 +6552,7 @@
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
@@ -6753,7 +6753,7 @@
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
@@ -7490,7 +7490,7 @@
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D106" s="2" t="inlineStr">
@@ -7959,7 +7959,7 @@
       </c>
       <c r="C113" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D113" s="2" t="inlineStr">
@@ -15530,7 +15530,7 @@
       </c>
       <c r="C226" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D226" s="2" t="inlineStr">
@@ -15798,7 +15798,7 @@
       </c>
       <c r="C230" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D230" s="2" t="inlineStr">
@@ -15932,7 +15932,7 @@
       </c>
       <c r="C232" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D232" s="2" t="inlineStr">
@@ -15999,7 +15999,7 @@
       </c>
       <c r="C233" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D233" s="2" t="inlineStr">
@@ -18947,7 +18947,7 @@
       </c>
       <c r="C277" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D277" s="2" t="inlineStr">
@@ -19215,7 +19215,7 @@
       </c>
       <c r="C281" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D281" s="2" t="inlineStr">
@@ -20555,7 +20555,7 @@
       </c>
       <c r="C301" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D301" s="2" t="inlineStr">
@@ -21024,7 +21024,7 @@
       </c>
       <c r="C308" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D308" s="2" t="inlineStr">
@@ -23436,7 +23436,7 @@
       </c>
       <c r="C344" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D344" s="2" t="inlineStr">
@@ -25848,7 +25848,7 @@
       </c>
       <c r="C380" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D380" s="2" t="inlineStr">
@@ -26183,7 +26183,7 @@
       </c>
       <c r="C385" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D385" s="2" t="inlineStr">
@@ -26853,7 +26853,7 @@
       </c>
       <c r="C395" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D395" s="2" t="inlineStr">
@@ -32347,7 +32347,7 @@
       </c>
       <c r="C477" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D477" s="2" t="inlineStr">
@@ -33017,7 +33017,7 @@
       </c>
       <c r="C487" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D487" s="2" t="inlineStr">
@@ -33084,7 +33084,7 @@
       </c>
       <c r="C488" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D488" s="2" t="inlineStr">
@@ -37841,7 +37841,7 @@
       </c>
       <c r="C559" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D559" s="2" t="inlineStr">
@@ -37908,7 +37908,7 @@
       </c>
       <c r="C560" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D560" s="2" t="inlineStr">
@@ -40186,7 +40186,7 @@
       </c>
       <c r="C594" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D594" s="2" t="inlineStr">
@@ -48494,7 +48494,7 @@
       </c>
       <c r="C718" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D718" s="2" t="inlineStr">
@@ -49365,7 +49365,7 @@
       </c>
       <c r="C731" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D731" s="2" t="inlineStr">
@@ -49499,7 +49499,7 @@
       </c>
       <c r="C733" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D733" s="2" t="inlineStr">
@@ -52447,7 +52447,7 @@
       </c>
       <c r="C777" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D777" s="2" t="inlineStr">
@@ -53921,7 +53921,7 @@
       </c>
       <c r="C799" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D799" s="2" t="inlineStr">
@@ -55462,7 +55462,7 @@
       </c>
       <c r="C822" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D822" s="2" t="inlineStr">
@@ -55529,7 +55529,7 @@
       </c>
       <c r="C823" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D823" s="2" t="inlineStr">
@@ -57003,7 +57003,7 @@
       </c>
       <c r="C845" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D845" s="2" t="inlineStr">
@@ -57204,7 +57204,7 @@
       </c>
       <c r="C848" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D848" s="2" t="inlineStr">
@@ -61224,7 +61224,7 @@
       </c>
       <c r="C908" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D908" s="2" t="inlineStr">
@@ -61760,7 +61760,7 @@
       </c>
       <c r="C916" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D916" s="2" t="inlineStr">
@@ -65043,7 +65043,7 @@
       </c>
       <c r="C965" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D965" s="2" t="inlineStr">
@@ -65311,7 +65311,7 @@
       </c>
       <c r="C969" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D969" s="2" t="inlineStr">
@@ -65780,7 +65780,7 @@
       </c>
       <c r="C976" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D976" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-03 04:18:36
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixas_42l.xlsx
+++ b/relatorio_analitico_caixas_42l.xlsx
@@ -1795,7 +1795,7 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -1996,7 +1996,7 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -4341,7 +4341,7 @@
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
@@ -6552,7 +6552,7 @@
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
@@ -7959,7 +7959,7 @@
       </c>
       <c r="C113" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D113" s="2" t="inlineStr">
@@ -18344,7 +18344,7 @@
       </c>
       <c r="C268" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D268" s="2" t="inlineStr">
@@ -18947,7 +18947,7 @@
       </c>
       <c r="C277" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D277" s="2" t="inlineStr">
@@ -20555,7 +20555,7 @@
       </c>
       <c r="C301" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D301" s="2" t="inlineStr">
@@ -23436,7 +23436,7 @@
       </c>
       <c r="C344" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D344" s="2" t="inlineStr">
@@ -23637,7 +23637,7 @@
       </c>
       <c r="C347" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D347" s="2" t="inlineStr">
@@ -26183,7 +26183,7 @@
       </c>
       <c r="C385" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D385" s="2" t="inlineStr">
@@ -26853,7 +26853,7 @@
       </c>
       <c r="C395" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D395" s="2" t="inlineStr">
@@ -28729,7 +28729,7 @@
       </c>
       <c r="C423" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D423" s="2" t="inlineStr">
@@ -32347,7 +32347,7 @@
       </c>
       <c r="C477" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D477" s="2" t="inlineStr">
@@ -32414,7 +32414,7 @@
       </c>
       <c r="C478" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D478" s="2" t="inlineStr">
@@ -32749,7 +32749,7 @@
       </c>
       <c r="C483" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D483" s="2" t="inlineStr">
@@ -35496,7 +35496,7 @@
       </c>
       <c r="C524" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D524" s="2" t="inlineStr">
@@ -40186,7 +40186,7 @@
       </c>
       <c r="C594" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D594" s="2" t="inlineStr">
@@ -45613,7 +45613,7 @@
       </c>
       <c r="C675" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D675" s="2" t="inlineStr">
@@ -48494,7 +48494,7 @@
       </c>
       <c r="C718" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D718" s="2" t="inlineStr">
@@ -52447,7 +52447,7 @@
       </c>
       <c r="C777" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D777" s="2" t="inlineStr">
@@ -52581,7 +52581,7 @@
       </c>
       <c r="C779" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D779" s="2" t="inlineStr">
@@ -52648,7 +52648,7 @@
       </c>
       <c r="C780" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D780" s="2" t="inlineStr">
@@ -53921,7 +53921,7 @@
       </c>
       <c r="C799" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D799" s="2" t="inlineStr">
@@ -55462,7 +55462,7 @@
       </c>
       <c r="C822" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D822" s="2" t="inlineStr">
@@ -56467,7 +56467,7 @@
       </c>
       <c r="C837" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D837" s="2" t="inlineStr">
@@ -57003,7 +57003,7 @@
       </c>
       <c r="C845" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D845" s="2" t="inlineStr">
@@ -57204,7 +57204,7 @@
       </c>
       <c r="C848" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D848" s="2" t="inlineStr">
@@ -61224,7 +61224,7 @@
       </c>
       <c r="C908" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D908" s="2" t="inlineStr">
@@ -61358,7 +61358,7 @@
       </c>
       <c r="C910" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D910" s="2" t="inlineStr">
@@ -61559,7 +61559,7 @@
       </c>
       <c r="C913" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D913" s="2" t="inlineStr">
@@ -63636,7 +63636,7 @@
       </c>
       <c r="C944" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D944" s="2" t="inlineStr">
@@ -64306,7 +64306,7 @@
       </c>
       <c r="C954" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D954" s="2" t="inlineStr">
@@ -65311,7 +65311,7 @@
       </c>
       <c r="C969" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D969" s="2" t="inlineStr">
@@ -66517,7 +66517,7 @@
       </c>
       <c r="C987" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D987" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-03 23:00:14
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixas_42l.xlsx
+++ b/relatorio_analitico_caixas_42l.xlsx
@@ -1795,7 +1795,7 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -1996,7 +1996,7 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -4341,7 +4341,7 @@
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
@@ -15999,7 +15999,7 @@
       </c>
       <c r="C233" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D233" s="2" t="inlineStr">
@@ -18947,7 +18947,7 @@
       </c>
       <c r="C277" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D277" s="2" t="inlineStr">
@@ -21024,7 +21024,7 @@
       </c>
       <c r="C308" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D308" s="2" t="inlineStr">
@@ -23637,7 +23637,7 @@
       </c>
       <c r="C347" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D347" s="2" t="inlineStr">
@@ -25848,7 +25848,7 @@
       </c>
       <c r="C380" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D380" s="2" t="inlineStr">
@@ -25982,7 +25982,7 @@
       </c>
       <c r="C382" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D382" s="2" t="inlineStr">
@@ -32347,7 +32347,7 @@
       </c>
       <c r="C477" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D477" s="2" t="inlineStr">
@@ -32883,7 +32883,7 @@
       </c>
       <c r="C485" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D485" s="2" t="inlineStr">
@@ -33017,7 +33017,7 @@
       </c>
       <c r="C487" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D487" s="2" t="inlineStr">
@@ -33084,7 +33084,7 @@
       </c>
       <c r="C488" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D488" s="2" t="inlineStr">
@@ -37841,7 +37841,7 @@
       </c>
       <c r="C559" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D559" s="2" t="inlineStr">
@@ -37908,7 +37908,7 @@
       </c>
       <c r="C560" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D560" s="2" t="inlineStr">
@@ -43000,7 +43000,7 @@
       </c>
       <c r="C636" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D636" s="2" t="inlineStr">
@@ -48427,7 +48427,7 @@
       </c>
       <c r="C717" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D717" s="2" t="inlineStr">
@@ -49365,7 +49365,7 @@
       </c>
       <c r="C731" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D731" s="2" t="inlineStr">
@@ -49499,7 +49499,7 @@
       </c>
       <c r="C733" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D733" s="2" t="inlineStr">
@@ -49566,7 +49566,7 @@
       </c>
       <c r="C734" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D734" s="2" t="inlineStr">
@@ -52715,7 +52715,7 @@
       </c>
       <c r="C781" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D781" s="2" t="inlineStr">
@@ -52782,7 +52782,7 @@
       </c>
       <c r="C782" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D782" s="2" t="inlineStr">
@@ -54055,7 +54055,7 @@
       </c>
       <c r="C801" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D801" s="2" t="inlineStr">
@@ -55663,7 +55663,7 @@
       </c>
       <c r="C825" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D825" s="2" t="inlineStr">
@@ -56601,7 +56601,7 @@
       </c>
       <c r="C839" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D839" s="2" t="inlineStr">
@@ -57338,7 +57338,7 @@
       </c>
       <c r="C850" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D850" s="2" t="inlineStr">
@@ -61358,7 +61358,7 @@
       </c>
       <c r="C910" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D910" s="2" t="inlineStr">
@@ -61492,7 +61492,7 @@
       </c>
       <c r="C912" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D912" s="2" t="inlineStr">
@@ -64306,7 +64306,7 @@
       </c>
       <c r="C954" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D954" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-04 00:39:54
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixas_42l.xlsx
+++ b/relatorio_analitico_caixas_42l.xlsx
@@ -1795,7 +1795,7 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -1996,7 +1996,7 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -7490,7 +7490,7 @@
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D106" s="2" t="inlineStr">
@@ -7959,7 +7959,7 @@
       </c>
       <c r="C113" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D113" s="2" t="inlineStr">
@@ -16669,7 +16669,7 @@
       </c>
       <c r="C243" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D243" s="2" t="inlineStr">
@@ -20555,7 +20555,7 @@
       </c>
       <c r="C301" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D301" s="2" t="inlineStr">
@@ -21024,7 +21024,7 @@
       </c>
       <c r="C308" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D308" s="2" t="inlineStr">
@@ -23436,7 +23436,7 @@
       </c>
       <c r="C344" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D344" s="2" t="inlineStr">
@@ -25848,7 +25848,7 @@
       </c>
       <c r="C380" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D380" s="2" t="inlineStr">
@@ -26116,7 +26116,7 @@
       </c>
       <c r="C384" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D384" s="2" t="inlineStr">
@@ -26183,7 +26183,7 @@
       </c>
       <c r="C385" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D385" s="2" t="inlineStr">
@@ -26853,7 +26853,7 @@
       </c>
       <c r="C395" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D395" s="2" t="inlineStr">
@@ -28729,7 +28729,7 @@
       </c>
       <c r="C423" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D423" s="2" t="inlineStr">
@@ -32883,7 +32883,7 @@
       </c>
       <c r="C485" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D485" s="2" t="inlineStr">
@@ -33017,7 +33017,7 @@
       </c>
       <c r="C487" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D487" s="2" t="inlineStr">
@@ -37841,7 +37841,7 @@
       </c>
       <c r="C559" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D559" s="2" t="inlineStr">
@@ -37908,7 +37908,7 @@
       </c>
       <c r="C560" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D560" s="2" t="inlineStr">
@@ -40186,7 +40186,7 @@
       </c>
       <c r="C594" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D594" s="2" t="inlineStr">
@@ -48427,7 +48427,7 @@
       </c>
       <c r="C717" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D717" s="2" t="inlineStr">
@@ -48494,7 +48494,7 @@
       </c>
       <c r="C718" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D718" s="2" t="inlineStr">
@@ -48963,7 +48963,7 @@
       </c>
       <c r="C725" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D725" s="2" t="inlineStr">
@@ -49499,7 +49499,7 @@
       </c>
       <c r="C733" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D733" s="2" t="inlineStr">
@@ -51442,7 +51442,7 @@
       </c>
       <c r="C762" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D762" s="2" t="inlineStr">
@@ -52514,7 +52514,7 @@
       </c>
       <c r="C778" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D778" s="2" t="inlineStr">
@@ -52581,7 +52581,7 @@
       </c>
       <c r="C779" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D779" s="2" t="inlineStr">
@@ -54055,7 +54055,7 @@
       </c>
       <c r="C801" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D801" s="2" t="inlineStr">
@@ -55730,7 +55730,7 @@
       </c>
       <c r="C826" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D826" s="2" t="inlineStr">
@@ -57338,7 +57338,7 @@
       </c>
       <c r="C850" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D850" s="2" t="inlineStr">
@@ -61894,7 +61894,7 @@
       </c>
       <c r="C918" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D918" s="2" t="inlineStr">
@@ -62363,7 +62363,7 @@
       </c>
       <c r="C925" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D925" s="2" t="inlineStr">
@@ -63837,7 +63837,7 @@
       </c>
       <c r="C947" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D947" s="2" t="inlineStr">
@@ -64440,7 +64440,7 @@
       </c>
       <c r="C956" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D956" s="2" t="inlineStr">
@@ -65177,7 +65177,7 @@
       </c>
       <c r="C967" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D967" s="2" t="inlineStr">
@@ -65445,7 +65445,7 @@
       </c>
       <c r="C971" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D971" s="2" t="inlineStr">
@@ -66651,7 +66651,7 @@
       </c>
       <c r="C989" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D989" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-04 02:20:49
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixas_42l.xlsx
+++ b/relatorio_analitico_caixas_42l.xlsx
@@ -6552,7 +6552,7 @@
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
@@ -6753,7 +6753,7 @@
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
@@ -15530,7 +15530,7 @@
       </c>
       <c r="C226" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D226" s="2" t="inlineStr">
@@ -15932,7 +15932,7 @@
       </c>
       <c r="C232" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D232" s="2" t="inlineStr">
@@ -15999,7 +15999,7 @@
       </c>
       <c r="C233" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D233" s="2" t="inlineStr">
@@ -16669,7 +16669,7 @@
       </c>
       <c r="C243" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D243" s="2" t="inlineStr">
@@ -19081,7 +19081,7 @@
       </c>
       <c r="C279" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D279" s="2" t="inlineStr">
@@ -19215,7 +19215,7 @@
       </c>
       <c r="C281" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D281" s="2" t="inlineStr">
@@ -21024,7 +21024,7 @@
       </c>
       <c r="C308" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D308" s="2" t="inlineStr">
@@ -26183,7 +26183,7 @@
       </c>
       <c r="C385" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D385" s="2" t="inlineStr">
@@ -26853,7 +26853,7 @@
       </c>
       <c r="C395" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D395" s="2" t="inlineStr">
@@ -32414,7 +32414,7 @@
       </c>
       <c r="C478" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D478" s="2" t="inlineStr">
@@ -32950,7 +32950,7 @@
       </c>
       <c r="C486" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D486" s="2" t="inlineStr">
@@ -33017,7 +33017,7 @@
       </c>
       <c r="C487" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D487" s="2" t="inlineStr">
@@ -37841,7 +37841,7 @@
       </c>
       <c r="C559" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D559" s="2" t="inlineStr">
@@ -40186,7 +40186,7 @@
       </c>
       <c r="C594" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D594" s="2" t="inlineStr">
@@ -45613,7 +45613,7 @@
       </c>
       <c r="C675" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D675" s="2" t="inlineStr">
@@ -48963,7 +48963,7 @@
       </c>
       <c r="C725" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D725" s="2" t="inlineStr">
@@ -51442,7 +51442,7 @@
       </c>
       <c r="C762" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D762" s="2" t="inlineStr">
@@ -52514,7 +52514,7 @@
       </c>
       <c r="C778" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D778" s="2" t="inlineStr">
@@ -52581,7 +52581,7 @@
       </c>
       <c r="C779" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D779" s="2" t="inlineStr">
@@ -52715,7 +52715,7 @@
       </c>
       <c r="C781" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D781" s="2" t="inlineStr">
@@ -52782,7 +52782,7 @@
       </c>
       <c r="C782" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D782" s="2" t="inlineStr">
@@ -55663,7 +55663,7 @@
       </c>
       <c r="C825" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D825" s="2" t="inlineStr">
@@ -55730,7 +55730,7 @@
       </c>
       <c r="C826" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D826" s="2" t="inlineStr">
@@ -56601,7 +56601,7 @@
       </c>
       <c r="C839" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D839" s="2" t="inlineStr">
@@ -57338,7 +57338,7 @@
       </c>
       <c r="C850" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D850" s="2" t="inlineStr">
@@ -61358,7 +61358,7 @@
       </c>
       <c r="C910" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D910" s="2" t="inlineStr">
@@ -61492,7 +61492,7 @@
       </c>
       <c r="C912" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D912" s="2" t="inlineStr">
@@ -61559,7 +61559,7 @@
       </c>
       <c r="C913" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D913" s="2" t="inlineStr">
@@ -63837,7 +63837,7 @@
       </c>
       <c r="C947" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D947" s="2" t="inlineStr">
@@ -64306,7 +64306,7 @@
       </c>
       <c r="C954" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D954" s="2" t="inlineStr">
@@ -64373,7 +64373,7 @@
       </c>
       <c r="C955" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D955" s="2" t="inlineStr">
@@ -64440,7 +64440,7 @@
       </c>
       <c r="C956" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D956" s="2" t="inlineStr">
@@ -65914,7 +65914,7 @@
       </c>
       <c r="C978" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D978" s="2" t="inlineStr">
@@ -66651,7 +66651,7 @@
       </c>
       <c r="C989" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D989" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-04 08:00:28
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixas_42l.xlsx
+++ b/relatorio_analitico_caixas_42l.xlsx
@@ -1996,7 +1996,7 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -4341,7 +4341,7 @@
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
@@ -6753,7 +6753,7 @@
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
@@ -15530,7 +15530,7 @@
       </c>
       <c r="C226" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D226" s="2" t="inlineStr">
@@ -15932,7 +15932,7 @@
       </c>
       <c r="C232" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D232" s="2" t="inlineStr">
@@ -18344,7 +18344,7 @@
       </c>
       <c r="C268" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D268" s="2" t="inlineStr">
@@ -18947,7 +18947,7 @@
       </c>
       <c r="C277" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D277" s="2" t="inlineStr">
@@ -19081,7 +19081,7 @@
       </c>
       <c r="C279" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D279" s="2" t="inlineStr">
@@ -20555,7 +20555,7 @@
       </c>
       <c r="C301" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D301" s="2" t="inlineStr">
@@ -21024,7 +21024,7 @@
       </c>
       <c r="C308" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D308" s="2" t="inlineStr">
@@ -25848,7 +25848,7 @@
       </c>
       <c r="C380" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D380" s="2" t="inlineStr">
@@ -25982,7 +25982,7 @@
       </c>
       <c r="C382" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D382" s="2" t="inlineStr">
@@ -26116,7 +26116,7 @@
       </c>
       <c r="C384" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D384" s="2" t="inlineStr">
@@ -28729,7 +28729,7 @@
       </c>
       <c r="C423" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D423" s="2" t="inlineStr">
@@ -32414,7 +32414,7 @@
       </c>
       <c r="C478" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D478" s="2" t="inlineStr">
@@ -32749,7 +32749,7 @@
       </c>
       <c r="C483" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D483" s="2" t="inlineStr">
@@ -32883,7 +32883,7 @@
       </c>
       <c r="C485" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D485" s="2" t="inlineStr">
@@ -32950,7 +32950,7 @@
       </c>
       <c r="C486" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D486" s="2" t="inlineStr">
@@ -33017,7 +33017,7 @@
       </c>
       <c r="C487" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D487" s="2" t="inlineStr">
@@ -37908,7 +37908,7 @@
       </c>
       <c r="C560" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D560" s="2" t="inlineStr">
@@ -48427,7 +48427,7 @@
       </c>
       <c r="C717" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D717" s="2" t="inlineStr">
@@ -49365,7 +49365,7 @@
       </c>
       <c r="C731" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D731" s="2" t="inlineStr">
@@ -49499,7 +49499,7 @@
       </c>
       <c r="C733" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D733" s="2" t="inlineStr">
@@ -49566,7 +49566,7 @@
       </c>
       <c r="C734" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D734" s="2" t="inlineStr">
@@ -52581,7 +52581,7 @@
       </c>
       <c r="C779" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D779" s="2" t="inlineStr">
@@ -52648,7 +52648,7 @@
       </c>
       <c r="C780" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D780" s="2" t="inlineStr">
@@ -55529,7 +55529,7 @@
       </c>
       <c r="C823" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D823" s="2" t="inlineStr">
@@ -57137,7 +57137,7 @@
       </c>
       <c r="C847" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D847" s="2" t="inlineStr">
@@ -61358,7 +61358,7 @@
       </c>
       <c r="C910" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D910" s="2" t="inlineStr">
@@ -61693,7 +61693,7 @@
       </c>
       <c r="C915" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D915" s="2" t="inlineStr">
@@ -61894,7 +61894,7 @@
       </c>
       <c r="C918" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D918" s="2" t="inlineStr">
@@ -62028,7 +62028,7 @@
       </c>
       <c r="C920" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D920" s="2" t="inlineStr">
@@ -62162,7 +62162,7 @@
       </c>
       <c r="C922" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D922" s="2" t="inlineStr">
@@ -64306,7 +64306,7 @@
       </c>
       <c r="C954" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D954" s="2" t="inlineStr">
@@ -64373,7 +64373,7 @@
       </c>
       <c r="C955" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D955" s="2" t="inlineStr">
@@ -64440,7 +64440,7 @@
       </c>
       <c r="C956" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D956" s="2" t="inlineStr">
@@ -65445,7 +65445,7 @@
       </c>
       <c r="C971" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D971" s="2" t="inlineStr">
@@ -66651,7 +66651,7 @@
       </c>
       <c r="C989" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D989" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-05 00:02:47
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixas_42l.xlsx
+++ b/relatorio_analitico_caixas_42l.xlsx
@@ -1996,7 +1996,7 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -4341,7 +4341,7 @@
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
@@ -6753,7 +6753,7 @@
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
@@ -7490,7 +7490,7 @@
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D106" s="2" t="inlineStr">
@@ -7959,7 +7959,7 @@
       </c>
       <c r="C113" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D113" s="2" t="inlineStr">
@@ -15999,7 +15999,7 @@
       </c>
       <c r="C233" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D233" s="2" t="inlineStr">
@@ -16669,7 +16669,7 @@
       </c>
       <c r="C243" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D243" s="2" t="inlineStr">
@@ -18344,7 +18344,7 @@
       </c>
       <c r="C268" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D268" s="2" t="inlineStr">
@@ -20555,7 +20555,7 @@
       </c>
       <c r="C301" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D301" s="2" t="inlineStr">
@@ -20890,7 +20890,7 @@
       </c>
       <c r="C306" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D306" s="2" t="inlineStr">
@@ -21024,7 +21024,7 @@
       </c>
       <c r="C308" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D308" s="2" t="inlineStr">
@@ -23637,7 +23637,7 @@
       </c>
       <c r="C347" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D347" s="2" t="inlineStr">
@@ -26116,7 +26116,7 @@
       </c>
       <c r="C384" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D384" s="2" t="inlineStr">
@@ -26853,7 +26853,7 @@
       </c>
       <c r="C395" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D395" s="2" t="inlineStr">
@@ -28729,7 +28729,7 @@
       </c>
       <c r="C423" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D423" s="2" t="inlineStr">
@@ -32749,7 +32749,7 @@
       </c>
       <c r="C483" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D483" s="2" t="inlineStr">
@@ -32883,7 +32883,7 @@
       </c>
       <c r="C485" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D485" s="2" t="inlineStr">
@@ -32950,7 +32950,7 @@
       </c>
       <c r="C486" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D486" s="2" t="inlineStr">
@@ -33017,7 +33017,7 @@
       </c>
       <c r="C487" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D487" s="2" t="inlineStr">
@@ -33084,7 +33084,7 @@
       </c>
       <c r="C488" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D488" s="2" t="inlineStr">
@@ -35496,7 +35496,7 @@
       </c>
       <c r="C524" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D524" s="2" t="inlineStr">
@@ -37841,7 +37841,7 @@
       </c>
       <c r="C559" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D559" s="2" t="inlineStr">
@@ -37908,7 +37908,7 @@
       </c>
       <c r="C560" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D560" s="2" t="inlineStr">
@@ -48427,7 +48427,7 @@
       </c>
       <c r="C717" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D717" s="2" t="inlineStr">
@@ -52581,7 +52581,7 @@
       </c>
       <c r="C779" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D779" s="2" t="inlineStr">
@@ -52648,7 +52648,7 @@
       </c>
       <c r="C780" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D780" s="2" t="inlineStr">
@@ -52782,7 +52782,7 @@
       </c>
       <c r="C782" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D782" s="2" t="inlineStr">
@@ -55529,7 +55529,7 @@
       </c>
       <c r="C823" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D823" s="2" t="inlineStr">
@@ -55663,7 +55663,7 @@
       </c>
       <c r="C825" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D825" s="2" t="inlineStr">
@@ -56601,7 +56601,7 @@
       </c>
       <c r="C839" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D839" s="2" t="inlineStr">
@@ -57338,7 +57338,7 @@
       </c>
       <c r="C850" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D850" s="2" t="inlineStr">
@@ -61358,7 +61358,7 @@
       </c>
       <c r="C910" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D910" s="2" t="inlineStr">
@@ -62363,7 +62363,7 @@
       </c>
       <c r="C925" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D925" s="2" t="inlineStr">
@@ -63837,7 +63837,7 @@
       </c>
       <c r="C947" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D947" s="2" t="inlineStr">
@@ -64373,7 +64373,7 @@
       </c>
       <c r="C955" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D955" s="2" t="inlineStr">
@@ -65177,7 +65177,7 @@
       </c>
       <c r="C967" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D967" s="2" t="inlineStr">
@@ -65445,7 +65445,7 @@
       </c>
       <c r="C971" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D971" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-05 03:31:23
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixas_42l.xlsx
+++ b/relatorio_analitico_caixas_42l.xlsx
@@ -4341,7 +4341,7 @@
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
@@ -6753,7 +6753,7 @@
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
@@ -7959,7 +7959,7 @@
       </c>
       <c r="C113" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D113" s="2" t="inlineStr">
@@ -15530,7 +15530,7 @@
       </c>
       <c r="C226" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D226" s="2" t="inlineStr">
@@ -16669,7 +16669,7 @@
       </c>
       <c r="C243" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D243" s="2" t="inlineStr">
@@ -18344,7 +18344,7 @@
       </c>
       <c r="C268" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D268" s="2" t="inlineStr">
@@ -18947,7 +18947,7 @@
       </c>
       <c r="C277" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D277" s="2" t="inlineStr">
@@ -19081,7 +19081,7 @@
       </c>
       <c r="C279" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D279" s="2" t="inlineStr">
@@ -19215,7 +19215,7 @@
       </c>
       <c r="C281" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D281" s="2" t="inlineStr">
@@ -20555,7 +20555,7 @@
       </c>
       <c r="C301" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D301" s="2" t="inlineStr">
@@ -23436,7 +23436,7 @@
       </c>
       <c r="C344" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D344" s="2" t="inlineStr">
@@ -23637,7 +23637,7 @@
       </c>
       <c r="C347" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D347" s="2" t="inlineStr">
@@ -25982,7 +25982,7 @@
       </c>
       <c r="C382" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D382" s="2" t="inlineStr">
@@ -26116,7 +26116,7 @@
       </c>
       <c r="C384" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D384" s="2" t="inlineStr">
@@ -26853,7 +26853,7 @@
       </c>
       <c r="C395" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D395" s="2" t="inlineStr">
@@ -32414,7 +32414,7 @@
       </c>
       <c r="C478" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D478" s="2" t="inlineStr">
@@ -32749,7 +32749,7 @@
       </c>
       <c r="C483" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D483" s="2" t="inlineStr">
@@ -32883,7 +32883,7 @@
       </c>
       <c r="C485" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D485" s="2" t="inlineStr">
@@ -32950,7 +32950,7 @@
       </c>
       <c r="C486" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D486" s="2" t="inlineStr">
@@ -33017,7 +33017,7 @@
       </c>
       <c r="C487" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D487" s="2" t="inlineStr">
@@ -33084,7 +33084,7 @@
       </c>
       <c r="C488" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D488" s="2" t="inlineStr">
@@ -35496,7 +35496,7 @@
       </c>
       <c r="C524" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D524" s="2" t="inlineStr">
@@ -37841,7 +37841,7 @@
       </c>
       <c r="C559" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D559" s="2" t="inlineStr">
@@ -37908,7 +37908,7 @@
       </c>
       <c r="C560" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D560" s="2" t="inlineStr">
@@ -40186,7 +40186,7 @@
       </c>
       <c r="C594" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D594" s="2" t="inlineStr">
@@ -45613,7 +45613,7 @@
       </c>
       <c r="C675" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D675" s="2" t="inlineStr">
@@ -48427,7 +48427,7 @@
       </c>
       <c r="C717" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D717" s="2" t="inlineStr">
@@ -48494,7 +48494,7 @@
       </c>
       <c r="C718" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D718" s="2" t="inlineStr">
@@ -48963,7 +48963,7 @@
       </c>
       <c r="C725" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D725" s="2" t="inlineStr">
@@ -49365,7 +49365,7 @@
       </c>
       <c r="C731" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D731" s="2" t="inlineStr">
@@ -49499,7 +49499,7 @@
       </c>
       <c r="C733" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D733" s="2" t="inlineStr">
@@ -51442,7 +51442,7 @@
       </c>
       <c r="C762" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D762" s="2" t="inlineStr">
@@ -52581,7 +52581,7 @@
       </c>
       <c r="C779" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D779" s="2" t="inlineStr">
@@ -55596,7 +55596,7 @@
       </c>
       <c r="C824" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D824" s="2" t="inlineStr">
@@ -55663,7 +55663,7 @@
       </c>
       <c r="C825" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D825" s="2" t="inlineStr">
@@ -56601,7 +56601,7 @@
       </c>
       <c r="C839" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D839" s="2" t="inlineStr">
@@ -57137,7 +57137,7 @@
       </c>
       <c r="C847" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D847" s="2" t="inlineStr">
@@ -57338,7 +57338,7 @@
       </c>
       <c r="C850" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D850" s="2" t="inlineStr">
@@ -61559,7 +61559,7 @@
       </c>
       <c r="C913" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D913" s="2" t="inlineStr">
@@ -61693,7 +61693,7 @@
       </c>
       <c r="C915" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D915" s="2" t="inlineStr">
@@ -62363,7 +62363,7 @@
       </c>
       <c r="C925" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D925" s="2" t="inlineStr">
@@ -63770,7 +63770,7 @@
       </c>
       <c r="C946" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D946" s="2" t="inlineStr">
@@ -65177,7 +65177,7 @@
       </c>
       <c r="C967" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D967" s="2" t="inlineStr">
@@ -65445,7 +65445,7 @@
       </c>
       <c r="C971" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D971" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-05 06:41:38
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixas_42l.xlsx
+++ b/relatorio_analitico_caixas_42l.xlsx
@@ -1795,7 +1795,7 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -4341,7 +4341,7 @@
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
@@ -18344,7 +18344,7 @@
       </c>
       <c r="C268" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D268" s="2" t="inlineStr">
@@ -18947,7 +18947,7 @@
       </c>
       <c r="C277" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D277" s="2" t="inlineStr">
@@ -19215,7 +19215,7 @@
       </c>
       <c r="C281" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D281" s="2" t="inlineStr">
@@ -20555,7 +20555,7 @@
       </c>
       <c r="C301" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D301" s="2" t="inlineStr">
@@ -23436,7 +23436,7 @@
       </c>
       <c r="C344" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D344" s="2" t="inlineStr">
@@ -25982,7 +25982,7 @@
       </c>
       <c r="C382" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D382" s="2" t="inlineStr">
@@ -26116,7 +26116,7 @@
       </c>
       <c r="C384" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D384" s="2" t="inlineStr">
@@ -26183,7 +26183,7 @@
       </c>
       <c r="C385" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D385" s="2" t="inlineStr">
@@ -26853,7 +26853,7 @@
       </c>
       <c r="C395" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D395" s="2" t="inlineStr">
@@ -28729,7 +28729,7 @@
       </c>
       <c r="C423" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D423" s="2" t="inlineStr">
@@ -32414,7 +32414,7 @@
       </c>
       <c r="C478" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D478" s="2" t="inlineStr">
@@ -32749,7 +32749,7 @@
       </c>
       <c r="C483" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D483" s="2" t="inlineStr">
@@ -32883,7 +32883,7 @@
       </c>
       <c r="C485" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D485" s="2" t="inlineStr">
@@ -33017,7 +33017,7 @@
       </c>
       <c r="C487" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D487" s="2" t="inlineStr">
@@ -33084,7 +33084,7 @@
       </c>
       <c r="C488" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D488" s="2" t="inlineStr">
@@ -37841,7 +37841,7 @@
       </c>
       <c r="C559" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D559" s="2" t="inlineStr">
@@ -37908,7 +37908,7 @@
       </c>
       <c r="C560" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D560" s="2" t="inlineStr">
@@ -45613,7 +45613,7 @@
       </c>
       <c r="C675" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D675" s="2" t="inlineStr">
@@ -49499,7 +49499,7 @@
       </c>
       <c r="C733" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D733" s="2" t="inlineStr">
@@ -49566,7 +49566,7 @@
       </c>
       <c r="C734" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D734" s="2" t="inlineStr">
@@ -52514,7 +52514,7 @@
       </c>
       <c r="C778" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D778" s="2" t="inlineStr">
@@ -52581,7 +52581,7 @@
       </c>
       <c r="C779" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D779" s="2" t="inlineStr">
@@ -52782,7 +52782,7 @@
       </c>
       <c r="C782" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D782" s="2" t="inlineStr">
@@ -54055,7 +54055,7 @@
       </c>
       <c r="C801" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D801" s="2" t="inlineStr">
@@ -55596,7 +55596,7 @@
       </c>
       <c r="C824" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D824" s="2" t="inlineStr">
@@ -56601,7 +56601,7 @@
       </c>
       <c r="C839" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D839" s="2" t="inlineStr">
@@ -57137,7 +57137,7 @@
       </c>
       <c r="C847" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D847" s="2" t="inlineStr">
@@ -57338,7 +57338,7 @@
       </c>
       <c r="C850" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D850" s="2" t="inlineStr">
@@ -61693,7 +61693,7 @@
       </c>
       <c r="C915" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D915" s="2" t="inlineStr">
@@ -61894,7 +61894,7 @@
       </c>
       <c r="C918" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D918" s="2" t="inlineStr">
@@ -62162,7 +62162,7 @@
       </c>
       <c r="C922" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D922" s="2" t="inlineStr">
@@ -62363,7 +62363,7 @@
       </c>
       <c r="C925" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D925" s="2" t="inlineStr">
@@ -63770,7 +63770,7 @@
       </c>
       <c r="C946" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D946" s="2" t="inlineStr">
@@ -63837,7 +63837,7 @@
       </c>
       <c r="C947" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D947" s="2" t="inlineStr">
@@ -64306,7 +64306,7 @@
       </c>
       <c r="C954" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D954" s="2" t="inlineStr">
@@ -65177,7 +65177,7 @@
       </c>
       <c r="C967" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D967" s="2" t="inlineStr">
@@ -65914,7 +65914,7 @@
       </c>
       <c r="C978" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D978" s="2" t="inlineStr">
@@ -66651,7 +66651,7 @@
       </c>
       <c r="C989" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D989" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-05 09:11:32
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixas_42l.xlsx
+++ b/relatorio_analitico_caixas_42l.xlsx
@@ -1996,7 +1996,7 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -6552,7 +6552,7 @@
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
@@ -7490,7 +7490,7 @@
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D106" s="2" t="inlineStr">
@@ -7959,7 +7959,7 @@
       </c>
       <c r="C113" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D113" s="2" t="inlineStr">
@@ -17205,7 +17205,7 @@
       </c>
       <c r="C251" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D251" s="2" t="inlineStr">
@@ -18344,7 +18344,7 @@
       </c>
       <c r="C268" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D268" s="2" t="inlineStr">
@@ -18947,7 +18947,7 @@
       </c>
       <c r="C277" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D277" s="2" t="inlineStr">
@@ -21024,7 +21024,7 @@
       </c>
       <c r="C308" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D308" s="2" t="inlineStr">
@@ -23436,7 +23436,7 @@
       </c>
       <c r="C344" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D344" s="2" t="inlineStr">
@@ -23637,7 +23637,7 @@
       </c>
       <c r="C347" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D347" s="2" t="inlineStr">
@@ -25982,7 +25982,7 @@
       </c>
       <c r="C382" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D382" s="2" t="inlineStr">
@@ -26116,7 +26116,7 @@
       </c>
       <c r="C384" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D384" s="2" t="inlineStr">
@@ -26183,7 +26183,7 @@
       </c>
       <c r="C385" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D385" s="2" t="inlineStr">
@@ -26853,7 +26853,7 @@
       </c>
       <c r="C395" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D395" s="2" t="inlineStr">
@@ -28729,7 +28729,7 @@
       </c>
       <c r="C423" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D423" s="2" t="inlineStr">
@@ -32347,7 +32347,7 @@
       </c>
       <c r="C477" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D477" s="2" t="inlineStr">
@@ -32414,7 +32414,7 @@
       </c>
       <c r="C478" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D478" s="2" t="inlineStr">
@@ -32749,7 +32749,7 @@
       </c>
       <c r="C483" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D483" s="2" t="inlineStr">
@@ -32950,7 +32950,7 @@
       </c>
       <c r="C486" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D486" s="2" t="inlineStr">
@@ -35496,7 +35496,7 @@
       </c>
       <c r="C524" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D524" s="2" t="inlineStr">
@@ -49365,7 +49365,7 @@
       </c>
       <c r="C731" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D731" s="2" t="inlineStr">
@@ -49499,7 +49499,7 @@
       </c>
       <c r="C733" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D733" s="2" t="inlineStr">
@@ -52514,7 +52514,7 @@
       </c>
       <c r="C778" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D778" s="2" t="inlineStr">
@@ -55730,7 +55730,7 @@
       </c>
       <c r="C826" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D826" s="2" t="inlineStr">
@@ -61358,7 +61358,7 @@
       </c>
       <c r="C910" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D910" s="2" t="inlineStr">
@@ -61492,7 +61492,7 @@
       </c>
       <c r="C912" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D912" s="2" t="inlineStr">
@@ -61693,7 +61693,7 @@
       </c>
       <c r="C915" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D915" s="2" t="inlineStr">
@@ -62028,7 +62028,7 @@
       </c>
       <c r="C920" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D920" s="2" t="inlineStr">
@@ -62162,7 +62162,7 @@
       </c>
       <c r="C922" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D922" s="2" t="inlineStr">
@@ -64306,7 +64306,7 @@
       </c>
       <c r="C954" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D954" s="2" t="inlineStr">
@@ -66651,7 +66651,7 @@
       </c>
       <c r="C989" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D989" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-05 16:21:24
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixas_42l.xlsx
+++ b/relatorio_analitico_caixas_42l.xlsx
@@ -1795,7 +1795,7 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -1996,7 +1996,7 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -6753,7 +6753,7 @@
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
@@ -16669,7 +16669,7 @@
       </c>
       <c r="C243" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D243" s="2" t="inlineStr">
@@ -18344,7 +18344,7 @@
       </c>
       <c r="C268" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D268" s="2" t="inlineStr">
@@ -20555,7 +20555,7 @@
       </c>
       <c r="C301" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D301" s="2" t="inlineStr">
@@ -21024,7 +21024,7 @@
       </c>
       <c r="C308" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D308" s="2" t="inlineStr">
@@ -26116,7 +26116,7 @@
       </c>
       <c r="C384" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D384" s="2" t="inlineStr">
@@ -26183,7 +26183,7 @@
       </c>
       <c r="C385" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D385" s="2" t="inlineStr">
@@ -28729,7 +28729,7 @@
       </c>
       <c r="C423" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D423" s="2" t="inlineStr">
@@ -32414,7 +32414,7 @@
       </c>
       <c r="C478" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D478" s="2" t="inlineStr">
@@ -32950,7 +32950,7 @@
       </c>
       <c r="C486" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D486" s="2" t="inlineStr">
@@ -33017,7 +33017,7 @@
       </c>
       <c r="C487" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D487" s="2" t="inlineStr">
@@ -33084,7 +33084,7 @@
       </c>
       <c r="C488" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D488" s="2" t="inlineStr">
@@ -35496,7 +35496,7 @@
       </c>
       <c r="C524" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D524" s="2" t="inlineStr">
@@ -37841,7 +37841,7 @@
       </c>
       <c r="C559" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D559" s="2" t="inlineStr">
@@ -40186,7 +40186,7 @@
       </c>
       <c r="C594" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D594" s="2" t="inlineStr">
@@ -48427,7 +48427,7 @@
       </c>
       <c r="C717" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D717" s="2" t="inlineStr">
@@ -48494,7 +48494,7 @@
       </c>
       <c r="C718" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D718" s="2" t="inlineStr">
@@ -48963,7 +48963,7 @@
       </c>
       <c r="C725" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D725" s="2" t="inlineStr">
@@ -49365,7 +49365,7 @@
       </c>
       <c r="C731" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D731" s="2" t="inlineStr">
@@ -49499,7 +49499,7 @@
       </c>
       <c r="C733" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D733" s="2" t="inlineStr">
@@ -49566,7 +49566,7 @@
       </c>
       <c r="C734" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D734" s="2" t="inlineStr">
@@ -52581,7 +52581,7 @@
       </c>
       <c r="C779" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D779" s="2" t="inlineStr">
@@ -52782,7 +52782,7 @@
       </c>
       <c r="C782" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D782" s="2" t="inlineStr">
@@ -54055,7 +54055,7 @@
       </c>
       <c r="C801" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D801" s="2" t="inlineStr">
@@ -55529,7 +55529,7 @@
       </c>
       <c r="C823" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D823" s="2" t="inlineStr">
@@ -55596,7 +55596,7 @@
       </c>
       <c r="C824" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D824" s="2" t="inlineStr">
@@ -55663,7 +55663,7 @@
       </c>
       <c r="C825" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D825" s="2" t="inlineStr">
@@ -61492,7 +61492,7 @@
       </c>
       <c r="C912" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D912" s="2" t="inlineStr">
@@ -61559,7 +61559,7 @@
       </c>
       <c r="C913" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D913" s="2" t="inlineStr">
@@ -61894,7 +61894,7 @@
       </c>
       <c r="C918" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D918" s="2" t="inlineStr">
@@ -62162,7 +62162,7 @@
       </c>
       <c r="C922" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D922" s="2" t="inlineStr">
@@ -63770,7 +63770,7 @@
       </c>
       <c r="C946" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D946" s="2" t="inlineStr">
@@ -63837,7 +63837,7 @@
       </c>
       <c r="C947" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D947" s="2" t="inlineStr">
@@ -64306,7 +64306,7 @@
       </c>
       <c r="C954" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D954" s="2" t="inlineStr">
@@ -65177,7 +65177,7 @@
       </c>
       <c r="C967" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D967" s="2" t="inlineStr">
@@ -65914,7 +65914,7 @@
       </c>
       <c r="C978" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D978" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-05 22:04:10
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixas_42l.xlsx
+++ b/relatorio_analitico_caixas_42l.xlsx
@@ -1795,7 +1795,7 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -4341,7 +4341,7 @@
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
@@ -6552,7 +6552,7 @@
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
@@ -6753,7 +6753,7 @@
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
@@ -7490,7 +7490,7 @@
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D106" s="2" t="inlineStr">
@@ -7959,7 +7959,7 @@
       </c>
       <c r="C113" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D113" s="2" t="inlineStr">
@@ -15999,7 +15999,7 @@
       </c>
       <c r="C233" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D233" s="2" t="inlineStr">
@@ -18344,7 +18344,7 @@
       </c>
       <c r="C268" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D268" s="2" t="inlineStr">
@@ -18947,7 +18947,7 @@
       </c>
       <c r="C277" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D277" s="2" t="inlineStr">
@@ -19215,7 +19215,7 @@
       </c>
       <c r="C281" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D281" s="2" t="inlineStr">
@@ -20890,7 +20890,7 @@
       </c>
       <c r="C306" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D306" s="2" t="inlineStr">
@@ -21024,7 +21024,7 @@
       </c>
       <c r="C308" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D308" s="2" t="inlineStr">
@@ -23637,7 +23637,7 @@
       </c>
       <c r="C347" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D347" s="2" t="inlineStr">
@@ -26183,7 +26183,7 @@
       </c>
       <c r="C385" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D385" s="2" t="inlineStr">
@@ -26853,7 +26853,7 @@
       </c>
       <c r="C395" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D395" s="2" t="inlineStr">
@@ -28729,7 +28729,7 @@
       </c>
       <c r="C423" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D423" s="2" t="inlineStr">
@@ -32950,7 +32950,7 @@
       </c>
       <c r="C486" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D486" s="2" t="inlineStr">
@@ -33017,7 +33017,7 @@
       </c>
       <c r="C487" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D487" s="2" t="inlineStr">
@@ -33084,7 +33084,7 @@
       </c>
       <c r="C488" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D488" s="2" t="inlineStr">
@@ -35496,7 +35496,7 @@
       </c>
       <c r="C524" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D524" s="2" t="inlineStr">
@@ -37841,7 +37841,7 @@
       </c>
       <c r="C559" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D559" s="2" t="inlineStr">
@@ -48427,7 +48427,7 @@
       </c>
       <c r="C717" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D717" s="2" t="inlineStr">
@@ -48494,7 +48494,7 @@
       </c>
       <c r="C718" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D718" s="2" t="inlineStr">
@@ -49365,7 +49365,7 @@
       </c>
       <c r="C731" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D731" s="2" t="inlineStr">
@@ -49499,7 +49499,7 @@
       </c>
       <c r="C733" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D733" s="2" t="inlineStr">
@@ -49566,7 +49566,7 @@
       </c>
       <c r="C734" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D734" s="2" t="inlineStr">
@@ -51442,7 +51442,7 @@
       </c>
       <c r="C762" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D762" s="2" t="inlineStr">
@@ -52581,7 +52581,7 @@
       </c>
       <c r="C779" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D779" s="2" t="inlineStr">
@@ -52715,7 +52715,7 @@
       </c>
       <c r="C781" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D781" s="2" t="inlineStr">
@@ -52782,7 +52782,7 @@
       </c>
       <c r="C782" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D782" s="2" t="inlineStr">
@@ -56601,7 +56601,7 @@
       </c>
       <c r="C839" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D839" s="2" t="inlineStr">
@@ -61358,7 +61358,7 @@
       </c>
       <c r="C910" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D910" s="2" t="inlineStr">
@@ -61492,7 +61492,7 @@
       </c>
       <c r="C912" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D912" s="2" t="inlineStr">
@@ -61559,7 +61559,7 @@
       </c>
       <c r="C913" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D913" s="2" t="inlineStr">
@@ -62363,7 +62363,7 @@
       </c>
       <c r="C925" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D925" s="2" t="inlineStr">
@@ -65177,7 +65177,7 @@
       </c>
       <c r="C967" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D967" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-08 12:51:10
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixas_42l.xlsx
+++ b/relatorio_analitico_caixas_42l.xlsx
@@ -1996,7 +1996,7 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -4341,7 +4341,7 @@
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
@@ -6552,7 +6552,7 @@
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
@@ -6820,7 +6820,7 @@
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr">
@@ -15597,7 +15597,7 @@
       </c>
       <c r="C227" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D227" s="2" t="inlineStr">
@@ -15865,7 +15865,7 @@
       </c>
       <c r="C231" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D231" s="2" t="inlineStr">
@@ -16133,7 +16133,7 @@
       </c>
       <c r="C235" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D235" s="2" t="inlineStr">
@@ -16803,7 +16803,7 @@
       </c>
       <c r="C245" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D245" s="2" t="inlineStr">
@@ -17339,7 +17339,7 @@
       </c>
       <c r="C253" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D253" s="2" t="inlineStr">
@@ -19148,7 +19148,7 @@
       </c>
       <c r="C280" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D280" s="2" t="inlineStr">
@@ -19282,7 +19282,7 @@
       </c>
       <c r="C282" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D282" s="2" t="inlineStr">
@@ -21225,7 +21225,7 @@
       </c>
       <c r="C311" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D311" s="2" t="inlineStr">
@@ -23905,7 +23905,7 @@
       </c>
       <c r="C351" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D351" s="2" t="inlineStr">
@@ -26451,7 +26451,7 @@
       </c>
       <c r="C389" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D389" s="2" t="inlineStr">
@@ -26652,7 +26652,7 @@
       </c>
       <c r="C392" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D392" s="2" t="inlineStr">
@@ -27322,7 +27322,7 @@
       </c>
       <c r="C402" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D402" s="2" t="inlineStr">
@@ -29198,7 +29198,7 @@
       </c>
       <c r="C430" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D430" s="2" t="inlineStr">
@@ -32883,7 +32883,7 @@
       </c>
       <c r="C485" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D485" s="2" t="inlineStr">
@@ -33352,7 +33352,7 @@
       </c>
       <c r="C492" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D492" s="2" t="inlineStr">
@@ -33419,7 +33419,7 @@
       </c>
       <c r="C493" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D493" s="2" t="inlineStr">
@@ -33486,7 +33486,7 @@
       </c>
       <c r="C494" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D494" s="2" t="inlineStr">
@@ -38310,7 +38310,7 @@
       </c>
       <c r="C566" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D566" s="2" t="inlineStr">
@@ -38377,7 +38377,7 @@
       </c>
       <c r="C567" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D567" s="2" t="inlineStr">
@@ -40655,7 +40655,7 @@
       </c>
       <c r="C601" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D601" s="2" t="inlineStr">
@@ -43469,7 +43469,7 @@
       </c>
       <c r="C643" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D643" s="2" t="inlineStr">
@@ -49499,7 +49499,7 @@
       </c>
       <c r="C733" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D733" s="2" t="inlineStr">
@@ -49901,7 +49901,7 @@
       </c>
       <c r="C739" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D739" s="2" t="inlineStr">
@@ -50035,7 +50035,7 @@
       </c>
       <c r="C741" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D741" s="2" t="inlineStr">
@@ -50102,7 +50102,7 @@
       </c>
       <c r="C742" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D742" s="2" t="inlineStr">
@@ -53117,7 +53117,7 @@
       </c>
       <c r="C787" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D787" s="2" t="inlineStr">
@@ -53318,7 +53318,7 @@
       </c>
       <c r="C790" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D790" s="2" t="inlineStr">
@@ -54591,7 +54591,7 @@
       </c>
       <c r="C809" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D809" s="2" t="inlineStr">
@@ -56132,7 +56132,7 @@
       </c>
       <c r="C832" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D832" s="2" t="inlineStr">
@@ -62028,7 +62028,7 @@
       </c>
       <c r="C920" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D920" s="2" t="inlineStr">
@@ -62095,7 +62095,7 @@
       </c>
       <c r="C921" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D921" s="2" t="inlineStr">
@@ -62430,7 +62430,7 @@
       </c>
       <c r="C926" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D926" s="2" t="inlineStr">
@@ -62564,7 +62564,7 @@
       </c>
       <c r="C928" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D928" s="2" t="inlineStr">
@@ -64306,7 +64306,7 @@
       </c>
       <c r="C954" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D954" s="2" t="inlineStr">
@@ -64373,7 +64373,7 @@
       </c>
       <c r="C955" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D955" s="2" t="inlineStr">
@@ -64842,7 +64842,7 @@
       </c>
       <c r="C962" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D962" s="2" t="inlineStr">
@@ -64976,7 +64976,7 @@
       </c>
       <c r="C964" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D964" s="2" t="inlineStr">
@@ -65713,7 +65713,7 @@
       </c>
       <c r="C975" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D975" s="2" t="inlineStr">
@@ -65981,7 +65981,7 @@
       </c>
       <c r="C979" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D979" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-08 13:31:18
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixas_42l.xlsx
+++ b/relatorio_analitico_caixas_42l.xlsx
@@ -1795,7 +1795,7 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -1996,7 +1996,7 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -4341,7 +4341,7 @@
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
@@ -6820,7 +6820,7 @@
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr">
@@ -7557,7 +7557,7 @@
       </c>
       <c r="C107" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D107" s="2" t="inlineStr">
@@ -15597,7 +15597,7 @@
       </c>
       <c r="C227" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D227" s="2" t="inlineStr">
@@ -15865,7 +15865,7 @@
       </c>
       <c r="C231" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D231" s="2" t="inlineStr">
@@ -16066,7 +16066,7 @@
       </c>
       <c r="C234" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D234" s="2" t="inlineStr">
@@ -16133,7 +16133,7 @@
       </c>
       <c r="C235" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D235" s="2" t="inlineStr">
@@ -18478,7 +18478,7 @@
       </c>
       <c r="C270" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D270" s="2" t="inlineStr">
@@ -19148,7 +19148,7 @@
       </c>
       <c r="C280" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D280" s="2" t="inlineStr">
@@ -23905,7 +23905,7 @@
       </c>
       <c r="C351" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D351" s="2" t="inlineStr">
@@ -26250,7 +26250,7 @@
       </c>
       <c r="C386" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D386" s="2" t="inlineStr">
@@ -26384,7 +26384,7 @@
       </c>
       <c r="C388" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D388" s="2" t="inlineStr">
@@ -26652,7 +26652,7 @@
       </c>
       <c r="C392" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D392" s="2" t="inlineStr">
@@ -29198,7 +29198,7 @@
       </c>
       <c r="C430" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D430" s="2" t="inlineStr">
@@ -33218,7 +33218,7 @@
       </c>
       <c r="C490" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D490" s="2" t="inlineStr">
@@ -33352,7 +33352,7 @@
       </c>
       <c r="C492" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D492" s="2" t="inlineStr">
@@ -33419,7 +33419,7 @@
       </c>
       <c r="C493" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D493" s="2" t="inlineStr">
@@ -33486,7 +33486,7 @@
       </c>
       <c r="C494" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D494" s="2" t="inlineStr">
@@ -33553,7 +33553,7 @@
       </c>
       <c r="C495" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D495" s="2" t="inlineStr">
@@ -40655,7 +40655,7 @@
       </c>
       <c r="C601" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D601" s="2" t="inlineStr">
@@ -48963,7 +48963,7 @@
       </c>
       <c r="C725" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D725" s="2" t="inlineStr">
@@ -49901,7 +49901,7 @@
       </c>
       <c r="C739" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D739" s="2" t="inlineStr">
@@ -50035,7 +50035,7 @@
       </c>
       <c r="C741" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D741" s="2" t="inlineStr">
@@ -51978,7 +51978,7 @@
       </c>
       <c r="C770" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D770" s="2" t="inlineStr">
@@ -53117,7 +53117,7 @@
       </c>
       <c r="C787" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D787" s="2" t="inlineStr">
@@ -53184,7 +53184,7 @@
       </c>
       <c r="C788" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D788" s="2" t="inlineStr">
@@ -53318,7 +53318,7 @@
       </c>
       <c r="C790" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D790" s="2" t="inlineStr">
@@ -54591,7 +54591,7 @@
       </c>
       <c r="C809" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D809" s="2" t="inlineStr">
@@ -56132,7 +56132,7 @@
       </c>
       <c r="C832" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D832" s="2" t="inlineStr">
@@ -57673,7 +57673,7 @@
       </c>
       <c r="C855" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D855" s="2" t="inlineStr">
@@ -62028,7 +62028,7 @@
       </c>
       <c r="C920" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D920" s="2" t="inlineStr">
@@ -62430,7 +62430,7 @@
       </c>
       <c r="C926" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D926" s="2" t="inlineStr">
@@ -62564,7 +62564,7 @@
       </c>
       <c r="C928" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D928" s="2" t="inlineStr">
@@ -64373,7 +64373,7 @@
       </c>
       <c r="C955" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D955" s="2" t="inlineStr">
@@ -64909,7 +64909,7 @@
       </c>
       <c r="C963" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D963" s="2" t="inlineStr">
@@ -67187,7 +67187,7 @@
       </c>
       <c r="C997" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D997" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-08 14:25:38
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixas_42l.xlsx
+++ b/relatorio_analitico_caixas_42l.xlsx
@@ -19282,7 +19282,7 @@
       </c>
       <c r="C282" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D282" s="2" t="inlineStr">
@@ -21225,7 +21225,7 @@
       </c>
       <c r="C311" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D311" s="2" t="inlineStr">
@@ -26250,7 +26250,7 @@
       </c>
       <c r="C386" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D386" s="2" t="inlineStr">
@@ -26652,7 +26652,7 @@
       </c>
       <c r="C392" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D392" s="2" t="inlineStr">
@@ -33218,7 +33218,7 @@
       </c>
       <c r="C490" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D490" s="2" t="inlineStr">
@@ -33419,7 +33419,7 @@
       </c>
       <c r="C493" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D493" s="2" t="inlineStr">
@@ -33553,7 +33553,7 @@
       </c>
       <c r="C495" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D495" s="2" t="inlineStr">
@@ -43469,7 +43469,7 @@
       </c>
       <c r="C643" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D643" s="2" t="inlineStr">
@@ -46082,7 +46082,7 @@
       </c>
       <c r="C682" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D682" s="2" t="inlineStr">
@@ -48896,7 +48896,7 @@
       </c>
       <c r="C724" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D724" s="2" t="inlineStr">
@@ -49499,7 +49499,7 @@
       </c>
       <c r="C733" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D733" s="2" t="inlineStr">
@@ -53050,7 +53050,7 @@
       </c>
       <c r="C786" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D786" s="2" t="inlineStr">
@@ -53117,7 +53117,7 @@
       </c>
       <c r="C787" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D787" s="2" t="inlineStr">
@@ -53318,7 +53318,7 @@
       </c>
       <c r="C790" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D790" s="2" t="inlineStr">
@@ -56132,7 +56132,7 @@
       </c>
       <c r="C832" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D832" s="2" t="inlineStr">
@@ -56266,7 +56266,7 @@
       </c>
       <c r="C834" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D834" s="2" t="inlineStr">
@@ -57137,7 +57137,7 @@
       </c>
       <c r="C847" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D847" s="2" t="inlineStr">
@@ -62028,7 +62028,7 @@
       </c>
       <c r="C920" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D920" s="2" t="inlineStr">
@@ -62430,7 +62430,7 @@
       </c>
       <c r="C926" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D926" s="2" t="inlineStr">
@@ -62899,7 +62899,7 @@
       </c>
       <c r="C933" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D933" s="2" t="inlineStr">
@@ -64842,7 +64842,7 @@
       </c>
       <c r="C962" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D962" s="2" t="inlineStr">
@@ -64976,7 +64976,7 @@
       </c>
       <c r="C964" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D964" s="2" t="inlineStr">
@@ -65713,7 +65713,7 @@
       </c>
       <c r="C975" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D975" s="2" t="inlineStr">
@@ -67187,7 +67187,7 @@
       </c>
       <c r="C997" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D997" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-08 14:34:32
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixas_42l.xlsx
+++ b/relatorio_analitico_caixas_42l.xlsx
@@ -1795,7 +1795,7 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -1996,7 +1996,7 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -4341,7 +4341,7 @@
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
@@ -7557,7 +7557,7 @@
       </c>
       <c r="C107" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D107" s="2" t="inlineStr">
@@ -8026,7 +8026,7 @@
       </c>
       <c r="C114" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D114" s="2" t="inlineStr">
@@ -16133,7 +16133,7 @@
       </c>
       <c r="C235" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D235" s="2" t="inlineStr">
@@ -18478,7 +18478,7 @@
       </c>
       <c r="C270" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D270" s="2" t="inlineStr">
@@ -19282,7 +19282,7 @@
       </c>
       <c r="C282" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D282" s="2" t="inlineStr">
@@ -19416,7 +19416,7 @@
       </c>
       <c r="C284" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D284" s="2" t="inlineStr">
@@ -23905,7 +23905,7 @@
       </c>
       <c r="C351" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D351" s="2" t="inlineStr">
@@ -26116,7 +26116,7 @@
       </c>
       <c r="C384" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D384" s="2" t="inlineStr">
@@ -26451,7 +26451,7 @@
       </c>
       <c r="C389" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="D389" s="2" t="inlineStr">
@@ -26585,7 +26585,7 @@
       </c>
       <c r="C391" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D391" s="2" t="inlineStr">
@@ -27322,7 +27322,7 @@
       </c>
       <c r="C402" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D402" s="2" t="inlineStr">
@@ -32883,7 +32883,7 @@
       </c>
       <c r="C485" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D485" s="2" t="inlineStr">
@@ -33218,7 +33218,7 @@
       </c>
       <c r="C490" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D490" s="2" t="inlineStr">
@@ -33419,7 +33419,7 @@
       </c>
       <c r="C493" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D493" s="2" t="inlineStr">
@@ -33486,7 +33486,7 @@
       </c>
       <c r="C494" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D494" s="2" t="inlineStr">
@@ -33553,7 +33553,7 @@
       </c>
       <c r="C495" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D495" s="2" t="inlineStr">
@@ -49499,7 +49499,7 @@
       </c>
       <c r="C733" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D733" s="2" t="inlineStr">
@@ -49901,7 +49901,7 @@
       </c>
       <c r="C739" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D739" s="2" t="inlineStr">
@@ -50102,7 +50102,7 @@
       </c>
       <c r="C742" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D742" s="2" t="inlineStr">
@@ -53117,7 +53117,7 @@
       </c>
       <c r="C787" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D787" s="2" t="inlineStr">
@@ -53184,7 +53184,7 @@
       </c>
       <c r="C788" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D788" s="2" t="inlineStr">
@@ -53251,7 +53251,7 @@
       </c>
       <c r="C789" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D789" s="2" t="inlineStr">
@@ -54591,7 +54591,7 @@
       </c>
       <c r="C809" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D809" s="2" t="inlineStr">
@@ -57137,7 +57137,7 @@
       </c>
       <c r="C847" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D847" s="2" t="inlineStr">
@@ -61894,7 +61894,7 @@
       </c>
       <c r="C918" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D918" s="2" t="inlineStr">
@@ -62028,7 +62028,7 @@
       </c>
       <c r="C920" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D920" s="2" t="inlineStr">
@@ -64842,7 +64842,7 @@
       </c>
       <c r="C962" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D962" s="2" t="inlineStr">
@@ -64976,7 +64976,7 @@
       </c>
       <c r="C964" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D964" s="2" t="inlineStr">
@@ -65713,7 +65713,7 @@
       </c>
       <c r="C975" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D975" s="2" t="inlineStr">
@@ -66450,7 +66450,7 @@
       </c>
       <c r="C986" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D986" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-08 15:46:41
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixas_42l.xlsx
+++ b/relatorio_analitico_caixas_42l.xlsx
@@ -8026,7 +8026,7 @@
       </c>
       <c r="C114" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D114" s="2" t="inlineStr">
@@ -15597,7 +15597,7 @@
       </c>
       <c r="C227" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D227" s="2" t="inlineStr">
@@ -15865,7 +15865,7 @@
       </c>
       <c r="C231" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D231" s="2" t="inlineStr">
@@ -18478,7 +18478,7 @@
       </c>
       <c r="C270" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D270" s="2" t="inlineStr">
@@ -19148,7 +19148,7 @@
       </c>
       <c r="C280" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D280" s="2" t="inlineStr">
@@ -19416,7 +19416,7 @@
       </c>
       <c r="C284" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D284" s="2" t="inlineStr">
@@ -20756,7 +20756,7 @@
       </c>
       <c r="C304" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D304" s="2" t="inlineStr">
@@ -23637,7 +23637,7 @@
       </c>
       <c r="C347" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D347" s="2" t="inlineStr">
@@ -23905,7 +23905,7 @@
       </c>
       <c r="C351" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D351" s="2" t="inlineStr">
@@ -26116,7 +26116,7 @@
       </c>
       <c r="C384" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D384" s="2" t="inlineStr">
@@ -26250,7 +26250,7 @@
       </c>
       <c r="C386" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D386" s="2" t="inlineStr">
@@ -26451,7 +26451,7 @@
       </c>
       <c r="C389" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="D389" s="2" t="inlineStr">
@@ -26652,7 +26652,7 @@
       </c>
       <c r="C392" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D392" s="2" t="inlineStr">
@@ -27322,7 +27322,7 @@
       </c>
       <c r="C402" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D402" s="2" t="inlineStr">
@@ -29198,7 +29198,7 @@
       </c>
       <c r="C430" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D430" s="2" t="inlineStr">
@@ -32816,7 +32816,7 @@
       </c>
       <c r="C484" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D484" s="2" t="inlineStr">
@@ -32883,7 +32883,7 @@
       </c>
       <c r="C485" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D485" s="2" t="inlineStr">
@@ -33218,7 +33218,7 @@
       </c>
       <c r="C490" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D490" s="2" t="inlineStr">
@@ -33553,7 +33553,7 @@
       </c>
       <c r="C495" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D495" s="2" t="inlineStr">
@@ -38310,7 +38310,7 @@
       </c>
       <c r="C566" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D566" s="2" t="inlineStr">
@@ -38377,7 +38377,7 @@
       </c>
       <c r="C567" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D567" s="2" t="inlineStr">
@@ -40655,7 +40655,7 @@
       </c>
       <c r="C601" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D601" s="2" t="inlineStr">
@@ -48963,7 +48963,7 @@
       </c>
       <c r="C725" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D725" s="2" t="inlineStr">
@@ -49901,7 +49901,7 @@
       </c>
       <c r="C739" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D739" s="2" t="inlineStr">
@@ -50035,7 +50035,7 @@
       </c>
       <c r="C741" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D741" s="2" t="inlineStr">
@@ -51978,7 +51978,7 @@
       </c>
       <c r="C770" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D770" s="2" t="inlineStr">
@@ -54591,7 +54591,7 @@
       </c>
       <c r="C809" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D809" s="2" t="inlineStr">
@@ -56132,7 +56132,7 @@
       </c>
       <c r="C832" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D832" s="2" t="inlineStr">
@@ -57137,7 +57137,7 @@
       </c>
       <c r="C847" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D847" s="2" t="inlineStr">
@@ -62095,7 +62095,7 @@
       </c>
       <c r="C921" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D921" s="2" t="inlineStr">
@@ -62229,7 +62229,7 @@
       </c>
       <c r="C923" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D923" s="2" t="inlineStr">
@@ -62564,7 +62564,7 @@
       </c>
       <c r="C928" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D928" s="2" t="inlineStr">
@@ -62899,7 +62899,7 @@
       </c>
       <c r="C933" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D933" s="2" t="inlineStr">
@@ -64306,7 +64306,7 @@
       </c>
       <c r="C954" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D954" s="2" t="inlineStr">
@@ -64373,7 +64373,7 @@
       </c>
       <c r="C955" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D955" s="2" t="inlineStr">
@@ -64909,7 +64909,7 @@
       </c>
       <c r="C963" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D963" s="2" t="inlineStr">
@@ -66450,7 +66450,7 @@
       </c>
       <c r="C986" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D986" s="2" t="inlineStr">
@@ -67187,7 +67187,7 @@
       </c>
       <c r="C997" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D997" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-08 17:48:38
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixas_42l.xlsx
+++ b/relatorio_analitico_caixas_42l.xlsx
@@ -1996,7 +1996,7 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -4341,7 +4341,7 @@
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
@@ -6552,7 +6552,7 @@
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
@@ -8026,7 +8026,7 @@
       </c>
       <c r="C114" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D114" s="2" t="inlineStr">
@@ -15597,7 +15597,7 @@
       </c>
       <c r="C227" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D227" s="2" t="inlineStr">
@@ -16803,7 +16803,7 @@
       </c>
       <c r="C245" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D245" s="2" t="inlineStr">
@@ -18478,7 +18478,7 @@
       </c>
       <c r="C270" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D270" s="2" t="inlineStr">
@@ -19282,7 +19282,7 @@
       </c>
       <c r="C282" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D282" s="2" t="inlineStr">
@@ -19416,7 +19416,7 @@
       </c>
       <c r="C284" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D284" s="2" t="inlineStr">
@@ -21225,7 +21225,7 @@
       </c>
       <c r="C311" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D311" s="2" t="inlineStr">
@@ -23637,7 +23637,7 @@
       </c>
       <c r="C347" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D347" s="2" t="inlineStr">
@@ -23905,7 +23905,7 @@
       </c>
       <c r="C351" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D351" s="2" t="inlineStr">
@@ -26116,7 +26116,7 @@
       </c>
       <c r="C384" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D384" s="2" t="inlineStr">
@@ -26451,7 +26451,7 @@
       </c>
       <c r="C389" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D389" s="2" t="inlineStr">
@@ -26585,7 +26585,7 @@
       </c>
       <c r="C391" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D391" s="2" t="inlineStr">
@@ -27322,7 +27322,7 @@
       </c>
       <c r="C402" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D402" s="2" t="inlineStr">
@@ -29198,7 +29198,7 @@
       </c>
       <c r="C430" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D430" s="2" t="inlineStr">
@@ -32816,7 +32816,7 @@
       </c>
       <c r="C484" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D484" s="2" t="inlineStr">
@@ -33486,7 +33486,7 @@
       </c>
       <c r="C494" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D494" s="2" t="inlineStr">
@@ -38310,7 +38310,7 @@
       </c>
       <c r="C566" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D566" s="2" t="inlineStr">
@@ -40655,7 +40655,7 @@
       </c>
       <c r="C601" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D601" s="2" t="inlineStr">
@@ -48963,7 +48963,7 @@
       </c>
       <c r="C725" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D725" s="2" t="inlineStr">
@@ -49901,7 +49901,7 @@
       </c>
       <c r="C739" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D739" s="2" t="inlineStr">
@@ -50035,7 +50035,7 @@
       </c>
       <c r="C741" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D741" s="2" t="inlineStr">
@@ -53050,7 +53050,7 @@
       </c>
       <c r="C786" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D786" s="2" t="inlineStr">
@@ -53117,7 +53117,7 @@
       </c>
       <c r="C787" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D787" s="2" t="inlineStr">
@@ -53318,7 +53318,7 @@
       </c>
       <c r="C790" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D790" s="2" t="inlineStr">
@@ -54591,7 +54591,7 @@
       </c>
       <c r="C809" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D809" s="2" t="inlineStr">
@@ -56065,7 +56065,7 @@
       </c>
       <c r="C831" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D831" s="2" t="inlineStr">
@@ -56132,7 +56132,7 @@
       </c>
       <c r="C832" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D832" s="2" t="inlineStr">
@@ -56266,7 +56266,7 @@
       </c>
       <c r="C834" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D834" s="2" t="inlineStr">
@@ -57673,7 +57673,7 @@
       </c>
       <c r="C855" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D855" s="2" t="inlineStr">
@@ -57874,7 +57874,7 @@
       </c>
       <c r="C858" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D858" s="2" t="inlineStr">
@@ -62430,7 +62430,7 @@
       </c>
       <c r="C926" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D926" s="2" t="inlineStr">
@@ -62564,7 +62564,7 @@
       </c>
       <c r="C928" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D928" s="2" t="inlineStr">
@@ -64909,7 +64909,7 @@
       </c>
       <c r="C963" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D963" s="2" t="inlineStr">
@@ -64976,7 +64976,7 @@
       </c>
       <c r="C964" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D964" s="2" t="inlineStr">
@@ -66450,7 +66450,7 @@
       </c>
       <c r="C986" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D986" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-08 19:09:22
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixas_42l.xlsx
+++ b/relatorio_analitico_caixas_42l.xlsx
@@ -1795,7 +1795,7 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -4341,7 +4341,7 @@
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
@@ -16066,7 +16066,7 @@
       </c>
       <c r="C234" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D234" s="2" t="inlineStr">
@@ -16133,7 +16133,7 @@
       </c>
       <c r="C235" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D235" s="2" t="inlineStr">
@@ -16803,7 +16803,7 @@
       </c>
       <c r="C245" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D245" s="2" t="inlineStr">
@@ -21225,7 +21225,7 @@
       </c>
       <c r="C311" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D311" s="2" t="inlineStr">
@@ -23637,7 +23637,7 @@
       </c>
       <c r="C347" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D347" s="2" t="inlineStr">
@@ -26451,7 +26451,7 @@
       </c>
       <c r="C389" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D389" s="2" t="inlineStr">
@@ -29198,7 +29198,7 @@
       </c>
       <c r="C430" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D430" s="2" t="inlineStr">
@@ -33486,7 +33486,7 @@
       </c>
       <c r="C494" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D494" s="2" t="inlineStr">
@@ -38310,7 +38310,7 @@
       </c>
       <c r="C566" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D566" s="2" t="inlineStr">
@@ -38377,7 +38377,7 @@
       </c>
       <c r="C567" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D567" s="2" t="inlineStr">
@@ -43469,7 +43469,7 @@
       </c>
       <c r="C643" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D643" s="2" t="inlineStr">
@@ -46082,7 +46082,7 @@
       </c>
       <c r="C682" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D682" s="2" t="inlineStr">
@@ -48963,7 +48963,7 @@
       </c>
       <c r="C725" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D725" s="2" t="inlineStr">
@@ -49901,7 +49901,7 @@
       </c>
       <c r="C739" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D739" s="2" t="inlineStr">
@@ -50035,7 +50035,7 @@
       </c>
       <c r="C741" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D741" s="2" t="inlineStr">
@@ -51978,7 +51978,7 @@
       </c>
       <c r="C770" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D770" s="2" t="inlineStr">
@@ -53318,7 +53318,7 @@
       </c>
       <c r="C790" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D790" s="2" t="inlineStr">
@@ -56132,7 +56132,7 @@
       </c>
       <c r="C832" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D832" s="2" t="inlineStr">
@@ -56199,7 +56199,7 @@
       </c>
       <c r="C833" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D833" s="2" t="inlineStr">
@@ -57137,7 +57137,7 @@
       </c>
       <c r="C847" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D847" s="2" t="inlineStr">
@@ -62028,7 +62028,7 @@
       </c>
       <c r="C920" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D920" s="2" t="inlineStr">
@@ -62095,7 +62095,7 @@
       </c>
       <c r="C921" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D921" s="2" t="inlineStr">
@@ -62430,7 +62430,7 @@
       </c>
       <c r="C926" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D926" s="2" t="inlineStr">
@@ -62564,7 +62564,7 @@
       </c>
       <c r="C928" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D928" s="2" t="inlineStr">
@@ -62899,7 +62899,7 @@
       </c>
       <c r="C933" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D933" s="2" t="inlineStr">
@@ -64373,7 +64373,7 @@
       </c>
       <c r="C955" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D955" s="2" t="inlineStr">
@@ -64909,7 +64909,7 @@
       </c>
       <c r="C963" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D963" s="2" t="inlineStr">
@@ -64976,7 +64976,7 @@
       </c>
       <c r="C964" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D964" s="2" t="inlineStr">
@@ -65713,7 +65713,7 @@
       </c>
       <c r="C975" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D975" s="2" t="inlineStr">
@@ -66450,7 +66450,7 @@
       </c>
       <c r="C986" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D986" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-08 19:18:59
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixas_42l.xlsx
+++ b/relatorio_analitico_caixas_42l.xlsx
@@ -1795,7 +1795,7 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -1996,7 +1996,7 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -6552,7 +6552,7 @@
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
@@ -8026,7 +8026,7 @@
       </c>
       <c r="C114" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D114" s="2" t="inlineStr">
@@ -16133,7 +16133,7 @@
       </c>
       <c r="C235" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D235" s="2" t="inlineStr">
@@ -16803,7 +16803,7 @@
       </c>
       <c r="C245" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D245" s="2" t="inlineStr">
@@ -20756,7 +20756,7 @@
       </c>
       <c r="C304" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D304" s="2" t="inlineStr">
@@ -21091,7 +21091,7 @@
       </c>
       <c r="C309" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D309" s="2" t="inlineStr">
@@ -23637,7 +23637,7 @@
       </c>
       <c r="C347" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D347" s="2" t="inlineStr">
@@ -26652,7 +26652,7 @@
       </c>
       <c r="C392" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D392" s="2" t="inlineStr">
@@ -32883,7 +32883,7 @@
       </c>
       <c r="C485" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D485" s="2" t="inlineStr">
@@ -33218,7 +33218,7 @@
       </c>
       <c r="C490" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D490" s="2" t="inlineStr">
@@ -33486,7 +33486,7 @@
       </c>
       <c r="C494" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D494" s="2" t="inlineStr">
@@ -33553,7 +33553,7 @@
       </c>
       <c r="C495" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D495" s="2" t="inlineStr">
@@ -38310,7 +38310,7 @@
       </c>
       <c r="C566" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D566" s="2" t="inlineStr">
@@ -40655,7 +40655,7 @@
       </c>
       <c r="C601" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D601" s="2" t="inlineStr">
@@ -43469,7 +43469,7 @@
       </c>
       <c r="C643" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D643" s="2" t="inlineStr">
@@ -46082,7 +46082,7 @@
       </c>
       <c r="C682" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D682" s="2" t="inlineStr">
@@ -48896,7 +48896,7 @@
       </c>
       <c r="C724" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D724" s="2" t="inlineStr">
@@ -48963,7 +48963,7 @@
       </c>
       <c r="C725" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D725" s="2" t="inlineStr">
@@ -49499,7 +49499,7 @@
       </c>
       <c r="C733" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D733" s="2" t="inlineStr">
@@ -49901,7 +49901,7 @@
       </c>
       <c r="C739" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D739" s="2" t="inlineStr">
@@ -53184,7 +53184,7 @@
       </c>
       <c r="C788" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D788" s="2" t="inlineStr">
@@ -53251,7 +53251,7 @@
       </c>
       <c r="C789" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D789" s="2" t="inlineStr">
@@ -53318,7 +53318,7 @@
       </c>
       <c r="C790" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D790" s="2" t="inlineStr">
@@ -56065,7 +56065,7 @@
       </c>
       <c r="C831" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D831" s="2" t="inlineStr">
@@ -62028,7 +62028,7 @@
       </c>
       <c r="C920" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D920" s="2" t="inlineStr">
@@ -62430,7 +62430,7 @@
       </c>
       <c r="C926" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D926" s="2" t="inlineStr">
@@ -62564,7 +62564,7 @@
       </c>
       <c r="C928" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D928" s="2" t="inlineStr">
@@ -64306,7 +64306,7 @@
       </c>
       <c r="C954" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D954" s="2" t="inlineStr">
@@ -64373,7 +64373,7 @@
       </c>
       <c r="C955" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D955" s="2" t="inlineStr">
@@ -64909,7 +64909,7 @@
       </c>
       <c r="C963" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D963" s="2" t="inlineStr">
@@ -64976,7 +64976,7 @@
       </c>
       <c r="C964" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D964" s="2" t="inlineStr">
@@ -65713,7 +65713,7 @@
       </c>
       <c r="C975" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D975" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-08 19:45:49
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixas_42l.xlsx
+++ b/relatorio_analitico_caixas_42l.xlsx
@@ -7557,7 +7557,7 @@
       </c>
       <c r="C107" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D107" s="2" t="inlineStr">
@@ -8026,7 +8026,7 @@
       </c>
       <c r="C114" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D114" s="2" t="inlineStr">
@@ -15865,7 +15865,7 @@
       </c>
       <c r="C231" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D231" s="2" t="inlineStr">
@@ -16066,7 +16066,7 @@
       </c>
       <c r="C234" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D234" s="2" t="inlineStr">
@@ -16803,7 +16803,7 @@
       </c>
       <c r="C245" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D245" s="2" t="inlineStr">
@@ -21091,7 +21091,7 @@
       </c>
       <c r="C309" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D309" s="2" t="inlineStr">
@@ -21225,7 +21225,7 @@
       </c>
       <c r="C311" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D311" s="2" t="inlineStr">
@@ -23637,7 +23637,7 @@
       </c>
       <c r="C347" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D347" s="2" t="inlineStr">
@@ -23905,7 +23905,7 @@
       </c>
       <c r="C351" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D351" s="2" t="inlineStr">
@@ -26384,7 +26384,7 @@
       </c>
       <c r="C388" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D388" s="2" t="inlineStr">
@@ -27322,7 +27322,7 @@
       </c>
       <c r="C402" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D402" s="2" t="inlineStr">
@@ -33218,7 +33218,7 @@
       </c>
       <c r="C490" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D490" s="2" t="inlineStr">
@@ -33352,7 +33352,7 @@
       </c>
       <c r="C492" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D492" s="2" t="inlineStr">
@@ -35965,7 +35965,7 @@
       </c>
       <c r="C531" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D531" s="2" t="inlineStr">
@@ -38310,7 +38310,7 @@
       </c>
       <c r="C566" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D566" s="2" t="inlineStr">
@@ -38377,7 +38377,7 @@
       </c>
       <c r="C567" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D567" s="2" t="inlineStr">
@@ -40655,7 +40655,7 @@
       </c>
       <c r="C601" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D601" s="2" t="inlineStr">
@@ -43469,7 +43469,7 @@
       </c>
       <c r="C643" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D643" s="2" t="inlineStr">
@@ -48896,7 +48896,7 @@
       </c>
       <c r="C724" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D724" s="2" t="inlineStr">
@@ -53117,7 +53117,7 @@
       </c>
       <c r="C787" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D787" s="2" t="inlineStr">
@@ -53251,7 +53251,7 @@
       </c>
       <c r="C789" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D789" s="2" t="inlineStr">
@@ -54591,7 +54591,7 @@
       </c>
       <c r="C809" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D809" s="2" t="inlineStr">
@@ -56132,7 +56132,7 @@
       </c>
       <c r="C832" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D832" s="2" t="inlineStr">
@@ -57673,7 +57673,7 @@
       </c>
       <c r="C855" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D855" s="2" t="inlineStr">
@@ -57874,7 +57874,7 @@
       </c>
       <c r="C858" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D858" s="2" t="inlineStr">
@@ -64976,7 +64976,7 @@
       </c>
       <c r="C964" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D964" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-08 20:17:15
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixas_42l.xlsx
+++ b/relatorio_analitico_caixas_42l.xlsx
@@ -1795,7 +1795,7 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -6820,7 +6820,7 @@
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr">
@@ -19148,7 +19148,7 @@
       </c>
       <c r="C280" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D280" s="2" t="inlineStr">
@@ -19416,7 +19416,7 @@
       </c>
       <c r="C284" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D284" s="2" t="inlineStr">
@@ -21091,7 +21091,7 @@
       </c>
       <c r="C309" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D309" s="2" t="inlineStr">
@@ -23637,7 +23637,7 @@
       </c>
       <c r="C347" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D347" s="2" t="inlineStr">
@@ -26384,7 +26384,7 @@
       </c>
       <c r="C388" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D388" s="2" t="inlineStr">
@@ -26652,7 +26652,7 @@
       </c>
       <c r="C392" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D392" s="2" t="inlineStr">
@@ -27322,7 +27322,7 @@
       </c>
       <c r="C402" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D402" s="2" t="inlineStr">
@@ -33218,7 +33218,7 @@
       </c>
       <c r="C490" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D490" s="2" t="inlineStr">
@@ -33352,7 +33352,7 @@
       </c>
       <c r="C492" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D492" s="2" t="inlineStr">
@@ -33419,7 +33419,7 @@
       </c>
       <c r="C493" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D493" s="2" t="inlineStr">
@@ -33553,7 +33553,7 @@
       </c>
       <c r="C495" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D495" s="2" t="inlineStr">
@@ -43469,7 +43469,7 @@
       </c>
       <c r="C643" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D643" s="2" t="inlineStr">
@@ -46082,7 +46082,7 @@
       </c>
       <c r="C682" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D682" s="2" t="inlineStr">
@@ -48963,7 +48963,7 @@
       </c>
       <c r="C725" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D725" s="2" t="inlineStr">
@@ -49499,7 +49499,7 @@
       </c>
       <c r="C733" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D733" s="2" t="inlineStr">
@@ -49901,7 +49901,7 @@
       </c>
       <c r="C739" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D739" s="2" t="inlineStr">
@@ -51978,7 +51978,7 @@
       </c>
       <c r="C770" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D770" s="2" t="inlineStr">
@@ -53117,7 +53117,7 @@
       </c>
       <c r="C787" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D787" s="2" t="inlineStr">
@@ -53251,7 +53251,7 @@
       </c>
       <c r="C789" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D789" s="2" t="inlineStr">
@@ -54591,7 +54591,7 @@
       </c>
       <c r="C809" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D809" s="2" t="inlineStr">
@@ -56065,7 +56065,7 @@
       </c>
       <c r="C831" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D831" s="2" t="inlineStr">
@@ -56199,7 +56199,7 @@
       </c>
       <c r="C833" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D833" s="2" t="inlineStr">
@@ -57673,7 +57673,7 @@
       </c>
       <c r="C855" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D855" s="2" t="inlineStr">
@@ -62028,7 +62028,7 @@
       </c>
       <c r="C920" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D920" s="2" t="inlineStr">
@@ -62229,7 +62229,7 @@
       </c>
       <c r="C923" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D923" s="2" t="inlineStr">
@@ -62430,7 +62430,7 @@
       </c>
       <c r="C926" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D926" s="2" t="inlineStr">
@@ -62564,7 +62564,7 @@
       </c>
       <c r="C928" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D928" s="2" t="inlineStr">
@@ -64373,7 +64373,7 @@
       </c>
       <c r="C955" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D955" s="2" t="inlineStr">
@@ -64909,7 +64909,7 @@
       </c>
       <c r="C963" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D963" s="2" t="inlineStr">
@@ -65713,7 +65713,7 @@
       </c>
       <c r="C975" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D975" s="2" t="inlineStr">
@@ -67187,7 +67187,7 @@
       </c>
       <c r="C997" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D997" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-08 20:36:32
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixas_42l.xlsx
+++ b/relatorio_analitico_caixas_42l.xlsx
@@ -1795,7 +1795,7 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -4341,7 +4341,7 @@
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
@@ -6820,7 +6820,7 @@
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr">
@@ -15597,7 +15597,7 @@
       </c>
       <c r="C227" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D227" s="2" t="inlineStr">
@@ -16066,7 +16066,7 @@
       </c>
       <c r="C234" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D234" s="2" t="inlineStr">
@@ -19148,7 +19148,7 @@
       </c>
       <c r="C280" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D280" s="2" t="inlineStr">
@@ -21225,7 +21225,7 @@
       </c>
       <c r="C311" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D311" s="2" t="inlineStr">
@@ -23637,7 +23637,7 @@
       </c>
       <c r="C347" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D347" s="2" t="inlineStr">
@@ -23905,7 +23905,7 @@
       </c>
       <c r="C351" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D351" s="2" t="inlineStr">
@@ -26250,7 +26250,7 @@
       </c>
       <c r="C386" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D386" s="2" t="inlineStr">
@@ -26451,7 +26451,7 @@
       </c>
       <c r="C389" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="D389" s="2" t="inlineStr">
@@ -26652,7 +26652,7 @@
       </c>
       <c r="C392" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D392" s="2" t="inlineStr">
@@ -27322,7 +27322,7 @@
       </c>
       <c r="C402" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D402" s="2" t="inlineStr">
@@ -32816,7 +32816,7 @@
       </c>
       <c r="C484" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D484" s="2" t="inlineStr">
@@ -33218,7 +33218,7 @@
       </c>
       <c r="C490" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D490" s="2" t="inlineStr">
@@ -33352,7 +33352,7 @@
       </c>
       <c r="C492" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D492" s="2" t="inlineStr">
@@ -35965,7 +35965,7 @@
       </c>
       <c r="C531" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D531" s="2" t="inlineStr">
@@ -38377,7 +38377,7 @@
       </c>
       <c r="C567" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D567" s="2" t="inlineStr">
@@ -43469,7 +43469,7 @@
       </c>
       <c r="C643" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D643" s="2" t="inlineStr">
@@ -48896,7 +48896,7 @@
       </c>
       <c r="C724" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D724" s="2" t="inlineStr">
@@ -48963,7 +48963,7 @@
       </c>
       <c r="C725" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D725" s="2" t="inlineStr">
@@ -49499,7 +49499,7 @@
       </c>
       <c r="C733" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D733" s="2" t="inlineStr">
@@ -49901,7 +49901,7 @@
       </c>
       <c r="C739" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D739" s="2" t="inlineStr">
@@ -50035,7 +50035,7 @@
       </c>
       <c r="C741" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D741" s="2" t="inlineStr">
@@ -51978,7 +51978,7 @@
       </c>
       <c r="C770" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D770" s="2" t="inlineStr">
@@ -53184,7 +53184,7 @@
       </c>
       <c r="C788" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D788" s="2" t="inlineStr">
@@ -53251,7 +53251,7 @@
       </c>
       <c r="C789" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D789" s="2" t="inlineStr">
@@ -53318,7 +53318,7 @@
       </c>
       <c r="C790" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D790" s="2" t="inlineStr">
@@ -54591,7 +54591,7 @@
       </c>
       <c r="C809" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D809" s="2" t="inlineStr">
@@ -56065,7 +56065,7 @@
       </c>
       <c r="C831" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D831" s="2" t="inlineStr">
@@ -56266,7 +56266,7 @@
       </c>
       <c r="C834" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D834" s="2" t="inlineStr">
@@ -62430,7 +62430,7 @@
       </c>
       <c r="C926" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D926" s="2" t="inlineStr">
@@ -62564,7 +62564,7 @@
       </c>
       <c r="C928" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D928" s="2" t="inlineStr">
@@ -64306,7 +64306,7 @@
       </c>
       <c r="C954" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D954" s="2" t="inlineStr">
@@ -64842,7 +64842,7 @@
       </c>
       <c r="C962" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D962" s="2" t="inlineStr">
@@ -64909,7 +64909,7 @@
       </c>
       <c r="C963" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D963" s="2" t="inlineStr">
@@ -65981,7 +65981,7 @@
       </c>
       <c r="C979" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D979" s="2" t="inlineStr">
@@ -66450,7 +66450,7 @@
       </c>
       <c r="C986" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D986" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-08 21:44:15
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixas_42l.xlsx
+++ b/relatorio_analitico_caixas_42l.xlsx
@@ -1996,7 +1996,7 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -4341,7 +4341,7 @@
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
@@ -6552,7 +6552,7 @@
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
@@ -15865,7 +15865,7 @@
       </c>
       <c r="C231" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D231" s="2" t="inlineStr">
@@ -16133,7 +16133,7 @@
       </c>
       <c r="C235" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D235" s="2" t="inlineStr">
@@ -18478,7 +18478,7 @@
       </c>
       <c r="C270" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D270" s="2" t="inlineStr">
@@ -19148,7 +19148,7 @@
       </c>
       <c r="C280" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D280" s="2" t="inlineStr">
@@ -21225,7 +21225,7 @@
       </c>
       <c r="C311" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D311" s="2" t="inlineStr">
@@ -26116,7 +26116,7 @@
       </c>
       <c r="C384" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D384" s="2" t="inlineStr">
@@ -26250,7 +26250,7 @@
       </c>
       <c r="C386" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D386" s="2" t="inlineStr">
@@ -26585,7 +26585,7 @@
       </c>
       <c r="C391" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D391" s="2" t="inlineStr">
@@ -26652,7 +26652,7 @@
       </c>
       <c r="C392" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D392" s="2" t="inlineStr">
@@ -27322,7 +27322,7 @@
       </c>
       <c r="C402" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D402" s="2" t="inlineStr">
@@ -29198,7 +29198,7 @@
       </c>
       <c r="C430" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D430" s="2" t="inlineStr">
@@ -32816,7 +32816,7 @@
       </c>
       <c r="C484" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D484" s="2" t="inlineStr">
@@ -32883,7 +32883,7 @@
       </c>
       <c r="C485" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D485" s="2" t="inlineStr">
@@ -33218,7 +33218,7 @@
       </c>
       <c r="C490" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D490" s="2" t="inlineStr">
@@ -33486,7 +33486,7 @@
       </c>
       <c r="C494" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D494" s="2" t="inlineStr">
@@ -35965,7 +35965,7 @@
       </c>
       <c r="C531" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D531" s="2" t="inlineStr">
@@ -38310,7 +38310,7 @@
       </c>
       <c r="C566" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D566" s="2" t="inlineStr">
@@ -43469,7 +43469,7 @@
       </c>
       <c r="C643" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D643" s="2" t="inlineStr">
@@ -46082,7 +46082,7 @@
       </c>
       <c r="C682" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D682" s="2" t="inlineStr">
@@ -48896,7 +48896,7 @@
       </c>
       <c r="C724" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D724" s="2" t="inlineStr">
@@ -48963,7 +48963,7 @@
       </c>
       <c r="C725" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D725" s="2" t="inlineStr">
@@ -53050,7 +53050,7 @@
       </c>
       <c r="C786" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D786" s="2" t="inlineStr">
@@ -53251,7 +53251,7 @@
       </c>
       <c r="C789" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D789" s="2" t="inlineStr">
@@ -54591,7 +54591,7 @@
       </c>
       <c r="C809" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D809" s="2" t="inlineStr">
@@ -56065,7 +56065,7 @@
       </c>
       <c r="C831" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D831" s="2" t="inlineStr">
@@ -56132,7 +56132,7 @@
       </c>
       <c r="C832" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D832" s="2" t="inlineStr">
@@ -57137,7 +57137,7 @@
       </c>
       <c r="C847" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D847" s="2" t="inlineStr">
@@ -57874,7 +57874,7 @@
       </c>
       <c r="C858" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D858" s="2" t="inlineStr">
@@ -61894,7 +61894,7 @@
       </c>
       <c r="C918" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D918" s="2" t="inlineStr">
@@ -62028,7 +62028,7 @@
       </c>
       <c r="C920" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D920" s="2" t="inlineStr">
@@ -62564,7 +62564,7 @@
       </c>
       <c r="C928" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D928" s="2" t="inlineStr">
@@ -62698,7 +62698,7 @@
       </c>
       <c r="C930" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D930" s="2" t="inlineStr">
@@ -62899,7 +62899,7 @@
       </c>
       <c r="C933" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D933" s="2" t="inlineStr">
@@ -64373,7 +64373,7 @@
       </c>
       <c r="C955" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D955" s="2" t="inlineStr">
@@ -64976,7 +64976,7 @@
       </c>
       <c r="C964" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D964" s="2" t="inlineStr">
@@ -65713,7 +65713,7 @@
       </c>
       <c r="C975" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D975" s="2" t="inlineStr">
@@ -67187,7 +67187,7 @@
       </c>
       <c r="C997" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D997" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-08 22:09:15
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixas_42l.xlsx
+++ b/relatorio_analitico_caixas_42l.xlsx
@@ -1996,7 +1996,7 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -4341,7 +4341,7 @@
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
@@ -6820,7 +6820,7 @@
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr">
@@ -7557,7 +7557,7 @@
       </c>
       <c r="C107" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D107" s="2" t="inlineStr">
@@ -15865,7 +15865,7 @@
       </c>
       <c r="C231" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D231" s="2" t="inlineStr">
@@ -16066,7 +16066,7 @@
       </c>
       <c r="C234" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D234" s="2" t="inlineStr">
@@ -16803,7 +16803,7 @@
       </c>
       <c r="C245" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D245" s="2" t="inlineStr">
@@ -18478,7 +18478,7 @@
       </c>
       <c r="C270" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D270" s="2" t="inlineStr">
@@ -19148,7 +19148,7 @@
       </c>
       <c r="C280" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D280" s="2" t="inlineStr">
@@ -19416,7 +19416,7 @@
       </c>
       <c r="C284" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D284" s="2" t="inlineStr">
@@ -21225,7 +21225,7 @@
       </c>
       <c r="C311" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D311" s="2" t="inlineStr">
@@ -26116,7 +26116,7 @@
       </c>
       <c r="C384" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D384" s="2" t="inlineStr">
@@ -26250,7 +26250,7 @@
       </c>
       <c r="C386" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D386" s="2" t="inlineStr">
@@ -26451,7 +26451,7 @@
       </c>
       <c r="C389" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D389" s="2" t="inlineStr">
@@ -26652,7 +26652,7 @@
       </c>
       <c r="C392" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D392" s="2" t="inlineStr">
@@ -27322,7 +27322,7 @@
       </c>
       <c r="C402" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D402" s="2" t="inlineStr">
@@ -32883,7 +32883,7 @@
       </c>
       <c r="C485" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D485" s="2" t="inlineStr">
@@ -33486,7 +33486,7 @@
       </c>
       <c r="C494" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D494" s="2" t="inlineStr">
@@ -33553,7 +33553,7 @@
       </c>
       <c r="C495" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D495" s="2" t="inlineStr">
@@ -35965,7 +35965,7 @@
       </c>
       <c r="C531" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D531" s="2" t="inlineStr">
@@ -38310,7 +38310,7 @@
       </c>
       <c r="C566" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D566" s="2" t="inlineStr">
@@ -40655,7 +40655,7 @@
       </c>
       <c r="C601" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D601" s="2" t="inlineStr">
@@ -46082,7 +46082,7 @@
       </c>
       <c r="C682" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D682" s="2" t="inlineStr">
@@ -50035,7 +50035,7 @@
       </c>
       <c r="C741" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D741" s="2" t="inlineStr">
@@ -53117,7 +53117,7 @@
       </c>
       <c r="C787" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D787" s="2" t="inlineStr">
@@ -53251,7 +53251,7 @@
       </c>
       <c r="C789" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D789" s="2" t="inlineStr">
@@ -54591,7 +54591,7 @@
       </c>
       <c r="C809" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D809" s="2" t="inlineStr">
@@ -56065,7 +56065,7 @@
       </c>
       <c r="C831" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D831" s="2" t="inlineStr">
@@ -56132,7 +56132,7 @@
       </c>
       <c r="C832" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D832" s="2" t="inlineStr">
@@ -57137,7 +57137,7 @@
       </c>
       <c r="C847" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D847" s="2" t="inlineStr">
@@ -57874,7 +57874,7 @@
       </c>
       <c r="C858" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D858" s="2" t="inlineStr">
@@ -61894,7 +61894,7 @@
       </c>
       <c r="C918" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D918" s="2" t="inlineStr">
@@ -62229,7 +62229,7 @@
       </c>
       <c r="C923" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D923" s="2" t="inlineStr">
@@ -62430,7 +62430,7 @@
       </c>
       <c r="C926" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D926" s="2" t="inlineStr">
@@ -64306,7 +64306,7 @@
       </c>
       <c r="C954" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D954" s="2" t="inlineStr">
@@ -64842,7 +64842,7 @@
       </c>
       <c r="C962" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D962" s="2" t="inlineStr">
@@ -65713,7 +65713,7 @@
       </c>
       <c r="C975" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D975" s="2" t="inlineStr">
@@ -65981,7 +65981,7 @@
       </c>
       <c r="C979" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D979" s="2" t="inlineStr">
@@ -67187,7 +67187,7 @@
       </c>
       <c r="C997" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D997" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-09 10:43:25
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixas_42l.xlsx
+++ b/relatorio_analitico_caixas_42l.xlsx
@@ -991,7 +991,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -4542,7 +4542,7 @@
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
@@ -7021,7 +7021,7 @@
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
@@ -7758,7 +7758,7 @@
       </c>
       <c r="C110" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D110" s="2" t="inlineStr">
@@ -8227,7 +8227,7 @@
       </c>
       <c r="C117" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D117" s="2" t="inlineStr">
@@ -16267,7 +16267,7 @@
       </c>
       <c r="C237" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D237" s="2" t="inlineStr">
@@ -17004,7 +17004,7 @@
       </c>
       <c r="C248" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D248" s="2" t="inlineStr">
@@ -19349,7 +19349,7 @@
       </c>
       <c r="C283" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D283" s="2" t="inlineStr">
@@ -19483,7 +19483,7 @@
       </c>
       <c r="C285" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D285" s="2" t="inlineStr">
@@ -23838,7 +23838,7 @@
       </c>
       <c r="C350" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D350" s="2" t="inlineStr">
@@ -24106,7 +24106,7 @@
       </c>
       <c r="C354" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D354" s="2" t="inlineStr">
@@ -26317,7 +26317,7 @@
       </c>
       <c r="C387" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D387" s="2" t="inlineStr">
@@ -33486,7 +33486,7 @@
       </c>
       <c r="C494" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D494" s="2" t="inlineStr">
@@ -33687,7 +33687,7 @@
       </c>
       <c r="C497" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D497" s="2" t="inlineStr">
@@ -33754,7 +33754,7 @@
       </c>
       <c r="C498" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D498" s="2" t="inlineStr">
@@ -36233,7 +36233,7 @@
       </c>
       <c r="C535" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D535" s="2" t="inlineStr">
@@ -40923,7 +40923,7 @@
       </c>
       <c r="C605" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D605" s="2" t="inlineStr">
@@ -46350,7 +46350,7 @@
       </c>
       <c r="C686" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D686" s="2" t="inlineStr">
@@ -49231,7 +49231,7 @@
       </c>
       <c r="C729" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D729" s="2" t="inlineStr">
@@ -49767,7 +49767,7 @@
       </c>
       <c r="C737" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D737" s="2" t="inlineStr">
@@ -50169,7 +50169,7 @@
       </c>
       <c r="C743" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D743" s="2" t="inlineStr">
@@ -56400,7 +56400,7 @@
       </c>
       <c r="C836" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D836" s="2" t="inlineStr">
@@ -62363,7 +62363,7 @@
       </c>
       <c r="C925" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D925" s="2" t="inlineStr">
@@ -62430,7 +62430,7 @@
       </c>
       <c r="C926" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D926" s="2" t="inlineStr">
@@ -62564,7 +62564,7 @@
       </c>
       <c r="C928" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D928" s="2" t="inlineStr">
@@ -62765,7 +62765,7 @@
       </c>
       <c r="C931" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D931" s="2" t="inlineStr">
@@ -62899,7 +62899,7 @@
       </c>
       <c r="C933" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D933" s="2" t="inlineStr">
@@ -64641,7 +64641,7 @@
       </c>
       <c r="C959" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D959" s="2" t="inlineStr">
@@ -64708,7 +64708,7 @@
       </c>
       <c r="C960" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D960" s="2" t="inlineStr">
@@ -65177,7 +65177,7 @@
       </c>
       <c r="C967" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D967" s="2" t="inlineStr">
@@ -66316,7 +66316,7 @@
       </c>
       <c r="C984" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D984" s="2" t="inlineStr">
@@ -67522,7 +67522,7 @@
       </c>
       <c r="C1002" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D1002" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-09 11:05:09
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixas_42l.xlsx
+++ b/relatorio_analitico_caixas_42l.xlsx
@@ -991,7 +991,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -1929,7 +1929,7 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -7021,7 +7021,7 @@
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
@@ -8227,7 +8227,7 @@
       </c>
       <c r="C117" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D117" s="2" t="inlineStr">
@@ -15798,7 +15798,7 @@
       </c>
       <c r="C230" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D230" s="2" t="inlineStr">
@@ -16334,7 +16334,7 @@
       </c>
       <c r="C238" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D238" s="2" t="inlineStr">
@@ -17004,7 +17004,7 @@
       </c>
       <c r="C248" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D248" s="2" t="inlineStr">
@@ -20957,7 +20957,7 @@
       </c>
       <c r="C307" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D307" s="2" t="inlineStr">
@@ -23838,7 +23838,7 @@
       </c>
       <c r="C350" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D350" s="2" t="inlineStr">
@@ -24106,7 +24106,7 @@
       </c>
       <c r="C354" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D354" s="2" t="inlineStr">
@@ -26317,7 +26317,7 @@
       </c>
       <c r="C387" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D387" s="2" t="inlineStr">
@@ -26853,7 +26853,7 @@
       </c>
       <c r="C395" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D395" s="2" t="inlineStr">
@@ -29466,7 +29466,7 @@
       </c>
       <c r="C434" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D434" s="2" t="inlineStr">
@@ -33486,7 +33486,7 @@
       </c>
       <c r="C494" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D494" s="2" t="inlineStr">
@@ -33754,7 +33754,7 @@
       </c>
       <c r="C498" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D498" s="2" t="inlineStr">
@@ -49164,7 +49164,7 @@
       </c>
       <c r="C728" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D728" s="2" t="inlineStr">
@@ -50169,7 +50169,7 @@
       </c>
       <c r="C743" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D743" s="2" t="inlineStr">
@@ -50303,7 +50303,7 @@
       </c>
       <c r="C745" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D745" s="2" t="inlineStr">
@@ -52313,7 +52313,7 @@
       </c>
       <c r="C775" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D775" s="2" t="inlineStr">
@@ -53653,7 +53653,7 @@
       </c>
       <c r="C795" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D795" s="2" t="inlineStr">
@@ -56467,7 +56467,7 @@
       </c>
       <c r="C837" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D837" s="2" t="inlineStr">
@@ -58209,7 +58209,7 @@
       </c>
       <c r="C863" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D863" s="2" t="inlineStr">
@@ -62363,7 +62363,7 @@
       </c>
       <c r="C925" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D925" s="2" t="inlineStr">
@@ -62899,7 +62899,7 @@
       </c>
       <c r="C933" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D933" s="2" t="inlineStr">
@@ -63234,7 +63234,7 @@
       </c>
       <c r="C938" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D938" s="2" t="inlineStr">
@@ -64708,7 +64708,7 @@
       </c>
       <c r="C960" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D960" s="2" t="inlineStr">
@@ -65311,7 +65311,7 @@
       </c>
       <c r="C969" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D969" s="2" t="inlineStr">
@@ -66048,7 +66048,7 @@
       </c>
       <c r="C980" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D980" s="2" t="inlineStr">
@@ -67522,7 +67522,7 @@
       </c>
       <c r="C1002" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D1002" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-09 11:14:13
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixas_42l.xlsx
+++ b/relatorio_analitico_caixas_42l.xlsx
@@ -991,7 +991,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -1929,7 +1929,7 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -2130,7 +2130,7 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -2197,7 +2197,7 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -7021,7 +7021,7 @@
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
@@ -16066,7 +16066,7 @@
       </c>
       <c r="C234" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D234" s="2" t="inlineStr">
@@ -16267,7 +16267,7 @@
       </c>
       <c r="C237" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D237" s="2" t="inlineStr">
@@ -19349,7 +19349,7 @@
       </c>
       <c r="C283" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D283" s="2" t="inlineStr">
@@ -20957,7 +20957,7 @@
       </c>
       <c r="C307" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D307" s="2" t="inlineStr">
@@ -21426,7 +21426,7 @@
       </c>
       <c r="C314" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D314" s="2" t="inlineStr">
@@ -23838,7 +23838,7 @@
       </c>
       <c r="C350" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D350" s="2" t="inlineStr">
@@ -24106,7 +24106,7 @@
       </c>
       <c r="C354" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D354" s="2" t="inlineStr">
@@ -26451,7 +26451,7 @@
       </c>
       <c r="C389" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D389" s="2" t="inlineStr">
@@ -26585,7 +26585,7 @@
       </c>
       <c r="C391" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D391" s="2" t="inlineStr">
@@ -27523,7 +27523,7 @@
       </c>
       <c r="C405" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D405" s="2" t="inlineStr">
@@ -29466,7 +29466,7 @@
       </c>
       <c r="C434" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D434" s="2" t="inlineStr">
@@ -33084,7 +33084,7 @@
       </c>
       <c r="C488" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D488" s="2" t="inlineStr">
@@ -33151,7 +33151,7 @@
       </c>
       <c r="C489" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D489" s="2" t="inlineStr">
@@ -33687,7 +33687,7 @@
       </c>
       <c r="C497" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D497" s="2" t="inlineStr">
@@ -33754,7 +33754,7 @@
       </c>
       <c r="C498" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D498" s="2" t="inlineStr">
@@ -33821,7 +33821,7 @@
       </c>
       <c r="C499" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D499" s="2" t="inlineStr">
@@ -36233,7 +36233,7 @@
       </c>
       <c r="C535" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D535" s="2" t="inlineStr">
@@ -43737,7 +43737,7 @@
       </c>
       <c r="C647" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D647" s="2" t="inlineStr">
@@ -49231,7 +49231,7 @@
       </c>
       <c r="C729" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D729" s="2" t="inlineStr">
@@ -49767,7 +49767,7 @@
       </c>
       <c r="C737" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D737" s="2" t="inlineStr">
@@ -50169,7 +50169,7 @@
       </c>
       <c r="C743" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D743" s="2" t="inlineStr">
@@ -50370,7 +50370,7 @@
       </c>
       <c r="C746" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D746" s="2" t="inlineStr">
@@ -52313,7 +52313,7 @@
       </c>
       <c r="C775" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D775" s="2" t="inlineStr">
@@ -53452,7 +53452,7 @@
       </c>
       <c r="C792" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D792" s="2" t="inlineStr">
@@ -56534,7 +56534,7 @@
       </c>
       <c r="C838" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D838" s="2" t="inlineStr">
@@ -57472,7 +57472,7 @@
       </c>
       <c r="C852" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D852" s="2" t="inlineStr">
@@ -58008,7 +58008,7 @@
       </c>
       <c r="C860" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D860" s="2" t="inlineStr">
@@ -62363,7 +62363,7 @@
       </c>
       <c r="C925" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D925" s="2" t="inlineStr">
@@ -62564,7 +62564,7 @@
       </c>
       <c r="C928" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D928" s="2" t="inlineStr">
@@ -62765,7 +62765,7 @@
       </c>
       <c r="C931" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D931" s="2" t="inlineStr">
@@ -64708,7 +64708,7 @@
       </c>
       <c r="C960" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D960" s="2" t="inlineStr">
@@ -65177,7 +65177,7 @@
       </c>
       <c r="C967" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D967" s="2" t="inlineStr">
@@ -65244,7 +65244,7 @@
       </c>
       <c r="C968" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D968" s="2" t="inlineStr">
@@ -65311,7 +65311,7 @@
       </c>
       <c r="C969" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D969" s="2" t="inlineStr">
@@ -66048,7 +66048,7 @@
       </c>
       <c r="C980" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D980" s="2" t="inlineStr">
@@ -66316,7 +66316,7 @@
       </c>
       <c r="C984" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D984" s="2" t="inlineStr">
@@ -66785,7 +66785,7 @@
       </c>
       <c r="C991" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D991" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-09 11:34:23
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixas_42l.xlsx
+++ b/relatorio_analitico_caixas_42l.xlsx
@@ -991,7 +991,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -2130,7 +2130,7 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -4542,7 +4542,7 @@
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
@@ -7021,7 +7021,7 @@
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
@@ -16066,7 +16066,7 @@
       </c>
       <c r="C234" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D234" s="2" t="inlineStr">
@@ -17004,7 +17004,7 @@
       </c>
       <c r="C248" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D248" s="2" t="inlineStr">
@@ -18679,7 +18679,7 @@
       </c>
       <c r="C273" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D273" s="2" t="inlineStr">
@@ -19617,7 +19617,7 @@
       </c>
       <c r="C287" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D287" s="2" t="inlineStr">
@@ -20957,7 +20957,7 @@
       </c>
       <c r="C307" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D307" s="2" t="inlineStr">
@@ -23838,7 +23838,7 @@
       </c>
       <c r="C350" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D350" s="2" t="inlineStr">
@@ -24106,7 +24106,7 @@
       </c>
       <c r="C354" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D354" s="2" t="inlineStr">
@@ -26585,7 +26585,7 @@
       </c>
       <c r="C391" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D391" s="2" t="inlineStr">
@@ -26853,7 +26853,7 @@
       </c>
       <c r="C395" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D395" s="2" t="inlineStr">
@@ -27523,7 +27523,7 @@
       </c>
       <c r="C405" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D405" s="2" t="inlineStr">
@@ -29466,7 +29466,7 @@
       </c>
       <c r="C434" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D434" s="2" t="inlineStr">
@@ -33084,7 +33084,7 @@
       </c>
       <c r="C488" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D488" s="2" t="inlineStr">
@@ -49231,7 +49231,7 @@
       </c>
       <c r="C729" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D729" s="2" t="inlineStr">
@@ -50169,7 +50169,7 @@
       </c>
       <c r="C743" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D743" s="2" t="inlineStr">
@@ -50303,7 +50303,7 @@
       </c>
       <c r="C745" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D745" s="2" t="inlineStr">
@@ -53385,7 +53385,7 @@
       </c>
       <c r="C791" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D791" s="2" t="inlineStr">
@@ -53653,7 +53653,7 @@
       </c>
       <c r="C795" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D795" s="2" t="inlineStr">
@@ -54926,7 +54926,7 @@
       </c>
       <c r="C814" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D814" s="2" t="inlineStr">
@@ -58209,7 +58209,7 @@
       </c>
       <c r="C863" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D863" s="2" t="inlineStr">
@@ -62363,7 +62363,7 @@
       </c>
       <c r="C925" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D925" s="2" t="inlineStr">
@@ -62564,7 +62564,7 @@
       </c>
       <c r="C928" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D928" s="2" t="inlineStr">
@@ -62765,7 +62765,7 @@
       </c>
       <c r="C931" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D931" s="2" t="inlineStr">
@@ -63234,7 +63234,7 @@
       </c>
       <c r="C938" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D938" s="2" t="inlineStr">
@@ -64641,7 +64641,7 @@
       </c>
       <c r="C959" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D959" s="2" t="inlineStr">
@@ -64708,7 +64708,7 @@
       </c>
       <c r="C960" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D960" s="2" t="inlineStr">
@@ -65177,7 +65177,7 @@
       </c>
       <c r="C967" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D967" s="2" t="inlineStr">
@@ -66048,7 +66048,7 @@
       </c>
       <c r="C980" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D980" s="2" t="inlineStr">
@@ -66316,7 +66316,7 @@
       </c>
       <c r="C984" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D984" s="2" t="inlineStr">
@@ -67522,7 +67522,7 @@
       </c>
       <c r="C1002" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D1002" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-09 12:06:20
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixas_42l.xlsx
+++ b/relatorio_analitico_caixas_42l.xlsx
@@ -1929,7 +1929,7 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -4542,7 +4542,7 @@
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
@@ -6753,7 +6753,7 @@
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
@@ -7021,7 +7021,7 @@
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
@@ -7758,7 +7758,7 @@
       </c>
       <c r="C110" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D110" s="2" t="inlineStr">
@@ -16267,7 +16267,7 @@
       </c>
       <c r="C237" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D237" s="2" t="inlineStr">
@@ -19617,7 +19617,7 @@
       </c>
       <c r="C287" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D287" s="2" t="inlineStr">
@@ -21426,7 +21426,7 @@
       </c>
       <c r="C314" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D314" s="2" t="inlineStr">
@@ -23838,7 +23838,7 @@
       </c>
       <c r="C350" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D350" s="2" t="inlineStr">
@@ -24106,7 +24106,7 @@
       </c>
       <c r="C354" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D354" s="2" t="inlineStr">
@@ -26317,7 +26317,7 @@
       </c>
       <c r="C387" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D387" s="2" t="inlineStr">
@@ -26451,7 +26451,7 @@
       </c>
       <c r="C389" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D389" s="2" t="inlineStr">
@@ -26652,7 +26652,7 @@
       </c>
       <c r="C392" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="D392" s="2" t="inlineStr">
@@ -26853,7 +26853,7 @@
       </c>
       <c r="C395" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D395" s="2" t="inlineStr">
@@ -33151,7 +33151,7 @@
       </c>
       <c r="C489" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D489" s="2" t="inlineStr">
@@ -33486,7 +33486,7 @@
       </c>
       <c r="C494" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D494" s="2" t="inlineStr">
@@ -33754,7 +33754,7 @@
       </c>
       <c r="C498" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D498" s="2" t="inlineStr">
@@ -33821,7 +33821,7 @@
       </c>
       <c r="C499" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D499" s="2" t="inlineStr">
@@ -36233,7 +36233,7 @@
       </c>
       <c r="C535" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D535" s="2" t="inlineStr">
@@ -38645,7 +38645,7 @@
       </c>
       <c r="C571" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D571" s="2" t="inlineStr">
@@ -40923,7 +40923,7 @@
       </c>
       <c r="C605" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D605" s="2" t="inlineStr">
@@ -46350,7 +46350,7 @@
       </c>
       <c r="C686" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D686" s="2" t="inlineStr">
@@ -49164,7 +49164,7 @@
       </c>
       <c r="C728" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D728" s="2" t="inlineStr">
@@ -49767,7 +49767,7 @@
       </c>
       <c r="C737" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D737" s="2" t="inlineStr">
@@ -50370,7 +50370,7 @@
       </c>
       <c r="C746" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D746" s="2" t="inlineStr">
@@ -53385,7 +53385,7 @@
       </c>
       <c r="C791" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D791" s="2" t="inlineStr">
@@ -53452,7 +53452,7 @@
       </c>
       <c r="C792" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D792" s="2" t="inlineStr">
@@ -53653,7 +53653,7 @@
       </c>
       <c r="C795" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D795" s="2" t="inlineStr">
@@ -56400,7 +56400,7 @@
       </c>
       <c r="C836" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D836" s="2" t="inlineStr">
@@ -56467,7 +56467,7 @@
       </c>
       <c r="C837" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D837" s="2" t="inlineStr">
@@ -57472,7 +57472,7 @@
       </c>
       <c r="C852" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D852" s="2" t="inlineStr">
@@ -62229,7 +62229,7 @@
       </c>
       <c r="C923" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D923" s="2" t="inlineStr">
@@ -62363,7 +62363,7 @@
       </c>
       <c r="C925" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D925" s="2" t="inlineStr">
@@ -62564,7 +62564,7 @@
       </c>
       <c r="C928" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D928" s="2" t="inlineStr">
@@ -64708,7 +64708,7 @@
       </c>
       <c r="C960" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D960" s="2" t="inlineStr">
@@ -65177,7 +65177,7 @@
       </c>
       <c r="C967" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D967" s="2" t="inlineStr">
@@ -66316,7 +66316,7 @@
       </c>
       <c r="C984" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D984" s="2" t="inlineStr">
@@ -66785,7 +66785,7 @@
       </c>
       <c r="C991" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D991" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-09 14:52:57
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixas_42l.xlsx
+++ b/relatorio_analitico_caixas_42l.xlsx
@@ -2130,7 +2130,7 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -7021,7 +7021,7 @@
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
@@ -7758,7 +7758,7 @@
       </c>
       <c r="C110" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D110" s="2" t="inlineStr">
@@ -16334,7 +16334,7 @@
       </c>
       <c r="C238" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D238" s="2" t="inlineStr">
@@ -17004,7 +17004,7 @@
       </c>
       <c r="C248" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D248" s="2" t="inlineStr">
@@ -19349,7 +19349,7 @@
       </c>
       <c r="C283" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D283" s="2" t="inlineStr">
@@ -19617,7 +19617,7 @@
       </c>
       <c r="C287" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D287" s="2" t="inlineStr">
@@ -20957,7 +20957,7 @@
       </c>
       <c r="C307" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D307" s="2" t="inlineStr">
@@ -21292,7 +21292,7 @@
       </c>
       <c r="C312" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D312" s="2" t="inlineStr">
@@ -21426,7 +21426,7 @@
       </c>
       <c r="C314" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D314" s="2" t="inlineStr">
@@ -24106,7 +24106,7 @@
       </c>
       <c r="C354" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D354" s="2" t="inlineStr">
@@ -26585,7 +26585,7 @@
       </c>
       <c r="C391" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D391" s="2" t="inlineStr">
@@ -26853,7 +26853,7 @@
       </c>
       <c r="C395" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D395" s="2" t="inlineStr">
@@ -27523,7 +27523,7 @@
       </c>
       <c r="C405" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D405" s="2" t="inlineStr">
@@ -33084,7 +33084,7 @@
       </c>
       <c r="C488" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D488" s="2" t="inlineStr">
@@ -33151,7 +33151,7 @@
       </c>
       <c r="C489" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D489" s="2" t="inlineStr">
@@ -33486,7 +33486,7 @@
       </c>
       <c r="C494" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D494" s="2" t="inlineStr">
@@ -33754,7 +33754,7 @@
       </c>
       <c r="C498" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D498" s="2" t="inlineStr">
@@ -33821,7 +33821,7 @@
       </c>
       <c r="C499" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D499" s="2" t="inlineStr">
@@ -38578,7 +38578,7 @@
       </c>
       <c r="C570" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D570" s="2" t="inlineStr">
@@ -49767,7 +49767,7 @@
       </c>
       <c r="C737" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D737" s="2" t="inlineStr">
@@ -50169,7 +50169,7 @@
       </c>
       <c r="C743" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D743" s="2" t="inlineStr">
@@ -50303,7 +50303,7 @@
       </c>
       <c r="C745" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D745" s="2" t="inlineStr">
@@ -53452,7 +53452,7 @@
       </c>
       <c r="C792" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D792" s="2" t="inlineStr">
@@ -53586,7 +53586,7 @@
       </c>
       <c r="C794" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D794" s="2" t="inlineStr">
@@ -53653,7 +53653,7 @@
       </c>
       <c r="C795" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D795" s="2" t="inlineStr">
@@ -56400,7 +56400,7 @@
       </c>
       <c r="C836" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D836" s="2" t="inlineStr">
@@ -56534,7 +56534,7 @@
       </c>
       <c r="C838" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D838" s="2" t="inlineStr">
@@ -57472,7 +57472,7 @@
       </c>
       <c r="C852" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D852" s="2" t="inlineStr">
@@ -62229,7 +62229,7 @@
       </c>
       <c r="C923" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D923" s="2" t="inlineStr">
@@ -62363,7 +62363,7 @@
       </c>
       <c r="C925" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D925" s="2" t="inlineStr">
@@ -62899,7 +62899,7 @@
       </c>
       <c r="C933" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D933" s="2" t="inlineStr">
@@ -64708,7 +64708,7 @@
       </c>
       <c r="C960" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D960" s="2" t="inlineStr">
@@ -65177,7 +65177,7 @@
       </c>
       <c r="C967" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D967" s="2" t="inlineStr">
@@ -65244,7 +65244,7 @@
       </c>
       <c r="C968" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D968" s="2" t="inlineStr">
@@ -66048,7 +66048,7 @@
       </c>
       <c r="C980" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D980" s="2" t="inlineStr">
@@ -66316,7 +66316,7 @@
       </c>
       <c r="C984" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D984" s="2" t="inlineStr">
@@ -66785,7 +66785,7 @@
       </c>
       <c r="C991" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D991" s="2" t="inlineStr">
@@ -67522,7 +67522,7 @@
       </c>
       <c r="C1002" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D1002" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-09 15:03:23
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixas_42l.xlsx
+++ b/relatorio_analitico_caixas_42l.xlsx
@@ -991,7 +991,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -1929,7 +1929,7 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -2197,7 +2197,7 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -4542,7 +4542,7 @@
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
@@ -6753,7 +6753,7 @@
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
@@ -7758,7 +7758,7 @@
       </c>
       <c r="C110" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D110" s="2" t="inlineStr">
@@ -15798,7 +15798,7 @@
       </c>
       <c r="C230" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D230" s="2" t="inlineStr">
@@ -16066,7 +16066,7 @@
       </c>
       <c r="C234" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D234" s="2" t="inlineStr">
@@ -16267,7 +16267,7 @@
       </c>
       <c r="C237" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D237" s="2" t="inlineStr">
@@ -16334,7 +16334,7 @@
       </c>
       <c r="C238" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D238" s="2" t="inlineStr">
@@ -17004,7 +17004,7 @@
       </c>
       <c r="C248" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D248" s="2" t="inlineStr">
@@ -18679,7 +18679,7 @@
       </c>
       <c r="C273" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D273" s="2" t="inlineStr">
@@ -19349,7 +19349,7 @@
       </c>
       <c r="C283" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D283" s="2" t="inlineStr">
@@ -19617,7 +19617,7 @@
       </c>
       <c r="C287" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D287" s="2" t="inlineStr">
@@ -20957,7 +20957,7 @@
       </c>
       <c r="C307" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D307" s="2" t="inlineStr">
@@ -21426,7 +21426,7 @@
       </c>
       <c r="C314" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D314" s="2" t="inlineStr">
@@ -24106,7 +24106,7 @@
       </c>
       <c r="C354" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D354" s="2" t="inlineStr">
@@ -26652,7 +26652,7 @@
       </c>
       <c r="C392" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="D392" s="2" t="inlineStr">
@@ -26786,7 +26786,7 @@
       </c>
       <c r="C394" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D394" s="2" t="inlineStr">
@@ -26853,7 +26853,7 @@
       </c>
       <c r="C395" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D395" s="2" t="inlineStr">
@@ -33084,7 +33084,7 @@
       </c>
       <c r="C488" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D488" s="2" t="inlineStr">
@@ -33151,7 +33151,7 @@
       </c>
       <c r="C489" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D489" s="2" t="inlineStr">
@@ -33687,7 +33687,7 @@
       </c>
       <c r="C497" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D497" s="2" t="inlineStr">
@@ -33754,7 +33754,7 @@
       </c>
       <c r="C498" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D498" s="2" t="inlineStr">
@@ -33821,7 +33821,7 @@
       </c>
       <c r="C499" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D499" s="2" t="inlineStr">
@@ -38578,7 +38578,7 @@
       </c>
       <c r="C570" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D570" s="2" t="inlineStr">
@@ -49164,7 +49164,7 @@
       </c>
       <c r="C728" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D728" s="2" t="inlineStr">
@@ -49231,7 +49231,7 @@
       </c>
       <c r="C729" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D729" s="2" t="inlineStr">
@@ -49767,7 +49767,7 @@
       </c>
       <c r="C737" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D737" s="2" t="inlineStr">
@@ -53385,7 +53385,7 @@
       </c>
       <c r="C791" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D791" s="2" t="inlineStr">
@@ -53653,7 +53653,7 @@
       </c>
       <c r="C795" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D795" s="2" t="inlineStr">
@@ -54926,7 +54926,7 @@
       </c>
       <c r="C814" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D814" s="2" t="inlineStr">
@@ -56400,7 +56400,7 @@
       </c>
       <c r="C836" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D836" s="2" t="inlineStr">
@@ -57472,7 +57472,7 @@
       </c>
       <c r="C852" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D852" s="2" t="inlineStr">
@@ -58209,7 +58209,7 @@
       </c>
       <c r="C863" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D863" s="2" t="inlineStr">
@@ -62229,7 +62229,7 @@
       </c>
       <c r="C923" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D923" s="2" t="inlineStr">
@@ -62363,7 +62363,7 @@
       </c>
       <c r="C925" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D925" s="2" t="inlineStr">
@@ -62430,7 +62430,7 @@
       </c>
       <c r="C926" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D926" s="2" t="inlineStr">
@@ -66048,7 +66048,7 @@
       </c>
       <c r="C980" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D980" s="2" t="inlineStr">
@@ -66785,7 +66785,7 @@
       </c>
       <c r="C991" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D991" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-09 18:02:05
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixas_42l.xlsx
+++ b/relatorio_analitico_caixas_42l.xlsx
@@ -1929,7 +1929,7 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -2130,7 +2130,7 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -4542,7 +4542,7 @@
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
@@ -8227,7 +8227,7 @@
       </c>
       <c r="C117" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D117" s="2" t="inlineStr">
@@ -16066,7 +16066,7 @@
       </c>
       <c r="C234" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D234" s="2" t="inlineStr">
@@ -17004,7 +17004,7 @@
       </c>
       <c r="C248" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D248" s="2" t="inlineStr">
@@ -19349,7 +19349,7 @@
       </c>
       <c r="C283" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D283" s="2" t="inlineStr">
@@ -20019,7 +20019,7 @@
       </c>
       <c r="C293" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D293" s="2" t="inlineStr">
@@ -20287,7 +20287,7 @@
       </c>
       <c r="C297" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D297" s="2" t="inlineStr">
@@ -22096,7 +22096,7 @@
       </c>
       <c r="C324" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D324" s="2" t="inlineStr">
@@ -24508,7 +24508,7 @@
       </c>
       <c r="C360" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D360" s="2" t="inlineStr">
@@ -24776,7 +24776,7 @@
       </c>
       <c r="C364" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D364" s="2" t="inlineStr">
@@ -27255,7 +27255,7 @@
       </c>
       <c r="C401" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D401" s="2" t="inlineStr">
@@ -28193,7 +28193,7 @@
       </c>
       <c r="C415" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D415" s="2" t="inlineStr">
@@ -33754,7 +33754,7 @@
       </c>
       <c r="C498" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D498" s="2" t="inlineStr">
@@ -33821,7 +33821,7 @@
       </c>
       <c r="C499" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D499" s="2" t="inlineStr">
@@ -34290,7 +34290,7 @@
       </c>
       <c r="C506" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D506" s="2" t="inlineStr">
@@ -34491,7 +34491,7 @@
       </c>
       <c r="C509" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D509" s="2" t="inlineStr">
@@ -39315,7 +39315,7 @@
       </c>
       <c r="C581" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D581" s="2" t="inlineStr">
@@ -41593,7 +41593,7 @@
       </c>
       <c r="C615" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D615" s="2" t="inlineStr">
@@ -50102,7 +50102,7 @@
       </c>
       <c r="C742" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D742" s="2" t="inlineStr">
@@ -50638,7 +50638,7 @@
       </c>
       <c r="C750" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D750" s="2" t="inlineStr">
@@ -51174,7 +51174,7 @@
       </c>
       <c r="C758" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D758" s="2" t="inlineStr">
@@ -53184,7 +53184,7 @@
       </c>
       <c r="C788" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D788" s="2" t="inlineStr">
@@ -54256,7 +54256,7 @@
       </c>
       <c r="C804" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D804" s="2" t="inlineStr">
@@ -54323,7 +54323,7 @@
       </c>
       <c r="C805" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D805" s="2" t="inlineStr">
@@ -54390,7 +54390,7 @@
       </c>
       <c r="C806" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D806" s="2" t="inlineStr">
@@ -54524,7 +54524,7 @@
       </c>
       <c r="C808" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D808" s="2" t="inlineStr">
@@ -58879,7 +58879,7 @@
       </c>
       <c r="C873" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D873" s="2" t="inlineStr">
@@ -59080,7 +59080,7 @@
       </c>
       <c r="C876" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D876" s="2" t="inlineStr">
@@ -63100,7 +63100,7 @@
       </c>
       <c r="C936" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D936" s="2" t="inlineStr">
@@ -63234,7 +63234,7 @@
       </c>
       <c r="C938" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D938" s="2" t="inlineStr">
@@ -63770,7 +63770,7 @@
       </c>
       <c r="C946" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D946" s="2" t="inlineStr">
@@ -63904,7 +63904,7 @@
       </c>
       <c r="C948" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D948" s="2" t="inlineStr">
@@ -66182,7 +66182,7 @@
       </c>
       <c r="C982" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D982" s="2" t="inlineStr">
@@ -66919,7 +66919,7 @@
       </c>
       <c r="C993" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D993" s="2" t="inlineStr">
@@ -67656,7 +67656,7 @@
       </c>
       <c r="C1004" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D1004" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-09 18:11:11
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixas_42l.xlsx
+++ b/relatorio_analitico_caixas_42l.xlsx
@@ -4542,7 +4542,7 @@
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
@@ -7021,7 +7021,7 @@
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
@@ -7758,7 +7758,7 @@
       </c>
       <c r="C110" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D110" s="2" t="inlineStr">
@@ -17004,7 +17004,7 @@
       </c>
       <c r="C248" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D248" s="2" t="inlineStr">
@@ -20287,7 +20287,7 @@
       </c>
       <c r="C297" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D297" s="2" t="inlineStr">
@@ -27121,7 +27121,7 @@
       </c>
       <c r="C399" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D399" s="2" t="inlineStr">
@@ -27255,7 +27255,7 @@
       </c>
       <c r="C401" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D401" s="2" t="inlineStr">
@@ -27523,7 +27523,7 @@
       </c>
       <c r="C405" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D405" s="2" t="inlineStr">
@@ -28193,7 +28193,7 @@
       </c>
       <c r="C415" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D415" s="2" t="inlineStr">
@@ -30136,7 +30136,7 @@
       </c>
       <c r="C444" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D444" s="2" t="inlineStr">
@@ -33754,7 +33754,7 @@
       </c>
       <c r="C498" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D498" s="2" t="inlineStr">
@@ -34290,7 +34290,7 @@
       </c>
       <c r="C506" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D506" s="2" t="inlineStr">
@@ -34424,7 +34424,7 @@
       </c>
       <c r="C508" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D508" s="2" t="inlineStr">
@@ -34491,7 +34491,7 @@
       </c>
       <c r="C509" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D509" s="2" t="inlineStr">
@@ -36903,7 +36903,7 @@
       </c>
       <c r="C545" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D545" s="2" t="inlineStr">
@@ -39248,7 +39248,7 @@
       </c>
       <c r="C580" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D580" s="2" t="inlineStr">
@@ -41593,7 +41593,7 @@
       </c>
       <c r="C615" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D615" s="2" t="inlineStr">
@@ -47020,7 +47020,7 @@
       </c>
       <c r="C696" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D696" s="2" t="inlineStr">
@@ -50035,7 +50035,7 @@
       </c>
       <c r="C741" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D741" s="2" t="inlineStr">
@@ -51040,7 +51040,7 @@
       </c>
       <c r="C756" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D756" s="2" t="inlineStr">
@@ -53184,7 +53184,7 @@
       </c>
       <c r="C788" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D788" s="2" t="inlineStr">
@@ -58343,7 +58343,7 @@
       </c>
       <c r="C865" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D865" s="2" t="inlineStr">
@@ -63234,7 +63234,7 @@
       </c>
       <c r="C938" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D938" s="2" t="inlineStr">
@@ -63435,7 +63435,7 @@
       </c>
       <c r="C941" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D941" s="2" t="inlineStr">
@@ -65579,7 +65579,7 @@
       </c>
       <c r="C973" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D973" s="2" t="inlineStr">
@@ -66048,7 +66048,7 @@
       </c>
       <c r="C980" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D980" s="2" t="inlineStr">
@@ -66182,7 +66182,7 @@
       </c>
       <c r="C982" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D982" s="2" t="inlineStr">
@@ -67187,7 +67187,7 @@
       </c>
       <c r="C997" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D997" s="2" t="inlineStr">
@@ -67656,7 +67656,7 @@
       </c>
       <c r="C1004" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D1004" s="2" t="inlineStr">
@@ -68393,7 +68393,7 @@
       </c>
       <c r="C1015" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D1015" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-09 19:11:17
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixas_42l.xlsx
+++ b/relatorio_analitico_caixas_42l.xlsx
@@ -991,7 +991,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -2197,7 +2197,7 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -4542,7 +4542,7 @@
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
@@ -15798,7 +15798,7 @@
       </c>
       <c r="C230" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D230" s="2" t="inlineStr">
@@ -16066,7 +16066,7 @@
       </c>
       <c r="C234" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D234" s="2" t="inlineStr">
@@ -16937,7 +16937,7 @@
       </c>
       <c r="C247" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D247" s="2" t="inlineStr">
@@ -17004,7 +17004,7 @@
       </c>
       <c r="C248" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D248" s="2" t="inlineStr">
@@ -17674,7 +17674,7 @@
       </c>
       <c r="C258" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D258" s="2" t="inlineStr">
@@ -19349,7 +19349,7 @@
       </c>
       <c r="C283" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D283" s="2" t="inlineStr">
@@ -21627,7 +21627,7 @@
       </c>
       <c r="C317" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D317" s="2" t="inlineStr">
@@ -21962,7 +21962,7 @@
       </c>
       <c r="C322" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D322" s="2" t="inlineStr">
@@ -22096,7 +22096,7 @@
       </c>
       <c r="C324" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D324" s="2" t="inlineStr">
@@ -24776,7 +24776,7 @@
       </c>
       <c r="C364" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D364" s="2" t="inlineStr">
@@ -27322,7 +27322,7 @@
       </c>
       <c r="C402" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="D402" s="2" t="inlineStr">
@@ -27523,7 +27523,7 @@
       </c>
       <c r="C405" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D405" s="2" t="inlineStr">
@@ -28193,7 +28193,7 @@
       </c>
       <c r="C415" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D415" s="2" t="inlineStr">
@@ -30136,7 +30136,7 @@
       </c>
       <c r="C444" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D444" s="2" t="inlineStr">
@@ -33754,7 +33754,7 @@
       </c>
       <c r="C498" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D498" s="2" t="inlineStr">
@@ -33821,7 +33821,7 @@
       </c>
       <c r="C499" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D499" s="2" t="inlineStr">
@@ -34156,7 +34156,7 @@
       </c>
       <c r="C504" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D504" s="2" t="inlineStr">
@@ -34290,7 +34290,7 @@
       </c>
       <c r="C506" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D506" s="2" t="inlineStr">
@@ -34424,7 +34424,7 @@
       </c>
       <c r="C508" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D508" s="2" t="inlineStr">
@@ -36903,7 +36903,7 @@
       </c>
       <c r="C545" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D545" s="2" t="inlineStr">
@@ -39248,7 +39248,7 @@
       </c>
       <c r="C580" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D580" s="2" t="inlineStr">
@@ -39315,7 +39315,7 @@
       </c>
       <c r="C581" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D581" s="2" t="inlineStr">
@@ -44407,7 +44407,7 @@
       </c>
       <c r="C657" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D657" s="2" t="inlineStr">
@@ -50035,7 +50035,7 @@
       </c>
       <c r="C741" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D741" s="2" t="inlineStr">
@@ -54323,7 +54323,7 @@
       </c>
       <c r="C805" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D805" s="2" t="inlineStr">
@@ -54524,7 +54524,7 @@
       </c>
       <c r="C808" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D808" s="2" t="inlineStr">
@@ -57405,7 +57405,7 @@
       </c>
       <c r="C851" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D851" s="2" t="inlineStr">
@@ -58879,7 +58879,7 @@
       </c>
       <c r="C873" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D873" s="2" t="inlineStr">
@@ -59080,7 +59080,7 @@
       </c>
       <c r="C876" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D876" s="2" t="inlineStr">
@@ -63100,7 +63100,7 @@
       </c>
       <c r="C936" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D936" s="2" t="inlineStr">
@@ -63301,7 +63301,7 @@
       </c>
       <c r="C939" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D939" s="2" t="inlineStr">
@@ -63904,7 +63904,7 @@
       </c>
       <c r="C948" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D948" s="2" t="inlineStr">
@@ -64105,7 +64105,7 @@
       </c>
       <c r="C951" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D951" s="2" t="inlineStr">
@@ -65512,7 +65512,7 @@
       </c>
       <c r="C972" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D972" s="2" t="inlineStr">
@@ -66048,7 +66048,7 @@
       </c>
       <c r="C980" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D980" s="2" t="inlineStr">
@@ -66115,7 +66115,7 @@
       </c>
       <c r="C981" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D981" s="2" t="inlineStr">
@@ -66182,7 +66182,7 @@
       </c>
       <c r="C982" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D982" s="2" t="inlineStr">
@@ -67656,7 +67656,7 @@
       </c>
       <c r="C1004" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D1004" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-09 20:54:29
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixas_42l.xlsx
+++ b/relatorio_analitico_caixas_42l.xlsx
@@ -991,7 +991,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -7021,7 +7021,7 @@
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
@@ -8227,7 +8227,7 @@
       </c>
       <c r="C117" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D117" s="2" t="inlineStr">
@@ -16066,7 +16066,7 @@
       </c>
       <c r="C234" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D234" s="2" t="inlineStr">
@@ -24776,7 +24776,7 @@
       </c>
       <c r="C364" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D364" s="2" t="inlineStr">
@@ -26987,7 +26987,7 @@
       </c>
       <c r="C397" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D397" s="2" t="inlineStr">
@@ -27255,7 +27255,7 @@
       </c>
       <c r="C401" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D401" s="2" t="inlineStr">
@@ -27322,7 +27322,7 @@
       </c>
       <c r="C402" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D402" s="2" t="inlineStr">
@@ -27456,7 +27456,7 @@
       </c>
       <c r="C404" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D404" s="2" t="inlineStr">
@@ -27523,7 +27523,7 @@
       </c>
       <c r="C405" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D405" s="2" t="inlineStr">
@@ -28193,7 +28193,7 @@
       </c>
       <c r="C415" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D415" s="2" t="inlineStr">
@@ -30136,7 +30136,7 @@
       </c>
       <c r="C444" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D444" s="2" t="inlineStr">
@@ -33754,7 +33754,7 @@
       </c>
       <c r="C498" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D498" s="2" t="inlineStr">
@@ -34290,7 +34290,7 @@
       </c>
       <c r="C506" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D506" s="2" t="inlineStr">
@@ -34357,7 +34357,7 @@
       </c>
       <c r="C507" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D507" s="2" t="inlineStr">
@@ -34491,7 +34491,7 @@
       </c>
       <c r="C509" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D509" s="2" t="inlineStr">
@@ -39248,7 +39248,7 @@
       </c>
       <c r="C580" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D580" s="2" t="inlineStr">
@@ -44407,7 +44407,7 @@
       </c>
       <c r="C657" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D657" s="2" t="inlineStr">
@@ -47020,7 +47020,7 @@
       </c>
       <c r="C696" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D696" s="2" t="inlineStr">
@@ -50035,7 +50035,7 @@
       </c>
       <c r="C741" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D741" s="2" t="inlineStr">
@@ -50102,7 +50102,7 @@
       </c>
       <c r="C742" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D742" s="2" t="inlineStr">
@@ -54256,7 +54256,7 @@
       </c>
       <c r="C804" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D804" s="2" t="inlineStr">
@@ -54323,7 +54323,7 @@
       </c>
       <c r="C805" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D805" s="2" t="inlineStr">
@@ -55797,7 +55797,7 @@
       </c>
       <c r="C827" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D827" s="2" t="inlineStr">
@@ -57405,7 +57405,7 @@
       </c>
       <c r="C851" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D851" s="2" t="inlineStr">
@@ -57472,7 +57472,7 @@
       </c>
       <c r="C852" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D852" s="2" t="inlineStr">
@@ -59080,7 +59080,7 @@
       </c>
       <c r="C876" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D876" s="2" t="inlineStr">
@@ -63100,7 +63100,7 @@
       </c>
       <c r="C936" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D936" s="2" t="inlineStr">
@@ -63770,7 +63770,7 @@
       </c>
       <c r="C946" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D946" s="2" t="inlineStr">
@@ -65512,7 +65512,7 @@
       </c>
       <c r="C972" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D972" s="2" t="inlineStr">
@@ -65579,7 +65579,7 @@
       </c>
       <c r="C973" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D973" s="2" t="inlineStr">
@@ -66115,7 +66115,7 @@
       </c>
       <c r="C981" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D981" s="2" t="inlineStr">
@@ -66182,7 +66182,7 @@
       </c>
       <c r="C982" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D982" s="2" t="inlineStr">
@@ -67656,7 +67656,7 @@
       </c>
       <c r="C1004" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D1004" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-09 21:06:28
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixas_42l.xlsx
+++ b/relatorio_analitico_caixas_42l.xlsx
@@ -991,7 +991,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -2130,7 +2130,7 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -16066,7 +16066,7 @@
       </c>
       <c r="C234" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D234" s="2" t="inlineStr">
@@ -20019,7 +20019,7 @@
       </c>
       <c r="C293" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D293" s="2" t="inlineStr">
@@ -21962,7 +21962,7 @@
       </c>
       <c r="C322" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D322" s="2" t="inlineStr">
@@ -24776,7 +24776,7 @@
       </c>
       <c r="C364" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D364" s="2" t="inlineStr">
@@ -27121,7 +27121,7 @@
       </c>
       <c r="C399" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D399" s="2" t="inlineStr">
@@ -27322,7 +27322,7 @@
       </c>
       <c r="C402" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="D402" s="2" t="inlineStr">
@@ -27523,7 +27523,7 @@
       </c>
       <c r="C405" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D405" s="2" t="inlineStr">
@@ -28193,7 +28193,7 @@
       </c>
       <c r="C415" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D415" s="2" t="inlineStr">
@@ -30136,7 +30136,7 @@
       </c>
       <c r="C444" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D444" s="2" t="inlineStr">
@@ -34290,7 +34290,7 @@
       </c>
       <c r="C506" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D506" s="2" t="inlineStr">
@@ -34357,7 +34357,7 @@
       </c>
       <c r="C507" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D507" s="2" t="inlineStr">
@@ -34491,7 +34491,7 @@
       </c>
       <c r="C509" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D509" s="2" t="inlineStr">
@@ -36903,7 +36903,7 @@
       </c>
       <c r="C545" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D545" s="2" t="inlineStr">
@@ -39248,7 +39248,7 @@
       </c>
       <c r="C580" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D580" s="2" t="inlineStr">
@@ -41593,7 +41593,7 @@
       </c>
       <c r="C615" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D615" s="2" t="inlineStr">
@@ -44407,7 +44407,7 @@
       </c>
       <c r="C657" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D657" s="2" t="inlineStr">
@@ -50638,7 +50638,7 @@
       </c>
       <c r="C750" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D750" s="2" t="inlineStr">
@@ -51040,7 +51040,7 @@
       </c>
       <c r="C756" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D756" s="2" t="inlineStr">
@@ -51174,7 +51174,7 @@
       </c>
       <c r="C758" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D758" s="2" t="inlineStr">
@@ -53184,7 +53184,7 @@
       </c>
       <c r="C788" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D788" s="2" t="inlineStr">
@@ -54323,7 +54323,7 @@
       </c>
       <c r="C805" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D805" s="2" t="inlineStr">
@@ -54390,7 +54390,7 @@
       </c>
       <c r="C806" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D806" s="2" t="inlineStr">
@@ -54524,7 +54524,7 @@
       </c>
       <c r="C808" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D808" s="2" t="inlineStr">
@@ -57271,7 +57271,7 @@
       </c>
       <c r="C849" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D849" s="2" t="inlineStr">
@@ -58343,7 +58343,7 @@
       </c>
       <c r="C865" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D865" s="2" t="inlineStr">
@@ -63100,7 +63100,7 @@
       </c>
       <c r="C936" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D936" s="2" t="inlineStr">
@@ -63301,7 +63301,7 @@
       </c>
       <c r="C939" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D939" s="2" t="inlineStr">
@@ -63770,7 +63770,7 @@
       </c>
       <c r="C946" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D946" s="2" t="inlineStr">
@@ -65512,7 +65512,7 @@
       </c>
       <c r="C972" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D972" s="2" t="inlineStr">
@@ -65579,7 +65579,7 @@
       </c>
       <c r="C973" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D973" s="2" t="inlineStr">
@@ -66048,7 +66048,7 @@
       </c>
       <c r="C980" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D980" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-09 21:25:39
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixas_42l.xlsx
+++ b/relatorio_analitico_caixas_42l.xlsx
@@ -991,7 +991,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -2130,7 +2130,7 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -2197,7 +2197,7 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -6753,7 +6753,7 @@
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
@@ -7021,7 +7021,7 @@
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
@@ -8227,7 +8227,7 @@
       </c>
       <c r="C117" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D117" s="2" t="inlineStr">
@@ -16066,7 +16066,7 @@
       </c>
       <c r="C234" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D234" s="2" t="inlineStr">
@@ -16937,7 +16937,7 @@
       </c>
       <c r="C247" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D247" s="2" t="inlineStr">
@@ -17674,7 +17674,7 @@
       </c>
       <c r="C258" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D258" s="2" t="inlineStr">
@@ -19349,7 +19349,7 @@
       </c>
       <c r="C283" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D283" s="2" t="inlineStr">
@@ -20019,7 +20019,7 @@
       </c>
       <c r="C293" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D293" s="2" t="inlineStr">
@@ -20153,7 +20153,7 @@
       </c>
       <c r="C295" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D295" s="2" t="inlineStr">
@@ -22096,7 +22096,7 @@
       </c>
       <c r="C324" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D324" s="2" t="inlineStr">
@@ -24776,7 +24776,7 @@
       </c>
       <c r="C364" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D364" s="2" t="inlineStr">
@@ -27121,7 +27121,7 @@
       </c>
       <c r="C399" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D399" s="2" t="inlineStr">
@@ -27322,7 +27322,7 @@
       </c>
       <c r="C402" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>2 C a 8 C</t>
         </is>
       </c>
       <c r="D402" s="2" t="inlineStr">
@@ -27523,7 +27523,7 @@
       </c>
       <c r="C405" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D405" s="2" t="inlineStr">
@@ -28193,7 +28193,7 @@
       </c>
       <c r="C415" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D415" s="2" t="inlineStr">
@@ -34290,7 +34290,7 @@
       </c>
       <c r="C506" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D506" s="2" t="inlineStr">
@@ -34491,7 +34491,7 @@
       </c>
       <c r="C509" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D509" s="2" t="inlineStr">
@@ -39248,7 +39248,7 @@
       </c>
       <c r="C580" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D580" s="2" t="inlineStr">
@@ -39315,7 +39315,7 @@
       </c>
       <c r="C581" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D581" s="2" t="inlineStr">
@@ -41593,7 +41593,7 @@
       </c>
       <c r="C615" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D615" s="2" t="inlineStr">
@@ -47020,7 +47020,7 @@
       </c>
       <c r="C696" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D696" s="2" t="inlineStr">
@@ -50035,7 +50035,7 @@
       </c>
       <c r="C741" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D741" s="2" t="inlineStr">
@@ -50638,7 +50638,7 @@
       </c>
       <c r="C750" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D750" s="2" t="inlineStr">
@@ -51040,7 +51040,7 @@
       </c>
       <c r="C756" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D756" s="2" t="inlineStr">
@@ -51174,7 +51174,7 @@
       </c>
       <c r="C758" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D758" s="2" t="inlineStr">
@@ -51241,7 +51241,7 @@
       </c>
       <c r="C759" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D759" s="2" t="inlineStr">
@@ -53184,7 +53184,7 @@
       </c>
       <c r="C788" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D788" s="2" t="inlineStr">
@@ -54256,7 +54256,7 @@
       </c>
       <c r="C804" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D804" s="2" t="inlineStr">
@@ -54323,7 +54323,7 @@
       </c>
       <c r="C805" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D805" s="2" t="inlineStr">
@@ -55797,7 +55797,7 @@
       </c>
       <c r="C827" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D827" s="2" t="inlineStr">
@@ -57472,7 +57472,7 @@
       </c>
       <c r="C852" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D852" s="2" t="inlineStr">
@@ -58879,7 +58879,7 @@
       </c>
       <c r="C873" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D873" s="2" t="inlineStr">
@@ -59080,7 +59080,7 @@
       </c>
       <c r="C876" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D876" s="2" t="inlineStr">
@@ -63301,7 +63301,7 @@
       </c>
       <c r="C939" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D939" s="2" t="inlineStr">
@@ -63904,7 +63904,7 @@
       </c>
       <c r="C948" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D948" s="2" t="inlineStr">
@@ -66182,7 +66182,7 @@
       </c>
       <c r="C982" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D982" s="2" t="inlineStr">
@@ -66919,7 +66919,7 @@
       </c>
       <c r="C993" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D993" s="2" t="inlineStr">
@@ -67187,7 +67187,7 @@
       </c>
       <c r="C997" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D997" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-09 21:36:25
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixas_42l.xlsx
+++ b/relatorio_analitico_caixas_42l.xlsx
@@ -991,7 +991,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -1929,7 +1929,7 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -4542,7 +4542,7 @@
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
@@ -6753,7 +6753,7 @@
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
@@ -15798,7 +15798,7 @@
       </c>
       <c r="C230" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D230" s="2" t="inlineStr">
@@ -16066,7 +16066,7 @@
       </c>
       <c r="C234" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D234" s="2" t="inlineStr">
@@ -17004,7 +17004,7 @@
       </c>
       <c r="C248" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D248" s="2" t="inlineStr">
@@ -18210,7 +18210,7 @@
       </c>
       <c r="C266" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D266" s="2" t="inlineStr">
@@ -20019,7 +20019,7 @@
       </c>
       <c r="C293" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D293" s="2" t="inlineStr">
@@ -20153,7 +20153,7 @@
       </c>
       <c r="C295" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D295" s="2" t="inlineStr">
@@ -20287,7 +20287,7 @@
       </c>
       <c r="C297" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D297" s="2" t="inlineStr">
@@ -22096,7 +22096,7 @@
       </c>
       <c r="C324" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D324" s="2" t="inlineStr">
@@ -24776,7 +24776,7 @@
       </c>
       <c r="C364" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D364" s="2" t="inlineStr">
@@ -27121,7 +27121,7 @@
       </c>
       <c r="C399" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D399" s="2" t="inlineStr">
@@ -27322,7 +27322,7 @@
       </c>
       <c r="C402" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D402" s="2" t="inlineStr">
@@ -27523,7 +27523,7 @@
       </c>
       <c r="C405" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D405" s="2" t="inlineStr">
@@ -33821,7 +33821,7 @@
       </c>
       <c r="C499" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D499" s="2" t="inlineStr">
@@ -34290,7 +34290,7 @@
       </c>
       <c r="C506" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D506" s="2" t="inlineStr">
@@ -41593,7 +41593,7 @@
       </c>
       <c r="C615" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D615" s="2" t="inlineStr">
@@ -50102,7 +50102,7 @@
       </c>
       <c r="C742" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D742" s="2" t="inlineStr">
@@ -51040,7 +51040,7 @@
       </c>
       <c r="C756" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D756" s="2" t="inlineStr">
@@ -51174,7 +51174,7 @@
       </c>
       <c r="C758" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D758" s="2" t="inlineStr">
@@ -54256,7 +54256,7 @@
       </c>
       <c r="C804" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D804" s="2" t="inlineStr">
@@ -54323,7 +54323,7 @@
       </c>
       <c r="C805" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D805" s="2" t="inlineStr">
@@ -54390,7 +54390,7 @@
       </c>
       <c r="C806" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D806" s="2" t="inlineStr">
@@ -57405,7 +57405,7 @@
       </c>
       <c r="C851" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D851" s="2" t="inlineStr">
@@ -63100,7 +63100,7 @@
       </c>
       <c r="C936" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D936" s="2" t="inlineStr">
@@ -63234,7 +63234,7 @@
       </c>
       <c r="C938" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D938" s="2" t="inlineStr">
@@ -63770,7 +63770,7 @@
       </c>
       <c r="C946" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D946" s="2" t="inlineStr">
@@ -63904,7 +63904,7 @@
       </c>
       <c r="C948" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D948" s="2" t="inlineStr">
@@ -64105,7 +64105,7 @@
       </c>
       <c r="C951" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D951" s="2" t="inlineStr">
@@ -65579,7 +65579,7 @@
       </c>
       <c r="C973" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D973" s="2" t="inlineStr">
@@ -66048,7 +66048,7 @@
       </c>
       <c r="C980" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D980" s="2" t="inlineStr">
@@ -66919,7 +66919,7 @@
       </c>
       <c r="C993" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D993" s="2" t="inlineStr">
@@ -67187,7 +67187,7 @@
       </c>
       <c r="C997" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D997" s="2" t="inlineStr">
@@ -67656,7 +67656,7 @@
       </c>
       <c r="C1004" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D1004" s="2" t="inlineStr">
@@ -68393,7 +68393,7 @@
       </c>
       <c r="C1015" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D1015" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-09 22:25:27
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixas_42l.xlsx
+++ b/relatorio_analitico_caixas_42l.xlsx
@@ -991,7 +991,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -1929,7 +1929,7 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -2197,7 +2197,7 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -4542,7 +4542,7 @@
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
@@ -6753,7 +6753,7 @@
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
@@ -8227,7 +8227,7 @@
       </c>
       <c r="C117" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D117" s="2" t="inlineStr">
@@ -15798,7 +15798,7 @@
       </c>
       <c r="C230" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D230" s="2" t="inlineStr">
@@ -17674,7 +17674,7 @@
       </c>
       <c r="C258" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D258" s="2" t="inlineStr">
@@ -20019,7 +20019,7 @@
       </c>
       <c r="C293" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D293" s="2" t="inlineStr">
@@ -20153,7 +20153,7 @@
       </c>
       <c r="C295" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D295" s="2" t="inlineStr">
@@ -21962,7 +21962,7 @@
       </c>
       <c r="C322" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D322" s="2" t="inlineStr">
@@ -24508,7 +24508,7 @@
       </c>
       <c r="C360" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D360" s="2" t="inlineStr">
@@ -24776,7 +24776,7 @@
       </c>
       <c r="C364" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D364" s="2" t="inlineStr">
@@ -27255,7 +27255,7 @@
       </c>
       <c r="C401" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D401" s="2" t="inlineStr">
@@ -28193,7 +28193,7 @@
       </c>
       <c r="C415" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D415" s="2" t="inlineStr">
@@ -30136,7 +30136,7 @@
       </c>
       <c r="C444" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D444" s="2" t="inlineStr">
@@ -34424,7 +34424,7 @@
       </c>
       <c r="C508" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D508" s="2" t="inlineStr">
@@ -34491,7 +34491,7 @@
       </c>
       <c r="C509" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D509" s="2" t="inlineStr">
@@ -39248,7 +39248,7 @@
       </c>
       <c r="C580" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D580" s="2" t="inlineStr">
@@ -39315,7 +39315,7 @@
       </c>
       <c r="C581" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D581" s="2" t="inlineStr">
@@ -41593,7 +41593,7 @@
       </c>
       <c r="C615" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D615" s="2" t="inlineStr">
@@ -44407,7 +44407,7 @@
       </c>
       <c r="C657" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D657" s="2" t="inlineStr">
@@ -50638,7 +50638,7 @@
       </c>
       <c r="C750" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D750" s="2" t="inlineStr">
@@ -51040,7 +51040,7 @@
       </c>
       <c r="C756" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D756" s="2" t="inlineStr">
@@ -51174,7 +51174,7 @@
       </c>
       <c r="C758" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D758" s="2" t="inlineStr">
@@ -53184,7 +53184,7 @@
       </c>
       <c r="C788" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D788" s="2" t="inlineStr">
@@ -54256,7 +54256,7 @@
       </c>
       <c r="C804" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D804" s="2" t="inlineStr">
@@ -55797,7 +55797,7 @@
       </c>
       <c r="C827" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D827" s="2" t="inlineStr">
@@ -57405,7 +57405,7 @@
       </c>
       <c r="C851" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D851" s="2" t="inlineStr">
@@ -57472,7 +57472,7 @@
       </c>
       <c r="C852" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D852" s="2" t="inlineStr">
@@ -58879,7 +58879,7 @@
       </c>
       <c r="C873" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D873" s="2" t="inlineStr">
@@ -59080,7 +59080,7 @@
       </c>
       <c r="C876" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D876" s="2" t="inlineStr">
@@ -63100,7 +63100,7 @@
       </c>
       <c r="C936" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D936" s="2" t="inlineStr">
@@ -63636,7 +63636,7 @@
       </c>
       <c r="C944" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D944" s="2" t="inlineStr">
@@ -66048,7 +66048,7 @@
       </c>
       <c r="C980" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D980" s="2" t="inlineStr">
@@ -66182,7 +66182,7 @@
       </c>
       <c r="C982" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D982" s="2" t="inlineStr">
@@ -66919,7 +66919,7 @@
       </c>
       <c r="C993" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D993" s="2" t="inlineStr">
@@ -67187,7 +67187,7 @@
       </c>
       <c r="C997" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D997" s="2" t="inlineStr">
@@ -67656,7 +67656,7 @@
       </c>
       <c r="C1004" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D1004" s="2" t="inlineStr">
@@ -68393,7 +68393,7 @@
       </c>
       <c r="C1015" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D1015" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-09 22:45:47
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixas_42l.xlsx
+++ b/relatorio_analitico_caixas_42l.xlsx
@@ -991,7 +991,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -4542,7 +4542,7 @@
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
@@ -6753,7 +6753,7 @@
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
@@ -7021,7 +7021,7 @@
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
@@ -8227,7 +8227,7 @@
       </c>
       <c r="C117" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D117" s="2" t="inlineStr">
@@ -16066,7 +16066,7 @@
       </c>
       <c r="C234" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D234" s="2" t="inlineStr">
@@ -16937,7 +16937,7 @@
       </c>
       <c r="C247" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D247" s="2" t="inlineStr">
@@ -17004,7 +17004,7 @@
       </c>
       <c r="C248" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D248" s="2" t="inlineStr">
@@ -17674,7 +17674,7 @@
       </c>
       <c r="C258" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D258" s="2" t="inlineStr">
@@ -20287,7 +20287,7 @@
       </c>
       <c r="C297" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D297" s="2" t="inlineStr">
@@ -21627,7 +21627,7 @@
       </c>
       <c r="C317" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D317" s="2" t="inlineStr">
@@ -24776,7 +24776,7 @@
       </c>
       <c r="C364" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D364" s="2" t="inlineStr">
@@ -27523,7 +27523,7 @@
       </c>
       <c r="C405" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D405" s="2" t="inlineStr">
@@ -34290,7 +34290,7 @@
       </c>
       <c r="C506" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D506" s="2" t="inlineStr">
@@ -34357,7 +34357,7 @@
       </c>
       <c r="C507" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D507" s="2" t="inlineStr">
@@ -34491,7 +34491,7 @@
       </c>
       <c r="C509" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D509" s="2" t="inlineStr">
@@ -36903,7 +36903,7 @@
       </c>
       <c r="C545" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D545" s="2" t="inlineStr">
@@ -44407,7 +44407,7 @@
       </c>
       <c r="C657" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D657" s="2" t="inlineStr">
@@ -50035,7 +50035,7 @@
       </c>
       <c r="C741" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D741" s="2" t="inlineStr">
@@ -50638,7 +50638,7 @@
       </c>
       <c r="C750" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D750" s="2" t="inlineStr">
@@ -51040,7 +51040,7 @@
       </c>
       <c r="C756" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D756" s="2" t="inlineStr">
@@ -51241,7 +51241,7 @@
       </c>
       <c r="C759" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D759" s="2" t="inlineStr">
@@ -53184,7 +53184,7 @@
       </c>
       <c r="C788" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D788" s="2" t="inlineStr">
@@ -54256,7 +54256,7 @@
       </c>
       <c r="C804" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D804" s="2" t="inlineStr">
@@ -54323,7 +54323,7 @@
       </c>
       <c r="C805" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D805" s="2" t="inlineStr">
@@ -54524,7 +54524,7 @@
       </c>
       <c r="C808" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D808" s="2" t="inlineStr">
@@ -55797,7 +55797,7 @@
       </c>
       <c r="C827" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D827" s="2" t="inlineStr">
@@ -57405,7 +57405,7 @@
       </c>
       <c r="C851" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D851" s="2" t="inlineStr">
@@ -58343,7 +58343,7 @@
       </c>
       <c r="C865" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D865" s="2" t="inlineStr">
@@ -63234,7 +63234,7 @@
       </c>
       <c r="C938" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D938" s="2" t="inlineStr">
@@ -63636,7 +63636,7 @@
       </c>
       <c r="C944" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D944" s="2" t="inlineStr">
@@ -63770,7 +63770,7 @@
       </c>
       <c r="C946" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D946" s="2" t="inlineStr">
@@ -63904,7 +63904,7 @@
       </c>
       <c r="C948" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D948" s="2" t="inlineStr">
@@ -64105,7 +64105,7 @@
       </c>
       <c r="C951" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D951" s="2" t="inlineStr">
@@ -65512,7 +65512,7 @@
       </c>
       <c r="C972" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D972" s="2" t="inlineStr">
@@ -66048,7 +66048,7 @@
       </c>
       <c r="C980" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D980" s="2" t="inlineStr">
@@ -66919,7 +66919,7 @@
       </c>
       <c r="C993" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D993" s="2" t="inlineStr">
@@ -68393,7 +68393,7 @@
       </c>
       <c r="C1015" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D1015" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-09 22:55:39
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixas_42l.xlsx
+++ b/relatorio_analitico_caixas_42l.xlsx
@@ -4542,7 +4542,7 @@
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
@@ -7021,7 +7021,7 @@
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
@@ -8227,7 +8227,7 @@
       </c>
       <c r="C117" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D117" s="2" t="inlineStr">
@@ -17004,7 +17004,7 @@
       </c>
       <c r="C248" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D248" s="2" t="inlineStr">
@@ -20019,7 +20019,7 @@
       </c>
       <c r="C293" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D293" s="2" t="inlineStr">
@@ -21627,7 +21627,7 @@
       </c>
       <c r="C317" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D317" s="2" t="inlineStr">
@@ -24508,7 +24508,7 @@
       </c>
       <c r="C360" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D360" s="2" t="inlineStr">
@@ -27121,7 +27121,7 @@
       </c>
       <c r="C399" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D399" s="2" t="inlineStr">
@@ -27523,7 +27523,7 @@
       </c>
       <c r="C405" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D405" s="2" t="inlineStr">
@@ -28193,7 +28193,7 @@
       </c>
       <c r="C415" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D415" s="2" t="inlineStr">
@@ -34357,7 +34357,7 @@
       </c>
       <c r="C507" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D507" s="2" t="inlineStr">
@@ -34424,7 +34424,7 @@
       </c>
       <c r="C508" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D508" s="2" t="inlineStr">
@@ -34491,7 +34491,7 @@
       </c>
       <c r="C509" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D509" s="2" t="inlineStr">
@@ -36903,7 +36903,7 @@
       </c>
       <c r="C545" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D545" s="2" t="inlineStr">
@@ -50035,7 +50035,7 @@
       </c>
       <c r="C741" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D741" s="2" t="inlineStr">
@@ -50102,7 +50102,7 @@
       </c>
       <c r="C742" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D742" s="2" t="inlineStr">
@@ -50638,7 +50638,7 @@
       </c>
       <c r="C750" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D750" s="2" t="inlineStr">
@@ -51040,7 +51040,7 @@
       </c>
       <c r="C756" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D756" s="2" t="inlineStr">
@@ -51241,7 +51241,7 @@
       </c>
       <c r="C759" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D759" s="2" t="inlineStr">
@@ -53184,7 +53184,7 @@
       </c>
       <c r="C788" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D788" s="2" t="inlineStr">
@@ -54256,7 +54256,7 @@
       </c>
       <c r="C804" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D804" s="2" t="inlineStr">
@@ -54323,7 +54323,7 @@
       </c>
       <c r="C805" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D805" s="2" t="inlineStr">
@@ -55797,7 +55797,7 @@
       </c>
       <c r="C827" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D827" s="2" t="inlineStr">
@@ -57271,7 +57271,7 @@
       </c>
       <c r="C849" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D849" s="2" t="inlineStr">
@@ -57338,7 +57338,7 @@
       </c>
       <c r="C850" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D850" s="2" t="inlineStr">
@@ -63234,7 +63234,7 @@
       </c>
       <c r="C938" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D938" s="2" t="inlineStr">
@@ -63301,7 +63301,7 @@
       </c>
       <c r="C939" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D939" s="2" t="inlineStr">
@@ -63636,7 +63636,7 @@
       </c>
       <c r="C944" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D944" s="2" t="inlineStr">
@@ -65512,7 +65512,7 @@
       </c>
       <c r="C972" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D972" s="2" t="inlineStr">
@@ -66115,7 +66115,7 @@
       </c>
       <c r="C981" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D981" s="2" t="inlineStr">
@@ -66919,7 +66919,7 @@
       </c>
       <c r="C993" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D993" s="2" t="inlineStr">
@@ -67187,7 +67187,7 @@
       </c>
       <c r="C997" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D997" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-09 23:04:56
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixas_42l.xlsx
+++ b/relatorio_analitico_caixas_42l.xlsx
@@ -2197,7 +2197,7 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -7021,7 +7021,7 @@
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
@@ -7758,7 +7758,7 @@
       </c>
       <c r="C110" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D110" s="2" t="inlineStr">
@@ -8227,7 +8227,7 @@
       </c>
       <c r="C117" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D117" s="2" t="inlineStr">
@@ -15798,7 +15798,7 @@
       </c>
       <c r="C230" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D230" s="2" t="inlineStr">
@@ -16066,7 +16066,7 @@
       </c>
       <c r="C234" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D234" s="2" t="inlineStr">
@@ -16937,7 +16937,7 @@
       </c>
       <c r="C247" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D247" s="2" t="inlineStr">
@@ -20287,7 +20287,7 @@
       </c>
       <c r="C297" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D297" s="2" t="inlineStr">
@@ -24508,7 +24508,7 @@
       </c>
       <c r="C360" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D360" s="2" t="inlineStr">
@@ -27255,7 +27255,7 @@
       </c>
       <c r="C401" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D401" s="2" t="inlineStr">
@@ -27523,7 +27523,7 @@
       </c>
       <c r="C405" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D405" s="2" t="inlineStr">
@@ -33821,7 +33821,7 @@
       </c>
       <c r="C499" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D499" s="2" t="inlineStr">
@@ -34424,7 +34424,7 @@
       </c>
       <c r="C508" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D508" s="2" t="inlineStr">
@@ -34491,7 +34491,7 @@
       </c>
       <c r="C509" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D509" s="2" t="inlineStr">
@@ -41593,7 +41593,7 @@
       </c>
       <c r="C615" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D615" s="2" t="inlineStr">
@@ -50102,7 +50102,7 @@
       </c>
       <c r="C742" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D742" s="2" t="inlineStr">
@@ -50638,7 +50638,7 @@
       </c>
       <c r="C750" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D750" s="2" t="inlineStr">
@@ -51040,7 +51040,7 @@
       </c>
       <c r="C756" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D756" s="2" t="inlineStr">
@@ -53184,7 +53184,7 @@
       </c>
       <c r="C788" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D788" s="2" t="inlineStr">
@@ -54524,7 +54524,7 @@
       </c>
       <c r="C808" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D808" s="2" t="inlineStr">
@@ -55797,7 +55797,7 @@
       </c>
       <c r="C827" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D827" s="2" t="inlineStr">
@@ -57338,7 +57338,7 @@
       </c>
       <c r="C850" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D850" s="2" t="inlineStr">
@@ -57405,7 +57405,7 @@
       </c>
       <c r="C851" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D851" s="2" t="inlineStr">
@@ -58343,7 +58343,7 @@
       </c>
       <c r="C865" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D865" s="2" t="inlineStr">
@@ -63301,7 +63301,7 @@
       </c>
       <c r="C939" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D939" s="2" t="inlineStr">
@@ -63636,7 +63636,7 @@
       </c>
       <c r="C944" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D944" s="2" t="inlineStr">
@@ -63770,7 +63770,7 @@
       </c>
       <c r="C946" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D946" s="2" t="inlineStr">
@@ -63904,7 +63904,7 @@
       </c>
       <c r="C948" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D948" s="2" t="inlineStr">
@@ -64105,7 +64105,7 @@
       </c>
       <c r="C951" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D951" s="2" t="inlineStr">
@@ -65512,7 +65512,7 @@
       </c>
       <c r="C972" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D972" s="2" t="inlineStr">
@@ -65579,7 +65579,7 @@
       </c>
       <c r="C973" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D973" s="2" t="inlineStr">
@@ -66048,7 +66048,7 @@
       </c>
       <c r="C980" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D980" s="2" t="inlineStr">
@@ -66115,7 +66115,7 @@
       </c>
       <c r="C981" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D981" s="2" t="inlineStr">
@@ -67656,7 +67656,7 @@
       </c>
       <c r="C1004" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D1004" s="2" t="inlineStr">
@@ -68393,7 +68393,7 @@
       </c>
       <c r="C1015" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D1015" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-09 23:25:00
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixas_42l.xlsx
+++ b/relatorio_analitico_caixas_42l.xlsx
@@ -991,7 +991,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -2197,7 +2197,7 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -4542,7 +4542,7 @@
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
@@ -6753,7 +6753,7 @@
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
@@ -7758,7 +7758,7 @@
       </c>
       <c r="C110" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D110" s="2" t="inlineStr">
@@ -16066,7 +16066,7 @@
       </c>
       <c r="C234" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D234" s="2" t="inlineStr">
@@ -18210,7 +18210,7 @@
       </c>
       <c r="C266" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D266" s="2" t="inlineStr">
@@ -19349,7 +19349,7 @@
       </c>
       <c r="C283" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D283" s="2" t="inlineStr">
@@ -20019,7 +20019,7 @@
       </c>
       <c r="C293" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D293" s="2" t="inlineStr">
@@ -20153,7 +20153,7 @@
       </c>
       <c r="C295" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D295" s="2" t="inlineStr">
@@ -24508,7 +24508,7 @@
       </c>
       <c r="C360" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D360" s="2" t="inlineStr">
@@ -27255,7 +27255,7 @@
       </c>
       <c r="C401" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D401" s="2" t="inlineStr">
@@ -28193,7 +28193,7 @@
       </c>
       <c r="C415" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D415" s="2" t="inlineStr">
@@ -33821,7 +33821,7 @@
       </c>
       <c r="C499" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D499" s="2" t="inlineStr">
@@ -34424,7 +34424,7 @@
       </c>
       <c r="C508" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D508" s="2" t="inlineStr">
@@ -34491,7 +34491,7 @@
       </c>
       <c r="C509" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D509" s="2" t="inlineStr">
@@ -39248,7 +39248,7 @@
       </c>
       <c r="C580" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D580" s="2" t="inlineStr">
@@ -41593,7 +41593,7 @@
       </c>
       <c r="C615" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D615" s="2" t="inlineStr">
@@ -44407,7 +44407,7 @@
       </c>
       <c r="C657" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D657" s="2" t="inlineStr">
@@ -47020,7 +47020,7 @@
       </c>
       <c r="C696" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D696" s="2" t="inlineStr">
@@ -50035,7 +50035,7 @@
       </c>
       <c r="C741" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D741" s="2" t="inlineStr">
@@ -50102,7 +50102,7 @@
       </c>
       <c r="C742" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D742" s="2" t="inlineStr">
@@ -50638,7 +50638,7 @@
       </c>
       <c r="C750" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D750" s="2" t="inlineStr">
@@ -51040,7 +51040,7 @@
       </c>
       <c r="C756" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D756" s="2" t="inlineStr">
@@ -51241,7 +51241,7 @@
       </c>
       <c r="C759" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D759" s="2" t="inlineStr">
@@ -53184,7 +53184,7 @@
       </c>
       <c r="C788" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D788" s="2" t="inlineStr">
@@ -54323,7 +54323,7 @@
       </c>
       <c r="C805" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D805" s="2" t="inlineStr">
@@ -57338,7 +57338,7 @@
       </c>
       <c r="C850" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D850" s="2" t="inlineStr">
@@ -57405,7 +57405,7 @@
       </c>
       <c r="C851" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D851" s="2" t="inlineStr">
@@ -58879,7 +58879,7 @@
       </c>
       <c r="C873" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D873" s="2" t="inlineStr">
@@ -59080,7 +59080,7 @@
       </c>
       <c r="C876" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D876" s="2" t="inlineStr">
@@ -63100,7 +63100,7 @@
       </c>
       <c r="C936" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D936" s="2" t="inlineStr">
@@ -63234,7 +63234,7 @@
       </c>
       <c r="C938" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D938" s="2" t="inlineStr">
@@ -63301,7 +63301,7 @@
       </c>
       <c r="C939" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D939" s="2" t="inlineStr">
@@ -64105,7 +64105,7 @@
       </c>
       <c r="C951" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D951" s="2" t="inlineStr">
@@ -65512,7 +65512,7 @@
       </c>
       <c r="C972" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D972" s="2" t="inlineStr">
@@ -65579,7 +65579,7 @@
       </c>
       <c r="C973" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D973" s="2" t="inlineStr">
@@ -66919,7 +66919,7 @@
       </c>
       <c r="C993" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D993" s="2" t="inlineStr">
@@ -68393,7 +68393,7 @@
       </c>
       <c r="C1015" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D1015" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-09 23:37:46
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixas_42l.xlsx
+++ b/relatorio_analitico_caixas_42l.xlsx
@@ -991,7 +991,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -1929,7 +1929,7 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -2130,7 +2130,7 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -4542,7 +4542,7 @@
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
@@ -7758,7 +7758,7 @@
       </c>
       <c r="C110" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D110" s="2" t="inlineStr">
@@ -16066,7 +16066,7 @@
       </c>
       <c r="C234" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D234" s="2" t="inlineStr">
@@ -17674,7 +17674,7 @@
       </c>
       <c r="C258" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D258" s="2" t="inlineStr">
@@ -27255,7 +27255,7 @@
       </c>
       <c r="C401" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D401" s="2" t="inlineStr">
@@ -28193,7 +28193,7 @@
       </c>
       <c r="C415" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D415" s="2" t="inlineStr">
@@ -34156,7 +34156,7 @@
       </c>
       <c r="C504" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D504" s="2" t="inlineStr">
@@ -34357,7 +34357,7 @@
       </c>
       <c r="C507" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D507" s="2" t="inlineStr">
@@ -34424,7 +34424,7 @@
       </c>
       <c r="C508" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D508" s="2" t="inlineStr">
@@ -36903,7 +36903,7 @@
       </c>
       <c r="C545" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D545" s="2" t="inlineStr">
@@ -39248,7 +39248,7 @@
       </c>
       <c r="C580" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D580" s="2" t="inlineStr">
@@ -39315,7 +39315,7 @@
       </c>
       <c r="C581" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D581" s="2" t="inlineStr">
@@ -41593,7 +41593,7 @@
       </c>
       <c r="C615" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D615" s="2" t="inlineStr">
@@ -47020,7 +47020,7 @@
       </c>
       <c r="C696" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D696" s="2" t="inlineStr">
@@ -51040,7 +51040,7 @@
       </c>
       <c r="C756" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D756" s="2" t="inlineStr">
@@ -53184,7 +53184,7 @@
       </c>
       <c r="C788" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D788" s="2" t="inlineStr">
@@ -57338,7 +57338,7 @@
       </c>
       <c r="C850" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D850" s="2" t="inlineStr">
@@ -57405,7 +57405,7 @@
       </c>
       <c r="C851" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D851" s="2" t="inlineStr">
@@ -58879,7 +58879,7 @@
       </c>
       <c r="C873" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D873" s="2" t="inlineStr">
@@ -63100,7 +63100,7 @@
       </c>
       <c r="C936" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D936" s="2" t="inlineStr">
@@ -63636,7 +63636,7 @@
       </c>
       <c r="C944" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D944" s="2" t="inlineStr">
@@ -63770,7 +63770,7 @@
       </c>
       <c r="C946" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D946" s="2" t="inlineStr">
@@ -64105,7 +64105,7 @@
       </c>
       <c r="C951" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D951" s="2" t="inlineStr">
@@ -65512,7 +65512,7 @@
       </c>
       <c r="C972" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D972" s="2" t="inlineStr">
@@ -66048,7 +66048,7 @@
       </c>
       <c r="C980" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D980" s="2" t="inlineStr">
@@ -66115,7 +66115,7 @@
       </c>
       <c r="C981" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D981" s="2" t="inlineStr">
@@ -66919,7 +66919,7 @@
       </c>
       <c r="C993" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D993" s="2" t="inlineStr">
@@ -67187,7 +67187,7 @@
       </c>
       <c r="C997" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D997" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-09-09 23:44:56
</commit_message>
<xml_diff>
--- a/relatorio_analitico_caixas_42l.xlsx
+++ b/relatorio_analitico_caixas_42l.xlsx
@@ -991,7 +991,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -2197,7 +2197,7 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -4542,7 +4542,7 @@
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
@@ -6753,7 +6753,7 @@
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
@@ -7021,7 +7021,7 @@
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
@@ -7758,7 +7758,7 @@
       </c>
       <c r="C110" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D110" s="2" t="inlineStr">
@@ -17004,7 +17004,7 @@
       </c>
       <c r="C248" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D248" s="2" t="inlineStr">
@@ -18210,7 +18210,7 @@
       </c>
       <c r="C266" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D266" s="2" t="inlineStr">
@@ -20019,7 +20019,7 @@
       </c>
       <c r="C293" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D293" s="2" t="inlineStr">
@@ -20287,7 +20287,7 @@
       </c>
       <c r="C297" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D297" s="2" t="inlineStr">
@@ -22096,7 +22096,7 @@
       </c>
       <c r="C324" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D324" s="2" t="inlineStr">
@@ -27255,7 +27255,7 @@
       </c>
       <c r="C401" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D401" s="2" t="inlineStr">
@@ -27322,7 +27322,7 @@
       </c>
       <c r="C402" s="2" t="inlineStr">
         <is>
-          <t>2 C a 8 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D402" s="2" t="inlineStr">
@@ -27523,7 +27523,7 @@
       </c>
       <c r="C405" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D405" s="2" t="inlineStr">
@@ -33754,7 +33754,7 @@
       </c>
       <c r="C498" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D498" s="2" t="inlineStr">
@@ -33821,7 +33821,7 @@
       </c>
       <c r="C499" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D499" s="2" t="inlineStr">
@@ -34156,7 +34156,7 @@
       </c>
       <c r="C504" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D504" s="2" t="inlineStr">
@@ -34290,7 +34290,7 @@
       </c>
       <c r="C506" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D506" s="2" t="inlineStr">
@@ -34357,7 +34357,7 @@
       </c>
       <c r="C507" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D507" s="2" t="inlineStr">
@@ -34491,7 +34491,7 @@
       </c>
       <c r="C509" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D509" s="2" t="inlineStr">
@@ -36903,7 +36903,7 @@
       </c>
       <c r="C545" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D545" s="2" t="inlineStr">
@@ -39248,7 +39248,7 @@
       </c>
       <c r="C580" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D580" s="2" t="inlineStr">
@@ -44407,7 +44407,7 @@
       </c>
       <c r="C657" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-15 C a -30 C</t>
         </is>
       </c>
       <c r="D657" s="2" t="inlineStr">
@@ -47020,7 +47020,7 @@
       </c>
       <c r="C696" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D696" s="2" t="inlineStr">
@@ -50035,7 +50035,7 @@
       </c>
       <c r="C741" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D741" s="2" t="inlineStr">
@@ -50638,7 +50638,7 @@
       </c>
       <c r="C750" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D750" s="2" t="inlineStr">
@@ -51174,7 +51174,7 @@
       </c>
       <c r="C758" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D758" s="2" t="inlineStr">
@@ -53184,7 +53184,7 @@
       </c>
       <c r="C788" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D788" s="2" t="inlineStr">
@@ -54256,7 +54256,7 @@
       </c>
       <c r="C804" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D804" s="2" t="inlineStr">
@@ -54323,7 +54323,7 @@
       </c>
       <c r="C805" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D805" s="2" t="inlineStr">
@@ -54390,7 +54390,7 @@
       </c>
       <c r="C806" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D806" s="2" t="inlineStr">
@@ -54457,7 +54457,7 @@
       </c>
       <c r="C807" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-25 C a -15 C</t>
         </is>
       </c>
       <c r="D807" s="2" t="inlineStr">
@@ -57271,7 +57271,7 @@
       </c>
       <c r="C849" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D849" s="2" t="inlineStr">
@@ -59080,7 +59080,7 @@
       </c>
       <c r="C876" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D876" s="2" t="inlineStr">
@@ -63234,7 +63234,7 @@
       </c>
       <c r="C938" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D938" s="2" t="inlineStr">
@@ -63301,7 +63301,7 @@
       </c>
       <c r="C939" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D939" s="2" t="inlineStr">
@@ -63636,7 +63636,7 @@
       </c>
       <c r="C944" s="2" t="inlineStr">
         <is>
-          <t>-15 C a -30 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D944" s="2" t="inlineStr">
@@ -65512,7 +65512,7 @@
       </c>
       <c r="C972" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D972" s="2" t="inlineStr">
@@ -65579,7 +65579,7 @@
       </c>
       <c r="C973" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D973" s="2" t="inlineStr">
@@ -67187,7 +67187,7 @@
       </c>
       <c r="C997" s="2" t="inlineStr">
         <is>
-          <t>-25 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D997" s="2" t="inlineStr">
@@ -67656,7 +67656,7 @@
       </c>
       <c r="C1004" s="2" t="inlineStr">
         <is>
-          <t>-30 C a -15 C</t>
+          <t>-35 C a -15 C</t>
         </is>
       </c>
       <c r="D1004" s="2" t="inlineStr">
@@ -68393,7 +68393,7 @@
       </c>
       <c r="C1015" s="2" t="inlineStr">
         <is>
-          <t>-35 C a -15 C</t>
+          <t>-30 C a -15 C</t>
         </is>
       </c>
       <c r="D1015" s="2" t="inlineStr">

</xml_diff>